<commit_message>
Update competition data 2026-08-17
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2 weeks ago - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
+          <t>Sep 4, 2025 · 3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -464,22 +464,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.poidata.io/report/engineer/south-africa</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -492,17 +496,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Two South Africans on the shortlist for the 2026 Africa Prize for Engineering Innovation</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/two-south-africans-on-the-shortlist-for-the-2026-africa-prize-for-engineering-innovation-2026-08-04</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2 weeks ago - Two South African innovators have been shortlisted for the UK Royal Academy of Engineering’s Africa Prize for Engineering Innovation 2026. This is the continent’s richest award aimed at promoting engineering innovation and entrepreneurship ...</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -512,24 +516,24 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>newsletters@creamermedia.co.za, advertising@creamermedia.co.za, newsdesk@engineeringnews.co.za, subscriptions@creamermedia.co.za, chanel@engineeringnews.co.za</t>
+          <t>info@ieomsociety.org</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3 days ago - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -537,22 +541,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>VUT inspires future engineers through Bridge Building Competition – Vaal University of Technology</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://vut.ac.za/vut-inspires-future-engineers-through-bridge-building-competition/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3 weeks ago - “VUT Ekhaya Alumni and SAICE STAR Vaal hosted the 2026 Bridge Building Competition, inspiring 16 Vaal schools through practical engineering, creativity and STEM education.”</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa. Find out more</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -565,17 +573,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>South Africa · South Korea · Spain · Sri Lanka · Sudan · Sweden · Switzerland · Syrian Arab Republic · Taiwan · Tajikistan · Tanzania · Thailand · Togo · Trinidad and Tobago · Tunisia · Turkey · Uganda · Ukraine · United Arab Emirates · United Kingdom ·</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -588,17 +596,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Engineering Conferences in South Africa 2025-2026</t>
+          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
+          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
+          <t>2 weeks ago - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -611,17 +619,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -629,26 +637,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
+          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.thecasecentre.org/products/view?id=189255</t>
+          <t>https://www.poidata.io/report/engineer/south-africa</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
+          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -661,17 +665,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Two South Africans on the shortlist for the 2026 Africa Prize for Engineering Innovation</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.engineeringnews.co.za/article/two-south-africans-on-the-shortlist-for-the-2026-africa-prize-for-engineering-innovation-2026-08-04</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>2 weeks ago - Two South African innovators have been shortlisted for the UK Royal Academy of Engineering’s Africa Prize for Engineering Innovation 2026. This is the continent’s richest award aimed at promoting engineering innovation and entrepreneurship ...</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -679,22 +683,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>newsletters@creamermedia.co.za, newsdesk@engineeringnews.co.za, chanel@engineeringnews.co.za, subscriptions@creamermedia.co.za, advertising@creamermedia.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>South Africa International Industrial Expo | Innovation Bridge</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show ...</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
+          <t>AI Expo Africa 2026 – Join the Largest AI Event &amp; Trade Community in Africa TODAY! Our business audience is a buyer / supplier focused community and comprised of Enterprise decision makers / CxOs, allied to AI Cloud platform providers, Tier 1 / 2 deployment &amp; service providers, AI start ups / innovators, investors, educators, government and AI ecosystem community builders.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -702,22 +710,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>enquiries@aiexpoafrica.com</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Two landmark exhibitions set to transform industrial technology and renewable energy in South Africa</t>
+          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/two-landmark-exhibitions-set-to-transform-industrial-technology-and-renewable-energy-in-south-africa-2025-10-24</t>
+          <t>https://10times.com/southafrica/tradeshows</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>October 24, 2025 - South Africa’s industrial and clean energy sectors celebrated a landmark moment today with the official launch of RE+ South Africa 2026 and the Cape Industrial Technology Exhibition (CITE) 2027.</t>
+          <t>South Africa trade shows, find and compare 964 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 174 upcoming expos in 2026-2027 1. South Africa Infrastructure &amp; Water Expo, 2.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -725,26 +737,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>newsletters@creamermedia.co.za, advertising@creamermedia.co.za, newsdesk@engineeringnews.co.za, subscriptions@creamermedia.co.za, chanel@engineeringnews.co.za</t>
-        </is>
-      </c>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>KZN Industrial Technology Exhibition</t>
+          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://www.kznindustrial.co.za/</t>
+          <t>https://manufacturingindaba.co.za/exhibition/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
+          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -754,24 +762,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>john@email.com</t>
+          <t>lene@hotdesigns.co.za</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
+          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://madeinafricaevent.co.za/</t>
+          <t>https://innovationweek.co.za/</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
+          <t>SA Innovation Week 2026 is South Africa’s official national innovation platform accelerating implementation, commercialisation and impact.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -779,22 +787,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>info@pixal8media.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Trade Shows Worldwide - South Africa - 2026/2027</t>
+          <t>IT &amp; Technology Events in South Africa, List of all South ...</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://www.eventseye.com/fairs/c1_trade-shows_south-africa.html</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>South Africa Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in South Africa</t>
+          <t>18 hours ago · Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -807,17 +819,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Exhibition | Innovation Festival Durban | South Africa</t>
+          <t>South Africa International Industrial Expo | Innovation Bridge</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://www.innovationfestival.durban/exhibition</t>
+          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities.</t>
+          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -825,26 +837,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>sithabile@innovate.durban, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, Erika@innovate.durban, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Discover Innovation Hub's Pavilion at Organic &amp; Natural Products Expo - Organic &amp; Natural Products Portal</t>
+          <t>Two landmark exhibitions set to transform industrial technology and renewable energy in South Africa</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://www.organicandnaturalportal.com/innovation-hub-organic-expo/</t>
+          <t>https://www.engineeringnews.co.za/article/two-landmark-exhibitions-set-to-transform-industrial-technology-and-renewable-energy-in-south-africa-2025-10-24</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2 weeks ago - Gathering producers, retailers, buyers, and conscious consumers under one roof, the expo serves as Africa’s premier showcase for sustainability, health, and wellness innovation. A standout highlight of this year’s exhibition is The Innovation Hub Pavilion, hosting a curated line-up of forward-thinking South African small, medium, and micro-enterprises (SMMEs).</t>
+          <t>October 24, 2025 - South Africa’s industrial and clean energy sectors celebrated a landmark moment today with the official launch of RE+ South Africa 2026 and the Cape Industrial Technology Exhibition (CITE) 2027.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -852,22 +860,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>newsletters@creamermedia.co.za, newsdesk@engineeringnews.co.za, chanel@engineeringnews.co.za, subscriptions@creamermedia.co.za, advertising@creamermedia.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
+          <t>KZN Industrial Technology Exhibition</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://manufacturingindaba.co.za/exhibition/</t>
+          <t>https://www.kznindustrial.co.za/</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
+          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -875,22 +887,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>john@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>International Science, Innovation &amp; Technology Expo (INSITE)</t>
+          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://www.dsti.gov.za/index.php/resource-center/27-temp/dst-links/3-international-science-innovation-a-technology-expo</t>
+          <t>https://madeinafricaevent.co.za/</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>The essence of INSITE INSITE is an international, biennial must-see Science and Technology event in South Africa, the only one of its kind in Africa that creates new frontiers for global challenges · INSITE aims to assemble the worlds leading innovators and scientists in one place, stimulating ...</t>
+          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -903,17 +919,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AAXO - The Association of African Exhibition Organisers</t>
+          <t>Trade Shows Worldwide - South Africa - 2026/2027</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.aaxo.co.za/</t>
+          <t>https://www.eventseye.com/fairs/c1_trade-shows_south-africa.html</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>February 20, 2026 - CAPE TOWN, South Africa – The inaugural Festival of Eventing (FOE) brought together 350 event professionals, 85 speakers, and 10 countries under one roof for a two-day showcase of innovation, inspiration, and industry connection.</t>
+          <t>South Africa Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in South Africa</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -926,17 +942,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
+          <t>In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community’s challenges and how community members view the impact of these challenges on their daily lives.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -944,22 +960,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
+          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -967,26 +987,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
-        </is>
-      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EWB Design Challenge | Aston University</t>
+          <t>Engineering for People Design Challenge | Department of ...</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
+          <t>Aug 4, 2025 · This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but under-resourced neighbourhood on the eastern edge of Johannesburg. Home to around 46,000 people, Makers Valley is a community rich in creativity, activism ...</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -994,22 +1010,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
+          <t>Oct 16, 2024 · STEM-focused NGO Engineers Without Borders UK has launched its 2025 Engineering for People Design Challenge. Organised in conjunction with sister organisation Engineers Without Borders South Africa, as well as the Makers Valley Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1017,26 +1037,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>ied@ied.org.uk</t>
-        </is>
-      </c>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Latest Community Engineering Design Competition Announced</t>
+          <t>Engineering For People Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
+          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
+          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1044,22 +1060,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Real-world research: Engineering team designs South African trolley system; science students investigate heavy metals | University of Wisconsin - Stout</t>
+          <t>Engineering for People Design Challenge - Engineers Without ...</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
+          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>May 15, 2025 - Research ranged from heavy metals ... Borders’ international design challenge. Nearly 90 students in 23 teams addressed the EWB challenge. One group focused on engineering a safer, more accessible transportation system in South ...</t>
+          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1067,26 +1087,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>dolanm@uwstout.edu, frischj@uwstout.edu</t>
-        </is>
-      </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Engineering for people, that’s the challenge | Engineers Without Borders</t>
+          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.rs-online.com/designspark/an-introduction-to-engineering-for-people-design-challenge</t>
+          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>That’s exactly what the annual Engineering for People Design Challenge asks participants to do. The competition, delivered in partnership by Engineers without Borders South Africa and Engineers Without Borders UK, encourages engineering students and those collaborating with engineers to broaden their awareness of how their decisions change the world.</t>
+          <t>Oct 24, 2024 · The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1094,22 +1110,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>team@crowdsolve.net</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of Engineering</t>
+          <t>EWB Design Challenge | Aston University</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
+          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1122,17 +1142,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2024 25 Engineering for People Design Challenge Makers Valley - Engineering for people Design - Studocu</t>
+          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.studocu.com/en-gb/document/swansea-university/engineering-for-people-hackathon/2024-25-engineering-for-people-design-challenge-makers-valley/115269605</t>
+          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
+          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1140,22 +1160,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>ied@ied.org.uk</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Inspiring, building and shaping a future fit engineering community – EWB-I</t>
+          <t>Real-world research: Engineering team designs South African trolley system; science students investigate heavy metals | University of Wisconsin - Stout</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.ewb-international.org/home/inspiring-building-and-shaping-a-future-fit-engineering-community/</t>
+          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>February 27, 2025 - The challenge, delivered during ... career, encourages individuals to broaden their awareness of the social, environmental and economic implications of their engineering solutions. Since 2011, the Design Challenge has been delivered in Cameroon, South Africa, the UK and Ireland and the USA to over 70,000 students...</t>
+          <t>May 15, 2025 - Research ranged from heavy metals ... Borders’ international design challenge. Nearly 90 students in 23 teams addressed the EWB challenge. One group focused on engineering a safer, more accessible transportation system in South ...</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1165,24 +1189,24 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>admin@ewb-international.org</t>
+          <t>dolanm@uwstout.edu, frischj@uwstout.edu</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1190,22 +1214,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1213,22 +1241,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
+          <t>Sep 4, 2025 · 3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1236,22 +1268,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>National Student Competition | ORSSA</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://www.orssa.org.za/studentcomp</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>National Student Competitions The Operations Research Society of South Africa The home of decision intelligence The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1259,22 +1295,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, email@example.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Engineering in South Africa: 24 Best universities Ranked</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://edurank.org/engineering/za/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
+          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1287,17 +1327,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1310,17 +1350,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2210</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1333,86 +1373,98 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
+          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 ...</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
+          <t>https://techspojoburg.co.za/</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
+          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>university engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr"/>
+          <t>tech expo South Africa</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>info@techspojoburg.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2025</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7 ...</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2025</t>
+          <t>Where Business, Tech and Innovation Collide in Cape Town! TECHSPO Cape Town is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>university engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr"/>
+          <t>tech expo South Africa</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>info@techspocapetown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>Africa Tech Festival</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>university engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr"/>
+          <t>tech expo South Africa</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>customerservices@informaconnect.com, support@informaconnect.com, customerservices@knect365.com, salesenquiries@africatechfestival.com, support@knect365.com, dataprivacy@informaconnect.com, dataprivacy@knect365.com</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>IT &amp; Technology Events in South Africa | 10times</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>https://techspojoburg.co.za/</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>February 20, 2026 - TECHSPO Johannesburg 2026 is a two day technology expo taking place September 28th to 29th, 2026 at the luxurious Hyatt Regency Johannesburg, Johannesburg, South Africa. TECHSPO Johannesburg brings together developers, brands, marketers, technology ...</t>
+          <t>18 hours ago · Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1420,26 +1472,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>info@techspojoburg.co.za</t>
-        </is>
-      </c>
+      <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://10times.com/johannesburg-za/technology</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
+          <t>3 days ago · Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1447,26 +1495,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>info@techspocapetown.co.za</t>
-        </is>
-      </c>
+      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa, List of all South Africa Technology Business Expo &amp; Events</t>
+          <t>IT Indaba 2026 – Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>New York Small Business Expo (Spring)07 MayNew York , USA · AFROZUM Fair · 07-09 May · Johannesburg , South Africa · AFROZUM Fair07-09 MayJohannesburg , South Africa · Nigeria Industries &amp; Manufacturing Summit · 18-20 May · Abuja , Nigeria ...</t>
+          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what’s next before everyone else does. Only 2,500 ...</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1479,17 +1523,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
+          <t>TECHSPO Johannesburg Technology ExpoJohannesburg Technology ...</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
+          <t>https://techspojoburg.co.za/johannesburg-technology-expo/</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
+          <t>TECHSPO Johannesburg is a 2-day technology expo taking place September 28 – 29, 2026 at the luxurious NH Johannesburg Sandton Hotel, Toronto, Ontario. TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1497,135 +1541,127 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>atinfo@techspo.coor, name@example.com, u003einfo@techspo.co</t>
-        </is>
-      </c>
+      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
+          <t>Maker Faire Africa - Wikipedia</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://africatechnologyexpo.com/</t>
+          <t>https://en.wikipedia.org/wiki/Maker_Faire_Africa</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
+          <t>Maker Faire Africa, Cairo, October 2011 Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds (Nubian Cheetah). Maker Faire Africa aims to engage with on ...</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>tech expo South Africa</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>partner@africatechnologyexpo.com, johndoe@email.com, info@sparkafrica.co</t>
-        </is>
-      </c>
+          <t>maker faire South Africa</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Home - Mediatech Africa | South Africa</t>
+          <t>Maker Faire Africa — Grokipedia</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://www.mediatech.co.za/</t>
+          <t>https://grokipedia.com/page/maker_faire_africa</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
+          <t>Maker Faire Africa Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>tech expo South Africa</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>claire@mediatech.co.za, simon@mediatech.co.za</t>
-        </is>
-      </c>
+          <t>maker faire South Africa</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference - AI Expo Africa | 28 - 29 October SCC Johannesburg South Africa</t>
+          <t>Maker Faire |</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://makerfaire.com/</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>(2 Day Event) 28th-29th October 2026 Sandton Convention Centre, JHB, South Africa · AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade ...</t>
+          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>tech expo South Africa</t>
+          <t>maker faire South Africa</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>enquiries@aiexpoafrica.com</t>
+          <t>fancybox_loading@2x.gif, pr@make.co, fancybox_sprite@2x.png, chosen-sprite@2x.png</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 – Africa's biggest IT Conference and Expo</t>
+          <t>Upcoming Faires - Maker Faire</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://makerfaire.com/upcoming-faires/</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>The inaugural 2025 IT Indaba promises to bring together 3,000+ IT professionals and tech influencers who are involved in the procurement of systems, tools, platforms and services, along with user experience developers who deal with the core processes and client interfaces of the business.</t>
+          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>tech expo South Africa</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr"/>
+          <t>maker faire South Africa</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>fancybox_loading@2x.gif, pr@make.co, fancybox_sprite@2x.png, chosen-sprite@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Discover Tech Conferences Events &amp; Activities in South Africa | Eventbrite</t>
+          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
+          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Save this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South AfricaShare this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South Africa</t>
+          <t>Aug 21, 2015 · DIRECTIONS THE CAPE TOWN MAKER FAIRE The Lookout, V&amp;A Waterfront Granger Bay Boulevard, V &amp; A Waterfront, Cape Town, 8002, South Africa Get Directions Fri Aug 21, 13:00 - Sun Aug 23, 17:00 The Lookout, V&amp;A Waterfront View Map Payments are secure and encrypted</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>tech expo South Africa</t>
+          <t>maker faire South Africa</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -1633,44 +1669,44 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>HOME | MAKERS FEST</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://www.industryevents.com/events/techspo-johannesburg-2026-technology-expo-internet-mobile-adtech-martech-saas</t>
+          <t>https://www.makersfestival.co.za/</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg – Where Business, Tech and Innovation Collide in Johannesburg, South Africa. TECHSPO Johannesburg Technology Expo returns September 28-29, 2026 to the NH Johannesburg Sandton Hotel in Johannesburg, South Africa.</t>
+          <t>On 8 &amp; 9 November 2025 at The Ostrich in Cape Town, join 2,000+ visitors each day for maker demos, a curated market, and family activities. It’s Africa’s first hands-on festival for creativity and craftsmanship — and everything you make, you take home.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>tech expo South Africa</t>
+          <t>maker faire South Africa</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>your@email.com, events@techspojoburg.co.za, you@company.com, colleague@company.com, support@industryevents.com</t>
+          <t>8c4075d5481d476e945486754f783364@sentry.io, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, example@mysite.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, warren@makersfestival.co.za, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Maker Faire Africa - Wikipedia</t>
+          <t>Maker Faire groups | Meetup</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Maker_Faire_Africa</t>
+          <t>https://www.meetup.com/topics/maker-faire/za/</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>March 7, 2025 - Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds ...</t>
+          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1683,22 +1719,22 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Maker Faire - Wikipedia</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Maker_Faire</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>May 3, 2026 - Maker Faires are also held in Europe, Asia, South America and Africa.</t>
+          <t>All these Olympiads and Competitions have a positive impact on education and on educational institutions in South Africa, but there is still a need to build stronger collaboration among teachers, schools, universities and educational authorities in order to meet the challenges of STEM education in South Africa today.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>maker faire South Africa</t>
+          <t>stem competition South Africa</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -1706,45 +1742,49 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
+          <t>STEM Scholars — 2026 STEM &amp; Entrepreneurship Discovery Initiative</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
+          <t>https://stemscholars.co.za/</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
+          <t>Building South Africa's Next Generation of Innovators The STEM &amp; Entrepreneurship Discovery Initiative connects learners with a world that's often invisible from inside a classroom — and equips them with skills that last far beyond the competition.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>maker faire South Africa</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr"/>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>you@school.co.za, inforeg@justice.gov.za, marushka@stemscholars.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://makerfairecapetown.wordpress.com/about/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>maker faire South Africa</t>
+          <t>stem competition South Africa</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
@@ -1752,49 +1792,49 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
+          <t>High School STEM Competition | Capetown 2026</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>http://capetown.makerfaire.com/</t>
+          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>May 29, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
+          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the ‘first author’. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>maker faire South Africa</t>
+          <t>stem competition South Africa</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>pr@make.co, fancybox_loading@2x.gif, chosen-sprite@2x.png, fancybox_sprite@2x.png</t>
+          <t>info@ieomsociety.org</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Blog : Maker Faire Africa</t>
+          <t>ASTEMI SA</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>http://makerfaireafrica.com/blog/</t>
+          <t>https://www.astemi.co.za/</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>December 31, 2021 - You can help them out on the new South African crowdfunding site, ThundaFund. ... One of the most ambitions items at Maker Faire Africa this year in Johannesburg, South Africa is Samuel Ngobeni’s “art car”. He’s a designer from Germinston, who has spent the last three years building his ANIMAL car, from the ground up, that means the frame and all.</t>
+          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>maker faire South Africa</t>
+          <t>stem competition South Africa</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
@@ -1802,22 +1842,22 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
+          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://contemporaryand.com/fr/events/maker-faire-africa-comes-to-johannesburg</t>
+          <t>https://www.samsung.com/za/solvefortomorrow/</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
+          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>maker faire South Africa</t>
+          <t>stem competition South Africa</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
@@ -1825,195 +1865,211 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Jo’Burg – AfriGadget</t>
+          <t>Applications for 2026 Samsung Solve For Tomorrow Now Open!</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://www.afrigadget.com/2014/07/08/maker-faire-africa-comes-to-joburg/</t>
+          <t>https://news.samsung.com/za/applications-for-2026-samsung-solve-for-tomorrow-now-open</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Maker Faire Africa 2014 will bring together over 5,000 attendees, along with featured inventors, world-class makers, self-made entrepreneurs &amp; workshop experts from South Africa, across the continent, and around the world, to manufacture real solutions for some of Africa’s most pressing ...</t>
+          <t>Feb 23, 2026 · The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges – with entries open until 06 March 2026. This is a transformative ...</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>maker faire South Africa</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr"/>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>ssapr.newsroom@samsung.com, ssasft@samsung.com</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Why Africa needs Maker Faire | ZDNET</t>
+          <t>Robotics Competition | WRO South Africa | Gauteng</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://www.zdnet.com/article/why-africa-needs-maker-faire/</t>
+          <t>https://www.wrosa.co.za/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>July 24, 2014 - Unlike other Maker Faires, Okafor said that it's not enough to simply hold the event in an African city and see who turns up. Two volunteers are currently working in South Africa to discover inventors in rural areas and neighbouring countries such as Zambia and Botswana who they can encourage to attend and show off their work.</t>
+          <t>WRO South Africa ( World Robot Olympiad ) is a robotics competition which brings together young people from all over the world to develop their creativity and problem-solving skills.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>maker faire South Africa</t>
+          <t>robotics competition South Africa</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>brand_licensing@ziffdavis.com</t>
+          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>South Africa Archivi - Maker Faire Rome</t>
+          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://2019.makerfairerome.eu/en/tag/south-africa/</t>
+          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>... It is the most important event in the world of innovation. Is a showcase of invention, creativity, and resourcefulness. Maker Faire gathers together tech enthusiasts, crafters, educators, tinkerers, schools, universities, research institutes, artists, students, and corporations.</t>
+          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in the leading UN-based global robotics competition, focusing on the critical area of agriculture and food security.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>maker faire South Africa</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr"/>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, info@thecortexhub.africa, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>StemCo - StemCo 2026 International Competitions</t>
+          <t>Robotics for Good Youth Challenge South Africa</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>https://stemco.org/</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>June 10, 2026 - BEST YOURSELF WITH STEMCO! Platform for the world’s brightest. ... Thanks to the participating 25 countries in 2019. Singapore, Albania, Australia, Azerbaijan, Canada, Germany, India, Indonesia, Japan, Jordan, Kazakhstan, Kyrgyzstan, Malawi, Mongolia, Nigeria, Myanmar, South Africa, Tajikistan, Turkey, Turkmenistan, Ukraine, The United States, Uzbekistan, Vietnam</t>
+          <t>Oct 31, 2025 · The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge, organized by ITU and The Cortex Hub, in partnership with Google.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
+          <t>robotics competition South Africa</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>awaisnaeem786@gmail.com, havtt@fermat.edu.vn, t.azizakhon@gmail.com, bestyourself@stemco.org, name@example.com, example@mail.com, education@missmaneducation.com, altasismail@gmail.com, info.iksc@kangaroo.org.pk, stemcomongolia@gmail.com, hkoffice@missmaneducation.com, info@missmaneducation.com</t>
+          <t>name@example.com</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Southafrica 2024</t>
+          <t>Robotics for Good Youth Challenge South Africa</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa/</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, ...</t>
+          <t>Apr 25, 2025 · The Robotics for Good Youth Challenge South Africa is a national event in a global robotics competition on disaster response, leading to the AI for Good Summit 2025.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
+          <t>robotics competition South Africa</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>info@ieomsociety.org</t>
+          <t>name@example.com</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Samsung opens Solve for Tomorrow 2026 STEM competition to all South African public schools</t>
+          <t>Competition &amp; Judge Registration | WROSA</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
+          <t>https://www.wrosa.co.za/teamregistration</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>February 27, 2026 - Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
+          <t>World Robot Olympiad South Africa Team Registration 2026 Physical Events - Team Registration Team Registrations are now open! Register your teams by clicking on the button below. Team registrations will close at 12:00 on the 1st of June. No Late Registrations will be accepted. Registrations Have Closed</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr"/>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Roboticon 2026: South Africa Showcases Robotics for Culture ...</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.ubuntutimes.co.za/roboticon-2026-south-africa-showcases-robotics-for-culture-education-and-innovation/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Local, regional and national competitions with thousands of · Multi-level events of two or more rounds that become increasingly challenging and culminate in top-level Olympiads. Enrichment programmes to inspire promising young South Africans to pursue STEMI</t>
+          <t>Jul 2, 2026 · The event, partnered with the World Robotics Olympiad, positions South Africa as a leader in educational robotics and entrepreneurial innovation.” South Africa’s robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr"/>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>adverts@ubuntutimes.co.za, newspaper-rec300@2x.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions 2022 – SAASTA</t>
+          <t>Home | Roboticon 2026</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://saasta.ac.za/astemi-competitions-2</t>
+          <t>https://roboticon.resolute.education/</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>Join us for the ultimate robotics showcase as Resolute proudly sponsors the World Robotics Olympiad (WRO) South Africa! This year, we're bringing together two worlds for the biggest robotics event of the year – Roboticon and the WRO Nationals, happening on the same day at the same venue.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
+          <t>robotics competition South Africa</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -2021,99 +2077,99 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026 Season - Africa's Global STEM Celebration</t>
+          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://www.stemfestival.org/competitions/</t>
+          <t>https://safcec.org.za/</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>April 30, 2026 - ... The Elementary, Junior, and Senior Robotics categories at STEM Festival are dedicated to advancing the World Robot Olympiad (WRO) across the Niger Delta and South-South Nigeria, working with ArcLights Foundation.</t>
+          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr"/>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>communication@safcec.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Competition – Eskom Expo for Young Scientists</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://exposcience.co.za/category/competition/</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Aqil Variava business cities Damien ... Gray STEMI Vuyo Nzimande · Eskom Expo for Young Scientists is an exposition, or science fair, where students have a chance to show others their projects about their own scientific investigations. At the annual prestigious Eskom Expo for Young Scientists International Science Fair (ISF), selected students from 35 Expo Regions in South Africa then compete ...</t>
+          <t>Sep 4, 2025 · 3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>support@exposcience.co.za</t>
+          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SA young scientists selected for global competition at Regeneron ISEF in the USA - Eskom</t>
+          <t>ICE Africa – Supporting Civil Engineers in Africa</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://www.eskom.co.za/sa-young-scientists-selected-for-global-competition-at-regeneron-isef-in-the-usa/</t>
+          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>May 6, 2025 - Regeneron ISEF 2025, the world’s largest pre-college science, technology, engineering and mathematics (STEM) competition, will take place from 10 to 16 May in Columbus, Ohio in the USA.</t>
+          <t>ICE Africa supports civil engineers across the continent, providing access to qualifications, training, and networking opportunities for professional growth.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>MediaDesk@eskom.co.za</t>
-        </is>
-      </c>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>STEAM Pitch Competition - STEM AFRICA FEST 2024</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://stemafricafest.com/steam-pitch-competition/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Join STEM Africa Fest , celebrating science, technology, engineering, and mathematics. Experience hands-on learning, industry leaders, and innovation across Africa.</t>
+          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
@@ -2121,29 +2177,586 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Rural youth lead in robotics at national STEM competition</t>
+          <t>Home - SAICE</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://iol.co.za/news/education/2025-09-15-rural-youth-lead-in-robotics-at-national-stem-competition/</t>
+          <t>https://saice.org.za/</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>September 15, 2025 - Discover how South Africa's brightest young minds are tackling real-world challenges with innovative solutions at the inaugural AlgoAtWork RoboRumble STEM Innovation Challenge, where ideas like autonomous robots and smart PPE systems are set ...</t>
+          <t>The South African Institution of Civil Engineering (SAICE) is the industry body for civil engineering professionals in South Africa. Our aim is to, promote growth, excellence and sustainability in the industry.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>lee.rondganger@inl.co.za, londiwe.gumede@inl.co.za, philippa.larkin@inl.co.za, nobuntu.mgijima@volt.africa, ashley.lechman@inl.co.za, mendy.mtshali@inl.co.za</t>
-        </is>
-      </c>
+          <t>membership@saice.org.za, communications@saice.org.za, marketing@saice.org.za, executiveadmin@saice.org.za, civilinfo@saice.org.za, barbara@avenue.co.za, accounts@saice.org.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Jul 7, 2026 · 19 June 2026 marked an exciting celebration of Youth Month as aspiring young engineers from across Gauteng gathered for the 2026 SAICE Johannesburg Branch Schools Bridge Building Competition. Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in ...</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Awards 2025 - SAICE</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>https://saice.org.za/awards-2025/</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Learn about SAICE's award categories, submission guidelines, key dates and how to nominate project and professionals.</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>membership@saice.org.za, communications@saice.org.za, marketing@saice.org.za, civilinfo@saice.org.za, accounts@saice.org.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>How to compete at the WSZA National Competitions 2025</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Competitions | Capetown 2026</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>ASTEMI Competitions – SAASTA</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>APPLY NOW! WORLDSKILLS SOUTH AFRICA NATIONAL COMPETITION 2025</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>SAIMechE</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>https://www.saimeche.org.za/</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>How to compete at the WSZA National Competitions 2025</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>South African Institute of Electrical Engineers</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>https://www.saiee.org.za/</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>South African Institute of Electrical Engineers 18a Gill Street Observatory Johannesburg South Africa Phone: +27 (0)11 487 3003 Email: reception@saiee.org.za Powered by</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>glueup-logo-white@2x.png, reception@saiee.org.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Competitions | ESG</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>https://za.rs-online.com/web/content/m/competition</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>example@email.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>ASTEMI Competitions – SAASTA</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Apr 30, 2026 · IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa) Deadline: April 30, 2026 May 15, 2026</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Competitions – SAASTA</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>https://www.saasta.ac.za/competitions/</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>https://hackon.co.za/</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Hackathons en South Africa</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>https://za.allhackathons.com/</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Aug 22, 2025 · Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>AI Hackathon | Sebaka</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>https://sebakasouthafrica.co.za/index.html</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Sebaka Mentorship &amp; Hackathons — Build an AI Agent for Software Quality Engineering.</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>https://hackon.co.za/partners/</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>South Africa Policy Hackathon Hello Ladies, Happy New Year. Some of you may be interested in this workshop. The workshop is flagged for South African nationals working at research and innovation offices, accelerators, innovation hubs and incubators, tech centers, and start-ups working on dual-use...</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Build the Future with Entelect Hackathons</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>https://challenge.entelect.co.za/</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Build the Future with Entelect Hackathons Join South Africa’s premier optimisation-first developer competition platform. Compete, iterate, and outperform the best.</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Young Engineers Movement (YEM) - ORT SA</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>MICT SETA National Skills Challenge 2026 | Empowering ...</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>https://www.cxia4irhack.co.za/</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Mar 27, 2026 · The MICT SETA National Skills Challenge 2026 is a 2-day innovation sprint that brings together students from universities and colleges across South Africa to solve real industry challenges through technology, creativity, and collaboration. Tackling real-world challenges in manufacturing, engineering, and technology through collaborative innovation.</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update competition data 2026-08-18
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E94"/>
+  <dimension ref="A1:E118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,7 +466,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
         </is>
       </c>
     </row>
@@ -483,7 +483,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>ASTEMI is a collaboration that ... &amp; Competitions to a broader base of learners and educators. ASTEMI is a national non-profit organization of independent organizations; teachers, public organisations and volunteers dedicated to improving and promoting science education and providing recognition for outstanding achievement by both learners and teachers. To promote excellence in Science, Technology, Engineering, Mathematics and Innovation in South African ...</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -496,17 +496,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+          <t>Some of our sparkling achievements ... and competitions. The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the · National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation ...</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -514,26 +514,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -550,17 +546,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa. Find out more</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -568,22 +564,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+          <t>Faculty of Engineering Students to Represent South Africa at ...</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://www.su.ac.za/en/innovus/news/faculty-engineering-students-represent-south-africa-global-space-competition?language=en</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
+          <t>Apr 15, 2026 · The competition offers the team an opportunity to showcase South African engineering talent on an international stage while benchmarking their skills against global peers. Beyond the event, the team aims to bring back new knowledge and inspiration, contributing to the growth of local expertise in space science and engineering.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -596,17 +596,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2 weeks ago - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -619,17 +619,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
+          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
+          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
+          <t>2 weeks ago - South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -642,17 +642,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
+          <t>VUT inspires future engineers through Bridge Building Competition – Vaal University of Technology</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.poidata.io/report/engineer/south-africa</t>
+          <t>https://vut.ac.za/vut-inspires-future-engineers-through-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
+          <t>3 weeks ago - Supported by the ArcelorMittal Science Centre, Institution of Structural Engineers (IStructE), Fundi, South African Institution of Civil Engineering Future Leaders Panel (SAICE FLP) Vaal and maVuti Shop, the initiative challenged learners to design and construct bridge models using simple ...</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -665,17 +665,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Two South Africans on the shortlist for the 2026 Africa Prize for Engineering Innovation</t>
+          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/two-south-africans-on-the-shortlist-for-the-2026-africa-prize-for-engineering-innovation-2026-08-04</t>
+          <t>https://www.poidata.io/report/engineer/south-africa</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2 weeks ago - Two South African innovators have been shortlisted for the UK Royal Academy of Engineering’s Africa Prize for Engineering Innovation 2026. This is the continent’s richest award aimed at promoting engineering innovation and entrepreneurship ...</t>
+          <t>June 22, 2026 - Our comprehensive list of 1,582 Engineers in South Africa empowers you to reach the right audience through multiple channels. Here are key ways this data can give you a competitive edge in the Engineers industry.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -683,16 +683,12 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>newsletters@creamermedia.co.za, newsdesk@engineeringnews.co.za, chanel@engineeringnews.co.za, subscriptions@creamermedia.co.za, advertising@creamermedia.co.za</t>
-        </is>
-      </c>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show ...</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -702,7 +698,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AI Expo Africa 2026 – Join the Largest AI Event &amp; Trade Community in Africa TODAY! Our business audience is a buyer / supplier focused community and comprised of Enterprise decision makers / CxOs, allied to AI Cloud platform providers, Tier 1 / 2 deployment &amp; service providers, AI start ups / innovators, investors, educators, government and AI ecosystem community builders.</t>
+          <t>AI Expo Africa 2026 - Join the Largest AI Event &amp; Trade Community in Africa TODAY! Our business audience is a buyer / supplier focused community and comprised of Enterprise decision makers / CxOs, allied to AI Cloud platform providers, Tier 1 / 2 deployment &amp; service providers, AI start ups / innovators, investors, educators, government and AI ecosystem community builders.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -719,17 +715,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
+          <t>Africa Tech Festival</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/tradeshows</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>South Africa trade shows, find and compare 964 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 174 upcoming expos in 2026-2027 1. South Africa Infrastructure &amp; Water Expo, 2.</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -737,22 +733,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>customerservices@informaconnect.com, salesenquiries@africatechfestival.com, support@informaconnect.com, customerservices@knect365.com, dataprivacy@knect365.com, dataprivacy@informaconnect.com, support@knect365.com</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
+          <t>Exhibitions in South Africa 2026-2027 - ExpoTobi</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://manufacturingindaba.co.za/exhibition/</t>
+          <t>https://expotobi.com/country/south-africa/exhibitions</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
+          <t>All Exhibitions in South Africa 2026-2027 | Full and accurate description of events for various business sectors | Schedule, tickets, travel arrangements and participation</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -760,11 +760,7 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>lene@hotdesigns.co.za</t>
-        </is>
-      </c>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -779,7 +775,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SA Innovation Week 2026 is South Africa’s official national innovation platform accelerating implementation, commercialisation and impact.</t>
+          <t>SA Innovation Week 2026 is South Africa's official national innovation platform accelerating implementation, commercialisation and impact.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -796,7 +792,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa, List of all South ...</t>
+          <t>IT &amp; Technology Events in South Africa | 10times</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -806,7 +802,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>18 hours ago · Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -819,17 +815,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>South Africa International Industrial Expo | Innovation Bridge</t>
+          <t>DigiMarCon Africa 2027 - Cape Town, South Africa · October 6</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
+          <t>https://digimarconafrica.com/</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
+          <t>The Premier Digital Marketing, Media and Advertising Conference &amp; Exhibition held annually in Cape Town, South Africa! Join your peers for 2 days jam packed with digital marketing best practices, latest trends and strategy, also check out the next generation of technology &amp; innovation; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year ...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -837,22 +833,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>info@digimarconafrica.com</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Two landmark exhibitions set to transform industrial technology and renewable energy in South Africa</t>
+          <t>Manufacturing Indaba Exhibition 2026 - Manufacturing Expo</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/two-landmark-exhibitions-set-to-transform-industrial-technology-and-renewable-energy-in-south-africa-2025-10-24</t>
+          <t>https://manufacturingindaba.co.za/exhibition/</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>October 24, 2025 - South Africa’s industrial and clean energy sectors celebrated a landmark moment today with the official launch of RE+ South Africa 2026 and the Cape Industrial Technology Exhibition (CITE) 2027.</t>
+          <t>Manufacturing Indaba Exhibition 2026: Africa's leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -860,26 +860,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>newsletters@creamermedia.co.za, newsdesk@engineeringnews.co.za, chanel@engineeringnews.co.za, subscriptions@creamermedia.co.za, advertising@creamermedia.co.za</t>
-        </is>
-      </c>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>KZN Industrial Technology Exhibition</t>
+          <t>TECHSPO Cape Town 2027 - Technology Expo · October 6</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://www.kznindustrial.co.za/</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
+          <t>Where Business, Tech and Innovation Collide in Cape Town! TECHSPO Cape Town is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -889,24 +885,24 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>john@email.com</t>
+          <t>info@techspocapetown.co.za</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
+          <t>TECHSPO Joburg 2026 - Technology Expo · October 10</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://madeinafricaevent.co.za/</t>
+          <t>https://techspojoburg.co.za/</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
+          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -914,22 +910,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>info@techspojoburg.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Trade Shows Worldwide - South Africa - 2026/2027</t>
+          <t>Home - AWIEF</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.eventseye.com/fairs/c1_trade-shows_south-africa.html</t>
+          <t>https://www.awieforum.org/</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>South Africa Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in South Africa</t>
+          <t>"Events like AWIEF bring together private sector leaders, government, policymakers, and entrepreneurs to unlock real opportunities for women and youth, and to turn Africa's prosperity potential into reality."</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -937,22 +937,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>info@awieforum.org</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community’s challenges and how community members view the impact of these challenges on their daily lives.</t>
+          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -960,26 +964,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
-        </is>
-      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
+          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -987,22 +987,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of ...</t>
+          <t>EWB Design Challenge | Aston University</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Aug 4, 2025 · This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but under-resourced neighbourhood on the eastern edge of Johannesburg. Home to around 46,000 people, Makers Valley is a community rich in creativity, activism ...</t>
+          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1010,26 +1014,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
-        </is>
-      </c>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Latest Community Engineering Design Competition Announced</t>
+          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
+          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Oct 16, 2024 · STEM-focused NGO Engineers Without Borders UK has launched its 2025 Engineering for People Design Challenge. Organised in conjunction with sister organisation Engineers Without Borders South Africa, as well as the Makers Valley Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg.</t>
+          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1037,22 +1037,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ied@ied.org.uk</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Engineering For People Design Challenge - EWBSA</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
+          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1060,26 +1064,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
-        </is>
-      </c>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge - Engineers Without ...</t>
+          <t>Engineering for people, that’s the challenge | Engineers Without Borders</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
+          <t>https://www.rs-online.com/designspark/an-introduction-to-engineering-for-people-design-challenge</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
+          <t>That’s exactly what the annual Engineering for People Design Challenge asks participants to do. The competition, delivered in partnership by Engineers without Borders South Africa and Engineers Without Borders UK, encourages engineering students and those collaborating with engineers to broaden their awareness of how their decisions change the world.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1092,17 +1092,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
+          <t>Real-world research: Engineering team designs South African trolley system; science students investigate heavy metals | University of Wisconsin - Stout</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
+          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Oct 24, 2024 · The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
+          <t>May 15, 2025 - Research ranged from heavy metals ... Borders’ international design challenge. Nearly 90 students in 23 teams addressed the EWB challenge. One group focused on engineering a safer, more accessible transportation system in South ...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1112,24 +1112,24 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>team@crowdsolve.net</t>
+          <t>dolanm@uwstout.edu, frischj@uwstout.edu</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>EWB Design Challenge | Aston University</t>
+          <t>Engineering for People Design Challenge | Department of Engineering</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
+          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1137,22 +1137,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>web-editor@eng.cam.ac.uk, marketing@eng.cam.ac.uk</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
+          <t>Inspiring, building and shaping a future fit engineering community – EWB-I</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
+          <t>https://www.ewb-international.org/home/inspiring-building-and-shaping-a-future-fit-engineering-community/</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
+          <t>February 27, 2025 - The challenge, delivered during ... career, encourages individuals to broaden their awareness of the social, environmental and economic implications of their engineering solutions. Since 2011, the Design Challenge has been delivered in Cameroon, South Africa, the UK and Ireland and the USA to over 70,000 students...</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1162,24 +1166,24 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ied@ied.org.uk</t>
+          <t>admin@ewb-international.org</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Real-world research: Engineering team designs South African trolley system; science students investigate heavy metals | University of Wisconsin - Stout</t>
+          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
+          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>May 15, 2025 - Research ranged from heavy metals ... Borders’ international design challenge. Nearly 90 students in 23 teams addressed the EWB challenge. One group focused on engineering a safer, more accessible transportation system in South ...</t>
+          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1187,26 +1191,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>dolanm@uwstout.edu, frischj@uwstout.edu</t>
-        </is>
-      </c>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1214,26 +1214,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1241,26 +1237,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
+          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Sep 4, 2025 · 3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1268,26 +1260,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
-        </is>
-      </c>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>National Student Competition | ORSSA</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://www.orssa.org.za/studentcomp</t>
+          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>National Student Competitions The Operations Research Society of South Africa The home of decision intelligence The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1295,26 +1283,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, email@example.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+          <t>Engineering in South Africa: 24 Best universities Ranked</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://edurank.org/engineering/za/</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
+          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1327,17 +1311,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>University Overall Rankings - Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>University Overall Rankings - Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1350,17 +1334,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2210</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1373,98 +1357,86 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 ...</t>
+          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://techspojoburg.co.za/</t>
+          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
+          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>tech expo South Africa</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>info@techspojoburg.co.za</t>
-        </is>
-      </c>
+          <t>university engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7 ...</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Where Business, Tech and Innovation Collide in Cape Town! TECHSPO Cape Town is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>tech expo South Africa</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>info@techspocapetown.co.za</t>
-        </is>
-      </c>
+          <t>university engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Africa Tech Festival</t>
+          <t>5 Best Universities to Study Engineering in South Africa</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://globalscholarships.com/best-universities-engineering-south-africa/</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
+          <t>May 9, 2026 - Its diplomas and BEngTech degrees can support routes to registration with the Engineering Council of South Africa as engineering technicians or engineering technologists after the required practical experience. ... Degree/s Offered: Bachelor’s, Master’s, Ph.D. South Africa’s oldest university, the University of Cape Town, is one of the best engineering schools in South Africa.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>tech expo South Africa</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>customerservices@informaconnect.com, support@informaconnect.com, customerservices@knect365.com, salesenquiries@africatechfestival.com, support@knect365.com, dataprivacy@informaconnect.com, dataprivacy@knect365.com</t>
-        </is>
-      </c>
+          <t>university engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 ...</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://techspojoburg.co.za/</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>18 hours ago · Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1472,22 +1444,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>info@techspojoburg.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
+          <t>Africa Tech Festival</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://10times.com/johannesburg-za/technology</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>3 days ago · Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1495,22 +1471,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>customerservices@informaconnect.com, salesenquiries@africatechfestival.com, support@informaconnect.com, customerservices@knect365.com, dataprivacy@knect365.com, dataprivacy@informaconnect.com, support@knect365.com</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 – Africa's biggest IT Conference and Expo</t>
+          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://10times.com/johannesburg-za/technology</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what’s next before everyone else does. Only 2,500 ...</t>
+          <t>4 days ago · Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1523,17 +1503,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology ExpoJohannesburg Technology ...</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7 ...</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://techspojoburg.co.za/johannesburg-technology-expo/</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg is a 2-day technology expo taking place September 28 – 29, 2026 at the luxurious NH Johannesburg Sandton Hotel, Toronto, Ontario. TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
+          <t>Where Business, Tech and Innovation Collide in Cape Town! TECHSPO Cape Town is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1541,27 +1521,31 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>info@techspocapetown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Maker Faire Africa - Wikipedia</t>
+          <t>IT &amp; Technology Events in South Africa | 10times</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Maker_Faire_Africa</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Maker Faire Africa, Cairo, October 2011 Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds (Nubian Cheetah). Maker Faire Africa aims to engage with on ...</t>
+          <t>Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>maker faire South Africa</t>
+          <t>tech expo South Africa</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
@@ -1569,22 +1553,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Maker Faire Africa — Grokipedia</t>
+          <t>IT Indaba 2026 – Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://grokipedia.com/page/maker_faire_africa</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Maker Faire Africa Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
+          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what’s next before everyone else does. Only 2,500 ...</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>maker faire South Africa</t>
+          <t>tech expo South Africa</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
@@ -1592,121 +1576,121 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Maker Faire |</t>
+          <t>TECHSPO Johannesburg Technology ExpoJohannesburg Technology ...</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://makerfaire.com/</t>
+          <t>https://techspojoburg.co.za/johannesburg-technology-expo/</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
+          <t>TECHSPO Johannesburg is a 2-day technology expo taking place September 28 – 29, 2026 at the luxurious NH Johannesburg Sandton Hotel, Toronto, Ontario. TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>maker faire South Africa</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>fancybox_loading@2x.gif, pr@make.co, fancybox_sprite@2x.png, chosen-sprite@2x.png</t>
-        </is>
-      </c>
+          <t>tech expo South Africa</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Upcoming Faires - Maker Faire</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://makerfaire.com/upcoming-faires/</t>
+          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
+          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>maker faire South Africa</t>
+          <t>tech expo South Africa</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>fancybox_loading@2x.gif, pr@make.co, fancybox_sprite@2x.png, chosen-sprite@2x.png</t>
+          <t>name@example.com, u003einfo@techspo.co, atinfo@techspo.coor</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
+          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
+          <t>https://africatechnologyexpo.com/</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Aug 21, 2015 · DIRECTIONS THE CAPE TOWN MAKER FAIRE The Lookout, V&amp;A Waterfront Granger Bay Boulevard, V &amp; A Waterfront, Cape Town, 8002, South Africa Get Directions Fri Aug 21, 13:00 - Sun Aug 23, 17:00 The Lookout, V&amp;A Waterfront View Map Payments are secure and encrypted</t>
+          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>maker faire South Africa</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr"/>
+          <t>tech expo South Africa</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>info@sparkafrica.co, partner@africatechnologyexpo.com, johndoe@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>HOME | MAKERS FEST</t>
+          <t>Home - Mediatech Africa | South Africa</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://www.makersfestival.co.za/</t>
+          <t>https://www.mediatech.co.za/</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>On 8 &amp; 9 November 2025 at The Ostrich in Cape Town, join 2,000+ visitors each day for maker demos, a curated market, and family activities. It’s Africa’s first hands-on festival for creativity and craftsmanship — and everything you make, you take home.</t>
+          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>maker faire South Africa</t>
+          <t>tech expo South Africa</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>8c4075d5481d476e945486754f783364@sentry.io, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, example@mysite.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, warren@makersfestival.co.za, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com</t>
+          <t>simon@mediatech.co.za, claire@mediatech.co.za</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Maker Faire groups | Meetup</t>
+          <t>Maker Faire Africa - Wikipedia</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/topics/maker-faire/za/</t>
+          <t>https://en.wikipedia.org/wiki/Maker_Faire_Africa</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
+          <t>Maker Faire Africa, Cairo, October 2011 Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds (Nubian Cheetah). Maker Faire Africa aims to engage with on ...</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1719,122 +1703,130 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Home | Makers Fest</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.makersfestival.co.za/</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>All these Olympiads and Competitions have a positive impact on education and on educational institutions in South Africa, but there is still a need to build stronger collaboration among teachers, schools, universities and educational authorities in order to meet the challenges of STEM education in South Africa today.</t>
+          <t>On 8 &amp; 9 November 2025 at The Ostrich in Cape Town, join 2,000+ visitors each day for maker demos, a curated market, and family activities. It's Africa's first hands-on festival for creativity and craftsmanship — and everything you make, you take home.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr"/>
+          <t>maker faire South Africa</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, example@mysite.com, 8c4075d5481d476e945486754f783364@sentry.io, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, warren@makersfestival.co.za, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>STEM Scholars — 2026 STEM &amp; Entrepreneurship Discovery Initiative</t>
+          <t>Makers Fair | Experience Culture - Join the Fair</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://stemscholars.co.za/</t>
+          <t>https://www.makersfair.co.za/</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Building South Africa's Next Generation of Innovators The STEM &amp; Entrepreneurship Discovery Initiative connects learners with a world that's often invisible from inside a classroom — and equips them with skills that last far beyond the competition.</t>
+          <t>Discover Southern African arts, crafts, food, and wine at the Makers Fair. Join us for cultural celebration and early ticket updates in Johannesburg 2026.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
+          <t>maker faire South Africa</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>you@school.co.za, inforeg@justice.gov.za, marushka@stemscholars.co.za</t>
+          <t>user@domain.com</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>About | Explore Unique Maker Culture — Join Now — Makers Fair</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.makersfair.co.za/about</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>Discover South African and Pan-African craftsmanship at Makers Fair, a women-led event celebrating sustainable design, art, and culture. Join us today!</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr"/>
+          <t>maker faire South Africa</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>user@domain.com</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Capetown 2026</t>
+          <t>Maker Faire |</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
+          <t>https://makerfaire.com/</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the ‘first author’. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
+          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
+          <t>maker faire South Africa</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>info@ieomsociety.org</t>
+          <t>pr@make.co, fancybox_loading@2x.gif, fancybox_sprite@2x.png, chosen-sprite@2x.png</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ASTEMI SA</t>
+          <t>Makers Festival SA | Cape Town - Facebook</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/</t>
+          <t>https://www.facebook.com/61574201023378/</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
+          <t>Makers Festival SA , Cape Town. 1,474 likes · 2 talking about this · 8 were here. Africa's first festival of creativity, craftsmanship &amp; community. Makers, live demos, food, music &amp; workshops for...</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
+          <t>maker faire South Africa</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
@@ -1842,334 +1834,318 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
+          <t>Upcoming Faires - Maker Faire</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/za/solvefortomorrow/</t>
+          <t>https://makerfaire.com/upcoming-faires/</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
+          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr"/>
+          <t>maker faire South Africa</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>pr@make.co, fancybox_loading@2x.gif, fancybox_sprite@2x.png, chosen-sprite@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Applications for 2026 Samsung Solve For Tomorrow Now Open!</t>
+          <t>Makers Festival South Africa 2025 - Child Magazine</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://news.samsung.com/za/applications-for-2026-samsung-solve-for-tomorrow-now-open</t>
+          <t>https://www.childmag.co.za/etn/makers-festival-south-africa-2025/</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Feb 23, 2026 · The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges – with entries open until 06 March 2026. This is a transformative ...</t>
+          <t>Makers Festival South Africa 2025 Africa's first festival of creativity, craftsmanship &amp; community. Makers, live demos, food, music &amp; workshops for all ages. Craft. Create. Connect. The first of its kind in Africa, Makers Festival is a groundbreaking celebration of creativity, craftsmanship, and community.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>ssapr.newsroom@samsung.com, ssasft@samsung.com</t>
-        </is>
-      </c>
+          <t>maker faire South Africa</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Robotics Competition | WRO South Africa | Gauteng</t>
+          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://www.wrosa.co.za/</t>
+          <t>https://capetown.makerfaire.com/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>WRO South Africa ( World Robot Olympiad ) is a robotics competition which brings together young people from all over the world to develop their creativity and problem-solving skills.</t>
+          <t>Jump into the Make: community and bring a Maker Faire to your town, city, or region! Spark curiosity, rally makers of all ages, and plug your local scene into a global movement fueled by creativity, resilience, innovation, and hands-on learning.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>robotics competition South Africa</t>
+          <t>maker faire South Africa</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com</t>
+          <t>pr@make.co, fancybox_loading@2x.gif, fancybox_sprite@2x.png, chosen-sprite@2x.png</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
+          <t>Makers Festival SA - Whats on in Cape Town</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
+          <t>https://whatsonincapetown.com/event/makers-festival-sa/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in the leading UN-based global robotics competition, focusing on the critical area of agriculture and food security.</t>
+          <t>Makers Festival SA Event information The first of its kind in Africa, Makers Festival is a groundbreaking celebration of creativity, craftsmanship, and community. Bringing together artists, makers, and craftsmen from across the country, it's more than just a festival — it's the start of something big. What sets it apart?</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>robotics competition South Africa</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, info@thecortexhub.africa, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com</t>
-        </is>
-      </c>
+          <t>maker faire South Africa</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Oct 31, 2025 · The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge, organized by ITU and The Cortex Hub, in partnership with Google.</t>
+          <t>All these Olympiads and Competitions have a positive impact on education and on educational institutions in South Africa, but there is still a need to build stronger collaboration among teachers, schools, universities and educational authorities in order to meet the challenges of STEM education in South Africa today.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>robotics competition South Africa</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>name@example.com</t>
-        </is>
-      </c>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa</t>
+          <t>STEM Scholars — 2026 STEM &amp; Entrepreneurship Discovery Initiative</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa/</t>
+          <t>https://stemscholars.co.za/</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Apr 25, 2025 · The Robotics for Good Youth Challenge South Africa is a national event in a global robotics competition on disaster response, leading to the AI for Good Summit 2025.</t>
+          <t>Building South Africa's Next Generation of Innovators The STEM &amp; Entrepreneurship Discovery Initiative connects learners with a world that's often invisible from inside a classroom — and equips them with skills that last far beyond the competition.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>robotics competition South Africa</t>
+          <t>stem competition South Africa</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>name@example.com</t>
+          <t>marushka@stemscholars.co.za, inforeg@justice.gov.za, you@school.co.za</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Competition &amp; Judge Registration | WROSA</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://www.wrosa.co.za/teamregistration</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>World Robot Olympiad South Africa Team Registration 2026 Physical Events - Team Registration Team Registrations are now open! Register your teams by clicking on the button below. Team registrations will close at 12:00 on the 1st of June. No Late Registrations will be accepted. Registrations Have Closed</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>robotics competition South Africa</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com</t>
-        </is>
-      </c>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Roboticon 2026: South Africa Showcases Robotics for Culture ...</t>
+          <t>ASTEMI SA</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://www.ubuntutimes.co.za/roboticon-2026-south-africa-showcases-robotics-for-culture-education-and-innovation/</t>
+          <t>https://www.astemi.co.za/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Jul 2, 2026 · The event, partnered with the World Robotics Olympiad, positions South Africa as a leader in educational robotics and entrepreneurial innovation.” South Africa’s robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation.</t>
+          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>robotics competition South Africa</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>adverts@ubuntutimes.co.za, newspaper-rec300@2x.jpg</t>
-        </is>
-      </c>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Home | Roboticon 2026</t>
+          <t>High School STEM Competition | Capetown 2026</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://roboticon.resolute.education/</t>
+          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Join us for the ultimate robotics showcase as Resolute proudly sponsors the World Robotics Olympiad (WRO) South Africa! This year, we're bringing together two worlds for the biggest robotics event of the year – Roboticon and the WRO Nationals, happening on the same day at the same venue.</t>
+          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the ‘first author’. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>robotics competition South Africa</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr"/>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
+          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://safcec.org.za/</t>
+          <t>https://www.samsung.com/za/solvefortomorrow/</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
+          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>communication@safcec.org.za</t>
-        </is>
-      </c>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
+          <t>StemCo - StemCo 2026 International Competitions</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://stemco.org/</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Sep 4, 2025 · 3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>June 10, 2026 - BEST YOURSELF WITH STEMCO! Platform for the world’s brightest. ... Thanks to the participating 25 countries in 2019. Singapore, Albania, Australia, Azerbaijan, Canada, Germany, India, Indonesia, Japan, Jordan, Kazakhstan, Kyrgyzstan, Malawi, Mongolia, Nigeria, Myanmar, South Africa, Tajikistan, Turkey, Turkmenistan, Ukraine, The United States, Uzbekistan, Vietnam</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
-        </is>
-      </c>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ICE Africa – Supporting Civil Engineers in Africa</t>
+          <t>High School STEM Competition | Southafrica 2024</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
+          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>ICE Africa supports civil engineers across the continent, providing access to qualifications, training, and networking opportunities for professional growth.</t>
+          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, ...</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr"/>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+          <t>Samsung opens Solve for Tomorrow 2026 STEM competition to all South African public schools</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
+          <t>February 27, 2026 - Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
+          <t>stem competition South Africa</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
@@ -2177,99 +2153,99 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Home - SAICE</t>
+          <t>ASTEMI Competitions 2022 – SAASTA</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://saice.org.za/</t>
+          <t>https://saasta.ac.za/astemi-competitions-2</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) is the industry body for civil engineering professionals in South Africa. Our aim is to, promote growth, excellence and sustainability in the industry.</t>
+          <t>National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>membership@saice.org.za, communications@saice.org.za, marketing@saice.org.za, executiveadmin@saice.org.za, civilinfo@saice.org.za, barbara@avenue.co.za, accounts@saice.org.za</t>
-        </is>
-      </c>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
+          <t>Robotics Competition | WRO South Africa | Gauteng</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
+          <t>https://www.wrosa.co.za/</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Jul 7, 2026 · 19 June 2026 marked an exciting celebration of Youth Month as aspiring young engineers from across Gauteng gathered for the 2026 SAICE Johannesburg Branch Schools Bridge Building Competition. Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in ...</t>
+          <t>WRO South Africa ( World Robot Olympiad ) is a robotics competition which brings together young people from all over the world to develop their creativity and problem-solving skills.</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr"/>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Awards 2025 - SAICE</t>
+          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>https://saice.org.za/awards-2025/</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Learn about SAICE's award categories, submission guidelines, key dates and how to nominate project and professionals.</t>
+          <t>April 14, 2026 - This National Event, to be held at the Sandton Convention Centre in Johannesburg, South Africa, as part of AI for Good Impact Africa, at AI Expo Africa 2025, is a qualifying tournament leading to the Grand Finale in Geneva during the AI for ...</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
+          <t>robotics competition South Africa</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>membership@saice.org.za, communications@saice.org.za, marketing@saice.org.za, civilinfo@saice.org.za, accounts@saice.org.za</t>
+          <t>name@example.com</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>FIRST South Africa – Robotics Programs for School Children</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://firstsa.org/</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+          <t>From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way. FIRST Tech Challenge students learn to think like engineers. Teams ...</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>robotics competition South Africa</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
@@ -2277,49 +2253,45 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>WorldSkillsZA Mobile Robotics Provincial Competition 2024</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://worldskillsza.dhet.gov.za/site/WSZA-Prov-Comp/Provincial-Competitions.aspx</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+          <t>The WorldSkills South Africa (WSZA) will be having its Mobile Robotics Combined Provincial Competitions in Lephalale TVET College from the 07th - 10th October 2023. the first 3 days will be focused on training and the last day will be the actual Mobile Robotics competition.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>robotics competition South Africa</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
@@ -2327,72 +2299,72 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+          <t>South African Robotics Competitions and Schools</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://www.sciencexpo.org.za/robotics.html</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
+          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr"/>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>marna.vanzyl@imbewu.foundation, webmaster@sciencexpo.org.za, madelien@imbewu.foundation</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Limpopo Learners Represent South Africa at Global Robotics Finals in Switzerland - African Times</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.atnews.co.za/limpopo-learners-represent-south-africa-at-global-robotics-finals-in-switzerland/</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>July 7, 2026 - The international competition, taking place from 7 to 10 July 2026 at the Palexpo International Exhibition and Convention Centre in Geneva, brings together some of the world’s brightest young innovators to develop technological solutions to ...</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>APPLY NOW! WORLDSKILLS SOUTH AFRICA NATIONAL COMPETITION 2025</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - AfrikaBot</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
+          <t>https://www.saiee.org.za/displaycustomlink.aspx?name=AfrikaBot</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
+          <t>AfrikaBot is affordable because you can build a competitive robot for a lot less with the correct advice. AfrikaBOT is South Africa's first robotics competition for high school teenagers and university undergraduates who are smart enough to build their own robots from electronic parts rather ...</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>robotics competition South Africa</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
@@ -2400,122 +2372,126 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>SAIMechE</t>
+          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://www.saimeche.org.za/</t>
+          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
+          <t>The Robotics for Good Youth Challenge national competition will be held in Johannesburg, South Africa, at the Sandton Convention Centre on the 31st October 2025.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr"/>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>info@thecortexhub.africa, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>Robotics for Good Youth Challenge South Africa - Limpopo - AI for Good</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-limpopo/</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+          <t>December 8, 2025 - This Regional Event is a qualifying tournament leading to the Robotics for Good Youth Challenge South Africa National Event, to be held on 31 October at the Sandton Convention Centre in Johannesbourg, as part of AI for Good Impact Africa, at ...</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr"/>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>name@example.com</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers</t>
+          <t>The South African Institution of Civil Engineering (SAICE)</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/</t>
+          <t>https://www.facebook.com/SAICECIVIL/posts/-capture-engineering-excellencethe-2026-pps-photo-competition-is-now-open-for-en/1448856900617968/</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers 18a Gill Street Observatory Johannesburg South Africa Phone: +27 (0)11 487 3003 Email: reception@saiee.org.za Powered by</t>
+          <t>📸 Capture Engineering Excellence. The 2026 PPS Photo Competition is now open for entries! Whether you've captured engineering innovation in action, impressive infrastructure, or the people behind the profession, this is your chance to showcase civil engineering at its best.</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, reception@saiee.org.za</t>
-        </is>
-      </c>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Competitions | ESG</t>
+          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://za.rs-online.com/web/content/m/competition</t>
+          <t>https://safcec.org.za/</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
+          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>example@email.com</t>
+          <t>communication@safcec.org.za</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>ICE Africa - Supporting Civil Engineers in Africa</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>ICE Africa supports civil engineers across the continent, providing access to qualifications, training, and networking opportunities for professional growth.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E84" t="inlineStr"/>
@@ -2523,22 +2499,22 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 · IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa) Deadline: April 30, 2026 May 15, 2026</t>
+          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
@@ -2546,95 +2522,103 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>info@ieomsociety.org</t>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>SAICE National Bridge Building Competition 2025 - avenue.co.za</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.avenue.co.za/post/saice-national-bridge-building-competition-2025</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>SAICE initiated the National Bridge Building Competition in 1991, and 34 years later, this exciting competition is still an enormous success and enjoyed by learners across country.Did you know, many a civil engineer has referred to this very competition as the turning point in their decision to choose civil engineering as a career?There is considerable value in partnering with SAICE and ...</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr"/>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, barbara@avenue.co.za, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
+          <t>Home - SAICE</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://hackon.co.za/</t>
+          <t>https://saice.org.za/</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) is the industry body for civil engineering professionals in South Africa. Our aim is to, promote growth, excellence and sustainability in the industry.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr"/>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>accounts@saice.org.za, civilinfo@saice.org.za, communications@saice.org.za, barbara@avenue.co.za, membership@saice.org.za, marketing@saice.org.za, executiveadmin@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Hackathons en South Africa</t>
+          <t>SAICE Aqualibrium 2025: High School Students Rise to the Challenge in ...</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://za.allhackathons.com/</t>
+          <t>https://southafricatoday.net/environment/saice-aqualibrium-2025-high-school-students-rise-to-the-challenge-in-national-water-competition/</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Aug 22, 2025 · Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
+          <t>The South African Institution of Civil Engineering (SAICE) hosted the thrilling 2025 Aqualibrium Competition National Finals this past week, which brought together high school students from schools all over South Africa at the Sci-Bono Discovery Centre in Johannesburg. The event continues to be an important platform for fostering engineering talent, inspiring young minds, and raising awareness ...</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
@@ -2642,68 +2626,76 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>AI Hackathon | Sebaka</t>
+          <t>Home - cidb</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://sebakasouthafrica.co.za/index.html</t>
+          <t>https://www.cidb.org.za/</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Sebaka Mentorship &amp; Hackathons — Build an AI Agent for Software Quality Engineering.</t>
+          <t>Partnering with you to achieve South Africa's construction industry success Established by Act 38 of 2000, cidb helps to transform the construction industry through inclusivity, high ethical standards, and amplifies contributions made by industry participants towards South Africa's economy and society.</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr"/>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Group-272@2x-300x270.jpg, Group-274@2x-300x269.jpg, Group-274@2x.jpg, Group-270@2x-300x270.jpg, Group-270@2x.jpg, Group-272@2x.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
+          <t>Awards 2025 - SAICE</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://hackon.co.za/partners/</t>
+          <t>https://saice.org.za/awards-2025/</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>South Africa Policy Hackathon Hello Ladies, Happy New Year. Some of you may be interested in this workshop. The workshop is flagged for South African nationals working at research and innovation offices, accelerators, innovation hubs and incubators, tech centers, and start-ups working on dual-use...</t>
+          <t>Learn about SAICE's award categories, submission guidelines, key dates and how to nominate project and professionals.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr"/>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>accounts@saice.org.za, civilinfo@saice.org.za, communications@saice.org.za, membership@saice.org.za, marketing@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Build the Future with Entelect Hackathons</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://challenge.entelect.co.za/</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Build the Future with Entelect Hackathons Join South Africa’s premier optimisation-first developer competition platform. Compete, iterate, and outperform the best.</t>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
@@ -2711,52 +2703,636 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Young Engineers Movement (YEM) - ORT SA</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
+          <t>info@ieomsociety.org</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>MICT SETA National Skills Challenge 2026 | Empowering ...</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://www.cxia4irhack.co.za/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Mar 27, 2026 · The MICT SETA National Skills Challenge 2026 is a 2-day innovation sprint that brings together students from universities and colleges across South Africa to solve real industry challenges through technology, creativity, and collaboration. Tackling real-world challenges in manufacturing, engineering, and technology through collaborative innovation.</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Competitions South Africa - Live Giveaways &amp; Prize Draws | Freehub</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>https://freehub.co.za/competitions/</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Browse live South African competitions, giveaways and prize draws. Find car, cash, voucher, tech and holiday competitions with clear entry rules and official source links.</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>The Department of Trade Industry and Competition</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>https://www.thedtic.gov.za/</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>The Minister of Trade, Industry and Competition, Mr Parks Tau has categorically reiterated that transformation and economic inclusion are moral and economic imperatives central to South Africa's democratic political order.</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>ThedticRFQenquiries@thedtic.gov.za, contactus@thedtic.gov.za, CGumede@thedtic.gov.za, VZitha@thedtic.gov.za, ERafapa@thedtic.gov.za, rajeshri@thedtic.gov.za, PKonza@thedtic.gov.za, NGovender@thedtic.gov.za, ALeGrange@thedtic.gov.za, SNgonyama@thedtic.gov.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>PDF Apply Now! Worldskills South Africa National Competition 2025</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>SAIMechE</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>https://www.saimeche.org.za/</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>South African Institute of Electrical Engineers</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>https://www.saiee.org.za/</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>South African Institute of Electrical Engineers (SAIEE) About Us See Member Benefits · Become a SAIEE Member today! SAIEE Membership · Earn CPD credits · About Training Academy · Join a SAIEE Centre near you! Centres · South African Institute of Electrical Engineers (SAIEE) 01 ·</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>reception@saiee.org.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>How to compete at the WSZA National Competitions 2025</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>ASTEMI Competitions – SAASTA</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Apr 30, 2026 · IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa) Deadline: April 30, 2026 May 15, 2026</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Competitions | ESG</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>https://za.rs-online.com/web/content/m/competition</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>example@email.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Home | Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>https://ebe.uct.ac.za/department-electrical-engineering</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>At the UCT Department of Electrical Engineering we are at the cutting edge of research and teaching, not just locally, but across Africa and globally. Become a part of our creative and stimulating degree programmes where students learn to solve known problems and conceive responses to challenges that have not yet been recognised.</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - SAIEE National Student Project Competition</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>https://www.saiee.org.za/calendar/EventDetails.aspx?eeid=29281</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>The SAIEE National Students Project Competition will be held at the North-West University (Potchefstroom Campus) on 21 November 2019</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>At the Centre for High Performance Computing (CHPC) Conference hosted in Cape Town at the end of last year, four current fourth-year electrical engineering students were crowned national champions in the Student Cluster Competition for 2025.</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>https://hackon.co.za/</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
+      <c r="E112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Hackathons en South Africa</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>https://za.allhackathons.com/</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Aug 22, 2025 · Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>AI Hackathon | Sebaka</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>https://sebakasouthafrica.co.za/index.html</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Sebaka Mentorship &amp; Hackathons — Build an AI Agent for Software Quality Engineering.</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>ICEP - Tshwane Varsity Hackathon</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>https://tvh.icep.co.za/</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Tshwane Varsity Hackathon South Africa's premier inter-university hackathon competition. Join hundreds of students for 53 hours of coding, innovation, and`` fun!</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>info@tvh.co.za, MagasengQM@tut.ac.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>https://hackon.co.za/partners/</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>South Africa Policy Hackathon Hello Ladies, Happy New Year. Some of you may be interested in this workshop. The workshop is flagged for South African nationals working at research and innovation offices, accelerators, innovation hubs and incubators, tech centers, and start-ups working on dual-use...</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Young Engineers Movement (YEM) - ORT SA</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>marketing@ortsa.org.za, info@ortsa.org.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>CompeteHub - Where Champions Are Made</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>https://www.devpluxe.co.za/</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>About DevPluxe Empowering South Africa ' s next generation of innovators We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update competition data 2026-08-19
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E118"/>
+  <dimension ref="A1:E121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Sep 4, 2025 · 3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -464,26 +464,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ASTEMI is a collaboration that ... &amp; Competitions to a broader base of learners and educators. ASTEMI is a national non-profit organization of independent organizations; teachers, public organisations and volunteers dedicated to improving and promoting science education and providing recognition for outstanding achievement by both learners and teachers. To promote excellence in Science, Technology, Engineering, Mathematics and Innovation in South African ...</t>
+          <t>Sep 4, 2025 · 3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -491,22 +487,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Some of our sparkling achievements ... and competitions. The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the · National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation ...</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -514,22 +514,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -546,17 +550,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -564,26 +568,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Faculty of Engineering Students to Represent South Africa at ...</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.su.ac.za/en/innovus/news/faculty-engineering-students-represent-south-africa-global-space-competition?language=en</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Apr 15, 2026 · The competition offers the team an opportunity to showcase South African engineering talent on an international stage while benchmarking their skills against global peers. Beyond the event, the team aims to bring back new knowledge and inspiration, contributing to the growth of local expertise in space science and engineering.</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa. Find out more</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -596,17 +596,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
+          <t>2 weeks ago - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -619,17 +619,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
+          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2 weeks ago - South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
+          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -642,17 +642,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>VUT inspires future engineers through Bridge Building Competition – Vaal University of Technology</t>
+          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://vut.ac.za/vut-inspires-future-engineers-through-bridge-building-competition/</t>
+          <t>https://www.poidata.io/report/engineer/south-africa</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>3 weeks ago - Supported by the ArcelorMittal Science Centre, Institution of Structural Engineers (IStructE), Fundi, South African Institution of Civil Engineering Future Leaders Panel (SAICE FLP) Vaal and maVuti Shop, the initiative challenged learners to design and construct bridge models using simple ...</t>
+          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -665,17 +665,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
+          <t>Two South Africans on the shortlist for the 2026 Africa Prize for Engineering Innovation</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://www.poidata.io/report/engineer/south-africa</t>
+          <t>https://www.engineeringnews.co.za/article/two-south-africans-on-the-shortlist-for-the-2026-africa-prize-for-engineering-innovation-2026-08-04</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>June 22, 2026 - Our comprehensive list of 1,582 Engineers in South Africa empowers you to reach the right audience through multiple channels. Here are key ways this data can give you a competitive edge in the Engineers industry.</t>
+          <t>2 weeks ago - Two South African innovators have been shortlisted for the UK Royal Academy of Engineering’s Africa Prize for Engineering Innovation 2026. This is the continent’s richest award aimed at promoting engineering innovation and entrepreneurship ...</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -683,12 +683,16 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>newsletters@creamermedia.co.za, advertising@creamermedia.co.za, newsdesk@engineeringnews.co.za, subscriptions@creamermedia.co.za, chanel@engineeringnews.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show ...</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -698,7 +702,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AI Expo Africa 2026 - Join the Largest AI Event &amp; Trade Community in Africa TODAY! Our business audience is a buyer / supplier focused community and comprised of Enterprise decision makers / CxOs, allied to AI Cloud platform providers, Tier 1 / 2 deployment &amp; service providers, AI start ups / innovators, investors, educators, government and AI ecosystem community builders.</t>
+          <t>AI Expo Africa 2026 – Join the Largest AI Event &amp; Trade Community in Africa TODAY! Our business audience is a buyer / supplier focused community and comprised of Enterprise decision makers / CxOs, allied to AI Cloud platform providers, Tier 1 / 2 deployment &amp; service providers, AI start ups / innovators, investors, educators, government and AI ecosystem community builders.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -715,17 +719,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Africa Tech Festival</t>
+          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://innovationweek.co.za/</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
+          <t>SA Innovation Week 2026 is South Africa’s official national innovation platform accelerating implementation, commercialisation and impact.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -735,24 +739,24 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>customerservices@informaconnect.com, salesenquiries@africatechfestival.com, support@informaconnect.com, customerservices@knect365.com, dataprivacy@knect365.com, dataprivacy@informaconnect.com, support@knect365.com</t>
+          <t>info@pixal8media.co.za</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Exhibitions in South Africa 2026-2027 - ExpoTobi</t>
+          <t>Innovations events in South Africa 2026-2027 - ExpoTobi</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://expotobi.com/country/south-africa/exhibitions</t>
+          <t>https://expotobi.com/country/south-africa/sector/innovations</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>All Exhibitions in South Africa 2026-2027 | Full and accurate description of events for various business sectors | Schedule, tickets, travel arrangements and participation</t>
+          <t>Innovations events in South Africa Full and accurate description of Innovations events Schedule, tickets, accommodation, travel arrangement and participation</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -765,17 +769,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
+          <t>Exhibitions in South Africa 2026-2027 - ExpoTobi</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://innovationweek.co.za/</t>
+          <t>https://expotobi.com/country/south-africa/exhibitions</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SA Innovation Week 2026 is South Africa's official national innovation platform accelerating implementation, commercialisation and impact.</t>
+          <t>7 hours ago · All Exhibitions in South Africa 2026-2027 | Full and accurate description of events for various business sectors | Schedule, tickets, travel arrangements and participation</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -783,26 +787,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>info@pixal8media.co.za</t>
-        </is>
-      </c>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>South Africa International Industrial Expo | Innovation Bridge</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -815,17 +815,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>DigiMarCon Africa 2027 - Cape Town, South Africa · October 6</t>
+          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://digimarconafrica.com/</t>
+          <t>https://madeinafricaevent.co.za/</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>The Premier Digital Marketing, Media and Advertising Conference &amp; Exhibition held annually in Cape Town, South Africa! Join your peers for 2 days jam packed with digital marketing best practices, latest trends and strategy, also check out the next generation of technology &amp; innovation; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year ...</t>
+          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -833,16 +833,12 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>info@digimarconafrica.com</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Manufacturing Indaba Exhibition 2026 - Manufacturing Expo</t>
+          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -852,7 +848,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Manufacturing Indaba Exhibition 2026: Africa's leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
+          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -865,17 +861,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 - Technology Expo · October 6</t>
+          <t>Two landmark exhibitions set to transform industrial technology and renewable energy in South Africa</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://www.engineeringnews.co.za/article/two-landmark-exhibitions-set-to-transform-industrial-technology-and-renewable-energy-in-south-africa-2025-10-24</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Where Business, Tech and Innovation Collide in Cape Town! TECHSPO Cape Town is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology.</t>
+          <t>October 24, 2025 - South Africa’s industrial and clean energy sectors celebrated a landmark moment today with the official launch of RE+ South Africa 2026 and the Cape Industrial Technology Exhibition (CITE) 2027.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -885,24 +881,24 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>info@techspocapetown.co.za</t>
+          <t>newsletters@creamermedia.co.za, advertising@creamermedia.co.za, newsdesk@engineeringnews.co.za, subscriptions@creamermedia.co.za, chanel@engineeringnews.co.za</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TECHSPO Joburg 2026 - Technology Expo · October 10</t>
+          <t>KZN Industrial Technology Exhibition</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://techspojoburg.co.za/</t>
+          <t>https://www.kznindustrial.co.za/</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
+          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -912,24 +908,24 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>info@techspojoburg.co.za</t>
+          <t>john@email.com</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Home - AWIEF</t>
+          <t>Exhibition | Innovation Festival Durban | South Africa</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.awieforum.org/</t>
+          <t>https://www.innovationfestival.durban/exhibition</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>"Events like AWIEF bring together private sector leaders, government, policymakers, and entrepreneurs to unlock real opportunities for women and youth, and to turn Africa's prosperity potential into reality."</t>
+          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -939,24 +935,24 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>info@awieforum.org</t>
+          <t>8c4075d5481d476e945486754f783364@sentry.io, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, Erika@innovate.durban, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, sithabile@innovate.durban, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
+          <t>Engineering For People Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
+          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
+          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -964,7 +960,11 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
+          <t>In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community's challenges and how community members view the impact of these challenges on their daily lives.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -989,24 +989,24 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
+          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EWB Design Challenge | Aston University</t>
+          <t>Engineering for People Design Challenge - Engineers Without Borders UK</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
+          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
+          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1019,17 +1019,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
+          <t>Engineering for People Design Challenge | Department of Engineering</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
+          <t>This year's design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but under-resourced neighbourhood on the eastern edge of Johannesburg. Home to around 46,000 people, Makers Valley is a community rich in creativity, activism ...</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1039,24 +1039,24 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ied@ied.org.uk</t>
+          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Latest Community Engineering Design Competition Announced</t>
+          <t>Engineering for People Design Challenge returns to Johannesburg!</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
+          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
+          <t>Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1069,17 +1069,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Engineering for people, that’s the challenge | Engineers Without Borders</t>
+          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://www.rs-online.com/designspark/an-introduction-to-engineering-for-people-design-challenge</t>
+          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>That’s exactly what the annual Engineering for People Design Challenge asks participants to do. The competition, delivered in partnership by Engineers without Borders South Africa and Engineers Without Borders UK, encourages engineering students and those collaborating with engineers to broaden their awareness of how their decisions change the world.</t>
+          <t>The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1087,22 +1087,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>team@crowdsolve.net</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Real-world research: Engineering team designs South African trolley system; science students investigate heavy metals | University of Wisconsin - Stout</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>May 15, 2025 - Research ranged from heavy metals ... Borders’ international design challenge. Nearly 90 students in 23 teams addressed the EWB challenge. One group focused on engineering a safer, more accessible transportation system in South ...</t>
+          <t>STEM-focused NGO Engineers Without Borders UK has launched its 2025 Engineering for People Design Challenge. Organised in conjunction with sister organisation Engineers Without Borders South Africa, as well as the Makers Valley Partnership, this year's challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1110,26 +1114,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>dolanm@uwstout.edu, frischj@uwstout.edu</t>
-        </is>
-      </c>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of Engineering</t>
+          <t>Engineers Without Borders | OU Design Show 2025</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://www.oudesignshow.org/designathon</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
+          <t>Makers Valley is a vibrant community of makers, creatives, and social enterprises in Johannesburg, South Africa. Engineers Without Borders UK has partnered with Makers Valley to engage students in design challenges focused on addressing local challenges and promoting sustainable development.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1137,26 +1137,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>web-editor@eng.cam.ac.uk, marketing@eng.cam.ac.uk</t>
-        </is>
-      </c>
+      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Inspiring, building and shaping a future fit engineering community – EWB-I</t>
+          <t>EWB-SA: Mid-Year Update - LinkedIn</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.ewb-international.org/home/inspiring-building-and-shaping-a-future-fit-engineering-community/</t>
+          <t>https://www.linkedin.com/pulse/ewb-sa-mid-year-update-ewbsa-uxo9f</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>February 27, 2025 - The challenge, delivered during ... career, encourages individuals to broaden their awareness of the social, environmental and economic implications of their engineering solutions. Since 2011, the Design Challenge has been delivered in Cameroon, South Africa, the UK and Ireland and the USA to over 70,000 students...</t>
+          <t>We wrapped up an extraordinary cycle of the 2023/24 Engineering for People Design Challenge in December 2024, with students across South Africa applying their creativity and empathy to solve real ...</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1164,26 +1160,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>admin@ewb-international.org</t>
-        </is>
-      </c>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
+          <t>Seven Cape Town Learners Just Won Gold At NASA</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
+          <t>https://www.2oceansvibe.com/technology/seven-cape-town-learners-just-won-gold-at-nasa/</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
+          <t>The South African team competed alongside 238 learners from 17 countries, with the final challenge requiring teams to produce a complete settlement design in roughly 48 hours and then pitch it to a client in a simulation designed to mirror the way real aerospace companies work.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1196,17 +1188,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
+          <t>University of Pretoria Faculty of Engineering, the Built Environment and Information Technology - Wikipedia</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
+          <t>https://en.wikipedia.org/wiki/University_of_Pretoria_Faculty_of_Engineering,_the_Built_Environment_and_Information_Technology</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
+          <t>June 18, 2026 - The university organises the annual SAE International sanctioned student automotive engineering Baja SAE competition in South Africa sponsored by Sasol. All undergraduate student participate in a compulsory community based project module as part of the university's wider community engagement ...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1219,17 +1211,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
+          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1242,17 +1234,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
+          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
+          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
+          <t>Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1265,17 +1257,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1311,17 +1303,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2025</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
+          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2025</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1357,17 +1349,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
+          <t>University Overall Rankings - Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
+          <t>University Overall Rankings - Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1380,17 +1372,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>University of South Africa</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
+          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-promotes-globally-recognised-engineering-qualifications</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>Unisa promotes globally recognised engineering qualifications</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1403,17 +1395,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>5 Best Universities to Study Engineering in South Africa</t>
+          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://globalscholarships.com/best-universities-engineering-south-africa/</t>
+          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>May 9, 2026 - Its diplomas and BEngTech degrees can support routes to registration with the Engineering Council of South Africa as engineering technicians or engineering technologists after the required practical experience. ... Degree/s Offered: Bachelor’s, Master’s, Ph.D. South Africa’s oldest university, the University of Cape Town, is one of the best engineering schools in South Africa.</t>
+          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1473,24 +1465,24 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>customerservices@informaconnect.com, salesenquiries@africatechfestival.com, support@informaconnect.com, customerservices@knect365.com, dataprivacy@knect365.com, dataprivacy@informaconnect.com, support@knect365.com</t>
+          <t>customerservices@informaconnect.com, support@informaconnect.com, dataprivacy@knect365.com, salesenquiries@africatechfestival.com, customerservices@knect365.com, support@knect365.com, dataprivacy@informaconnect.com</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7 ...</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://10times.com/johannesburg-za/technology</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>4 days ago · Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>Where Business, Tech and Innovation Collide in Cape Town! TECHSPO Cape Town is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1498,22 +1490,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>info@techspocapetown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7 ...</t>
+          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://10times.com/johannesburg-za/technology</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Where Business, Tech and Innovation Collide in Cape Town! TECHSPO Cape Town is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
+          <t>7 hours ago · Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1521,11 +1517,7 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>info@techspocapetown.co.za</t>
-        </is>
-      </c>
+      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1540,7 +1532,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>2 days ago · Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1553,17 +1545,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 – Africa's biggest IT Conference and Expo</t>
+          <t>Home - Mediatech Africa | South Africa</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://www.mediatech.co.za/</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what’s next before everyone else does. Only 2,500 ...</t>
+          <t>Mediatech Africa is the continent’s largest trade expo for professional AV, media, broadcast, and live entertainment technology. For 25 years, it’s been the industry’s meeting place — where manufacturers, integrators, creatives, and decision-makers come together to connect, discover new tech, and do business.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1571,7 +1563,11 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>simon@mediatech.co.za, claire@mediatech.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1619,7 +1615,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>name@example.com, u003einfo@techspo.co, atinfo@techspo.coor</t>
+          <t>name@example.com, atinfo@techspo.coor, u003einfo@techspo.co</t>
         </is>
       </c>
     </row>
@@ -1646,24 +1642,24 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>info@sparkafrica.co, partner@africatechnologyexpo.com, johndoe@email.com</t>
+          <t>partner@africatechnologyexpo.com, johndoe@email.com, info@sparkafrica.co</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Home - Mediatech Africa | South Africa</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference - AI Expo Africa | 28 - 29 October SCC Johannesburg South Africa</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://www.mediatech.co.za/</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
+          <t>(2 Day Event) 28th-29th October 2026 Sandton Convention Centre, JHB, South Africa · AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade ...</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1673,7 +1669,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>simon@mediatech.co.za, claire@mediatech.co.za</t>
+          <t>enquiries@aiexpoafrica.com</t>
         </is>
       </c>
     </row>
@@ -1703,17 +1699,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Home | Makers Fest</t>
+          <t>Maker Faire - Wikipedia</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://www.makersfestival.co.za/</t>
+          <t>https://en.wikipedia.org/wiki/Maker_Faire</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>On 8 &amp; 9 November 2025 at The Ostrich in Cape Town, join 2,000+ visitors each day for maker demos, a curated market, and family activities. It's Africa's first hands-on festival for creativity and craftsmanship — and everything you make, you take home.</t>
+          <t>Maker Faire is a convention of do it yourself (DIY) enthusiasts established by Make magazine in 2006. Participants come from a wide variety of interests, such as robotics, 3D printing, computers, arts and crafts, and hacker culture.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1721,26 +1717,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, example@mysite.com, 8c4075d5481d476e945486754f783364@sentry.io, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, warren@makersfestival.co.za, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Makers Fair | Experience Culture - Join the Fair</t>
+          <t>Maker Faire Africa — Grokipedia</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://www.makersfair.co.za/</t>
+          <t>https://grokipedia.com/page/maker_faire_africa</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Discover Southern African arts, crafts, food, and wine at the Makers Fair. Join us for cultural celebration and early ticket updates in Johannesburg 2026.</t>
+          <t>Maker Faire Africa Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1748,26 +1740,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>user@domain.com</t>
-        </is>
-      </c>
+      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>About | Explore Unique Maker Culture — Join Now — Makers Fair</t>
+          <t>Upcoming Faires - Maker Faire</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://www.makersfair.co.za/about</t>
+          <t>https://makerfaire.com/upcoming-faires/</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Discover South African and Pan-African craftsmanship at Makers Fair, a women-led event celebrating sustainable design, art, and culture. Join us today!</t>
+          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1777,7 +1765,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>user@domain.com</t>
+          <t>pr@make.co, fancybox_sprite@2x.png, chosen-sprite@2x.png, fancybox_loading@2x.gif</t>
         </is>
       </c>
     </row>
@@ -1804,24 +1792,24 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>pr@make.co, fancybox_loading@2x.gif, fancybox_sprite@2x.png, chosen-sprite@2x.png</t>
+          <t>pr@make.co, fancybox_sprite@2x.png, chosen-sprite@2x.png, fancybox_loading@2x.gif</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Makers Festival SA | Cape Town - Facebook</t>
+          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/61574201023378/</t>
+          <t>https://capetown.makerfaire.com/</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Makers Festival SA , Cape Town. 1,474 likes · 2 talking about this · 8 were here. Africa's first festival of creativity, craftsmanship &amp; community. Makers, live demos, food, music &amp; workshops for...</t>
+          <t>Jump into the Make: community and bring a Maker Faire to your town, city, or region! Spark curiosity, rally makers of all ages, and plug your local scene into a global movement fueled by creativity, resilience, innovation, and hands-on learning.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1829,22 +1817,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>pr@make.co, fancybox_sprite@2x.png, chosen-sprite@2x.png, fancybox_loading@2x.gif</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Upcoming Faires - Maker Faire</t>
+          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://makerfaire.com/upcoming-faires/</t>
+          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
+          <t>DIRECTIONS THE CAPE TOWN MAKER FAIRE The Lookout, V&amp;A Waterfront Granger Bay Boulevard, V &amp; A Waterfront, Cape Town, 8002, South Africa Get Directions Fri Aug 21, 13:00 - Sun Aug 23, 17:00 The Lookout, V&amp;A Waterfront View Map Payments are secure and encrypted</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1852,26 +1844,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>pr@make.co, fancybox_loading@2x.gif, fancybox_sprite@2x.png, chosen-sprite@2x.png</t>
-        </is>
-      </c>
+      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Makers Festival South Africa 2025 - Child Magazine</t>
+          <t>Home | Makers Fest</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://www.childmag.co.za/etn/makers-festival-south-africa-2025/</t>
+          <t>https://www.makersfestival.co.za/</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Makers Festival South Africa 2025 Africa's first festival of creativity, craftsmanship &amp; community. Makers, live demos, food, music &amp; workshops for all ages. Craft. Create. Connect. The first of its kind in Africa, Makers Festival is a groundbreaking celebration of creativity, craftsmanship, and community.</t>
+          <t>On 8 &amp; 9 November 2025 at The Ostrich in Cape Town, join 2,000+ visitors each day for maker demos, a curated market, and family activities. It's Africa's first hands-on festival for creativity and craftsmanship — and everything you make, you take home.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1879,22 +1867,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>8c4075d5481d476e945486754f783364@sentry.io, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, example@mysite.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, warren@makersfestival.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
+          <t>MakeAfrica - Le festival africain de l'innovation technologique et de ...</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://capetown.makerfaire.com/</t>
+          <t>https://makeafrica.tech/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Jump into the Make: community and bring a Maker Faire to your town, city, or region! Spark curiosity, rally makers of all ages, and plug your local scene into a global movement fueled by creativity, resilience, innovation, and hands-on learning.</t>
+          <t>Le festival africain de l'innovation technologique et de la culture maker Un événement africain pensé par des africains et qui vise à partager, créer, fabriquer et apprendre les uns des autres. Il regroupe stands de démonstration, ateliers de découverte, présentations et conférences autour des sujets liés à l'innovation, la créativité, la fabrication, le numérique, les ...</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1904,24 +1896,24 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>pr@make.co, fancybox_loading@2x.gif, fancybox_sprite@2x.png, chosen-sprite@2x.png</t>
+          <t>contact@makeafrica.tech</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Makers Festival SA - Whats on in Cape Town</t>
+          <t>Maker Faire groups | Meetup</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://whatsonincapetown.com/event/makers-festival-sa/</t>
+          <t>https://www.meetup.com/topics/maker-faire/za/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Makers Festival SA Event information The first of its kind in Africa, Makers Festival is a groundbreaking celebration of creativity, craftsmanship, and community. Bringing together artists, makers, and craftsmen from across the country, it's more than just a festival — it's the start of something big. What sets it apart?</t>
+          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1934,7 +1926,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1957,17 +1949,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>STEM Scholars — 2026 STEM &amp; Entrepreneurship Discovery Initiative</t>
+          <t>High School STEM Competition | Capetown 2026</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://stemscholars.co.za/</t>
+          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Building South Africa's Next Generation of Innovators The STEM &amp; Entrepreneurship Discovery Initiative connects learners with a world that's often invisible from inside a classroom — and equips them with skills that last far beyond the competition.</t>
+          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the 'first author'. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1977,24 +1969,24 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>marushka@stemscholars.co.za, inforeg@justice.gov.za, you@school.co.za</t>
+          <t>info@ieomsociety.org</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.samsung.com/za/solvefortomorrow/</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2007,17 +1999,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ASTEMI SA</t>
+          <t>South African Space Design Competition | Inspire Space Innovation ...</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
+          <t>Join the South African Space Design Competition to inspire space innovation, develop STEM skills, and compete for a trip to NASA. Perfect for high school students passionate about space.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2025,22 +2017,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>user@domain.com, info@zasdc.org</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Capetown 2026</t>
+          <t>Astemi Sa</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
+          <t>https://www.astemi.co.za/</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the ‘first author’. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
+          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2048,26 +2044,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/za/solvefortomorrow/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2080,17 +2072,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>StemCo - StemCo 2026 International Competitions</t>
+          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://stemco.org/</t>
+          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>June 10, 2026 - BEST YOURSELF WITH STEMCO! Platform for the world’s brightest. ... Thanks to the participating 25 countries in 2019. Singapore, Albania, Australia, Azerbaijan, Canada, Germany, India, Indonesia, Japan, Jordan, Kazakhstan, Kyrgyzstan, Malawi, Mongolia, Nigeria, Myanmar, South Africa, Tajikistan, Turkey, Turkmenistan, Ukraine, The United States, Uzbekistan, Vietnam</t>
+          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2103,17 +2095,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Southafrica 2024</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, ...</t>
+          <t>The IEOM High School/Middle School STEM Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2130,17 +2122,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Samsung opens Solve for Tomorrow 2026 STEM competition to all South African public schools</t>
+          <t>Applications for 2026 Samsung Solve For Tomorrow Now Open!</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
+          <t>https://news.samsung.com/za/applications-for-2026-samsung-solve-for-tomorrow-now-open</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>February 27, 2026 - Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
+          <t>The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries open until 06 March 2026. This is a transformative ...</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2153,17 +2145,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions 2022 – SAASTA</t>
+          <t>Register your school for Samsung Solve for Tomorrow 2026</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://saasta.ac.za/astemi-competitions-2</t>
+          <t>https://www.sowetan.co.za/careers/2026-03-03-register-your-school-for-samsung-solve-for-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>Register your school for Samsung Solve for Tomorrow 2026 STEM competition aims to transform and empower South African learners with critical skills to solve real-world challenges March 03, 2026 at 7:44 am</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2171,7 +2163,11 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ssasft@samsung.com</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2196,24 +2192,24 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
+          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
+          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
+          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>April 14, 2026 - This National Event, to be held at the Sandton Convention Centre in Johannesburg, South Africa, as part of AI for Good Impact Africa, at AI Expo Africa 2025, is a qualifying tournament leading to the Grand Finale in Geneva during the AI for ...</t>
+          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in the leading UN-based global robotics competition, focusing on the critical area of agriculture and food security.</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2223,24 +2219,24 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>name@example.com</t>
+          <t>8c4075d5481d476e945486754f783364@sentry.io, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, info@thecortexhub.africa, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>FIRST South Africa – Robotics Programs for School Children</t>
+          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://firstsa.org/</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way. FIRST Tech Challenge students learn to think like engineers. Teams ...</t>
+          <t>April 14, 2026 - This National Event, to be held at the Sandton Convention Centre in Johannesburg, South Africa, as part of AI for Good Impact Africa, at AI Expo Africa 2025, is a qualifying tournament leading to the Grand Finale in Geneva during the AI for ...</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2248,22 +2244,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>name@example.com</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>WorldSkillsZA Mobile Robotics Provincial Competition 2024</t>
+          <t>Robotics for Good Youth Challenge South Africa</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://worldskillsza.dhet.gov.za/site/WSZA-Prov-Comp/Provincial-Competitions.aspx</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa/</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>The WorldSkills South Africa (WSZA) will be having its Mobile Robotics Combined Provincial Competitions in Lephalale TVET College from the 07th - 10th October 2023. the first 3 days will be focused on training and the last day will be the actual Mobile Robotics competition.</t>
+          <t>Apr 25, 2025 · The Robotics for Good Youth Challenge South Africa is a national event in a global robotics competition on disaster response, leading to the AI for Good Summit 2025.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2271,22 +2271,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>name@example.com</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
+          <t>Roboticon 2026: South Africa Showcases Robotics for Culture ...</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
+          <t>https://www.ubuntutimes.co.za/roboticon-2026-south-africa-showcases-robotics-for-culture-education-and-innovation/</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
+          <t>Jul 2, 2026 · The event, partnered with the World Robotics Olympiad, positions South Africa as a leader in educational robotics and entrepreneurial innovation.” South Africa’s robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2294,22 +2298,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>newspaper-rec300@2x.jpg, adverts@ubuntutimes.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>South African Robotics Competitions and Schools</t>
+          <t>African Youth in Artificial Intelligence and Robotics</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://www.sciencexpo.org.za/robotics.html</t>
+          <t>https://ele-vate.co.za/african-youth-in-artificial-intelligence-and-robotics</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
+          <t>In partnership with the Government of the Republic of South Africa, the Second Edition of the Presidential African Youth in Artificial Intelligence and Robotics competition 2025 was hosted in Cape Town, South Africa.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2319,24 +2327,24 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>marna.vanzyl@imbewu.foundation, webmaster@sciencexpo.org.za, madelien@imbewu.foundation</t>
+          <t>innovationhub@ele-vate.co.za</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Limpopo Learners Represent South Africa at Global Robotics Finals in Switzerland - African Times</t>
+          <t>FIRST South Africa – Robotics Programs for School Children</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://www.atnews.co.za/limpopo-learners-represent-south-africa-at-global-robotics-finals-in-switzerland/</t>
+          <t>https://firstsa.org/</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>July 7, 2026 - The international competition, taking place from 7 to 10 July 2026 at the Palexpo International Exhibition and Convention Centre in Geneva, brings together some of the world’s brightest young innovators to develop technological solutions to ...</t>
+          <t>From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way. FIRST Tech Challenge students learn to think like engineers. Teams ...</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2349,17 +2357,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - AfrikaBot</t>
+          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/displaycustomlink.aspx?name=AfrikaBot</t>
+          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>AfrikaBot is affordable because you can build a competitive robot for a lot less with the correct advice. AfrikaBOT is South Africa's first robotics competition for high school teenagers and university undergraduates who are smart enough to build their own robots from electronic parts rather ...</t>
+          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2372,17 +2380,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
+          <t>South African Robotics Competitions and Schools</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
+          <t>https://www.sciencexpo.org.za/robotics.html</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge national competition will be held in Johannesburg, South Africa, at the Sandton Convention Centre on the 31st October 2025.</t>
+          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2392,24 +2400,24 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>info@thecortexhub.africa, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
+          <t>marna.vanzyl@imbewu.foundation, madelien@imbewu.foundation, webmaster@sciencexpo.org.za</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa - Limpopo - AI for Good</t>
+          <t>Limpopo Learners Represent South Africa at Global Robotics Finals in Switzerland - African Times</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-limpopo/</t>
+          <t>https://www.atnews.co.za/limpopo-learners-represent-south-africa-at-global-robotics-finals-in-switzerland/</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>December 8, 2025 - This Regional Event is a qualifying tournament leading to the Robotics for Good Youth Challenge South Africa National Event, to be held on 31 October at the Sandton Convention Centre in Johannesbourg, as part of AI for Good Impact Africa, at ...</t>
+          <t>July 7, 2026 - The international competition, taking place from 7 to 10 July 2026 at the Palexpo International Exhibition and Convention Centre in Geneva, brings together some of the world’s brightest young innovators to develop technological solutions to ...</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2419,24 +2427,24 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>name@example.com</t>
+          <t>rampedim@atnews.co.za, NkosiN@atnews.co.za</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE)</t>
+          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/SAICECIVIL/posts/-capture-engineering-excellencethe-2026-pps-photo-competition-is-now-open-for-en/1448856900617968/</t>
+          <t>https://safcec.org.za/</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>📸 Capture Engineering Excellence. The 2026 PPS Photo Competition is now open for entries! Whether you've captured engineering innovation in action, impressive infrastructure, or the people behind the profession, this is your chance to showcase civil engineering at its best.</t>
+          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2444,22 +2452,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>communication@safcec.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
+          <t>Competition Ts and Cs - SAICE</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://safcec.org.za/</t>
+          <t>https://saice.org.za/competition-ts-and-cs/</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
+          <t>Preamble These Terms and Conditions govern participation in the Know Your Sector Competition ("the Competition") conducted by the South African Institute of Civil Engineering ("SAICE"). Definitions SAICE: Shall mean the South African Institute of Civil Engineering. The Competition: Shall mean SAICE's Know Your Sector Competition. Entrant: Shall mean any individual who enters the ...</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2469,24 +2481,24 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>communication@safcec.org.za</t>
+          <t>accounts@saice.org.za, membership@saice.org.za, marketing@saice.org.za, communications@saice.org.za, civilinfo@saice.org.za</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ICE Africa - Supporting Civil Engineers in Africa</t>
+          <t>Civil Expo ITs 2026</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
+          <t>https://civilexpoits2026.com/</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>ICE Africa supports civil engineers across the continent, providing access to qualifications, training, and networking opportunities for professional growth.</t>
+          <t>Hi Cipo Pals! Civil Expo ITs 2026 Sovereign Structures, Resilient Societies This national civil engineering competition is your chance to put your engineering precision to the test and build real-world structural solutions. Step up and prove your skills on a national stage!</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2494,22 +2506,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>civilexpo.sipilits@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>SAICE's 34th International bridge competition inspires tomorrow's engineers</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://www.crown.co.za/africa-updates/33867-saice-s-34th-international-bridge-competition-inspires-tomorrow-s-engineers</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
+          <t>The South African Institution of Civil Engineering (SAICE) hosted its 34th International Bridge Building Competition at the Midrand Conference Centre, bringing together 21 teams of high school learners from across South Africa, alongside international participants from Eswatini, Uganda, and Zimbabwe.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2549,17 +2565,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>SAICE National Bridge Building Competition 2025 - avenue.co.za</t>
+          <t>Engineering the Future: 16 schools compete in SAICE's 33rd ...</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://www.avenue.co.za/post/saice-national-bridge-building-competition-2025</t>
+          <t>https://southafricatoday.net/lifestyle/education/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>SAICE initiated the National Bridge Building Competition in 1991, and 34 years later, this exciting competition is still an enormous success and enjoyed by learners across country.Did you know, many a civil engineer has referred to this very competition as the turning point in their decision to choose civil engineering as a career?There is considerable value in partnering with SAICE and ...</t>
+          <t>The South African Institution of Civil Engineering (SAICE) hosted its 33 rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland. The very first SAICE Bridge Building Competition was held in 1991, and it aimed to encourage high school learners to apply their knowledge of mathematics and science in a ...</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2567,26 +2583,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, barbara@avenue.co.za, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Home - SAICE</t>
+          <t>SAICE Aqualibrium 2025: High School Students Rise to the Challenge in ...</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://saice.org.za/</t>
+          <t>https://southafricatoday.net/environment/saice-aqualibrium-2025-high-school-students-rise-to-the-challenge-in-national-water-competition/</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) is the industry body for civil engineering professionals in South Africa. Our aim is to, promote growth, excellence and sustainability in the industry.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) hosted the thrilling 2025 Aqualibrium Competition National Finals this past week, which brought together high school students from schools all over South Africa at the Sci-Bono Discovery Centre in Johannesburg. The event continues to be an important platform for fostering engineering talent, inspiring young minds, and raising awareness ...</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2594,26 +2606,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>accounts@saice.org.za, civilinfo@saice.org.za, communications@saice.org.za, barbara@avenue.co.za, membership@saice.org.za, marketing@saice.org.za, executiveadmin@saice.org.za</t>
-        </is>
-      </c>
+      <c r="E88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>SAICE Aqualibrium 2025: High School Students Rise to the Challenge in ...</t>
+          <t>Home - SAICE</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://southafricatoday.net/environment/saice-aqualibrium-2025-high-school-students-rise-to-the-challenge-in-national-water-competition/</t>
+          <t>https://saice.org.za/</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) hosted the thrilling 2025 Aqualibrium Competition National Finals this past week, which brought together high school students from schools all over South Africa at the Sci-Bono Discovery Centre in Johannesburg. The event continues to be an important platform for fostering engineering talent, inspiring young minds, and raising awareness ...</t>
+          <t>The South African Institution of Civil Engineering (SAICE) is the industry body for civil engineering professionals in South Africa. Our aim is to, promote growth, excellence and sustainability in the industry.</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2621,22 +2629,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>accounts@saice.org.za, membership@saice.org.za, executiveadmin@saice.org.za, barbara@avenue.co.za, marketing@saice.org.za, communications@saice.org.za, civilinfo@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Home - cidb</t>
+          <t>SAICE Aqualibrium 2025: High School Students Rise to the Challenge in ...</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://www.cidb.org.za/</t>
+          <t>https://infrastructurenews.co.za/2025/05/14/saice-aqualibrium-2025-high-school-students-rise-to-the-challenge-in-national-water-competition/</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Partnering with you to achieve South Africa's construction industry success Established by Act 38 of 2000, cidb helps to transform the construction industry through inclusivity, high ethical standards, and amplifies contributions made by industry participants towards South Africa's economy and society.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) hosted the thrilling 2025 Aqualibrium Competition National Finals, which brought together high school students from schools all over South Africa at the Sci-Bono Discovery Centre.</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2644,26 +2656,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>Group-272@2x-300x270.jpg, Group-274@2x-300x269.jpg, Group-274@2x.jpg, Group-270@2x-300x270.jpg, Group-270@2x.jpg, Group-272@2x.jpg</t>
-        </is>
-      </c>
+      <c r="E90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Awards 2025 - SAICE</t>
+          <t>SAICE | Events and Awards</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://saice.org.za/awards-2025/</t>
+          <t>https://members.saice.org.za/events-and-awards</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Learn about SAICE's award categories, submission guidelines, key dates and how to nominate project and professionals.</t>
+          <t>The South African Institution Of Civil Engineering SAICE hosts the Awards Function annually to honour individuals, projects of excellence, as well as community-oriented initiatives. The annual awards function gives companies and individuals a unique opportunity to showcase their deserving projects and work to the industry.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2671,11 +2679,7 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>accounts@saice.org.za, civilinfo@saice.org.za, communications@saice.org.za, membership@saice.org.za, marketing@saice.org.za</t>
-        </is>
-      </c>
+      <c r="E91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2703,17 +2707,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2721,26 +2725,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2748,22 +2748,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2773,24 +2777,24 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+          <t>info@ieomsociety.org</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2803,17 +2807,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Competitions - Prized Competitions South Africa</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.prized.co.za/competitions/</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>Prized is home to Online Competitions in South Africa. Enter any competition that peaks your interest and join the Prized community.</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2821,26 +2825,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Competitions South Africa - Live Giveaways &amp; Prize Draws | Freehub</t>
+          <t>National Student Competition | ORSSA</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://freehub.co.za/competitions/</t>
+          <t>https://www.orssa.org.za/studentcomp</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Browse live South African competitions, giveaways and prize draws. Find car, cash, voucher, tech and holiday competitions with clear entry rules and official source links.</t>
+          <t>National Student Competitions The Operations Research Society of South Africa The home of decision intelligence The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2848,22 +2848,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, email@example.com</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>The Department of Trade Industry and Competition</t>
+          <t>PDF Apply Now! Worldskills South Africa National Competition 2025</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://www.thedtic.gov.za/</t>
+          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>The Minister of Trade, Industry and Competition, Mr Parks Tau has categorically reiterated that transformation and economic inclusion are moral and economic imperatives central to South Africa's democratic political order.</t>
+          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2871,26 +2875,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>ThedticRFQenquiries@thedtic.gov.za, contactus@thedtic.gov.za, CGumede@thedtic.gov.za, VZitha@thedtic.gov.za, ERafapa@thedtic.gov.za, rajeshri@thedtic.gov.za, PKonza@thedtic.gov.za, NGovender@thedtic.gov.za, ALeGrange@thedtic.gov.za, SNgonyama@thedtic.gov.za</t>
-        </is>
-      </c>
+      <c r="E99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>PDF Apply Now! Worldskills South Africa National Competition 2025</t>
+          <t>SAIMechE</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
+          <t>https://www.saimeche.org.za/</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
+          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2903,17 +2903,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>SAIMechE</t>
+          <t>Home - Icmeesa</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>https://www.saimeche.org.za/</t>
+          <t>http://icmeesa.org.za/</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
+          <t>Certificated Mechanical or Electrical Engineers in mining and factory are the professional engineering practitioners recognised by law in South Africa to accept legal responsibility to improve health and safety in mines and works. These Engineers need to provide solutions reliant on basic scientific, mathematical and engineering knowledge, supported by analysis and synthesis, and underpinned ...</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2921,22 +2921,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>info@icmeesa.org.za, icmeesa@icmeesa.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/</t>
+          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers (SAIEE) About Us See Member Benefits · Become a SAIEE Member today! SAIEE Membership · Earn CPD credits · About Training Academy · Join a SAIEE Centre near you! Centres · South African Institute of Electrical Engineers (SAIEE) 01 ·</t>
+          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2944,26 +2948,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>reception@saiee.org.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+      <c r="E102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - SAIEE National Student Project Competition</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://www.saiee.org.za/calendar/EventDetails.aspx?eeid=29281</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+          <t>The SAIEE National Students Project Competition will be held at the North-West University (Potchefstroom Campus) on 21 November 2019</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2976,17 +2976,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - IEEE ZA 5G Competition</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51397</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>Form templates: Template for a Cover Sheet for the Competition on Ideas, Designs and Applications for 5G and Beyond South Africa (.docx) [Click to Download] Template for a Resume for the Student (.docx) [Click to Download] ... Help (FAQ) • Privacy Statement • Terms &amp; Conditions The SAIEE is ...</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2999,17 +2999,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
+          <t>Student Design Competition | IEEE CASS</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
+          <t>https://ieee-cas.org/society-involvement/student-design-competition</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 · IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa) Deadline: April 30, 2026 May 15, 2026</t>
+          <t>East, Africa), Region 9 (Latin America), and Region 10 (Asia, Australia, Pacific), as well as ISCAS registration. The winning team will be awarded $3,000 USD. For details on how to participate in the 2026 Student Design Competition, click here. ... Undergraduate students would suggest and execute ...</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -3022,17 +3022,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Competitions | ESG</t>
+          <t>Top 100 Electrical Engineering Companies in South Africa (2026) | ensun</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://za.rs-online.com/web/content/m/competition</t>
+          <t>https://ensun.io/search/electrical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
+          <t>The competitive landscape is marked by both established firms and emerging startups, driving innovation and efficiency. Additionally, South Africa’s position in the broader global market allows for potential collaborations and export opportunities, particularly in green technologies. Understanding these factors is essential for anyone looking to engage with the Electrical Engineering ...</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -3040,26 +3040,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>example@email.com</t>
-        </is>
-      </c>
+      <c r="E106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>At the Centre for High Performance Computing (CHPC) Conference hosted in Cape Town at the end of last year, four current fourth-year electrical engineering students were crowned national champions in the Student Cluster Competition for 2025.</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3067,26 +3063,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Home | Electrical Engineering</t>
+          <t>Electrical Engineering Conferences in South Africa 2025/2026/2027 - Conference Index</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://ebe.uct.ac.za/department-electrical-engineering</t>
+          <t>https://conferenceindex.org/conferences/electrical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>At the UCT Department of Electrical Engineering we are at the cutting edge of research and teaching, not just locally, but across Africa and globally. Become a part of our creative and stimulating degree programmes where students learn to solve known problems and conceive responses to challenges that have not yet been recognised.</t>
+          <t>Electrical Engineering Conferences in South Africa 2025 2026 2027 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and ...</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3099,17 +3091,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
+          <t>7 Electrical Engineering Degree Programs in South Africa - Study Abroad | educations.com</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
+          <t>https://www.educations.com/electrical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
+          <t>Find the best fit for you - Compare 7 in Engineering Programs Electrical Engineering in South Africa for 2025/2026</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3122,17 +3114,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - SAIEE National Student Project Competition</t>
+          <t>Electrical And Electronics Engineering Conferences in South Africa 2026 | Conference Alerts</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/calendar/EventDetails.aspx?eeid=29281</t>
+          <t>https://conferencealerts.co.in/south-africa/electrical-and-electronics-engineering</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>The SAIEE National Students Project Competition will be held at the North-West University (Potchefstroom Campus) on 21 November 2019</t>
+          <t>Select your participation type (in-person, virtual, or hybrid), fill in your personal and professional details, and pay the registration fee if required. After registering, you’ll receive confirmation and access instructions. Some electrical and electronics engineering conferences in south africa also allow early-bird registration with discounted fees.</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3145,17 +3137,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>South African Institute of Electrical Engineers</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://www.saiee.org.za/</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>At the Centre for High Performance Computing (CHPC) Conference hosted in Cape Town at the end of last year, four current fourth-year electrical engineering students were crowned national champions in the Student Cluster Competition for 2025.</t>
+          <t>South African Institute of Electrical Engineers (SAIEE) About Us See Member Benefits · Become a SAIEE Member today! SAIEE Membership · Earn CPD credits · About Training Academy · Join a SAIEE Centre near you! Centres · South African Institute of Electrical Engineers (SAIEE) 01 ·</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3163,22 +3155,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>glueup-logo-white@2x.png, reception@saiee.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
+          <t>Hackathons en South Africa</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>https://hackon.co.za/</t>
+          <t>https://za.allhackathons.com/</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
+          <t>Aug 22, 2025 · Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -3191,17 +3187,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Hackathons en South Africa</t>
+          <t>AI Hackathon | Sebaka</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>https://za.allhackathons.com/</t>
+          <t>https://sebakasouthafrica.co.za/index.html</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Aug 22, 2025 · Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
+          <t>Sebaka Mentorship &amp; Hackathons — Build an AI Agent for Software Quality Engineering.</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -3214,17 +3210,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>AI Hackathon | Sebaka</t>
+          <t>Build the Future with Entelect Hackathons</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>https://sebakasouthafrica.co.za/index.html</t>
+          <t>https://challenge.entelect.co.za/</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Sebaka Mentorship &amp; Hackathons — Build an AI Agent for Software Quality Engineering.</t>
+          <t>Build the Future with Entelect Hackathons Join South Africa’s premier optimisation-first developer competition platform. Compete, iterate, and outperform the best.</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3237,17 +3233,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ICEP - Tshwane Varsity Hackathon</t>
+          <t>GirlCode | Hackathon 2026</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>https://tvh.icep.co.za/</t>
+          <t>https://www.girlcode.co.za/hackathon-2026</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Tshwane Varsity Hackathon South Africa's premier inter-university hackathon competition. Join hundreds of students for 53 hours of coding, innovation, and`` fun!</t>
+          <t>Building Africa's Next Generation of AI-Powered Female Innovators Join Africa's largest women-in-tech hackathon empowering innovators, creators, and future founders.</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3255,26 +3251,22 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>info@tvh.co.za, MagasengQM@tut.ac.za</t>
-        </is>
-      </c>
+      <c r="E115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
+          <t>Budding engineers showcase innovation at YEM hackathon | ITWeb</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>https://hackon.co.za/partners/</t>
+          <t>https://www.itweb.co.za/article/budding-engineers-showcase-innovation-at-yem-hackathon/kYbe97XbP4ZqAWpG</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>South Africa Policy Hackathon Hello Ladies, Happy New Year. Some of you may be interested in this workshop. The workshop is flagged for South African nationals working at research and innovation offices, accelerators, innovation hubs and incubators, tech centers, and start-ups working on dual-use...</t>
+          <t>June 30, 2026 - The hackathon was hosted by Johannesburg-based non-profit education and training organisation ORT South Africa, in partnership with JSE-listed industrial and engineering supplies firm Hudaco.</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -3282,22 +3274,26 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>enquiries@ombudsman.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Young Engineers Movement (YEM) - ORT SA</t>
+          <t>Young Engineers Shine as Inaugural YEM Hackathon Celebrates South Africa's Next Generation of Innovators</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
+          <t>https://novuspressbulletin.co.za/blog/young-engineers-shine-as-inaugural-yem-hackathon-celebrates-south-africa-s-next-generation-of-innovators</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
+          <t>June 30, 2026 - ... Johannesburg, June 2026 – After five inspiring days of innovation, collaboration, and problem-solving, the inaugural Young Engineers Movement (YEM) Hackathon, hosted by ORT South Africa in partnership with Hudaco, concluded with a vibrant ...</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3305,26 +3301,22 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t>marketing@ortsa.org.za, info@ortsa.org.za</t>
-        </is>
-      </c>
+      <c r="E117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>CompeteHub - Where Champions Are Made</t>
+          <t>Young Engineers Shine as Inaugural YEM Hackathon Celebrates South Africa's Next Generation of Innovators - Lifestyle &amp; Tech</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>https://www.devpluxe.co.za/</t>
+          <t>https://lifestyleandtech.co.za/company-news/article/2026-06-29/young-engineers-shine-as-inaugural-yem-hackathon-celebrates-south-africas-next-generation-of-innovators</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>About DevPluxe Empowering South Africa ' s next generation of innovators We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
+          <t>June 29, 2026 - After five inspiring days of innovation, collaboration, and problem-solving, the inaugural Young Engineers Movement (YEM) Hackathon, hosted by ORT South Africa in partnership with Hudaco, concluded with a vibrant exhibition showcasing the remarkable ...</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3333,6 +3325,83 @@
         </is>
       </c>
       <c r="E118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>ORT South Africa's inaugural YEM Hackathon empowers future STEM innovators</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>https://www.futuresa.co.za/bursaries-and-scholarships/ort-south-africa-yem-hackathon/</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>3 weeks ago - ORT South Africa's first Young Engineers Movement Hackathon saw 55 learners develop innovative STEM solutions during a five-day competition.</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>info@futuresa.co.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Houghton hackathon: Stepping stone for future engineers | Rosebank Killarney Gazette</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>https://www.citizen.co.za/rosebank-killarney-gazette/news-headlines/local-news/2026/06/23/houghton-hackathon-stepping-stone-for-future-engineers/</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>June 23, 2026 - Hosted by ORT South Africa in partnership with Hudaco, the hackathon has brought together 55 learners from underserved communities to work together in developing solutions to challenges they face in their communities.</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>55 learners from underserved schools showcase engineering innovations at Johannesburg hackathon</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>https://iol.co.za/saturday-star/2026-07-01-55-learners-from-underserved-schools-showcase-engineering-innovations-at-johannesburg-hackathon/</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>3 weeks ago - Fifty-five high school learners ... at the Young Engineers Movement (YEM) Hackathon Exhibition Day in Johannesburg last week, presenting working prototypes designed to solve real-world problems affecting their communities. The learners, accompanied by 11 teachers, took part in the five-day hackathon, hosted by ORT South Africa in partnership with Hudaco, from June 22 to 26....</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>yasmine.jacobs@iol.co.za, pholoso.manyama@iol.co.za, pholoso.manyama@inl.co.za, wendy.dondolo@inl.co.za, verna.vandiemen@inl.co.za</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update competition data 2026-08-20
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E121"/>
+  <dimension ref="A1:E106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,7 +456,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -479,7 +479,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sep 4, 2025 · 3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>Sep 4, 2025 · The Africa Prize for Engineering Innovation is open to individuals or teams based in sub-Saharan Africa who have a scalable engineering innovation with social or environmental impact potential.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -496,17 +496,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+          <t>Some of our sparkling achievements during 2014 – to help the NRF and DSI grow a representative science and technology workforce in the country – SAASTA has run a number of maths and science educator development programmes and a number of learner development programmes, including maths and science camps for learners with potential, olympiads and competitions. The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the · National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -514,26 +514,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -541,26 +537,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
+          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -573,17 +565,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa. Find out more</t>
+          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -596,17 +588,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
+          <t>National Student Competition | ORSSA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
+          <t>https://www.orssa.org.za/studentcomp</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2 weeks ago - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
+          <t>The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -614,22 +606,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, email@example.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
+          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
+          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
+          <t>2 weeks ago - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -685,24 +681,24 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>newsletters@creamermedia.co.za, advertising@creamermedia.co.za, newsdesk@engineeringnews.co.za, subscriptions@creamermedia.co.za, chanel@engineeringnews.co.za</t>
+          <t>subscriptions@creamermedia.co.za, chanel@engineeringnews.co.za, newsdesk@engineeringnews.co.za, advertising@creamermedia.co.za, newsletters@creamermedia.co.za</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show ...</t>
+          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://10times.com/southafrica/tradeshows</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AI Expo Africa 2026 – Join the Largest AI Event &amp; Trade Community in Africa TODAY! Our business audience is a buyer / supplier focused community and comprised of Enterprise decision makers / CxOs, allied to AI Cloud platform providers, Tier 1 / 2 deployment &amp; service providers, AI start ups / innovators, investors, educators, government and AI ecosystem community builders.</t>
+          <t>1 day ago · South Africa trade shows, find and compare 966 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 176 upcoming expos in 2026-2027 1. South Africa Infrastructure &amp; Water Expo, 2.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -710,11 +706,7 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>enquiries@aiexpoafrica.com</t>
-        </is>
-      </c>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -729,7 +721,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SA Innovation Week 2026 is South Africa’s official national innovation platform accelerating implementation, commercialisation and impact.</t>
+          <t>SAIW’ 26 is designed as a week-long national programme to feature provincial innovation engagements across South Africa. From 16 – 17 March, Provinces will showcase local innovation strengths, emerging enterprises and sectoral capabilities.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -769,17 +761,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Exhibitions in South Africa 2026-2027 - ExpoTobi</t>
+          <t>Africa Tech Festival</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://expotobi.com/country/south-africa/exhibitions</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>7 hours ago · All Exhibitions in South Africa 2026-2027 | Full and accurate description of events for various business sectors | Schedule, tickets, travel arrangements and participation</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -787,22 +779,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>dataprivacy@informaconnect.com, support@knect365.com, salesenquiries@africatechfestival.com, dataprivacy@knect365.com, customerservices@informaconnect.com, customerservices@knect365.com, support@informaconnect.com</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>South Africa International Industrial Expo | Innovation Bridge</t>
+          <t>IT &amp; Technology Events in South Africa, List of all South ...</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
+          <t>The BI + AI Innovation &amp; Tech Fest is a pioneering event that celebrates the intersection of Business Intelligence (BI) and Artificial Intelligence (AI), emphasizing the transformative power of technology...</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -815,17 +811,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
+          <t>South Africa International Industrial Expo | Innovation Bridge</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://madeinafricaevent.co.za/</t>
+          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
+          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -838,17 +834,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
+          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://manufacturingindaba.co.za/exhibition/</t>
+          <t>https://madeinafricaevent.co.za/</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
+          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -861,17 +857,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Two landmark exhibitions set to transform industrial technology and renewable energy in South Africa</t>
+          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/two-landmark-exhibitions-set-to-transform-industrial-technology-and-renewable-energy-in-south-africa-2025-10-24</t>
+          <t>https://manufacturingindaba.co.za/exhibition/</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>October 24, 2025 - South Africa’s industrial and clean energy sectors celebrated a landmark moment today with the official launch of RE+ South Africa 2026 and the Cape Industrial Technology Exhibition (CITE) 2027.</t>
+          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -879,26 +875,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>newsletters@creamermedia.co.za, advertising@creamermedia.co.za, newsdesk@engineeringnews.co.za, subscriptions@creamermedia.co.za, chanel@engineeringnews.co.za</t>
-        </is>
-      </c>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>KZN Industrial Technology Exhibition</t>
+          <t>Two landmark exhibitions set to transform industrial technology and renewable energy in South Africa</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://www.kznindustrial.co.za/</t>
+          <t>https://www.engineeringnews.co.za/article/two-landmark-exhibitions-set-to-transform-industrial-technology-and-renewable-energy-in-south-africa-2025-10-24</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
+          <t>October 24, 2025 - South Africa’s industrial and clean energy sectors celebrated a landmark moment today with the official launch of RE+ South Africa 2026 and the Cape Industrial Technology Exhibition (CITE) 2027.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -908,24 +900,24 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>john@email.com</t>
+          <t>subscriptions@creamermedia.co.za, chanel@engineeringnews.co.za, newsdesk@engineeringnews.co.za, advertising@creamermedia.co.za, newsletters@creamermedia.co.za</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Exhibition | Innovation Festival Durban | South Africa</t>
+          <t>KZN Industrial Technology Exhibition</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.innovationfestival.durban/exhibition</t>
+          <t>https://www.kznindustrial.co.za/</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities.</t>
+          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -935,24 +927,24 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>8c4075d5481d476e945486754f783364@sentry.io, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, Erika@innovate.durban, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, sithabile@innovate.durban, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com</t>
+          <t>john@email.com</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Engineering For People Design Challenge - EWBSA</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
+          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -960,26 +952,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
-        </is>
-      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>Engineering for People Design Challenge | Department of ...</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community's challenges and how community members view the impact of these challenges on their daily lives.</t>
+          <t>Aug 4, 2025 · The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -989,24 +977,24 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
+          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge - Engineers Without Borders UK</t>
+          <t>Engineering for People Design Challenge returns to Johannesburg!</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
+          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
+          <t>Sep 18, 2024 · Engineering for People Design Challenge returns to Johannesburg! Now entering its fourteenth year, we’re delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1019,17 +1007,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of Engineering</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>This year's design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but under-resourced neighbourhood on the eastern edge of Johannesburg. Home to around 46,000 people, Makers Valley is a community rich in creativity, activism ...</t>
+          <t>Oct 16, 2024 · Organised in conjunction with sister organisation Engineers Without Borders South Africa, as well as the Makers Valley Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1037,26 +1025,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
-        </is>
-      </c>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge returns to Johannesburg!</t>
+          <t>Engineering For People Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
+          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
+          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1069,17 +1053,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
+          <t>Engineering for People Design Challenge - Engineers Without ...</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
+          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
+          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1087,26 +1071,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>team@crowdsolve.net</t>
-        </is>
-      </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Latest Community Engineering Design Competition Announced</t>
+          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
+          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>STEM-focused NGO Engineers Without Borders UK has launched its 2025 Engineering for People Design Challenge. Organised in conjunction with sister organisation Engineers Without Borders South Africa, as well as the Makers Valley Partnership, this year's challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg.</t>
+          <t>Oct 24, 2024 · The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1114,22 +1094,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>team@crowdsolve.net</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Engineers Without Borders | OU Design Show 2025</t>
+          <t>EWB Design Challenge | Aston University</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.oudesignshow.org/designathon</t>
+          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Makers Valley is a vibrant community of makers, creatives, and social enterprises in Johannesburg, South Africa. Engineers Without Borders UK has partnered with Makers Valley to engage students in design challenges focused on addressing local challenges and promoting sustainable development.</t>
+          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1142,17 +1126,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>EWB-SA: Mid-Year Update - LinkedIn</t>
+          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/pulse/ewb-sa-mid-year-update-ewbsa-uxo9f</t>
+          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>We wrapped up an extraordinary cycle of the 2023/24 Engineering for People Design Challenge in December 2024, with students across South Africa applying their creativity and empathy to solve real ...</t>
+          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1160,22 +1144,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>ied@ied.org.uk</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Seven Cape Town Learners Just Won Gold At NASA</t>
+          <t>Real-world research: Engineering team designs South African trolley system; science students investigate heavy metals | University of Wisconsin - Stout</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.2oceansvibe.com/technology/seven-cape-town-learners-just-won-gold-at-nasa/</t>
+          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>The South African team competed alongside 238 learners from 17 countries, with the final challenge requiring teams to produce a complete settlement design in roughly 48 hours and then pitch it to a client in a simulation designed to mirror the way real aerospace companies work.</t>
+          <t>May 15, 2025 - Research ranged from heavy metals ... Borders’ international design challenge. Nearly 90 students in 23 teams addressed the EWB challenge. One group focused on engineering a safer, more accessible transportation system in South ...</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1183,22 +1171,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>frischj@uwstout.edu, dolanm@uwstout.edu</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>University of Pretoria Faculty of Engineering, the Built Environment and Information Technology - Wikipedia</t>
+          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/University_of_Pretoria_Faculty_of_Engineering,_the_Built_Environment_and_Information_Technology</t>
+          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>June 18, 2026 - The university organises the annual SAE International sanctioned student automotive engineering Baja SAE competition in South Africa sponsored by Sasol. All undergraduate student participate in a compulsory community based project module as part of the university's wider community engagement ...</t>
+          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1211,17 +1203,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
+          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
+          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
+          <t>Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1234,17 +1226,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
+          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1257,17 +1249,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
+          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1303,17 +1295,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1349,17 +1341,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2025</t>
+          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
+          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2025</t>
+          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1372,17 +1364,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>University of South Africa</t>
+          <t>University Overall Rankings - Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-promotes-globally-recognised-engineering-qualifications</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Unisa promotes globally recognised engineering qualifications</t>
+          <t>University Overall Rankings - Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1395,17 +1387,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1418,7 +1410,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 ...</t>
+          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1428,7 +1420,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
+          <t>February 20, 2026 - TECHSPO Johannesburg 2026 is a two day technology expo taking place September 28th to 29th, 2026 at the luxurious Hyatt Regency Johannesburg, Johannesburg, South Africa. TECHSPO Johannesburg brings together developers, brands, marketers, technology ...</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1465,14 +1457,14 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>customerservices@informaconnect.com, support@informaconnect.com, dataprivacy@knect365.com, salesenquiries@africatechfestival.com, customerservices@knect365.com, support@knect365.com, dataprivacy@informaconnect.com</t>
+          <t>dataprivacy@informaconnect.com, support@knect365.com, salesenquiries@africatechfestival.com, dataprivacy@knect365.com, customerservices@informaconnect.com, customerservices@knect365.com, support@informaconnect.com</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7 ...</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1482,7 +1474,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Where Business, Tech and Innovation Collide in Cape Town! TECHSPO Cape Town is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
+          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1499,17 +1491,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
+          <t>IT &amp; Technology Events in South Africa | 10times</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://10times.com/johannesburg-za/technology</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>7 hours ago · Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1522,17 +1514,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>Home - Mediatech Africa | South Africa</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://www.mediatech.co.za/</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2 days ago · Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>Mediatech Africa showcases the full range of professional tech driving AV, broadcast, media, &amp; live event production. From AV integration, unified communications &amp; display to pro audio, lighting, content creation, &amp; future tech — our sectors highlight the tools behind today’s connected experiences.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1545,17 +1537,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Home - Mediatech Africa | South Africa</t>
+          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://www.mediatech.co.za/</t>
+          <t>https://10times.com/johannesburg-za/technology</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Mediatech Africa is the continent’s largest trade expo for professional AV, media, broadcast, and live entertainment technology. For 25 years, it’s been the industry’s meeting place — where manufacturers, integrators, creatives, and decision-makers come together to connect, discover new tech, and do business.</t>
+          <t>6 days ago · Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1563,11 +1555,7 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>simon@mediatech.co.za, claire@mediatech.co.za</t>
-        </is>
-      </c>
+      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1582,7 +1570,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg is a 2-day technology expo taking place September 28 – 29, 2026 at the luxurious NH Johannesburg Sandton Hotel, Toronto, Ontario. TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
+          <t>TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1615,7 +1603,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>name@example.com, atinfo@techspo.coor, u003einfo@techspo.co</t>
+          <t>atinfo@techspo.coor, name@example.com, u003einfo@techspo.co</t>
         </is>
       </c>
     </row>
@@ -1642,24 +1630,24 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>partner@africatechnologyexpo.com, johndoe@email.com, info@sparkafrica.co</t>
+          <t>partner@africatechnologyexpo.com, info@sparkafrica.co, johndoe@email.com</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference - AI Expo Africa | 28 - 29 October SCC Johannesburg South Africa</t>
+          <t>IT Indaba 2026 – Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>(2 Day Event) 28th-29th October 2026 Sandton Convention Centre, JHB, South Africa · AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade ...</t>
+          <t>The inaugural 2025 IT Indaba promises to bring together 3,000+ IT professionals and tech influencers who are involved in the procurement of systems, tools, platforms and services, along with user experience developers who deal with the core processes and client interfaces of the business.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1667,11 +1655,7 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>enquiries@aiexpoafrica.com</t>
-        </is>
-      </c>
+      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1686,7 +1670,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Maker Faire Africa, Cairo, October 2011 Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds (Nubian Cheetah). Maker Faire Africa aims to engage with on ...</t>
+          <t>March 7, 2025 - Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds ...</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1732,7 +1716,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Maker Faire Africa Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
+          <t>Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1745,12 +1729,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Upcoming Faires - Maker Faire</t>
+          <t>Maker Faire |</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://makerfaire.com/upcoming-faires/</t>
+          <t>https://makerfaire.com/</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1765,24 +1749,24 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>pr@make.co, fancybox_sprite@2x.png, chosen-sprite@2x.png, fancybox_loading@2x.gif</t>
+          <t>fancybox_loading@2x.gif, chosen-sprite@2x.png, pr@make.co, fancybox_sprite@2x.png</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Maker Faire |</t>
+          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://makerfaire.com/</t>
+          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
+          <t>Aug 21, 2015 · We’re delighted to present the first ever Cape Town Maker Faire, hosted by Open Design in partnership with Trimble.Maker Faire is primarily designed as a forward-looking event, showcasing makers who are exploring new forms and new technologies.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1790,26 +1774,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>pr@make.co, fancybox_sprite@2x.png, chosen-sprite@2x.png, fancybox_loading@2x.gif</t>
-        </is>
-      </c>
+      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
+          <t>Maker Faire groups | Meetup</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://capetown.makerfaire.com/</t>
+          <t>https://www.meetup.com/topics/maker-faire/za/</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Jump into the Make: community and bring a Maker Faire to your town, city, or region! Spark curiosity, rally makers of all ages, and plug your local scene into a global movement fueled by creativity, resilience, innovation, and hands-on learning.</t>
+          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1817,26 +1797,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>pr@make.co, fancybox_sprite@2x.png, chosen-sprite@2x.png, fancybox_loading@2x.gif</t>
-        </is>
-      </c>
+      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
+          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
+          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>DIRECTIONS THE CAPE TOWN MAKER FAIRE The Lookout, V&amp;A Waterfront Granger Bay Boulevard, V &amp; A Waterfront, Cape Town, 8002, South Africa Get Directions Fri Aug 21, 13:00 - Sun Aug 23, 17:00 The Lookout, V&amp;A Waterfront View Map Payments are secure and encrypted</t>
+          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1849,17 +1825,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Home | Makers Fest</t>
+          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://www.makersfestival.co.za/</t>
+          <t>https://makerfairecapetown.wordpress.com/about/</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>On 8 &amp; 9 November 2025 at The Ostrich in Cape Town, join 2,000+ visitors each day for maker demos, a curated market, and family activities. It's Africa's first hands-on festival for creativity and craftsmanship — and everything you make, you take home.</t>
+          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1867,26 +1843,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>8c4075d5481d476e945486754f783364@sentry.io, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, example@mysite.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, warren@makersfestival.co.za</t>
-        </is>
-      </c>
+      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>MakeAfrica - Le festival africain de l'innovation technologique et de ...</t>
+          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://makeafrica.tech/</t>
+          <t>http://capetown.makerfaire.com/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Le festival africain de l'innovation technologique et de la culture maker Un événement africain pensé par des africains et qui vise à partager, créer, fabriquer et apprendre les uns des autres. Il regroupe stands de démonstration, ateliers de découverte, présentations et conférences autour des sujets liés à l'innovation, la créativité, la fabrication, le numérique, les ...</t>
+          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1896,24 +1868,24 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>contact@makeafrica.tech</t>
+          <t>fancybox_loading@2x.gif, chosen-sprite@2x.png, pr@make.co, fancybox_sprite@2x.png</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Maker Faire groups | Meetup</t>
+          <t>Blog : Maker Faire Africa</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/topics/maker-faire/za/</t>
+          <t>http://makerfaireafrica.com/blog/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
+          <t>December 31, 2021 - You can help them out on the new South African crowdfunding site, ThundaFund. ... One of the most ambitions items at Maker Faire Africa this year in Johannesburg, South Africa is Samuel Ngobeni’s “art car”. He’s a designer from Germinston, who has spent the last three years building his ANIMAL car, from the ground up, that means the frame and all.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1926,7 +1898,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1936,7 +1908,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>All these Olympiads and Competitions have a positive impact on education and on educational institutions in South Africa, but there is still a need to build stronger collaboration among teachers, schools, universities and educational authorities in order to meet the challenges of STEM education in South Africa today.</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1949,17 +1921,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Capetown 2026</t>
+          <t>Samsung Solve for Tomorrow 2026: STEM contest opens - tech.africa</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
+          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the 'first author'. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
+          <t>Feb 27, 2026 · Samsung Electronics South Africa has opened applications for the 2026 edition of Solve for Tomorrow (SFT), its annual science, technology, engineering, and mathematics (STEM) competition aimed at Grade 10 and 11 learners.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1967,26 +1939,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
+          <t>High School STEM Competition | Capetown 2026</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/za/solvefortomorrow/</t>
+          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
+          <t>High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas. Each submission can provide a summary of the STEM project. All projects must be presented at the IEOM Cape Town, South Africa 2026.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1999,17 +1967,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation ...</t>
+          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://www.samsung.com/za/solvefortomorrow/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Join the South African Space Design Competition to inspire space innovation, develop STEM skills, and compete for a trip to NASA. Perfect for high school students passionate about space.</t>
+          <t>Rooted in the belief that today’s youth hold the key to tomorrow’s progress, Solve for Tomorrow South Africa provides participants with the tools, mentorship, and platforms they need to turn ideas into action.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2017,16 +1985,12 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>user@domain.com, info@zasdc.org</t>
-        </is>
-      </c>
+      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Astemi Sa</t>
+          <t>ASTEMI SA</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2049,7 +2013,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2072,17 +2036,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
+          <t>StemCo - StemCo 2026 International Competitions</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
+          <t>https://stemco.org/</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
+          <t>June 10, 2026 - BEST YOURSELF WITH STEMCO! Platform for the world’s brightest. ... Thanks to the participating 25 countries in 2019. Singapore, Albania, Australia, Azerbaijan, Canada, Germany, India, Indonesia, Japan, Jordan, Kazakhstan, Kyrgyzstan, Malawi, Mongolia, Nigeria, Myanmar, South Africa, Tajikistan, Turkey, Turkmenistan, Ukraine, The United States, Uzbekistan, Vietnam</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2090,22 +2054,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>havtt@fermat.edu.vn, example@mail.com, bestyourself@stemco.org, hkoffice@missmaneducation.com, education@missmaneducation.com, name@example.com, info@missmaneducation.com, stemcomongolia@gmail.com, awaisnaeem786@gmail.com, info.iksc@kangaroo.org.pk, t.azizakhon@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>High School STEM Competition | Southafrica 2024</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>The IEOM High School/Middle School STEM Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects.</t>
+          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, ...</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2113,26 +2081,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Applications for 2026 Samsung Solve For Tomorrow Now Open!</t>
+          <t>2026 Season - Africa's Global STEM Celebration</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://news.samsung.com/za/applications-for-2026-samsung-solve-for-tomorrow-now-open</t>
+          <t>https://www.stemfestival.org/competitions/</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries open until 06 March 2026. This is a transformative ...</t>
+          <t>April 30, 2026 - ... The Elementary, Junior, and Senior Robotics categories at STEM Festival are dedicated to advancing the World Robot Olympiad (WRO) across the Niger Delta and South-South Nigeria, working with ArcLights Foundation.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2145,17 +2109,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Register your school for Samsung Solve for Tomorrow 2026</t>
+          <t>ASTEMI Competitions 2022 – SAASTA</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://www.sowetan.co.za/careers/2026-03-03-register-your-school-for-samsung-solve-for-tomorrow-2026/</t>
+          <t>https://saasta.ac.za/astemi-competitions-2</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Register your school for Samsung Solve for Tomorrow 2026 STEM competition aims to transform and empower South African learners with critical skills to solve real-world challenges March 03, 2026 at 7:44 am</t>
+          <t>National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2163,11 +2127,7 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>ssasft@samsung.com</t>
-        </is>
-      </c>
+      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2182,7 +2142,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>WRO South Africa ( World Robot Olympiad ) is a robotics competition which brings together young people from all over the world to develop their creativity and problem-solving skills.</t>
+          <t>All competing teams are ranked nationally, and from this ranking list, the top 10 to 15 teams are invited to attend and compete in the National event in Gauteng. Teams winning their category stand a chance to be invited to represent South Africa at the WRO international event.</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2192,24 +2152,24 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com</t>
+          <t>8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
+          <t>Robotics for Good Youth Challenge South Africa</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in the leading UN-based global robotics competition, focusing on the critical area of agriculture and food security.</t>
+          <t>Oct 31, 2025 · The Robotics for Good Youth Challenge is the leading UN-based global robotics championship, inviting students aged 10 to 18 to develop AI and robotics-based solutions to tackle global challenges.</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2219,24 +2179,24 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>8c4075d5481d476e945486754f783364@sentry.io, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, info@thecortexhub.africa, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com</t>
+          <t>name@example.com</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
+          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
+          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>April 14, 2026 - This National Event, to be held at the Sandton Convention Centre in Johannesburg, South Africa, as part of AI for Good Impact Africa, at AI Expo Africa 2025, is a qualifying tournament leading to the Grand Finale in Geneva during the AI for ...</t>
+          <t>This is a call for learners and teams from across South Africa who are passionate about robotics, innovation, and making a difference. Whether you’re experienced or just starting, this competition welcomes anyone eager to learn and innovate.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2246,7 +2206,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>name@example.com</t>
+          <t>8c4075d5481d476e945486754f783364@sentry.io, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, info@thecortexhub.africa, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -2263,7 +2223,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Apr 25, 2025 · The Robotics for Good Youth Challenge South Africa is a national event in a global robotics competition on disaster response, leading to the AI for Good Summit 2025.</t>
+          <t>Apr 25, 2025 · Experience the excitement as South African teams showcase their skills in a UN-based global robotics competition, focusing on the critical area of disaster response. This National Event is a qualifying tournament leading to the Grand Finale in Geneva during the AI for Good Global Summit 2025.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2290,7 +2250,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Jul 2, 2026 · The event, partnered with the World Robotics Olympiad, positions South Africa as a leader in educational robotics and entrepreneurial innovation.” South Africa’s robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation.</t>
+          <t>Jul 2, 2026 · South Africa’s robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation. Hosted at the Heartfelt Arena in Pretoria, the event is not only a showcase of technical skills but also a celebration of how robotics can address societal challenges.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2307,17 +2267,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>African Youth in Artificial Intelligence and Robotics</t>
+          <t>Home | Roboticon 2026</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://ele-vate.co.za/african-youth-in-artificial-intelligence-and-robotics</t>
+          <t>https://roboticon.resolute.education/</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>In partnership with the Government of the Republic of South Africa, the Second Edition of the Presidential African Youth in Artificial Intelligence and Robotics competition 2025 was hosted in Cape Town, South Africa.</t>
+          <t>Join us for the ultimate robotics showcase as Resolute proudly sponsors the World Robotics Olympiad (WRO) South Africa! This year, we're bringing together two worlds for the biggest robotics event of the year – Roboticon and the WRO Nationals, happening on the same day at the same venue.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2325,26 +2285,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>innovationhub@ele-vate.co.za</t>
-        </is>
-      </c>
+      <c r="E77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>FIRST South Africa – Robotics Programs for School Children</t>
+          <t>ROBO-RUMBLE 2026 — Innovation in Motion</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://firstsa.org/</t>
+          <t>https://roborumble.net/</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way. FIRST Tech Challenge students learn to think like engineers. Teams ...</t>
+          <t>South Africa's premier youth robotics &amp; technology competition. Robo Wars, Drone Racing, Grand Prix &amp; Innovation Challenge. August 2026.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2357,94 +2313,90 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
+          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
+          <t>https://safcec.org.za/</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
+          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>robotics competition South Africa</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr"/>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>communication@safcec.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>South African Robotics Competitions and Schools</t>
+          <t>The South African Institution of Civil Engineering</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://www.sciencexpo.org.za/robotics.html</t>
+          <t>https://civils.org.za/</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
+          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>robotics competition South Africa</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>marna.vanzyl@imbewu.foundation, madelien@imbewu.foundation, webmaster@sciencexpo.org.za</t>
-        </is>
-      </c>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Limpopo Learners Represent South Africa at Global Robotics Finals in Switzerland - African Times</t>
+          <t>SAICE’s 34th International Bridge Competition Inspires ...</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://www.atnews.co.za/limpopo-learners-represent-south-africa-at-global-robotics-finals-in-switzerland/</t>
+          <t>https://southafricatoday.net/lifestyle/education/saices-34th-international-bridge-competition-inspires-tomorrows-engineers/</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>July 7, 2026 - The international competition, taking place from 7 to 10 July 2026 at the Palexpo International Exhibition and Convention Centre in Geneva, brings together some of the world’s brightest young innovators to develop technological solutions to ...</t>
+          <t>Sep 1, 2025 · The South African Institution of Civil Engineering (SAICE) hosted its 34th International Bridge Building Competition at the Midrand Conference Centre, bringing together 21 teams of high school learners from across South Africa, alongside international participants from Eswatini, Uganda, and Zimbabwe.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>robotics competition South Africa</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>rampedim@atnews.co.za, NkosiN@atnews.co.za</t>
-        </is>
-      </c>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
+          <t>Home - SAICE</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://safcec.org.za/</t>
+          <t>https://saice.org.za/</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
+          <t>Through our divisions, branches and committees, we aim to advance professional knowledge and improve the practice of civil engineering in South Africa. Our purpose is to provide members with opportunities for professional development through continued learning opportunities and industry networking.</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2454,24 +2406,24 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>communication@safcec.org.za</t>
+          <t>marketing@saice.org.za, civilinfo@saice.org.za, barbara@avenue.co.za, executiveadmin@saice.org.za, membership@saice.org.za, communications@saice.org.za, accounts@saice.org.za</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Competition Ts and Cs - SAICE</t>
+          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://saice.org.za/competition-ts-and-cs/</t>
+          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Preamble These Terms and Conditions govern participation in the Know Your Sector Competition ("the Competition") conducted by the South African Institute of Civil Engineering ("SAICE"). Definitions SAICE: Shall mean the South African Institute of Civil Engineering. The Competition: Shall mean SAICE's Know Your Sector Competition. Entrant: Shall mean any individual who enters the ...</t>
+          <t>Jul 7, 2026 · Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in a shared commitment to developing South Africa’s future engineering talent.</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2479,26 +2431,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>accounts@saice.org.za, membership@saice.org.za, marketing@saice.org.za, communications@saice.org.za, civilinfo@saice.org.za</t>
-        </is>
-      </c>
+      <c r="E83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Civil Expo ITs 2026</t>
+          <t>Bridge Building Project Info - SAICE</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://civilexpoits2026.com/</t>
+          <t>https://saice.org.za/bridge-building-project-info/</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Hi Cipo Pals! Civil Expo ITs 2026 Sovereign Structures, Resilient Societies This national civil engineering competition is your chance to put your engineering precision to the test and build real-world structural solutions. Step up and prove your skills on a national stage!</t>
+          <t>These learners come from across South Africa as well as Eswatini and Zimbabwe. This competition exposes the learners to a practical application of a process through which civil engineering impact their daily lives.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2508,24 +2456,24 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>civilexpo.sipilits@gmail.com</t>
+          <t>marketing@saice.org.za, civilinfo@saice.org.za, membership@saice.org.za, communications@saice.org.za, accounts@saice.org.za, memory@saice.org.za</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SAICE's 34th International bridge competition inspires tomorrow's engineers</t>
+          <t>SAICE Aqualibrium 2025: High School Students Rise to the ...</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://www.crown.co.za/africa-updates/33867-saice-s-34th-international-bridge-competition-inspires-tomorrow-s-engineers</t>
+          <t>https://southafricatoday.net/environment/saice-aqualibrium-2025-high-school-students-rise-to-the-challenge-in-national-water-competition/</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) hosted its 34th International Bridge Building Competition at the Midrand Conference Centre, bringing together 21 teams of high school learners from across South Africa, alongside international participants from Eswatini, Uganda, and Zimbabwe.</t>
+          <t>May 14, 2025 · Each year, the Aqualibrium competition puts high school students in the shoes of actual civil engineers, putting their creativity and problem-solving abilities to the test by solving a challenging real-world problem.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2538,49 +2486,45 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Engineering the Future: 16 schools compete in SAICE's 33rd ...</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://southafricatoday.net/lifestyle/education/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) hosted its 33 rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland. The very first SAICE Bridge Building Competition was held in 1991, and it aimed to encourage high school learners to apply their knowledge of mathematics and science in a ...</t>
+          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
@@ -2588,22 +2532,22 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>SAICE Aqualibrium 2025: High School Students Rise to the Challenge in ...</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://southafricatoday.net/environment/saice-aqualibrium-2025-high-school-students-rise-to-the-challenge-in-national-water-competition/</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) hosted the thrilling 2025 Aqualibrium Competition National Finals this past week, which brought together high school students from schools all over South Africa at the Sci-Bono Discovery Centre in Johannesburg. The event continues to be an important platform for fostering engineering talent, inspiring young minds, and raising awareness ...</t>
+          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -2611,49 +2555,45 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Home - SAICE</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://saice.org.za/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) is the industry body for civil engineering professionals in South Africa. Our aim is to, promote growth, excellence and sustainability in the industry.</t>
+          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>accounts@saice.org.za, membership@saice.org.za, executiveadmin@saice.org.za, barbara@avenue.co.za, marketing@saice.org.za, communications@saice.org.za, civilinfo@saice.org.za</t>
-        </is>
-      </c>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>SAICE Aqualibrium 2025: High School Students Rise to the Challenge in ...</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://infrastructurenews.co.za/2025/05/14/saice-aqualibrium-2025-high-school-students-rise-to-the-challenge-in-national-water-competition/</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) hosted the thrilling 2025 Aqualibrium Competition National Finals, which brought together high school students from schools all over South Africa at the Sci-Bono Discovery Centre.</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -2661,22 +2601,22 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>SAICE | Events and Awards</t>
+          <t>APPLY NOW! WORLDSKILLS SOUTH AFRICA NATIONAL COMPETITION 2025</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://members.saice.org.za/events-and-awards</t>
+          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>The South African Institution Of Civil Engineering SAICE hosts the Awards Function annually to honour individuals, projects of excellence, as well as community-oriented initiatives. The annual awards function gives companies and individuals a unique opportunity to showcase their deserving projects and work to the industry.</t>
+          <t>ndidate with an accredited qualification in the related skill - Candida. e must not turn 23 years old in 2026 for the skills required. - Candidate applying for Aircraft Maintenance, Mechatr.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
@@ -2684,17 +2624,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>SAIMechE</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://www.saimeche.org.za/</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2707,7 +2647,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2717,12 +2657,12 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
@@ -2730,76 +2670,68 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+          <t>Apr 30, 2026 · IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa) Deadline: April 30, 2026 May 15, 2026</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Home | Electrical Engineering</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://ebe.uct.ac.za/department-electrical-engineering</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>Join the department’s research groups that, working closely with industry, stay at the forefront of electrical engineering trends worldwide.</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -2807,95 +2739,103 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Competitions - Prized Competitions South Africa</t>
+          <t>South African Institute of Electrical Engineers</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://www.prized.co.za/competitions/</t>
+          <t>https://www.saiee.org.za/</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Prized is home to Online Competitions in South Africa. Enter any competition that peaks your interest and join the Prized community.</t>
+          <t>Companies are composed of a number of job roles &amp; ... All equipment from massive ships to tiny devices h ... Earn your CPD credits today! Read it here.</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr"/>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>glueup-logo-white@2x.png, reception@saiee.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>National Student Competition | ORSSA</t>
+          <t>Competitions | ESG</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://www.orssa.org.za/studentcomp</t>
+          <t>https://za.rs-online.com/web/content/m/competition</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>National Student Competitions The Operations Research Society of South Africa The home of decision intelligence The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
+          <t>Find your next opportunity below, we stagger them throughout the year so make sure to check back regularly for up to date information. Good luck! The RS Student Project Fund 2026 provides successful applicants with up to R10 000 to spend on RS products.</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, email@example.com</t>
+          <t>example@email.com</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>PDF Apply Now! Worldskills South Africa National Competition 2025</t>
+          <t>Wits ENERGISE Centre Call for Participation Shaping the ...</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
+          <t>https://www.wits.ac.za/media/wits-university/faculties-and-schools/-engineering-and-the-built-environment/electrical-and-information-engineering/energise/wits-energise-centre-competition.pdf</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
+          <t>Join the ENERGISE Sustainable Business Model Competition 2026 and embark on guided academic training embedded in an international flagship project on the Just Energy Transition (JET) for the African-German Centre of Excellence held at Wits. Through iterative idea development, mentoring, and international exchange, participants co-develop application-oriented business model concepts addressing ...</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr"/>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>muhammed.aswat1@wits.ac.za</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>SAIMechE</t>
+          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://www.saimeche.org.za/</t>
+          <t>https://hackon.co.za/</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
+          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>engineering hackathon South Africa</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -2903,49 +2843,45 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Home - Icmeesa</t>
+          <t>Hackathons en South Africa</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>http://icmeesa.org.za/</t>
+          <t>https://za.allhackathons.com/</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Certificated Mechanical or Electrical Engineers in mining and factory are the professional engineering practitioners recognised by law in South Africa to accept legal responsibility to improve health and safety in mines and works. These Engineers need to provide solutions reliant on basic scientific, mathematical and engineering knowledge, supported by analysis and synthesis, and underpinned ...</t>
+          <t>Aug 22, 2025 · Join us for an electrifying hackathon where innovation meets security and finance! This event brings together developers, data scientists, cybersecurity experts, and FinTech enthusiasts to …</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>info@icmeesa.org.za, icmeesa@icmeesa.org.za</t>
-        </is>
-      </c>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
+          <t>AI Hackathon | Sebaka</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
+          <t>https://sebakasouthafrica.co.za/index.html</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
+          <t>Sebaka Mentorship &amp; Hackathons — Build an AI Agent for Software Quality Engineering.</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>engineering hackathon South Africa</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
@@ -2953,22 +2889,22 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - SAIEE National Student Project Competition</t>
+          <t>GirlCode | Hackathon 2026</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/calendar/EventDetails.aspx?eeid=29281</t>
+          <t>https://www.girlcode.co.za/hackathon-2026</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>The SAIEE National Students Project Competition will be held at the North-West University (Potchefstroom Campus) on 21 November 2019</t>
+          <t>What is the GirlCode Hackathon? The GirlCode Hackathon is an annual, all-women 30 hours coding marathon designed to address the gender gap in the tech industry by providing female developers with a high-intensity, real-world platform to showcase their technical talent, develop innovative solutions, and build crucial industry networks.</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>engineering hackathon South Africa</t>
         </is>
       </c>
       <c r="E103" t="inlineStr"/>
@@ -2976,22 +2912,22 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - IEEE ZA 5G Competition</t>
+          <t>Build the Future with Entelect Hackathons</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51397</t>
+          <t>https://challenge.entelect.co.za/</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Form templates: Template for a Cover Sheet for the Competition on Ideas, Designs and Applications for 5G and Beyond South Africa (.docx) [Click to Download] Template for a Resume for the Student (.docx) [Click to Download] ... Help (FAQ) • Privacy Statement • Terms &amp; Conditions The SAIEE is ...</t>
+          <t>Instead of focusing on building a once-off project, our hackathons centre around optimisation problems. Participants develop solutions that are tested, scored, and ranked based on performance, efficiency, and strategy.</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>engineering hackathon South Africa</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
@@ -2999,22 +2935,22 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Student Design Competition | IEEE CASS</t>
+          <t>Young Engineers Movement (YEM) - ORT SA</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://ieee-cas.org/society-involvement/student-design-competition</t>
+          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>East, Africa), Region 9 (Latin America), and Region 10 (Asia, Australia, Pacific), as well as ISCAS registration. The winning team will be awarded $3,000 USD. For details on how to participate in the 2026 Student Design Competition, click here. ... Undergraduate students would suggest and execute ...</t>
+          <t>The Young Engineers Movement (YEM) is an immersive engineering and technology hackathon designed to equip young South Africans with the skills, mindset and confidence needed to solve real-world challenges.</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>engineering hackathon South Africa</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
@@ -3022,386 +2958,25 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Top 100 Electrical Engineering Companies in South Africa (2026) | ensun</t>
+          <t>CompeteHub - Where Champions Are Made</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://ensun.io/search/electrical-engineering/south-africa</t>
+          <t>https://www.devpluxe.co.za/</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>The competitive landscape is marked by both established firms and emerging startups, driving innovation and efficiency. Additionally, South Africa’s position in the broader global market allows for potential collaborations and export opportunities, particularly in green technologies. Understanding these factors is essential for anyone looking to engage with the Electrical Engineering ...</t>
+          <t>Join thousands of developers, designers, and innovators competing in South Africa ' s most impactful tech hackathons. We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>engineering hackathon South Africa</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>At the Centre for High Performance Computing (CHPC) Conference hosted in Cape Town at the end of last year, four current fourth-year electrical engineering students were crowned national champions in the Student Cluster Competition for 2025.</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr"/>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>Electrical Engineering Conferences in South Africa 2025/2026/2027 - Conference Index</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>https://conferenceindex.org/conferences/electrical-engineering/south-africa</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>Electrical Engineering Conferences in South Africa 2025 2026 2027 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and ...</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr"/>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>7 Electrical Engineering Degree Programs in South Africa - Study Abroad | educations.com</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>https://www.educations.com/electrical-engineering/south-africa</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>Find the best fit for you - Compare 7 in Engineering Programs Electrical Engineering in South Africa for 2025/2026</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr"/>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>Electrical And Electronics Engineering Conferences in South Africa 2026 | Conference Alerts</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>https://conferencealerts.co.in/south-africa/electrical-and-electronics-engineering</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>Select your participation type (in-person, virtual, or hybrid), fill in your personal and professional details, and pay the registration fee if required. After registering, you’ll receive confirmation and access instructions. Some electrical and electronics engineering conferences in south africa also allow early-bird registration with discounted fees.</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E110" t="inlineStr"/>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>South African Institute of Electrical Engineers</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>https://www.saiee.org.za/</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>South African Institute of Electrical Engineers (SAIEE) About Us See Member Benefits · Become a SAIEE Member today! SAIEE Membership · Earn CPD credits · About Training Academy · Join a SAIEE Centre near you! Centres · South African Institute of Electrical Engineers (SAIEE) 01 ·</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, reception@saiee.org.za</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>Hackathons en South Africa</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>https://za.allhackathons.com/</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>Aug 22, 2025 · Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E112" t="inlineStr"/>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>AI Hackathon | Sebaka</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>https://sebakasouthafrica.co.za/index.html</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>Sebaka Mentorship &amp; Hackathons — Build an AI Agent for Software Quality Engineering.</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E113" t="inlineStr"/>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>Build the Future with Entelect Hackathons</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>https://challenge.entelect.co.za/</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>Build the Future with Entelect Hackathons Join South Africa’s premier optimisation-first developer competition platform. Compete, iterate, and outperform the best.</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr"/>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>GirlCode | Hackathon 2026</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>https://www.girlcode.co.za/hackathon-2026</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>Building Africa's Next Generation of AI-Powered Female Innovators Join Africa's largest women-in-tech hackathon empowering innovators, creators, and future founders.</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E115" t="inlineStr"/>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>Budding engineers showcase innovation at YEM hackathon | ITWeb</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>https://www.itweb.co.za/article/budding-engineers-showcase-innovation-at-yem-hackathon/kYbe97XbP4ZqAWpG</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>June 30, 2026 - The hackathon was hosted by Johannesburg-based non-profit education and training organisation ORT South Africa, in partnership with JSE-listed industrial and engineering supplies firm Hudaco.</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>enquiries@ombudsman.org.za</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>Young Engineers Shine as Inaugural YEM Hackathon Celebrates South Africa's Next Generation of Innovators</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>https://novuspressbulletin.co.za/blog/young-engineers-shine-as-inaugural-yem-hackathon-celebrates-south-africa-s-next-generation-of-innovators</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>June 30, 2026 - ... Johannesburg, June 2026 – After five inspiring days of innovation, collaboration, and problem-solving, the inaugural Young Engineers Movement (YEM) Hackathon, hosted by ORT South Africa in partnership with Hudaco, concluded with a vibrant ...</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr"/>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>Young Engineers Shine as Inaugural YEM Hackathon Celebrates South Africa's Next Generation of Innovators - Lifestyle &amp; Tech</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>https://lifestyleandtech.co.za/company-news/article/2026-06-29/young-engineers-shine-as-inaugural-yem-hackathon-celebrates-south-africas-next-generation-of-innovators</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>June 29, 2026 - After five inspiring days of innovation, collaboration, and problem-solving, the inaugural Young Engineers Movement (YEM) Hackathon, hosted by ORT South Africa in partnership with Hudaco, concluded with a vibrant exhibition showcasing the remarkable ...</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr"/>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>ORT South Africa's inaugural YEM Hackathon empowers future STEM innovators</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>https://www.futuresa.co.za/bursaries-and-scholarships/ort-south-africa-yem-hackathon/</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>3 weeks ago - ORT South Africa's first Young Engineers Movement Hackathon saw 55 learners develop innovative STEM solutions during a five-day competition.</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>info@futuresa.co.za</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>Houghton hackathon: Stepping stone for future engineers | Rosebank Killarney Gazette</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>https://www.citizen.co.za/rosebank-killarney-gazette/news-headlines/local-news/2026/06/23/houghton-hackathon-stepping-stone-for-future-engineers/</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>June 23, 2026 - Hosted by ORT South Africa in partnership with Hudaco, the hackathon has brought together 55 learners from underserved communities to work together in developing solutions to challenges they face in their communities.</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr"/>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>55 learners from underserved schools showcase engineering innovations at Johannesburg hackathon</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>https://iol.co.za/saturday-star/2026-07-01-55-learners-from-underserved-schools-showcase-engineering-innovations-at-johannesburg-hackathon/</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>3 weeks ago - Fifty-five high school learners ... at the Young Engineers Movement (YEM) Hackathon Exhibition Day in Johannesburg last week, presenting working prototypes designed to solve real-world problems affecting their communities. The learners, accompanied by 11 teachers, took part in the five-day hackathon, hosted by ORT South Africa in partnership with Hudaco, from June 22 to 26....</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>yasmine.jacobs@iol.co.za, pholoso.manyama@iol.co.za, pholoso.manyama@inl.co.za, wendy.dondolo@inl.co.za, verna.vandiemen@inl.co.za</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update competition data 2026-08-21
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>2 weeks ago - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -469,17 +469,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
+          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.poidata.io/report/engineer/south-africa</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sep 4, 2025 · The Africa Prize for Engineering Innovation is open to individuals or teams based in sub-Saharan Africa who have a scalable engineering innovation with social or environmental impact potential.</t>
+          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -487,26 +487,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>Two South Africans on the shortlist for the 2026 Africa Prize for Engineering Innovation</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.engineeringnews.co.za/article/two-south-africans-on-the-shortlist-for-the-2026-africa-prize-for-engineering-innovation-2026-08-04</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Some of our sparkling achievements during 2014 – to help the NRF and DSI grow a representative science and technology workforce in the country – SAASTA has run a number of maths and science educator development programmes and a number of learner development programmes, including maths and science camps for learners with potential, olympiads and competitions. The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the · National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>2 weeks ago - Two South African innovators have been shortlisted for the UK Royal Academy of Engineering’s Africa Prize for Engineering Innovation 2026. This is the continent’s richest award aimed at promoting engineering innovation and entrepreneurship ...</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -514,22 +510,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>chanel@engineeringnews.co.za, newsletters@creamermedia.co.za, advertising@creamermedia.co.za, subscriptions@creamermedia.co.za, newsdesk@engineeringnews.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
+          <t>1 week ago - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -542,17 +542,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -560,22 +560,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+          <t>Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions.</t>
+          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -588,17 +592,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>National Student Competition | ORSSA</t>
+          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.orssa.org.za/studentcomp</t>
+          <t>https://www.thecasecentre.org/products/view?id=189255</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
+          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -606,26 +610,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, email@example.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
+          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2 weeks ago - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
+          <t>South Africa · South Korea · Spain · Sri Lanka · Sudan · Sweden · Switzerland · Syrian Arab Republic · Taiwan · Tajikistan · Tanzania · Thailand · Togo · Trinidad and Tobago · Tunisia · Turkey · Uganda · Ukraine · United Arab Emirates · United Kingdom ·</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -638,17 +638,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.poidata.io/report/engineer/south-africa</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -661,17 +661,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Two South Africans on the shortlist for the 2026 Africa Prize for Engineering Innovation</t>
+          <t>Engineering News|Real-Economy News</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/two-south-africans-on-the-shortlist-for-the-2026-africa-prize-for-engineering-innovation-2026-08-04</t>
+          <t>https://www.engineeringnews.co.za/</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2 weeks ago - Two South African innovators have been shortlisted for the UK Royal Academy of Engineering’s Africa Prize for Engineering Innovation 2026. This is the continent’s richest award aimed at promoting engineering innovation and entrepreneurship ...</t>
+          <t>The competition invites South Africans to submit an original name for the new...</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -681,24 +681,24 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>subscriptions@creamermedia.co.za, chanel@engineeringnews.co.za, newsdesk@engineeringnews.co.za, advertising@creamermedia.co.za, newsletters@creamermedia.co.za</t>
+          <t>subscriptions@creamermedia.co.za, newsletters@creamermedia.co.za</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
+          <t>South Africa International Industrial Expo | Innovation Bridge</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/tradeshows</t>
+          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1 day ago · South Africa trade shows, find and compare 966 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 176 upcoming expos in 2026-2027 1. South Africa Infrastructure &amp; Water Expo, 2.</t>
+          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -711,17 +711,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
+          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://innovationweek.co.za/</t>
+          <t>https://madeinafricaevent.co.za/</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SAIW’ 26 is designed as a week-long national programme to feature provincial innovation engagements across South Africa. From 16 – 17 March, Provinces will showcase local innovation strengths, emerging enterprises and sectoral capabilities.</t>
+          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -729,26 +729,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>info@pixal8media.co.za</t>
-        </is>
-      </c>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Innovations events in South Africa 2026-2027 - ExpoTobi</t>
+          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://expotobi.com/country/south-africa/sector/innovations</t>
+          <t>https://manufacturingindaba.co.za/exhibition/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Innovations events in South Africa Full and accurate description of Innovations events Schedule, tickets, accommodation, travel arrangement and participation</t>
+          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -761,17 +757,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Africa Tech Festival</t>
+          <t>KZN Industrial Technology Exhibition</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://www.kznindustrial.co.za/</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
+          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -781,24 +777,24 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>dataprivacy@informaconnect.com, support@knect365.com, salesenquiries@africatechfestival.com, dataprivacy@knect365.com, customerservices@informaconnect.com, customerservices@knect365.com, support@informaconnect.com</t>
+          <t>john@email.com</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa, List of all South ...</t>
+          <t>Two landmark exhibitions set to transform industrial technology and renewable energy in South Africa</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://www.engineeringnews.co.za/article/two-landmark-exhibitions-set-to-transform-industrial-technology-and-renewable-energy-in-south-africa-2025-10-24</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>The BI + AI Innovation &amp; Tech Fest is a pioneering event that celebrates the intersection of Business Intelligence (BI) and Artificial Intelligence (AI), emphasizing the transformative power of technology...</t>
+          <t>October 24, 2025 - South Africa’s industrial and clean energy sectors celebrated a landmark moment today with the official launch of RE+ South Africa 2026 and the Cape Industrial Technology Exhibition (CITE) 2027.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -806,22 +802,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>chanel@engineeringnews.co.za, newsletters@creamermedia.co.za, advertising@creamermedia.co.za, subscriptions@creamermedia.co.za, newsdesk@engineeringnews.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>South Africa International Industrial Expo | Innovation Bridge</t>
+          <t>Exhibition | Innovation Festival Durban | South Africa</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
+          <t>https://www.innovationfestival.durban/exhibition</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
+          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -829,22 +829,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Erika@innovate.durban, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, sithabile@innovate.durban, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
+          <t>Trade Shows Worldwide - South Africa - 2026/2027</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://madeinafricaevent.co.za/</t>
+          <t>https://www.eventseye.com/fairs/c1_trade-shows_south-africa.html</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
+          <t>South Africa Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in South Africa</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -857,17 +861,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
+          <t>Discover Innovation Hub's Pavilion at Organic &amp; Natural Products Expo - Organic &amp; Natural Products Portal</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://manufacturingindaba.co.za/exhibition/</t>
+          <t>https://www.organicandnaturalportal.com/innovation-hub-organic-expo/</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
+          <t>2 weeks ago - Gathering producers, retailers, buyers, and conscious consumers under one roof, the expo serves as Africa’s premier showcase for sustainability, health, and wellness innovation. A standout highlight of this year’s exhibition is The Innovation Hub Pavilion, hosting a curated line-up of forward-thinking South African small, medium, and micro-enterprises (SMMEs).</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -880,17 +884,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Two landmark exhibitions set to transform industrial technology and renewable energy in South Africa</t>
+          <t>International Science, Innovation &amp; Technology Expo (INSITE)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/two-landmark-exhibitions-set-to-transform-industrial-technology-and-renewable-energy-in-south-africa-2025-10-24</t>
+          <t>https://www.dsti.gov.za/index.php/resource-center/27-temp/dst-links/3-international-science-innovation-a-technology-expo</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>October 24, 2025 - South Africa’s industrial and clean energy sectors celebrated a landmark moment today with the official launch of RE+ South Africa 2026 and the Cape Industrial Technology Exhibition (CITE) 2027.</t>
+          <t>The essence of INSITE INSITE is an international, biennial must-see Science and Technology event in South Africa, the only one of its kind in Africa that creates new frontiers for global challenges · INSITE aims to assemble the worlds leading innovators and scientists in one place, stimulating ...</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -898,26 +902,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>subscriptions@creamermedia.co.za, chanel@engineeringnews.co.za, newsdesk@engineeringnews.co.za, advertising@creamermedia.co.za, newsletters@creamermedia.co.za</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>KZN Industrial Technology Exhibition</t>
+          <t>AAXO - The Association of African Exhibition Organisers</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.kznindustrial.co.za/</t>
+          <t>https://www.aaxo.co.za/</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
+          <t>February 20, 2026 - CAPE TOWN, South Africa – The inaugural Festival of Eventing (FOE) brought together 350 event professionals, 85 speakers, and 10 countries under one roof for a two-day showcase of innovation, inspiration, and industry connection.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -925,26 +925,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>john@email.com</t>
-        </is>
-      </c>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
+          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -957,17 +953,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of ...</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Aug 4, 2025 · The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
+          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -977,24 +973,24 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
+          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge returns to Johannesburg!</t>
+          <t>EWB Design Challenge | Aston University</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
+          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Sep 18, 2024 · Engineering for People Design Challenge returns to Johannesburg! Now entering its fourteenth year, we’re delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
+          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1007,17 +1003,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Latest Community Engineering Design Competition Announced</t>
+          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
+          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Oct 16, 2024 · Organised in conjunction with sister organisation Engineers Without Borders South Africa, as well as the Makers Valley Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg.</t>
+          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1025,22 +1021,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ied@ied.org.uk</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Engineering For People Design Challenge - EWBSA</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
+          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1053,17 +1053,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge - Engineers Without ...</t>
+          <t>Real-world research: Engineering team designs South African trolley system; science students investigate heavy metals | University of Wisconsin - Stout</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
+          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
+          <t>May 15, 2025 - Research ranged from heavy metals ... Borders’ international design challenge. Nearly 90 students in 23 teams addressed the EWB challenge. One group focused on engineering a safer, more accessible transportation system in South ...</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1071,22 +1071,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>dolanm@uwstout.edu, frischj@uwstout.edu</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
+          <t>Engineering for people, that’s the challenge | Engineers Without Borders</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
+          <t>https://www.rs-online.com/designspark/an-introduction-to-engineering-for-people-design-challenge</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Oct 24, 2024 · The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
+          <t>That’s exactly what the annual Engineering for People Design Challenge asks participants to do. The competition, delivered in partnership by Engineers without Borders South Africa and Engineers Without Borders UK, encourages engineering students and those collaborating with engineers to broaden their awareness of how their decisions change the world.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1094,26 +1098,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>team@crowdsolve.net</t>
-        </is>
-      </c>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>EWB Design Challenge | Aston University</t>
+          <t>Engineering for People Design Challenge | Department of Engineering</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
+          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1121,22 +1121,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
+          <t>Launching Engineering for People Design challenge 2024 ...</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
+          <t>https://www.electronicspecifier.com/studentzone/studentzone-news/launching-engineering-for-people-design-challenge-2024-25-2/</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
+          <t>November 16, 2025 - Engineers Without Borders has launched the 2024/25 cycle of the award-winning Engineering for People Design Challenge in partnership with Engineers Without Borders South Africa and Makers Valley Partnership.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1144,26 +1148,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>ied@ied.org.uk</t>
-        </is>
-      </c>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Real-world research: Engineering team designs South African trolley system; science students investigate heavy metals | University of Wisconsin - Stout</t>
+          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
+          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>May 15, 2025 - Research ranged from heavy metals ... Borders’ international design challenge. Nearly 90 students in 23 teams addressed the EWB challenge. One group focused on engineering a safer, more accessible transportation system in South ...</t>
+          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1171,26 +1171,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>frischj@uwstout.edu, dolanm@uwstout.edu</t>
-        </is>
-      </c>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
+          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1198,22 +1194,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
+          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1221,22 +1221,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
+          <t>National Student Competition | ORSSA</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
+          <t>https://www.orssa.org.za/studentcomp</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
+          <t>The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1244,22 +1248,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, email@example.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1272,17 +1280,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Engineering in South Africa: 24 Best universities Ranked</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://edurank.org/engineering/za/</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
+          <t>Sep 4, 2025 · The Africa Prize for Engineering Innovation is open to individuals or teams based in sub-Saharan Africa who have a scalable engineering innovation with social or environmental impact potential.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1290,22 +1298,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Competitions – Enactus South Africa | National Expos ...</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://enactusza.org/what-we-do/competitions</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>Explore our national and international competitions that empower students to tackle challenges with entrepreneurial solutions and social impact at the core.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1313,22 +1325,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>adminsa@enactus.org, xmadlanga@enactus.org, marketingsa@enactus.org, liso@enactus.org</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
+          <t>Wits ENERGISE Centre Call for Participation - Wits University</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2210</t>
+          <t>https://www.wits.ac.za/media/wits-university/faculties-and-schools/-engineering-and-the-built-environment/electrical-and-information-engineering/energise/wits-energise-centre-competition.pdf</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
+          <t>Join the ENERGISE Sustainable Business Model Competition 2026 and embark on guided academic training embedded in an international flagship project on the Just Energy Transition (JET) for the African-German Centre of Excellence held at Wits. Through iterative idea development, mentoring, and international exchange, participants co-develop application-oriented business model concepts addressing ...</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1336,22 +1352,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>muhammed.aswat1@wits.ac.za</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
+          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
+          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
+          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1364,17 +1384,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2025</t>
+          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
+          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2025</t>
+          <t>Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1387,17 +1407,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
+          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1457,24 +1477,24 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>dataprivacy@informaconnect.com, support@knect365.com, salesenquiries@africatechfestival.com, dataprivacy@knect365.com, customerservices@informaconnect.com, customerservices@knect365.com, support@informaconnect.com</t>
+          <t>salesenquiries@africatechfestival.com, customerservices@informaconnect.com, support@informaconnect.com, customerservices@knect365.com, dataprivacy@knect365.com, support@knect365.com, dataprivacy@informaconnect.com</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>IT &amp; Technology Events in South Africa | 10times</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
+          <t>7 hours ago · Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1482,26 +1502,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>info@techspocapetown.co.za</t>
-        </is>
-      </c>
+      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>Home - Mediatech Africa | South Africa</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://www.mediatech.co.za/</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>Mediatech Africa showcases the full range of professional tech driving AV, broadcast, media, &amp; live event production. From AV integration, unified communications &amp; display to pro audio, lighting, content creation, &amp; future tech — our sectors highlight the tools behind today’s connected experiences.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1509,22 +1525,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>claire@mediatech.co.za, simon@mediatech.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Home - Mediatech Africa | South Africa</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://www.mediatech.co.za/</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Mediatech Africa showcases the full range of professional tech driving AV, broadcast, media, &amp; live event production. From AV integration, unified communications &amp; display to pro audio, lighting, content creation, &amp; future tech — our sectors highlight the tools behind today’s connected experiences.</t>
+          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1532,7 +1552,11 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>info@techspocapetown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1547,7 +1571,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>6 days ago · Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience.</t>
+          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1603,7 +1627,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>atinfo@techspo.coor, name@example.com, u003einfo@techspo.co</t>
+          <t>atinfo@techspo.coor, u003einfo@techspo.co, name@example.com</t>
         </is>
       </c>
     </row>
@@ -1637,17 +1661,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 – Africa's biggest IT Conference and Expo</t>
+          <t>HOME | Africa Tech Week</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://africatechweek.co.za/</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>The inaugural 2025 IT Indaba promises to bring together 3,000+ IT professionals and tech influencers who are involved in the procurement of systems, tools, platforms and services, along with user experience developers who deal with the core processes and client interfaces of the business.</t>
+          <t>May 11, 2026 - From sensational speakers, to top tech exhibitons, see what’s in store when you attend the 2-day Sentech Africa Tech Week Conference in 2025&gt;&gt; ... Sponsor, Speak, Attend! For more information on how you can be a part of the #ATW family, contact ...</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1693,7 +1717,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Maker Faire is a convention of do it yourself (DIY) enthusiasts established by Make magazine in 2006. Participants come from a wide variety of interests, such as robotics, 3D printing, computers, arts and crafts, and hacker culture.</t>
+          <t>May 3, 2026 - Maker Faires are also held in Europe, Asia, South America and Africa.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1706,17 +1730,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Maker Faire Africa — Grokipedia</t>
+          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://grokipedia.com/page/maker_faire_africa</t>
+          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
+          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1729,17 +1753,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Maker Faire |</t>
+          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://makerfaire.com/</t>
+          <t>https://makerfairecapetown.wordpress.com/about/</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
+          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1747,26 +1771,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>fancybox_loading@2x.gif, chosen-sprite@2x.png, pr@make.co, fancybox_sprite@2x.png</t>
-        </is>
-      </c>
+      <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
+          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
+          <t>http://capetown.makerfaire.com/</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Aug 21, 2015 · We’re delighted to present the first ever Cape Town Maker Faire, hosted by Open Design in partnership with Trimble.Maker Faire is primarily designed as a forward-looking event, showcasing makers who are exploring new forms and new technologies.</t>
+          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1774,22 +1794,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>fancybox_sprite@2x.png, fancybox_loading@2x.gif, pr@make.co, chosen-sprite@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Maker Faire groups | Meetup</t>
+          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/topics/maker-faire/za/</t>
+          <t>https://contemporaryand.com/fr/events/maker-faire-africa-comes-to-johannesburg</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
+          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1802,17 +1826,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
+          <t>Maker Faire Africa comes to Jo’Burg – AfriGadget</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
+          <t>https://www.afrigadget.com/2014/07/08/maker-faire-africa-comes-to-joburg/</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
+          <t>Maker Faire Africa 2014 will bring together over 5,000 attendees, along with featured inventors, world-class makers, self-made entrepreneurs &amp; workshop experts from South Africa, across the continent, and around the world, to manufacture real solutions for some of Africa’s most pressing ...</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1825,17 +1849,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
+          <t>Why Africa needs Maker Faire | ZDNET</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://makerfairecapetown.wordpress.com/about/</t>
+          <t>https://www.zdnet.com/article/why-africa-needs-maker-faire/</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
+          <t>July 24, 2014 - Unlike other Maker Faires, Okafor said that it's not enough to simply hold the event in an African city and see who turns up. Two volunteers are currently working in South Africa to discover inventors in rural areas and neighbouring countries such as Zambia and Botswana who they can encourage to attend and show off their work.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1843,22 +1867,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>brand_licensing@ziffdavis.com</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
+          <t>South Africa Archivi - Maker Faire Rome</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>http://capetown.makerfaire.com/</t>
+          <t>https://2019.makerfairerome.eu/en/tag/south-africa/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
+          <t>... It is the most important event in the world of innovation. Is a showcase of invention, creativity, and resourcefulness. Maker Faire gathers together tech enthusiasts, crafters, educators, tinkerers, schools, universities, research institutes, artists, students, and corporations.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1866,26 +1894,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>fancybox_loading@2x.gif, chosen-sprite@2x.png, pr@make.co, fancybox_sprite@2x.png</t>
-        </is>
-      </c>
+      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Blog : Maker Faire Africa</t>
+          <t>Maker Faire returning to South Africa in August - Hypertext</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>http://makerfaireafrica.com/blog/</t>
+          <t>https://htxt.co.za/2015/07/maker-faire-returning-to-south-africa-in-august/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>December 31, 2021 - You can help them out on the new South African crowdfunding site, ThundaFund. ... One of the most ambitions items at Maker Faire Africa this year in Johannesburg, South Africa is Samuel Ngobeni’s “art car”. He’s a designer from Germinston, who has spent the last three years building his ANIMAL car, from the ground up, that means the frame and all.</t>
+          <t>August 13, 2015 - Maker Faire will be held in Cape Town from 21st-23rd August at the V&amp;A Waterfront, with a Maker Faire Conference preceding the event on the 20th at The Lookout, V&amp;A Waterfront. The event is being backed by Maker Faire and Make: Magazine in the ...</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1962,22 +1986,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
+          <t>South African Space Design Competition | Inspire Space ...</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/za/solvefortomorrow/</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Rooted in the belief that today’s youth hold the key to tomorrow’s progress, Solve for Tomorrow South Africa provides participants with the tools, mentorship, and platforms they need to turn ideas into action.</t>
+          <t>Join the South African Space Design Competition to inspire space innovation, develop STEM skills, and compete for a trip to NASA. Perfect for high school students passionate about space.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -1985,22 +2013,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>user@domain.com, info@zasdc.org</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ASTEMI SA</t>
+          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/</t>
+          <t>https://www.samsung.com/za/solvefortomorrow/</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
+          <t>Rooted in the belief that today’s youth hold the key to tomorrow’s progress, Solve for Tomorrow South Africa provides participants with the tools, mentorship, and platforms they need to turn ideas into action.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2013,17 +2045,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>ASTEMI SA</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.astemi.co.za/</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2054,11 +2086,7 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>havtt@fermat.edu.vn, example@mail.com, bestyourself@stemco.org, hkoffice@missmaneducation.com, education@missmaneducation.com, name@example.com, info@missmaneducation.com, stemcomongolia@gmail.com, awaisnaeem786@gmail.com, info.iksc@kangaroo.org.pk, t.azizakhon@gmail.com</t>
-        </is>
-      </c>
+      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2081,22 +2109,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026 Season - Africa's Global STEM Celebration</t>
+          <t>ASTEMI Competitions 2022 – SAASTA</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://www.stemfestival.org/competitions/</t>
+          <t>https://saasta.ac.za/astemi-competitions-2</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>April 30, 2026 - ... The Elementary, Junior, and Senior Robotics categories at STEM Festival are dedicated to advancing the World Robot Olympiad (WRO) across the Niger Delta and South-South Nigeria, working with ArcLights Foundation.</t>
+          <t>National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2109,17 +2141,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions 2022 – SAASTA</t>
+          <t>2026 Season - Africa's Global STEM Celebration</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://saasta.ac.za/astemi-competitions-2</t>
+          <t>https://www.stemfestival.org/competitions/</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>April 30, 2026 - ... The Elementary, Junior, and Senior Robotics categories at STEM Festival are dedicated to advancing the World Robot Olympiad (WRO) across the Niger Delta and South-South Nigeria, working with ArcLights Foundation.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2150,26 +2182,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa</t>
+          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
+          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Oct 31, 2025 · The Robotics for Good Youth Challenge is the leading UN-based global robotics championship, inviting students aged 10 to 18 to develop AI and robotics-based solutions to tackle global challenges.</t>
+          <t>This is a call for learners and teams from across South Africa who are passionate about robotics, innovation, and making a difference. Whether you’re experienced or just starting, this competition welcomes anyone eager to learn and innovate.</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2179,24 +2207,24 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>name@example.com</t>
+          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, info@thecortexhub.africa, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
+          <t>Robotics for Good Youth Challenge South Africa</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>This is a call for learners and teams from across South Africa who are passionate about robotics, innovation, and making a difference. Whether you’re experienced or just starting, this competition welcomes anyone eager to learn and innovate.</t>
+          <t>Oct 31, 2025 · The Robotics for Good Youth Challenge is the leading UN-based global robotics championship, inviting students aged 10 to 18 to develop AI and robotics-based solutions to tackle global challenges.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2206,7 +2234,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>8c4075d5481d476e945486754f783364@sentry.io, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, info@thecortexhub.africa, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com</t>
+          <t>name@example.com</t>
         </is>
       </c>
     </row>
@@ -2313,17 +2341,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
+          <t>The South African Institution of Civil Engineering</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://safcec.org.za/</t>
+          <t>https://civils.org.za/</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
+          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2331,26 +2359,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>communication@safcec.org.za</t>
-        </is>
-      </c>
+      <c r="E79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering</t>
+          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://civils.org.za/</t>
+          <t>https://safcec.org.za/</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
+          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2358,22 +2382,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>communication@safcec.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SAICE’s 34th International Bridge Competition Inspires ...</t>
+          <t>Engineering the Future: 16 schools compete in SAICE’s 33rd ...</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://southafricatoday.net/lifestyle/education/saices-34th-international-bridge-competition-inspires-tomorrows-engineers/</t>
+          <t>https://southafricatoday.net/lifestyle/education/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Sep 1, 2025 · The South African Institution of Civil Engineering (SAICE) hosted its 34th International Bridge Building Competition at the Midrand Conference Centre, bringing together 21 teams of high school learners from across South Africa, alongside international participants from Eswatini, Uganda, and Zimbabwe.</t>
+          <t>Aug 30, 2024 · The South African Institution of Civil Engineering (SAICE) hosted its 33 rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2386,17 +2414,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Home - SAICE</t>
+          <t>ICE Africa – Supporting Civil Engineers in Africa</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://saice.org.za/</t>
+          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Through our divisions, branches and committees, we aim to advance professional knowledge and improve the practice of civil engineering in South Africa. Our purpose is to provide members with opportunities for professional development through continued learning opportunities and industry networking.</t>
+          <t>Click your country to find local events, competitions, and information on how you can get more involved. At the heart of everything we do in South Africa is ICE-SA, the volunteer ICE local association (formerly known as the Joint Civils Division).</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2404,26 +2432,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>marketing@saice.org.za, civilinfo@saice.org.za, barbara@avenue.co.za, executiveadmin@saice.org.za, membership@saice.org.za, communications@saice.org.za, accounts@saice.org.za</t>
-        </is>
-      </c>
+      <c r="E82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
+          <t>Home - SAICE</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
+          <t>https://saice.org.za/</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Jul 7, 2026 · Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in a shared commitment to developing South Africa’s future engineering talent.</t>
+          <t>Through our divisions, branches and committees, we aim to advance professional knowledge and improve the practice of civil engineering in South Africa. Our purpose is to provide members with opportunities for professional development through continued learning opportunities and industry networking.</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2431,22 +2455,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>barbara@avenue.co.za, communications@saice.org.za, membership@saice.org.za, accounts@saice.org.za, civilinfo@saice.org.za, marketing@saice.org.za, executiveadmin@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Bridge Building Project Info - SAICE</t>
+          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://saice.org.za/bridge-building-project-info/</t>
+          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>These learners come from across South Africa as well as Eswatini and Zimbabwe. This competition exposes the learners to a practical application of a process through which civil engineering impact their daily lives.</t>
+          <t>Jul 7, 2026 · Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in a shared commitment to developing South Africa’s future engineering talent.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2454,26 +2482,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>marketing@saice.org.za, civilinfo@saice.org.za, membership@saice.org.za, communications@saice.org.za, accounts@saice.org.za, memory@saice.org.za</t>
-        </is>
-      </c>
+      <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SAICE Aqualibrium 2025: High School Students Rise to the ...</t>
+          <t>Bridge Building Project Info - SAICE</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://southafricatoday.net/environment/saice-aqualibrium-2025-high-school-students-rise-to-the-challenge-in-national-water-competition/</t>
+          <t>https://saice.org.za/bridge-building-project-info/</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>May 14, 2025 · Each year, the Aqualibrium competition puts high school students in the shoes of actual civil engineers, putting their creativity and problem-solving abilities to the test by solving a challenging real-world problem.</t>
+          <t>These learners come from across South Africa as well as Eswatini and Zimbabwe. This competition exposes the learners to a practical application of a process through which civil engineering impact their daily lives.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2481,22 +2505,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>communications@saice.org.za, memory@saice.org.za, accounts@saice.org.za, civilinfo@saice.org.za, marketing@saice.org.za, membership@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2509,17 +2537,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2550,7 +2578,11 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2573,7 +2605,11 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2647,17 +2683,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2670,17 +2706,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 · IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa) Deadline: April 30, 2026 May 15, 2026</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2693,17 +2729,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Home | Electrical Engineering</t>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://ebe.uct.ac.za/department-electrical-engineering</t>
+          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Join the department’s research groups that, working closely with industry, stay at the forefront of electrical engineering trends worldwide.</t>
+          <t>Apr 30, 2026 · IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa) Deadline: April 30, 2026 May 15, 2026</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2716,17 +2752,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Electrical Engineering Conferences in South Africa 2026/2027 ...</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://conferenceindex.org/conferences/electrical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
+          <t>Electrical Engineering Conferences in South Africa 2026 2027 2028 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and symposiums.</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2866,17 +2902,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>AI Hackathon | Sebaka</t>
+          <t>Hackathons - challenge.entelect.co.za</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://sebakasouthafrica.co.za/index.html</t>
+          <t>https://challenge.entelect.co.za/hackathons</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Sebaka Mentorship &amp; Hackathons — Build an AI Agent for Software Quality Engineering.</t>
+          <t>Compete against the best university teams across South Africa. Prize Pool: Various cool prizes &amp; bragging rights! A hands-on practice problem statement for Hack-ademy workshop attendees, joining in person or online.</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2889,17 +2925,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>GirlCode | Hackathon 2026</t>
+          <t>Hackathons | Sebaka</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://www.girlcode.co.za/hackathon-2026</t>
+          <t>https://sebakasouthafrica.co.za/hackathons.html</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>What is the GirlCode Hackathon? The GirlCode Hackathon is an annual, all-women 30 hours coding marathon designed to address the gender gap in the tech industry by providing female developers with a high-intensity, real-world platform to showcase their technical talent, develop innovative solutions, and build crucial industry networks.</t>
+          <t>Sebaka Mentorship &amp; Hackathons — Build an AI Agent for Software Quality Engineering.</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2953,7 +2989,11 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">

</xml_diff>

<commit_message>
Update competition data 2026-08-22
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -469,17 +469,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
+          <t>VUT inspires future engineers through Bridge Building Competition – Vaal University of Technology</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.poidata.io/report/engineer/south-africa</t>
+          <t>https://vut.ac.za/vut-inspires-future-engineers-through-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
+          <t>3 weeks ago - “VUT Ekhaya Alumni and SAICE STAR Vaal hosted the 2026 Bridge Building Competition, inspiring 16 Vaal schools through practical engineering, creativity and STEM education.”</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -492,17 +492,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Two South Africans on the shortlist for the 2026 Africa Prize for Engineering Innovation</t>
+          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/two-south-africans-on-the-shortlist-for-the-2026-africa-prize-for-engineering-innovation-2026-08-04</t>
+          <t>https://www.poidata.io/report/engineer/south-africa</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2 weeks ago - Two South African innovators have been shortlisted for the UK Royal Academy of Engineering’s Africa Prize for Engineering Innovation 2026. This is the continent’s richest award aimed at promoting engineering innovation and entrepreneurship ...</t>
+          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -510,26 +510,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>chanel@engineeringnews.co.za, newsletters@creamermedia.co.za, advertising@creamermedia.co.za, subscriptions@creamermedia.co.za, newsdesk@engineeringnews.co.za</t>
-        </is>
-      </c>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
+          <t>Two South Africans on the shortlist for the 2026 Africa Prize for Engineering Innovation</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
+          <t>https://www.engineeringnews.co.za/article/two-south-africans-on-the-shortlist-for-the-2026-africa-prize-for-engineering-innovation-2026-08-04</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1 week ago - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
+          <t>2 weeks ago - Two South African innovators have been shortlisted for the UK Royal Academy of Engineering’s Africa Prize for Engineering Innovation 2026. This is the continent’s richest award aimed at promoting engineering innovation and entrepreneurship ...</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -537,22 +533,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>newsdesk@engineeringnews.co.za, subscriptions@creamermedia.co.za, newsletters@creamermedia.co.za, advertising@creamermedia.co.za, chanel@engineeringnews.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
+          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>1 week ago - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -560,11 +560,7 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -592,17 +588,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.thecasecentre.org/products/view?id=189255</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -610,22 +606,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://www.thecasecentre.org/products/view?id=189255</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>South Africa · South Korea · Spain · Sri Lanka · Sudan · Sweden · Switzerland · Syrian Arab Republic · Taiwan · Tajikistan · Tanzania · Thailand · Togo · Trinidad and Tobago · Tunisia · Turkey · Uganda · Ukraine · United Arab Emirates · United Kingdom ·</t>
+          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -638,17 +638,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Engineering News|Real-Economy News</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.engineeringnews.co.za/</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>The competition invites South Africans to submit an original name for the new...</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -656,22 +656,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>newsletters@creamermedia.co.za, subscriptions@creamermedia.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Engineering News|Real-Economy News</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/</t>
+          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>The competition invites South Africans to submit an original name for the new...</t>
+          <t>South Africa · South Korea · Spain · Sri Lanka · Sudan · Sweden · Switzerland · Syrian Arab Republic · Taiwan · Tajikistan · Tanzania · Thailand · Togo · Trinidad and Tobago · Tunisia · Turkey · Uganda · Ukraine · United Arab Emirates · United Kingdom ·</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -679,26 +683,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>subscriptions@creamermedia.co.za, newsletters@creamermedia.co.za</t>
-        </is>
-      </c>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>South Africa International Industrial Expo | Innovation Bridge</t>
+          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
+          <t>https://10times.com/southafrica/tradeshows</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
+          <t>3 days ago · South Africa trade shows, find and compare 964 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 174 upcoming expos in 2026-2027 1. South Africa Infrastructure &amp; Water Expo, 2.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -711,17 +711,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
+          <t>Africa Tech Festival</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://madeinafricaevent.co.za/</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -729,22 +729,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>support@informaconnect.com, dataprivacy@informaconnect.com, support@knect365.com, salesenquiries@africatechfestival.com, customerservices@knect365.com, dataprivacy@knect365.com, customerservices@informaconnect.com</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show ...</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://manufacturingindaba.co.za/exhibition/</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
+          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -752,22 +756,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>enquiries@aiexpoafrica.com</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>KZN Industrial Technology Exhibition</t>
+          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://www.kznindustrial.co.za/</t>
+          <t>https://innovationweek.co.za/</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
+          <t>SAIW’ 26 is designed as a week-long national programme to feature provincial innovation engagements across South Africa. From 16 – 17 March, Provinces will showcase local innovation strengths, emerging enterprises and sectoral capabilities.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -777,24 +785,24 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>john@email.com</t>
+          <t>info@pixal8media.co.za</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Two landmark exhibitions set to transform industrial technology and renewable energy in South Africa</t>
+          <t>Innovations events in South Africa 2026-2027 - ExpoTobi</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/two-landmark-exhibitions-set-to-transform-industrial-technology-and-renewable-energy-in-south-africa-2025-10-24</t>
+          <t>https://expotobi.com/country/south-africa/sector/innovations</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>October 24, 2025 - South Africa’s industrial and clean energy sectors celebrated a landmark moment today with the official launch of RE+ South Africa 2026 and the Cape Industrial Technology Exhibition (CITE) 2027.</t>
+          <t>Innovations events in South Africa Full and accurate description of Innovations events Schedule, tickets, accommodation, travel arrangement and participation</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -802,26 +810,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>chanel@engineeringnews.co.za, newsletters@creamermedia.co.za, advertising@creamermedia.co.za, subscriptions@creamermedia.co.za, newsdesk@engineeringnews.co.za</t>
-        </is>
-      </c>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Exhibition | Innovation Festival Durban | South Africa</t>
+          <t>IT &amp; Technology Events in South Africa, List of all South ...</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://www.innovationfestival.durban/exhibition</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities.</t>
+          <t>1 day ago · Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -829,26 +833,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Erika@innovate.durban, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, sithabile@innovate.durban, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Trade Shows Worldwide - South Africa - 2026/2027</t>
+          <t>South Africa International Industrial Expo | Innovation Bridge</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://www.eventseye.com/fairs/c1_trade-shows_south-africa.html</t>
+          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>South Africa Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in South Africa</t>
+          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -861,17 +861,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Discover Innovation Hub's Pavilion at Organic &amp; Natural Products Expo - Organic &amp; Natural Products Portal</t>
+          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://www.organicandnaturalportal.com/innovation-hub-organic-expo/</t>
+          <t>https://madeinafricaevent.co.za/</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2 weeks ago - Gathering producers, retailers, buyers, and conscious consumers under one roof, the expo serves as Africa’s premier showcase for sustainability, health, and wellness innovation. A standout highlight of this year’s exhibition is The Innovation Hub Pavilion, hosting a curated line-up of forward-thinking South African small, medium, and micro-enterprises (SMMEs).</t>
+          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -884,17 +884,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>International Science, Innovation &amp; Technology Expo (INSITE)</t>
+          <t>KZN Industrial Technology Exhibition</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://www.dsti.gov.za/index.php/resource-center/27-temp/dst-links/3-international-science-innovation-a-technology-expo</t>
+          <t>https://www.kznindustrial.co.za/</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>The essence of INSITE INSITE is an international, biennial must-see Science and Technology event in South Africa, the only one of its kind in Africa that creates new frontiers for global challenges · INSITE aims to assemble the worlds leading innovators and scientists in one place, stimulating ...</t>
+          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -902,22 +902,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>john@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AAXO - The Association of African Exhibition Organisers</t>
+          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.aaxo.co.za/</t>
+          <t>https://manufacturingindaba.co.za/exhibition/</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>February 20, 2026 - CAPE TOWN, South Africa – The inaugural Festival of Eventing (FOE) brought together 350 event professionals, 85 speakers, and 10 countries under one roof for a two-day showcase of innovation, inspiration, and industry connection.</t>
+          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -930,17 +934,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
+          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -948,22 +952,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>Engineering for People Design Challenge | Department of ...</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
+          <t>Aug 4, 2025 · The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -973,24 +981,24 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
+          <t>web-editor@eng.cam.ac.uk, marketing@eng.cam.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EWB Design Challenge | Aston University</t>
+          <t>Engineering for People Design Challenge returns to Johannesburg!</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
+          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
+          <t>Sep 18, 2024 · Engineering for People Design Challenge returns to Johannesburg! Now entering its fourteenth year, we’re delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1003,17 +1011,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
+          <t>Engineering For People Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
+          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
+          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1023,24 +1031,24 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ied@ied.org.uk</t>
+          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Latest Community Engineering Design Competition Announced</t>
+          <t>Engineering for People Design Challenge - Engineers Without ...</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
+          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
+          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1053,17 +1061,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Real-world research: Engineering team designs South African trolley system; science students investigate heavy metals | University of Wisconsin - Stout</t>
+          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
+          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>May 15, 2025 - Research ranged from heavy metals ... Borders’ international design challenge. Nearly 90 students in 23 teams addressed the EWB challenge. One group focused on engineering a safer, more accessible transportation system in South ...</t>
+          <t>Oct 24, 2024 · The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1073,24 +1081,24 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>dolanm@uwstout.edu, frischj@uwstout.edu</t>
+          <t>team@crowdsolve.net</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Engineering for people, that’s the challenge | Engineers Without Borders</t>
+          <t>EWB Design Challenge | Aston University</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.rs-online.com/designspark/an-introduction-to-engineering-for-people-design-challenge</t>
+          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>That’s exactly what the annual Engineering for People Design Challenge asks participants to do. The competition, delivered in partnership by Engineers without Borders South Africa and Engineers Without Borders UK, encourages engineering students and those collaborating with engineers to broaden their awareness of how their decisions change the world.</t>
+          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1103,17 +1111,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of Engineering</t>
+          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
+          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1123,24 +1131,24 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
+          <t>ied@ied.org.uk</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Launching Engineering for People Design challenge 2024 ...</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.electronicspecifier.com/studentzone/studentzone-news/launching-engineering-for-people-design-challenge-2024-25-2/</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>November 16, 2025 - Engineers Without Borders has launched the 2024/25 cycle of the award-winning Engineering for People Design Challenge in partnership with Engineers Without Borders South Africa and Makers Valley Partnership.</t>
+          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1153,17 +1161,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
+          <t>Real-world research: Engineering team designs South African trolley system; science students investigate heavy metals | University of Wisconsin - Stout</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
+          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
+          <t>May 15, 2025 - Research ranged from heavy metals ... Borders’ international design challenge. Nearly 90 students in 23 teams addressed the EWB challenge. One group focused on engineering a safer, more accessible transportation system in South ...</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1171,22 +1179,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>frischj@uwstout.edu, dolanm@uwstout.edu</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
+          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1194,26 +1206,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
+          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1221,26 +1229,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>National Student Competition | ORSSA</t>
+          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://www.orssa.org.za/studentcomp</t>
+          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
+          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1248,26 +1252,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, email@example.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions.</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1280,17 +1280,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Sep 4, 2025 · The Africa Prize for Engineering Innovation is open to individuals or teams based in sub-Saharan Africa who have a scalable engineering innovation with social or environmental impact potential.</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1298,26 +1298,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Competitions – Enactus South Africa | National Expos ...</t>
+          <t>Engineering in South Africa: 24 Best universities Ranked</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://enactusza.org/what-we-do/competitions</t>
+          <t>https://edurank.org/engineering/za/</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Explore our national and international competitions that empower students to tackle challenges with entrepreneurial solutions and social impact at the core.</t>
+          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1325,26 +1321,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>adminsa@enactus.org, xmadlanga@enactus.org, marketingsa@enactus.org, liso@enactus.org</t>
-        </is>
-      </c>
+      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Wits ENERGISE Centre Call for Participation - Wits University</t>
+          <t>University Overall Rankings - Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://www.wits.ac.za/media/wits-university/faculties-and-schools/-engineering-and-the-built-environment/electrical-and-information-engineering/energise/wits-energise-centre-competition.pdf</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Join the ENERGISE Sustainable Business Model Competition 2026 and embark on guided academic training embedded in an international flagship project on the Just Energy Transition (JET) for the African-German Centre of Excellence held at Wits. Through iterative idea development, mentoring, and international exchange, participants co-develop application-oriented business model concepts addressing ...</t>
+          <t>University Overall Rankings - Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1352,26 +1344,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>muhammed.aswat1@wits.ac.za</t>
-        </is>
-      </c>
+      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
+          <t>University of South Africa</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
+          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-promotes-globally-recognised-engineering-qualifications</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
+          <t>Unisa promotes globally recognised engineering qualifications</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1384,17 +1372,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
+          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1407,17 +1395,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1440,7 +1428,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>February 20, 2026 - TECHSPO Johannesburg 2026 is a two day technology expo taking place September 28th to 29th, 2026 at the luxurious Hyatt Regency Johannesburg, Johannesburg, South Africa. TECHSPO Johannesburg brings together developers, brands, marketers, technology ...</t>
+          <t>3 weeks ago - TECHSPO Johannesburg 2026 is a two day technology expo taking place September 28th to 29th, 2026 at the luxurious Hyatt Regency Johannesburg, Johannesburg, South Africa. TECHSPO Johannesburg brings together developers, brands, marketers, technology ...</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1457,17 +1445,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Africa Tech Festival</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
+          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1477,14 +1465,14 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>salesenquiries@africatechfestival.com, customerservices@informaconnect.com, support@informaconnect.com, customerservices@knect365.com, dataprivacy@knect365.com, support@knect365.com, dataprivacy@informaconnect.com</t>
+          <t>info@techspocapetown.co.za</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>IT &amp; Technology Events in South Africa, List of all South Africa Technology Business Expo &amp; Events</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1494,7 +1482,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>7 hours ago · Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>New York Small Business Expo (Spring)07 MayNew York , USA · AFROZUM Fair · 07-09 May · Johannesburg , South Africa · AFROZUM Fair07-09 MayJohannesburg , South Africa · Nigeria Industries &amp; Manufacturing Summit · 18-20 May · Abuja , Nigeria ...</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1507,17 +1495,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Home - Mediatech Africa | South Africa</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://www.mediatech.co.za/</t>
+          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Mediatech Africa showcases the full range of professional tech driving AV, broadcast, media, &amp; live event production. From AV integration, unified communications &amp; display to pro audio, lighting, content creation, &amp; future tech — our sectors highlight the tools behind today’s connected experiences.</t>
+          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1527,24 +1515,24 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>claire@mediatech.co.za, simon@mediatech.co.za</t>
+          <t>atinfo@techspo.coor, u003einfo@techspo.co</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://africatechnologyexpo.com/</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
+          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1554,24 +1542,24 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>info@techspocapetown.co.za</t>
+          <t>info@sparkafrica.co, johndoe@email.com, partner@africatechnologyexpo.com</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
+          <t>Home - Mediatech Africa | South Africa</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://10times.com/johannesburg-za/technology</t>
+          <t>https://www.mediatech.co.za/</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience.</t>
+          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1579,22 +1567,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>claire@mediatech.co.za, simon@mediatech.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology ExpoJohannesburg Technology ...</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference - AI Expo Africa | 28 - 29 October SCC Johannesburg South Africa</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://techspojoburg.co.za/johannesburg-technology-expo/</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
+          <t>(2 Day Event) 28th-29th October 2026 Sandton Convention Centre, JHB, South Africa · AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade ...</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1602,22 +1594,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>enquiries@aiexpoafrica.com</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
+          <t>Discover Tech Conferences Events &amp; Activities in South Africa | Eventbrite</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
+          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
+          <t>Save this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South AfricaShare this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1625,26 +1621,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>atinfo@techspo.coor, u003einfo@techspo.co, name@example.com</t>
-        </is>
-      </c>
+      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
+          <t>IT &amp; Technology Events in Johannesburg, List of all Johannesburg Technology Business Expo &amp; Events in South Africa</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://africatechnologyexpo.com/</t>
+          <t>https://10times.com/johannesburg-za/technology</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
+          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1652,26 +1644,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>partner@africatechnologyexpo.com, info@sparkafrica.co, johndoe@email.com</t>
-        </is>
-      </c>
+      <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>HOME | Africa Tech Week</t>
+          <t>FinancialContent - TECHSPO Cape Town 2026 Unites Business, Tech and Marketing Leaders for High-Impact Expo</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://africatechweek.co.za/</t>
+          <t>https://markets.financialcontent.com/stocks/article/abnewswire-2026-4-8-techspo-cape-town-2026-unites-business-tech-and-marketing-leaders-for-high-impact-expo</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>May 11, 2026 - From sensational speakers, to top tech exhibitons, see what’s in store when you attend the 2-day Sentech Africa Tech Week Conference in 2025&gt;&gt; ... Sponsor, Speak, Attend! For more information on how you can be a part of the #ATW family, contact ...</t>
+          <t>April 8, 2026 - Cape Town, South Africa - TECHSPO Cape Town Technology Expo returns October 1-2, 2026, to the V&amp;A Waterfront Cape Town Avenue Conference Venue, uniting business leaders, technologists, marketers, and innovators for a high-impact, two-day showcase ...</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1717,7 +1705,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>May 3, 2026 - Maker Faires are also held in Europe, Asia, South America and Africa.</t>
+          <t>Maker Faire is a convention of do it yourself (DIY) enthusiasts established by Make magazine in 2006. Participants come from a wide variety of interests, such as robotics, 3D printing, computers, arts and crafts, and hacker culture.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1730,17 +1718,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
+          <t>Upcoming Faires - Maker Faire</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
+          <t>https://makerfaire.com/upcoming-faires/</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
+          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1748,22 +1736,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>fancybox_loading@2x.gif, chosen-sprite@2x.png, fancybox_sprite@2x.png, pr@make.co</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
+          <t>Maker Faire Africa — Grokipedia</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://makerfairecapetown.wordpress.com/about/</t>
+          <t>https://grokipedia.com/page/maker_faire_africa</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
+          <t>Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1776,17 +1768,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
+          <t>Maker Faire |</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>http://capetown.makerfaire.com/</t>
+          <t>https://makerfaire.com/</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
+          <t>A city’s Maker community, turned up to full volume. Hundreds of exhibitors, interactive zones, live talks, and a stage that lifts up expert makers and thought leaders alongside a few legendary guests.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1796,24 +1788,24 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>fancybox_sprite@2x.png, fancybox_loading@2x.gif, pr@make.co, chosen-sprite@2x.png</t>
+          <t>fancybox_loading@2x.gif, chosen-sprite@2x.png, fancybox_sprite@2x.png, pr@make.co</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
+          <t>Maker Faire groups | Meetup</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://contemporaryand.com/fr/events/maker-faire-africa-comes-to-johannesburg</t>
+          <t>https://www.meetup.com/topics/maker-faire/za/</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
+          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1826,17 +1818,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Jo’Burg – AfriGadget</t>
+          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://www.afrigadget.com/2014/07/08/maker-faire-africa-comes-to-joburg/</t>
+          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Maker Faire Africa 2014 will bring together over 5,000 attendees, along with featured inventors, world-class makers, self-made entrepreneurs &amp; workshop experts from South Africa, across the continent, and around the world, to manufacture real solutions for some of Africa’s most pressing ...</t>
+          <t>Aug 21, 2015 · We’re delighted to present the first ever Cape Town Maker Faire, hosted by Open Design in partnership with Trimble.Maker Faire is primarily designed as a forward-looking event, showcasing makers who are exploring new forms and new technologies.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1849,17 +1841,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Why Africa needs Maker Faire | ZDNET</t>
+          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://www.zdnet.com/article/why-africa-needs-maker-faire/</t>
+          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>July 24, 2014 - Unlike other Maker Faires, Okafor said that it's not enough to simply hold the event in an African city and see who turns up. Two volunteers are currently working in South Africa to discover inventors in rural areas and neighbouring countries such as Zambia and Botswana who they can encourage to attend and show off their work.</t>
+          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1867,26 +1859,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>brand_licensing@ziffdavis.com</t>
-        </is>
-      </c>
+      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>South Africa Archivi - Maker Faire Rome</t>
+          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://2019.makerfairerome.eu/en/tag/south-africa/</t>
+          <t>https://makerfairecapetown.wordpress.com/about/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>... It is the most important event in the world of innovation. Is a showcase of invention, creativity, and resourcefulness. Maker Faire gathers together tech enthusiasts, crafters, educators, tinkerers, schools, universities, research institutes, artists, students, and corporations.</t>
+          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1899,17 +1887,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Maker Faire returning to South Africa in August - Hypertext</t>
+          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://htxt.co.za/2015/07/maker-faire-returning-to-south-africa-in-august/</t>
+          <t>http://capetown.makerfaire.com/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>August 13, 2015 - Maker Faire will be held in Cape Town from 21st-23rd August at the V&amp;A Waterfront, with a Maker Faire Conference preceding the event on the 20th at The Lookout, V&amp;A Waterfront. The event is being backed by Maker Faire and Make: Magazine in the ...</t>
+          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1917,22 +1905,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>fancybox_loading@2x.gif, chosen-sprite@2x.png, fancybox_sprite@2x.png, pr@make.co</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>StemCo - StemCo 2026 International Competitions</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://stemco.org/</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>June 10, 2026 - BEST YOURSELF WITH STEMCO! Platform for the world’s brightest. ... Thanks to the participating 25 countries in 2019. Singapore, Albania, Australia, Azerbaijan, Canada, Germany, India, Indonesia, Japan, Jordan, Kazakhstan, Kyrgyzstan, Malawi, Mongolia, Nigeria, Myanmar, South Africa, Tajikistan, Turkey, Turkmenistan, Ukraine, The United States, Uzbekistan, Vietnam</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1945,7 +1937,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Samsung Solve for Tomorrow 2026: STEM contest opens - tech.africa</t>
+          <t>Samsung opens Solve for Tomorrow 2026 STEM competition to all South African public schools</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1955,7 +1947,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Feb 27, 2026 · Samsung Electronics South Africa has opened applications for the 2026 edition of Solve for Tomorrow (SFT), its annual science, technology, engineering, and mathematics (STEM) competition aimed at Grade 10 and 11 learners.</t>
+          <t>February 27, 2026 - Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1968,17 +1960,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Capetown 2026</t>
+          <t>High School STEM Competition | Southafrica 2024</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
+          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas. Each submission can provide a summary of the STEM project. All projects must be presented at the IEOM Cape Town, South Africa 2026.</t>
+          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, ...</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1995,17 +1987,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space ...</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Join the South African Space Design Competition to inspire space innovation, develop STEM skills, and compete for a trip to NASA. Perfect for high school students passionate about space.</t>
+          <t>Local, regional and national competitions with thousands of · Multi-level events of two or more rounds that become increasingly challenging and culminate in top-level Olympiads. Enrichment programmes to inspire promising young South Africans to pursue STEMI</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2013,26 +2005,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>user@domain.com, info@zasdc.org</t>
-        </is>
-      </c>
+      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
+          <t>ASTEMI Competitions 2022 – SAASTA</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/za/solvefortomorrow/</t>
+          <t>https://saasta.ac.za/astemi-competitions-2</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Rooted in the belief that today’s youth hold the key to tomorrow’s progress, Solve for Tomorrow South Africa provides participants with the tools, mentorship, and platforms they need to turn ideas into action.</t>
+          <t>National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2045,17 +2033,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ASTEMI SA</t>
+          <t>2026 Season - Africa's Global STEM Celebration</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/</t>
+          <t>https://www.stemfestival.org/competitions/</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
+          <t>April 30, 2026 - ... The Elementary, Junior, and Senior Robotics categories at STEM Festival are dedicated to advancing the World Robot Olympiad (WRO) across the Niger Delta and South-South Nigeria, working with ArcLights Foundation.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2068,17 +2056,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>StemCo - StemCo 2026 International Competitions</t>
+          <t>STEAM Pitch Competition - STEM AFRICA FEST 2024</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://stemco.org/</t>
+          <t>https://stemafricafest.com/steam-pitch-competition/</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>June 10, 2026 - BEST YOURSELF WITH STEMCO! Platform for the world’s brightest. ... Thanks to the participating 25 countries in 2019. Singapore, Albania, Australia, Azerbaijan, Canada, Germany, India, Indonesia, Japan, Jordan, Kazakhstan, Kyrgyzstan, Malawi, Mongolia, Nigeria, Myanmar, South Africa, Tajikistan, Turkey, Turkmenistan, Ukraine, The United States, Uzbekistan, Vietnam</t>
+          <t>Join STEM Africa Fest , celebrating science, technology, engineering, and mathematics. Experience hands-on learning, industry leaders, and innovation across Africa.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2091,17 +2079,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Southafrica 2024</t>
+          <t>Competition – Eskom Expo for Young Scientists</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
+          <t>https://exposcience.co.za/category/competition/</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, ...</t>
+          <t>Aqil Variava business cities Damien ... Gray STEMI Vuyo Nzimande · Eskom Expo for Young Scientists is an exposition, or science fair, where students have a chance to show others their projects about their own scientific investigations. At the annual prestigious Eskom Expo for Young Scientists International Science Fair (ISF), selected students from 35 Expo Regions in South Africa then compete ...</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2111,24 +2099,24 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>info@ieomsociety.org</t>
+          <t>support@exposcience.co.za</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions 2022 – SAASTA</t>
+          <t>SA young scientists selected for global competition at Regeneron ISEF in the USA - Eskom</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://saasta.ac.za/astemi-competitions-2</t>
+          <t>https://www.eskom.co.za/sa-young-scientists-selected-for-global-competition-at-regeneron-isef-in-the-usa/</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>May 6, 2025 - Regeneron ISEF 2025, the world’s largest pre-college science, technology, engineering and mathematics (STEM) competition, will take place from 10 to 16 May in Columbus, Ohio in the USA.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2136,22 +2124,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>MediaDesk@eskom.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026 Season - Africa's Global STEM Celebration</t>
+          <t>Rural youth lead in robotics at national STEM competition</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://www.stemfestival.org/competitions/</t>
+          <t>https://iol.co.za/news/education/2025-09-15-rural-youth-lead-in-robotics-at-national-stem-competition/</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>April 30, 2026 - ... The Elementary, Junior, and Senior Robotics categories at STEM Festival are dedicated to advancing the World Robot Olympiad (WRO) across the Niger Delta and South-South Nigeria, working with ArcLights Foundation.</t>
+          <t>September 15, 2025 - Discover how South Africa's brightest young minds are tackling real-world challenges with innovative solutions at the inaugural AlgoAtWork RoboRumble STEM Innovation Challenge, where ideas like autonomous robots and smart PPE systems are set ...</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2159,7 +2151,11 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>philippa.larkin@inl.co.za, mendy.mtshali@inl.co.za, nobuntu.mgijima@volt.africa, ashley.lechman@inl.co.za, londiwe.gumede@inl.co.za, lee.rondganger@inl.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2182,7 +2178,11 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, info@thecortexhub.africa, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com</t>
+          <t>dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, info@thecortexhub.africa, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -2268,17 +2268,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Roboticon 2026: South Africa Showcases Robotics for Culture ...</t>
+          <t>Live Competitions — Nirvana Global Foundation</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://www.ubuntutimes.co.za/roboticon-2026-south-africa-showcases-robotics-for-culture-education-and-innovation/</t>
+          <t>https://nirvanaglobalfoundation.org/competition.html</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Jul 2, 2026 · South Africa’s robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation. Hosted at the Heartfelt Arena in Pretoria, the event is not only a showcase of technical skills but also a celebration of how robotics can address societal challenges.</t>
+          <t>Enjoy AI South Africa An international AI and robotics competition for young innovators. Teams build, program and compete with official ENJOY AI robotics kits across categories like Battle of Stars, Mining Expedition, Drone Cup and Inventions Trail — preparing learners for the global ENJOY AI stage.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2288,24 +2288,24 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>newspaper-rec300@2x.jpg, adverts@ubuntutimes.co.za</t>
+          <t>info@nirvanaglobalfoundation.org, coach@school.co.za</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Home | Roboticon 2026</t>
+          <t>ROBO-RUMBLE 2026 — Innovation in Motion</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://roboticon.resolute.education/</t>
+          <t>https://roborumble.net/</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Join us for the ultimate robotics showcase as Resolute proudly sponsors the World Robotics Olympiad (WRO) South Africa! This year, we're bringing together two worlds for the biggest robotics event of the year – Roboticon and the WRO Nationals, happening on the same day at the same venue.</t>
+          <t>South Africa's premier youth robotics &amp; technology competition. Robo Wars, Drone Racing, Grand Prix &amp; Innovation Challenge. August 2026.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2318,17 +2318,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ROBO-RUMBLE 2026 — Innovation in Motion</t>
+          <t>Home | Roboticon 2026</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://roborumble.net/</t>
+          <t>https://roboticon.resolute.education/</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>South Africa's premier youth robotics &amp; technology competition. Robo Wars, Drone Racing, Grand Prix &amp; Innovation Challenge. August 2026.</t>
+          <t>Join us for the ultimate robotics showcase as Resolute proudly sponsors the World Robotics Olympiad (WRO) South Africa! This year, we're bringing together two worlds for the biggest robotics event of the year – Roboticon and the WRO Nationals, happening on the same day at the same venue.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2341,17 +2341,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering</t>
+          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://civils.org.za/</t>
+          <t>https://safcec.org.za/</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
+          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2359,22 +2359,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>communication@safcec.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
+          <t>The South African Institution of Civil Engineering</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://safcec.org.za/</t>
+          <t>https://civils.org.za/</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
+          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2382,26 +2386,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>communication@safcec.org.za</t>
-        </is>
-      </c>
+      <c r="E80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Engineering the Future: 16 schools compete in SAICE’s 33rd ...</t>
+          <t>ICE Africa – Supporting Civil Engineers in Africa</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://southafricatoday.net/lifestyle/education/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
+          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Aug 30, 2024 · The South African Institution of Civil Engineering (SAICE) hosted its 33 rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
+          <t>Click your country to find local events, competitions, and information on how you can get more involved. At the heart of everything we do in South Africa is ICE-SA, the volunteer ICE local association (formerly known as the Joint Civils Division).</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2414,17 +2414,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ICE Africa – Supporting Civil Engineers in Africa</t>
+          <t>Engineering the Future: 16 schools compete in SAICE’s 33rd ...</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
+          <t>https://southafricatoday.net/lifestyle/education/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Click your country to find local events, competitions, and information on how you can get more involved. At the heart of everything we do in South Africa is ICE-SA, the volunteer ICE local association (formerly known as the Joint Civils Division).</t>
+          <t>Aug 30, 2024 · The South African Institution of Civil Engineering (SAICE) hosted its 33 rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2457,7 +2457,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>barbara@avenue.co.za, communications@saice.org.za, membership@saice.org.za, accounts@saice.org.za, civilinfo@saice.org.za, marketing@saice.org.za, executiveadmin@saice.org.za</t>
+          <t>communications@saice.org.za, civilinfo@saice.org.za, membership@saice.org.za, barbara@avenue.co.za, executiveadmin@saice.org.za, marketing@saice.org.za, accounts@saice.org.za</t>
         </is>
       </c>
     </row>
@@ -2507,7 +2507,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>communications@saice.org.za, memory@saice.org.za, accounts@saice.org.za, civilinfo@saice.org.za, marketing@saice.org.za, membership@saice.org.za</t>
+          <t>communications@saice.org.za, civilinfo@saice.org.za, membership@saice.org.za, memory@saice.org.za, marketing@saice.org.za, accounts@saice.org.za</t>
         </is>
       </c>
     </row>
@@ -2637,17 +2637,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>APPLY NOW! WORLDSKILLS SOUTH AFRICA NATIONAL COMPETITION 2025</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>ndidate with an accredited qualification in the related skill - Candida. e must not turn 23 years old in 2026 for the skills required. - Candidate applying for Aircraft Maintenance, Mechatr.</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2729,17 +2729,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
+          <t>Electrical Engineering Conferences in South Africa 2026/2027 ...</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
+          <t>https://conferenceindex.org/conferences/electrical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 · IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa) Deadline: April 30, 2026 May 15, 2026</t>
+          <t>Electrical Engineering Conferences in South Africa 2026 2027 2028 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and symposiums.</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2752,17 +2752,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Electrical Engineering Conferences in South Africa 2026/2027 ...</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://conferenceindex.org/conferences/electrical-engineering/south-africa</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Electrical Engineering Conferences in South Africa 2026 2027 2028 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and symposiums.</t>
+          <t>Sep 4, 2025 · The Africa Prize for Engineering Innovation is open to individuals or teams based in sub-Saharan Africa who have a scalable engineering innovation with social or environmental impact potential.</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2770,22 +2770,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers</t>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/</t>
+          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Companies are composed of a number of job roles &amp; ... All equipment from massive ships to tiny devices h ... Earn your CPD credits today! Read it here.</t>
+          <t>Apr 30, 2026 · IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa) Deadline: April 30, 2026 May 15, 2026</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2793,26 +2797,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, reception@saiee.org.za</t>
-        </is>
-      </c>
+      <c r="E97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Competitions | ESG</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://za.rs-online.com/web/content/m/competition</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Find your next opportunity below, we stagger them throughout the year so make sure to check back regularly for up to date information. Good luck! The RS Student Project Fund 2026 provides successful applicants with up to R10 000 to spend on RS products.</t>
+          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions.</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2820,26 +2820,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>example@email.com</t>
-        </is>
-      </c>
+      <c r="E98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Wits ENERGISE Centre Call for Participation Shaping the ...</t>
+          <t>South African Institute of Electrical Engineers</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://www.wits.ac.za/media/wits-university/faculties-and-schools/-engineering-and-the-built-environment/electrical-and-information-engineering/energise/wits-energise-centre-competition.pdf</t>
+          <t>https://www.saiee.org.za/</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Join the ENERGISE Sustainable Business Model Competition 2026 and embark on guided academic training embedded in an international flagship project on the Just Energy Transition (JET) for the African-German Centre of Excellence held at Wits. Through iterative idea development, mentoring, and international exchange, participants co-develop application-oriented business model concepts addressing ...</t>
+          <t>All equipment from massive ships to tiny devices h ... Earn your CPD credits today! Read it here.</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2849,7 +2845,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>muhammed.aswat1@wits.ac.za</t>
+          <t>reception@saiee.org.za, glueup-logo-white@2x.png</t>
         </is>
       </c>
     </row>
@@ -2902,17 +2898,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Hackathons - challenge.entelect.co.za</t>
+          <t>Build the Future with Entelect Hackathons</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://challenge.entelect.co.za/hackathons</t>
+          <t>https://challenge.entelect.co.za/</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Compete against the best university teams across South Africa. Prize Pool: Various cool prizes &amp; bragging rights! A hands-on practice problem statement for Hack-ademy workshop attendees, joining in person or online.</t>
+          <t>Instead of focusing on building a once-off project, our hackathons centre around optimisation problems. Participants develop solutions that are tested, scored, and ranked based on performance, efficiency, and strategy.</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2925,17 +2921,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Hackathons | Sebaka</t>
+          <t>Hackathons - challenge.entelect.co.za</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://sebakasouthafrica.co.za/hackathons.html</t>
+          <t>https://challenge.entelect.co.za/hackathons</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Sebaka Mentorship &amp; Hackathons — Build an AI Agent for Software Quality Engineering.</t>
+          <t>7 hours ago · Compete against the best university teams across South Africa. Prize Pool: Various cool prizes &amp; bragging rights! A hands-on practice problem statement for Hack-ademy workshop attendees, joining in person or online.</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2948,17 +2944,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Build the Future with Entelect Hackathons</t>
+          <t>Hackathons | Sebaka</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://challenge.entelect.co.za/</t>
+          <t>https://sebakasouthafrica.co.za/hackathons.html</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Instead of focusing on building a once-off project, our hackathons centre around optimisation problems. Participants develop solutions that are tested, scored, and ranked based on performance, efficiency, and strategy.</t>
+          <t>Sebaka Mentorship &amp; Hackathons — Build an AI Agent for Software Quality Engineering.</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2991,7 +2987,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
+          <t>marketing@ortsa.org.za, info@ortsa.org.za</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update competition data 2026-08-23
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E106"/>
+  <dimension ref="A1:E121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2 weeks ago - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -464,22 +464,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>VUT inspires future engineers through Bridge Building Competition – Vaal University of Technology</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://vut.ac.za/vut-inspires-future-engineers-through-bridge-building-competition/</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>3 weeks ago - “VUT Ekhaya Alumni and SAICE STAR Vaal hosted the 2026 Bridge Building Competition, inspiring 16 Vaal schools through practical engineering, creativity and STEM education.”</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -487,22 +491,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.poidata.io/report/engineer/south-africa</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -515,17 +523,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Two South Africans on the shortlist for the 2026 Africa Prize for Engineering Innovation</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/two-south-africans-on-the-shortlist-for-the-2026-africa-prize-for-engineering-innovation-2026-08-04</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2 weeks ago - Two South African innovators have been shortlisted for the UK Royal Academy of Engineering’s Africa Prize for Engineering Innovation 2026. This is the continent’s richest award aimed at promoting engineering innovation and entrepreneurship ...</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa. Find out more</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -533,26 +541,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>newsdesk@engineeringnews.co.za, subscriptions@creamermedia.co.za, newsletters@creamermedia.co.za, advertising@creamermedia.co.za, chanel@engineeringnews.co.za</t>
-        </is>
-      </c>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
+          <t>National Student Competition | ORSSA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
+          <t>https://www.orssa.org.za/studentcomp</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1 week ago - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
+          <t>National Student Competitions The Operations Research Society of South Africa The home of decision intelligence The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -560,22 +564,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, email@example.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Engineering Conferences in South Africa 2025-2026</t>
+          <t>Competitions - Enactus South Africa | National Expos, Challenges ...</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
+          <t>https://enactusza.org/what-we-do/competitions</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
+          <t>Enactus South Africa Competitions Enactus National Exposition The Enactus National Exposition is a dynamic annual event where student teams from across the country come together to showcase the progress and impact of their entrepreneurial projects.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -583,22 +591,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>liso@enactus.org, xmadlanga@enactus.org, adminsa@enactus.org, marketingsa@enactus.org</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -606,26 +618,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.thecasecentre.org/products/view?id=189255</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -638,17 +646,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Engineering News|Real-Economy News</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>The competition invites South Africans to submit an original name for the new...</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -658,24 +666,24 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>newsletters@creamermedia.co.za, subscriptions@creamermedia.co.za</t>
+          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>ECSA - Engineering Council of South Africa</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://www.ecsa.co.za/</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>South Africa · South Korea · Spain · Sri Lanka · Sudan · Sweden · Switzerland · Syrian Arab Republic · Taiwan · Tajikistan · Tanzania · Thailand · Togo · Trinidad and Tobago · Tunisia · Turkey · Uganda · Ukraine · United Arab Emirates · United Kingdom ·</t>
+          <t>The Engineering Council of South Africa is the only body in South Africa that is authorised to register engineering professionals and bestow the use of engineering titles, such as Pr Eng, Pr Tech Eng, Pr Techni Eng, Pr Cert Eng, on persons who have the requisite registration criteria.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -688,17 +696,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
+          <t>South Africa International Industrial Expo | Innovation Bridge</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/tradeshows</t>
+          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3 days ago · South Africa trade shows, find and compare 964 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 174 upcoming expos in 2026-2027 1. South Africa Infrastructure &amp; Water Expo, 2.</t>
+          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -711,17 +719,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Africa Tech Festival</t>
+          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://madeinafricaevent.co.za/</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
+          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -729,26 +737,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>support@informaconnect.com, dataprivacy@informaconnect.com, support@knect365.com, salesenquiries@africatechfestival.com, customerservices@knect365.com, dataprivacy@knect365.com, customerservices@informaconnect.com</t>
-        </is>
-      </c>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show ...</t>
+          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://manufacturingindaba.co.za/exhibition/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
+          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -756,26 +760,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>enquiries@aiexpoafrica.com</t>
-        </is>
-      </c>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
+          <t>KZN Industrial Technology Exhibition</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://innovationweek.co.za/</t>
+          <t>https://www.kznindustrial.co.za/</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SAIW’ 26 is designed as a week-long national programme to feature provincial innovation engagements across South Africa. From 16 – 17 March, Provinces will showcase local innovation strengths, emerging enterprises and sectoral capabilities.</t>
+          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -785,24 +785,24 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>info@pixal8media.co.za</t>
+          <t>john@email.com</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Innovations events in South Africa 2026-2027 - ExpoTobi</t>
+          <t>Two landmark exhibitions set to transform industrial technology and renewable energy in South Africa</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://expotobi.com/country/south-africa/sector/innovations</t>
+          <t>https://www.engineeringnews.co.za/article/two-landmark-exhibitions-set-to-transform-industrial-technology-and-renewable-energy-in-south-africa-2025-10-24</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Innovations events in South Africa Full and accurate description of Innovations events Schedule, tickets, accommodation, travel arrangement and participation</t>
+          <t>October 24, 2025 - South Africa’s industrial and clean energy sectors celebrated a landmark moment today with the official launch of RE+ South Africa 2026 and the Cape Industrial Technology Exhibition (CITE) 2027.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -810,22 +810,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>advertising@creamermedia.co.za, newsletters@creamermedia.co.za, subscriptions@creamermedia.co.za, newsdesk@engineeringnews.co.za, chanel@engineeringnews.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa, List of all South ...</t>
+          <t>Exhibition | Innovation Festival Durban | South Africa</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://www.innovationfestival.durban/exhibition</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1 day ago · Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -833,22 +837,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>c183baa23371454f99f417f6616b724d@sentry.wixpress.com, sithabile@innovate.durban, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, Erika@innovate.durban, 8c4075d5481d476e945486754f783364@sentry.io, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>South Africa International Industrial Expo | Innovation Bridge</t>
+          <t>International Science, Innovation &amp; Technology Expo (INSITE)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
+          <t>https://www.dsti.gov.za/index.php/resource-center/27-temp/dst-links/3-international-science-innovation-a-technology-expo</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
+          <t>The essence of INSITE INSITE is an international, biennial must-see Science and Technology event in South Africa, the only one of its kind in Africa that creates new frontiers for global challenges · INSITE aims to assemble the worlds leading innovators and scientists in one place, stimulating ...</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -861,17 +869,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
+          <t>Discover Innovation Hub's Pavilion at Organic &amp; Natural Products Expo - Organic &amp; Natural Products Portal</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://madeinafricaevent.co.za/</t>
+          <t>https://www.organicandnaturalportal.com/innovation-hub-organic-expo/</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
+          <t>2 weeks ago - Gathering producers, retailers, buyers, and conscious consumers under one roof, the expo serves as Africa’s premier showcase for sustainability, health, and wellness innovation. A standout highlight of this year’s exhibition is The Innovation Hub Pavilion, hosting a curated line-up of forward-thinking South African small, medium, and micro-enterprises (SMMEs).</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -884,17 +892,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>KZN Industrial Technology Exhibition</t>
+          <t>Trade Shows Worldwide - South Africa - 2026/2027</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://www.kznindustrial.co.za/</t>
+          <t>https://www.eventseye.com/fairs/c1_trade-shows_south-africa.html</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
+          <t>South Africa Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in South Africa</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -902,26 +910,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>john@email.com</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
+          <t>AAXO - The Association of African Exhibition Organisers</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://manufacturingindaba.co.za/exhibition/</t>
+          <t>https://www.aaxo.co.za/</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
+          <t>February 20, 2026 - CAPE TOWN, South Africa – The inaugural Festival of Eventing (FOE) brought together 350 event professionals, 85 speakers, and 10 countries under one roof for a two-day showcase of innovation, inspiration, and industry connection.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -934,17 +938,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
+          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -952,26 +956,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
-        </is>
-      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of ...</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Aug 4, 2025 · The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
+          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -981,24 +981,24 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>web-editor@eng.cam.ac.uk, marketing@eng.cam.ac.uk</t>
+          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge returns to Johannesburg!</t>
+          <t>EWB Design Challenge | Aston University</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
+          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Sep 18, 2024 · Engineering for People Design Challenge returns to Johannesburg! Now entering its fourteenth year, we’re delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
+          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1011,17 +1011,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Engineering For People Design Challenge - EWBSA</t>
+          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
+          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
+          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1031,24 +1031,24 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
+          <t>ied@ied.org.uk</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge - Engineers Without ...</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
+          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1061,17 +1061,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
+          <t>Real-world research: Engineering team designs South African trolley system; science students investigate heavy metals | University of Wisconsin - Stout</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
+          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Oct 24, 2024 · The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
+          <t>May 15, 2025 - Research ranged from heavy metals ... Borders’ international design challenge. Nearly 90 students in 23 teams addressed the EWB challenge. One group focused on engineering a safer, more accessible transportation system in South ...</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1081,24 +1081,24 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>team@crowdsolve.net</t>
+          <t>dolanm@uwstout.edu, frischj@uwstout.edu</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>EWB Design Challenge | Aston University</t>
+          <t>Engineering for people, that’s the challenge | Engineers Without Borders</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
+          <t>https://www.rs-online.com/designspark/an-introduction-to-engineering-for-people-design-challenge</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
+          <t>That’s exactly what the annual Engineering for People Design Challenge asks participants to do. The competition, delivered in partnership by Engineers without Borders South Africa and Engineers Without Borders UK, encourages engineering students and those collaborating with engineers to broaden their awareness of how their decisions change the world.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1111,17 +1111,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
+          <t>Engineering for People Design Challenge | Department of Engineering</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
+          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1129,26 +1129,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>ied@ied.org.uk</t>
-        </is>
-      </c>
+      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Latest Community Engineering Design Competition Announced</t>
+          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
+          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
+          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1161,17 +1157,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Real-world research: Engineering team designs South African trolley system; science students investigate heavy metals | University of Wisconsin - Stout</t>
+          <t>Launching Engineering for People Design challenge 2024 ...</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
+          <t>https://www.electronicspecifier.com/studentzone/studentzone-news/launching-engineering-for-people-design-challenge-2024-25-2/</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>May 15, 2025 - Research ranged from heavy metals ... Borders’ international design challenge. Nearly 90 students in 23 teams addressed the EWB challenge. One group focused on engineering a safer, more accessible transportation system in South ...</t>
+          <t>November 16, 2025 - Engineers Without Borders has launched the 2024/25 cycle of the award-winning Engineering for People Design Challenge in partnership with Engineers Without Borders South Africa and Makers Valley Partnership.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1179,26 +1175,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>frischj@uwstout.edu, dolanm@uwstout.edu</t>
-        </is>
-      </c>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1206,22 +1198,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1229,22 +1225,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
+          <t>National Student Competition | ORSSA</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
+          <t>https://www.orssa.org.za/studentcomp</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
+          <t>National Student Competitions The Operations Research Society of South Africa The home of decision intelligence The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1252,22 +1252,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, email@example.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1280,17 +1284,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1303,17 +1307,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Engineering in South Africa: 24 Best universities Ranked</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://edurank.org/engineering/za/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1326,17 +1330,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2025</t>
+          <t>Competitions - Enactus South Africa | National Expos, Challenges ...</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
+          <t>https://enactusza.org/what-we-do/competitions</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2025</t>
+          <t>Explore our national and international competitions that empower students to tackle challenges with entrepreneurial solutions and social impact at the core.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1344,22 +1348,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>liso@enactus.org, xmadlanga@enactus.org, adminsa@enactus.org, marketingsa@enactus.org</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>University of South Africa</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-promotes-globally-recognised-engineering-qualifications</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Unisa promotes globally recognised engineering qualifications</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1367,22 +1375,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
+          <t>Competitions - SABSA</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
+          <t>https://sabsa.co.za/competitions/</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
+          <t>African Business Concept Challenge ABCC is a virtual simulation-based business concept competition for African undergraduate and graduate students. The competition will challenge student teams to design a viable business concept that addresses a locally-relevant challenge or problem related to Agenda 2063, and inclusive and sustainable development.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1390,22 +1402,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>anne@sabsa.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
+          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa) Deadline: April 30, 2026 May 15, 2026</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1418,7 +1434,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 (Internet ...</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1428,7 +1444,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>3 weeks ago - TECHSPO Johannesburg 2026 is a two day technology expo taking place September 28th to 29th, 2026 at the luxurious Hyatt Regency Johannesburg, Johannesburg, South Africa. TECHSPO Johannesburg brings together developers, brands, marketers, technology ...</t>
+          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1445,17 +1461,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>Africa Tech Festival</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1465,24 +1481,24 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>info@techspocapetown.co.za</t>
+          <t>salesenquiries@africatechfestival.com, dataprivacy@informaconnect.com, customerservices@informaconnect.com, customerservices@knect365.com, support@informaconnect.com, dataprivacy@knect365.com, support@knect365.com</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa, List of all South Africa Technology Business Expo &amp; Events</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 - 7, 2027 ...</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>New York Small Business Expo (Spring)07 MayNew York , USA · AFROZUM Fair · 07-09 May · Johannesburg , South Africa · AFROZUM Fair07-09 MayJohannesburg , South Africa · Nigeria Industries &amp; Manufacturing Summit · 18-20 May · Abuja , Nigeria ...</t>
+          <t>The annual TECHSPO Cape Town 2027 Technology Expo returns October 6th to 7th, 2027 to the V&amp;A Waterfront Cape Town Avenue Conference Venue in Cape Town. TECHSPO Cape Town Technology Expo is the must-attend event to: Experience the Future of Technology &amp; Innovation Discover cutting-edge tech, game-changing tools, and innovators shaping tomorrow's digital world. See the latest advancements in ...</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1490,22 +1506,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>info@techspocapetown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
+          <t>TECHSPO Johannesburg Technology ExpoJohannesburg Technology Expo ...</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
+          <t>https://techspojoburg.co.za/johannesburg-technology-expo/</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
+          <t>TECHSPO Johannesburg is a 2-day technology expo taking place September 28 - 29, 2026 at the luxurious NH Johannesburg Sandton Hotel, Toronto, Ontario. TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1513,26 +1533,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>atinfo@techspo.coor, u003einfo@techspo.co</t>
-        </is>
-      </c>
+      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
+          <t>Tech Expo Africa - Enabling Development</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://africatechnologyexpo.com/</t>
+          <t>https://techexpo.africa/</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
+          <t>Tech Expo Africa is a social enterprise connecting African businesses with top tech and business leaders to drive innovation.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1542,7 +1558,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>info@sparkafrica.co, johndoe@email.com, partner@africatechnologyexpo.com</t>
+          <t>info@techexpo.africa</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1575,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
+          <t>Mediatech Africa is the continent's largest trade expo for professional AV, media, broadcast, and live entertainment technology. For 25 years, it's been the industry's meeting place — where manufacturers, integrators, creatives, and decision-makers come together to connect, discover new tech, and do business.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1569,24 +1585,24 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>claire@mediatech.co.za, simon@mediatech.co.za</t>
+          <t>simon@mediatech.co.za, claire@mediatech.co.za</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference - AI Expo Africa | 28 - 29 October SCC Johannesburg South Africa</t>
+          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://10times.com/johannesburg-za/technology</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>(2 Day Event) 28th-29th October 2026 Sandton Convention Centre, JHB, South Africa · AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade ...</t>
+          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1594,26 +1610,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>enquiries@aiexpoafrica.com</t>
-        </is>
-      </c>
+      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Discover Tech Conferences Events &amp; Activities in South Africa | Eventbrite</t>
+          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Save this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South AfricaShare this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South Africa</t>
+          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1626,17 +1638,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in Johannesburg, List of all Johannesburg Technology Business Expo &amp; Events in South Africa</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~…</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://10times.com/johannesburg-za/technology</t>
+          <t>https://www.industryevents.com/events/techspo-johannesburg-2026-technology-expo-internet-mobile-adtech-martech-saas</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience.</t>
+          <t>Exhibitions &amp; Tradeshows on 22 Sept 2026 - 23 Sept 2026 in South Africa. TECHSPO Johannesburg - Where Business, Tech and Innovation Collide in…</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1644,22 +1656,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>your@email.com, events@techspojoburg.co.za, colleague@company.com, you@company.com, support@industryevents.com</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>FinancialContent - TECHSPO Cape Town 2026 Unites Business, Tech and Marketing Leaders for High-Impact Expo</t>
+          <t>TECHSPO Cape Town 2026 Technology Expo (Internet ~ Mobile ~ AdTech ...</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://markets.financialcontent.com/stocks/article/abnewswire-2026-4-8-techspo-cape-town-2026-unites-business-tech-and-marketing-leaders-for-high-impact-expo</t>
+          <t>https://allevents.in/cape-town/techspo-cape-town-2026-technology-expo-internet-~-mobile-~-adtech-~-martech-~-saas/200030358413547</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>April 8, 2026 - Cape Town, South Africa - TECHSPO Cape Town Technology Expo returns October 1-2, 2026, to the V&amp;A Waterfront Cape Town Avenue Conference Venue, uniting business leaders, technologists, marketers, and innovators for a high-impact, two-day showcase ...</t>
+          <t>TECHSPO Cape Town Technology Expo returns October 1-2, 2026 to the V&amp;A Waterfront Cape Town Avenue Conference Venue in Cape Town, South Africa. This must-attend, two-day annual event brings together leading developers, marketers, innovators, and technology enthusiasts eager to showcase and explore the latest in tech and digital solutions.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1718,17 +1734,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Upcoming Faires - Maker Faire</t>
+          <t>HOME | MAKERS FEST</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://makerfaire.com/upcoming-faires/</t>
+          <t>https://www.makersfestival.co.za/</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
+          <t>On 8 &amp; 9 November 2025 at The Ostrich in Cape Town, join 2,000+ visitors each day for maker demos, a curated market, and family activities. It’s Africa’s first hands-on festival for creativity and craftsmanship — and everything you make, you take home. Tickets are on sale now.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1738,24 +1754,24 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>fancybox_loading@2x.gif, chosen-sprite@2x.png, fancybox_sprite@2x.png, pr@make.co</t>
+          <t>79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, warren@makersfestival.co.za, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, example@mysite.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Maker Faire Africa — Grokipedia</t>
+          <t>Upcoming Faires - Maker Faire</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://grokipedia.com/page/maker_faire_africa</t>
+          <t>https://makerfaire.com/upcoming-faires/</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
+          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1763,22 +1779,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>fancybox_loading@2x.gif, fancybox_sprite@2x.png, chosen-sprite@2x.png, pr@make.co</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Maker Faire |</t>
+          <t>Maker Faire Africa — Grokipedia</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://makerfaire.com/</t>
+          <t>https://grokipedia.com/page/maker_faire_africa</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>A city’s Maker community, turned up to full volume. Hundreds of exhibitors, interactive zones, live talks, and a stage that lifts up expert makers and thought leaders alongside a few legendary guests.</t>
+          <t>Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1786,26 +1806,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>fancybox_loading@2x.gif, chosen-sprite@2x.png, fancybox_sprite@2x.png, pr@make.co</t>
-        </is>
-      </c>
+      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Maker Faire groups | Meetup</t>
+          <t>Maker Faire |</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/topics/maker-faire/za/</t>
+          <t>https://makerfaire.com/</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
+          <t>A city’s Maker community, turned up to full volume. Hundreds of exhibitors, interactive zones, live talks, and a stage that lifts up expert makers and thought leaders alongside a few legendary guests.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1813,7 +1829,11 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>pr@make.co</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1907,7 +1927,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>fancybox_loading@2x.gif, chosen-sprite@2x.png, fancybox_sprite@2x.png, pr@make.co</t>
+          <t>fancybox_loading@2x.gif, fancybox_sprite@2x.png, chosen-sprite@2x.png, pr@make.co</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1952,11 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>t.azizakhon@gmail.com, hkoffice@missmaneducation.com, name@example.com, stemcomongolia@gmail.com, education@missmaneducation.com, info.iksc@kangaroo.org.pk, havtt@fermat.edu.vn, bestyourself@stemco.org, example@mail.com, awaisnaeem786@gmail.com, info@missmaneducation.com</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2153,7 +2177,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>philippa.larkin@inl.co.za, mendy.mtshali@inl.co.za, nobuntu.mgijima@volt.africa, ashley.lechman@inl.co.za, londiwe.gumede@inl.co.za, lee.rondganger@inl.co.za</t>
+          <t>ashley.lechman@inl.co.za, mendy.mtshali@inl.co.za, nobuntu.mgijima@volt.africa, lee.rondganger@inl.co.za, londiwe.gumede@inl.co.za, philippa.larkin@inl.co.za</t>
         </is>
       </c>
     </row>
@@ -2178,11 +2202,7 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2207,14 +2227,14 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, info@thecortexhub.africa, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com</t>
+          <t>79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, info@thecortexhub.africa, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa</t>
+          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2224,7 +2244,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Oct 31, 2025 · The Robotics for Good Youth Challenge is the leading UN-based global robotics championship, inviting students aged 10 to 18 to develop AI and robotics-based solutions to tackle global challenges.</t>
+          <t>April 14, 2026 - This National Event, to be held at the Sandton Convention Centre in Johannesburg, South Africa, as part of AI for Good Impact Africa, at AI Expo Africa 2025, is a qualifying tournament leading to the Grand Finale in Geneva during the AI for ...</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2268,17 +2288,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Live Competitions — Nirvana Global Foundation</t>
+          <t>Roboticon 2026: South Africa Showcases Robotics for Culture ...</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://nirvanaglobalfoundation.org/competition.html</t>
+          <t>https://www.ubuntutimes.co.za/roboticon-2026-south-africa-showcases-robotics-for-culture-education-and-innovation/</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Enjoy AI South Africa An international AI and robotics competition for young innovators. Teams build, program and compete with official ENJOY AI robotics kits across categories like Battle of Stars, Mining Expedition, Drone Cup and Inventions Trail — preparing learners for the global ENJOY AI stage.</t>
+          <t>Jul 2, 2026 · South Africa’s robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation. Hosted at the Heartfelt Arena in Pretoria, the event is not only a showcase of technical skills but also a celebration of how robotics can address societal challenges.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2288,24 +2308,24 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>info@nirvanaglobalfoundation.org, coach@school.co.za</t>
+          <t>adverts@ubuntutimes.co.za, newspaper-rec300@2x.jpg</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ROBO-RUMBLE 2026 — Innovation in Motion</t>
+          <t>Live Competitions — Nirvana Global Foundation</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://roborumble.net/</t>
+          <t>https://nirvanaglobalfoundation.org/competition.html</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>South Africa's premier youth robotics &amp; technology competition. Robo Wars, Drone Racing, Grand Prix &amp; Innovation Challenge. August 2026.</t>
+          <t>Enjoy AI South Africa An international AI and robotics competition for young innovators. Teams build, program and compete with official ENJOY AI robotics kits across categories like Battle of Stars, Mining Expedition, Drone Cup and Inventions Trail — preparing learners for the global ENJOY AI stage.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2313,22 +2333,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>info@nirvanaglobalfoundation.org, coach@school.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Home | Roboticon 2026</t>
+          <t>FIRST South Africa – Robotics Programs for School Children</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://roboticon.resolute.education/</t>
+          <t>https://firstsa.org/</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Join us for the ultimate robotics showcase as Resolute proudly sponsors the World Robotics Olympiad (WRO) South Africa! This year, we're bringing together two worlds for the biggest robotics event of the year – Roboticon and the WRO Nationals, happening on the same day at the same venue.</t>
+          <t>From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way. FIRST Tech Challenge students learn to think like engineers. Teams ...</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2341,90 +2365,94 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
+          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://safcec.org.za/</t>
+          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
+          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>communication@safcec.org.za</t>
-        </is>
-      </c>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering</t>
+          <t>South African Robotics Competitions and Schools</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://civils.org.za/</t>
+          <t>https://www.sciencexpo.org.za/robotics.html</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
+          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr"/>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>webmaster@sciencexpo.org.za, madelien@imbewu.foundation, marna.vanzyl@imbewu.foundation</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ICE Africa – Supporting Civil Engineers in Africa</t>
+          <t>Limpopo Learners Represent South Africa at Global Robotics Finals in Switzerland - African Times</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
+          <t>https://www.atnews.co.za/limpopo-learners-represent-south-africa-at-global-robotics-finals-in-switzerland/</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Click your country to find local events, competitions, and information on how you can get more involved. At the heart of everything we do in South Africa is ICE-SA, the volunteer ICE local association (formerly known as the Joint Civils Division).</t>
+          <t>July 7, 2026 - The international competition, taking place from 7 to 10 July 2026 at the Palexpo International Exhibition and Convention Centre in Geneva, brings together some of the world’s brightest young innovators to develop technological solutions to ...</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr"/>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>NkosiN@atnews.co.za, rampedim@atnews.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Engineering the Future: 16 schools compete in SAICE’s 33rd ...</t>
+          <t>The South African Institution of Civil Engineering</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://southafricatoday.net/lifestyle/education/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
+          <t>https://civils.org.za/</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Aug 30, 2024 · The South African Institution of Civil Engineering (SAICE) hosted its 33 rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
+          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2437,17 +2465,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Home - SAICE</t>
+          <t>Zutari Bursary Programme 2027: Fully Funded Engineering Bursaries for ...</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://saice.org.za/</t>
+          <t>https://careersandopportunities.com/2026/08/07/bursary/</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Through our divisions, branches and committees, we aim to advance professional knowledge and improve the practice of civil engineering in South Africa. Our purpose is to provide members with opportunities for professional development through continued learning opportunities and industry networking.</t>
+          <t>Applications are now open for the Zutari Bursary Programme 2027. Ten fully funded engineering bursaries are available for South African students studying Civil or Electrical Engineering. Apply by 31 August 2026.</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2455,26 +2483,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>communications@saice.org.za, civilinfo@saice.org.za, membership@saice.org.za, barbara@avenue.co.za, executiveadmin@saice.org.za, marketing@saice.org.za, accounts@saice.org.za</t>
-        </is>
-      </c>
+      <c r="E83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
+          <t>Zutari Bursary Programme 2027 Opens Applications for Civil and ...</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
+          <t>https://www.globalsouthopportunities.com/2026/08/10/zutari/</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Jul 7, 2026 · Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in a shared commitment to developing South Africa’s future engineering talent.</t>
+          <t>Zutari has opened applications for its 2027 Engineering Bursary Programme, offering financial and professional development support to South African students pursuing studies in Civil Engineering and Electrical Engineering. The engineering consulting company plans to award 10 bursaries for the 2027 academic year. The programme is aimed at young engineering talent, including matriculants and ...</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2487,17 +2511,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Bridge Building Project Info - SAICE</t>
+          <t>List of ALL Engineering Bursaries South Africa 2027</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://saice.org.za/bridge-building-project-info/</t>
+          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>These learners come from across South Africa as well as Eswatini and Zimbabwe. This competition exposes the learners to a practical application of a process through which civil engineering impact their daily lives.</t>
+          <t>How much can I earn within the Engineering field in South Africa? The engineering sector in South Africa offers a wide range of career opportunities across fields such as civil, mechanical, electrical, chemical, mining, and industrial engineering. Salaries vary depending on qualifications, experience, and industry, with entry-level roles typically starting at moderate levels and increasing ...</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2505,31 +2529,27 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>communications@saice.org.za, civilinfo@saice.org.za, membership@saice.org.za, memory@saice.org.za, marketing@saice.org.za, accounts@saice.org.za</t>
-        </is>
-      </c>
+      <c r="E85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>JG Afrika Bursary Programme 2027: Fund Your Civil Engineering Studies</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://southafricaportal.com/jg-afrika-bursary-civil-engineering-2027/</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
+          <t>JG Afrika Bursary Programme 2027: Civil Engineering Study Opportunity JG Afrika is inviting qualifying South African students to apply for its 2027 Bursary Programme. This opportunity […]</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
@@ -2537,22 +2557,22 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>SAICE's 34th International Bridge Competition Inspires Tomorrow's ...</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://southafricatoday.net/lifestyle/education/saices-34th-international-bridge-competition-inspires-tomorrows-engineers/</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) hosted its 34th International Bridge Building Competition at the Midrand Conference Centre, bringing together 21 teams of high school learners from across South Africa, alongside international participants from Eswatini, Uganda, and Zimbabwe.</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
@@ -2560,76 +2580,72 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>ICE Africa - Supporting Civil Engineers in Africa</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
+          <t>ICE Africa supports civil engineers across the continent, providing access to qualifications, training, and networking opportunities for professional growth.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Home - SAICE</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://saice.org.za/</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) is the industry body for civil engineering professionals in South Africa. Our aim is to, promote growth, excellence and sustainability in the industry.</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>info@ieomsociety.org</t>
+          <t>executiveadmin@saice.org.za, marketing@saice.org.za, civilinfo@saice.org.za, communications@saice.org.za, barbara@avenue.co.za, accounts@saice.org.za, membership@saice.org.za</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>19 June 2026 marked an exciting celebration of Youth Month as aspiring young engineers from across Gauteng gathered for the 2026 SAICE Johannesburg Branch Schools Bridge Building Competition. Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in ...</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -2637,40 +2653,44 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>Awards 2025 - SAICE</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://saice.org.za/awards-2025/</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>Learn about SAICE's award categories, submission guidelines, key dates and how to nominate project and professionals.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr"/>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>marketing@saice.org.za, civilinfo@saice.org.za, communications@saice.org.za, accounts@saice.org.za, membership@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>SAIMechE</t>
+          <t>List of ALL Engineering Bursaries South Africa 2027</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://www.saimeche.org.za/</t>
+          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
+          <t>How much can I earn within the Engineering field in South Africa? The engineering sector in South Africa offers a wide range of career opportunities across fields such as civil, mechanical, electrical, chemical, mining, and industrial engineering. Salaries vary depending on qualifications, experience, and industry, with entry-level roles typically starting at moderate levels and increasing ...</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2693,12 +2713,12 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
@@ -2706,7 +2726,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2716,12 +2736,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E94" t="inlineStr"/>
@@ -2729,95 +2749,99 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Electrical Engineering Conferences in South Africa 2026/2027 ...</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://conferenceindex.org/conferences/electrical-engineering/south-africa</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Electrical Engineering Conferences in South Africa 2026 2027 2028 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and symposiums.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr"/>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Sep 4, 2025 · The Africa Prize for Engineering Innovation is open to individuals or teams based in sub-Saharan Africa who have a scalable engineering innovation with social or environmental impact potential.</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 · IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa) Deadline: April 30, 2026 May 15, 2026</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr"/>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+          <t>Latest Engineering Bursaries in South Africa for 2027</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://ibursaries.co.za/list/field/engineering</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions.</t>
+          <t>Find the latest engineering bursaries in South Africa for 2027. Browse funding opportunities for civil, mechanical, electrical, mining and other engineering qualifications.</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
@@ -2825,49 +2849,45 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers</t>
+          <t>PDF Apply Now! Worldskills South Africa National Competition 2025</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/</t>
+          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>All equipment from massive ships to tiny devices h ... Earn your CPD credits today! Read it here.</t>
+          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>reception@saiee.org.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
+          <t>SAIMechE</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://hackon.co.za/</t>
+          <t>https://www.saimeche.org.za/</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
+          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -2875,45 +2895,49 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Hackathons en South Africa</t>
+          <t>Home - Icmeesa</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>https://za.allhackathons.com/</t>
+          <t>http://icmeesa.org.za/</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Aug 22, 2025 · Join us for an electrifying hackathon where innovation meets security and finance! This event brings together developers, data scientists, cybersecurity experts, and FinTech enthusiasts to …</t>
+          <t>Certificated Mechanical or Electrical Engineers in mining and factory are the professional engineering practitioners recognised by law in South Africa to accept legal responsibility to improve health and safety in mines and works. These Engineers need to provide solutions reliant on basic scientific, mathematical and engineering knowledge, supported by analysis and synthesis, and underpinned ...</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr"/>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>icmeesa@icmeesa.org.za, info@icmeesa.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Build the Future with Entelect Hackathons</t>
+          <t>Electrical Engineering Conferences in South Africa 2026/2027/2028</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://challenge.entelect.co.za/</t>
+          <t>https://conferenceindex.org/conferences/electrical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Instead of focusing on building a once-off project, our hackathons centre around optimisation problems. Participants develop solutions that are tested, scored, and ranked based on performance, efficiency, and strategy.</t>
+          <t>Electrical Engineering Conferences in South Africa 2026 2027 2028 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and symposiums.</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
@@ -2921,22 +2945,22 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Hackathons - challenge.entelect.co.za</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://challenge.entelect.co.za/hackathons</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>7 hours ago · Compete against the best university teams across South Africa. Prize Pool: Various cool prizes &amp; bragging rights! A hands-on practice problem statement for Hack-ademy workshop attendees, joining in person or online.</t>
+          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E103" t="inlineStr"/>
@@ -2944,75 +2968,444 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Hackathons | Sebaka</t>
+          <t>South African Institute of Electrical Engineers</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://sebakasouthafrica.co.za/hackathons.html</t>
+          <t>https://www.saiee.org.za/</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Sebaka Mentorship &amp; Hackathons — Build an AI Agent for Software Quality Engineering.</t>
+          <t>Centres South African Institute of Electrical Engineers (SAIEE) About Us See Member Benefits</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E104" t="inlineStr"/>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>glueup-logo-white@2x.png, reception@saiee.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Young Engineers Movement (YEM) - ORT SA</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>The Young Engineers Movement (YEM) is an immersive engineering and technology hackathon designed to equip young South Africans with the skills, mindset and confidence needed to solve real-world challenges.</t>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>marketing@ortsa.org.za, info@ortsa.org.za</t>
-        </is>
-      </c>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>CompeteHub - Where Champions Are Made</t>
+          <t>The Africa Prize for Engineering Innovation</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://www.devpluxe.co.za/</t>
+          <t>https://africaprize.raeng.org.uk/</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Join thousands of developers, designers, and innovators competing in South Africa ' s most impactful tech hackathons. We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
+          <t>The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators developing scalable engineering solutions to local challenges.</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>ASTEMI Competitions - SAASTA</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Zutari Bursary Programme 2027: Fully Funded Engineering Bursaries for ...</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>https://careersandopportunities.com/2026/08/07/bursary/</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Applications are now open for the Zutari Bursary Programme 2027. Ten fully funded engineering bursaries are available for South African students studying Civil or Electrical Engineering. Apply by 31 August 2026.</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Zutari Bursary Programme 2027 Opens Applications for Civil and ...</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>https://www.globalsouthopportunities.com/2026/08/10/zutari/</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Zutari has opened applications for its 2027 Engineering Bursary Programme, offering financial and professional development support to South African students pursuing studies in Civil Engineering and Electrical Engineering. The engineering consulting company plans to award 10 bursaries for the 2027 academic year. The programme is aimed at young engineering talent, including matriculants and ...</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>The Home of South African Hackathons</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>https://hackon.co.za/</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
+      <c r="E112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Hackathons en South Africa</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>https://za.allhackathons.com/</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Build the Future with Entelect Hackathons</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>https://challenge.entelect.co.za/</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Build the Future with Entelect Hackathons Join South Africa's premier optimisation-first developer competition platform. Compete, iterate, and outperform the best.</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Unisa hosts first-ever Hackathon to ignite student learning experience</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-hosts-first-ever-Hackathon-to-ignite-student-learning-experience</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Unisa's Information and Communication Technology Portfolio, in collaboration with the College of Science, Engineering and Technology, held the first-ever Unisa Hackathon on 3 and 4 July 2025, marking a major step in the university's journey to embed digital innovation and entrepreneurship into the students learning experience.</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>The Home of South African Hackathons</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>https://hackon.co.za/partners/</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>South Africa Policy Hackathon Hello Ladies, Happy New Year. Some of you may be interested in this workshop. The workshop is flagged for South African nationals working at research and innovation offices, accelerators, innovation hubs and incubators, tech centers, and start-ups working on dual-use...</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>ICEP - Tshwane Varsity Hackathon</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>https://tvh.icep.co.za/</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Tshwane Varsity Hackathon South Africa's premier inter-university hackathon competition. Join hundreds of students for 53 hours of coding, innovation, and`` fun!</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>MagasengQM@tut.ac.za, info@tvh.co.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Young Engineers Showcase Innovation at STEM Hackathon</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>https://www.futuresa.co.za/education/young-engineers-movement-stem/</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Young Engineers Build Solutions for Real-World Challenges at STEM Hackathon Fifty-five high school learners and 11 teachers from underserved South African schools will showcase working engineering and technology prototypes at the Young Engineers Movement (YEM) Hackathon Exhibition Day on 26 June 2026.</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>info@futuresa.co.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Hackathons | Sebaka</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>https://sebakasouthafrica.co.za/hackathons.html</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Sebaka Mentorship &amp; Hackathons — Build an AI Agent for Software Quality Engineering.</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Geekulcha Annual Hackathon 2025 Preparation | Sonke Platform</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>https://sonke.gklink.co/gkhack25</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Geekulcha Annual Hackathon 2025 FINISH WHAT YOU STARTED Join us for this year's edition of the hackathon to harness intelligence for sustainable development. Hosted in South Africa, Kenya and Virtual.</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>connect@geekulcha.dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Young Engineers Movement (YEM) - ORT SA</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>marketing@ortsa.org.za, info@ortsa.org.za</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update competition data 2026-08-25
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,17 +469,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>VUT inspires future engineers through Bridge Building Competition – Vaal University of Technology</t>
+          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://vut.ac.za/vut-inspires-future-engineers-through-bridge-building-competition/</t>
+          <t>https://www.poidata.io/report/engineer/south-africa</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1 month ago - “VUT Ekhaya Alumni and SAICE STAR Vaal hosted the 2026 Bridge Building Competition, inspiring 16 Vaal schools through practical engineering, creativity and STEM education.”</t>
+          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -492,17 +492,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
+          <t>Two South Africans on the shortlist for the 2026 Africa Prize for Engineering Innovation</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.poidata.io/report/engineer/south-africa</t>
+          <t>https://www.engineeringnews.co.za/article/two-south-africans-on-the-shortlist-for-the-2026-africa-prize-for-engineering-innovation-2026-08-04</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
+          <t>3 weeks ago - Two South African innovators have been shortlisted for the UK Royal Academy of Engineering’s Africa Prize for Engineering Innovation 2026. This is the continent’s richest award aimed at promoting engineering innovation and entrepreneurship ...</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -510,22 +510,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>chanel@engineeringnews.co.za, newsdesk@engineeringnews.co.za, advertising@creamermedia.co.za, newsletters@creamermedia.co.za, subscriptions@creamermedia.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Two South Africans on the shortlist for the 2026 Africa Prize for Engineering Innovation</t>
+          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/two-south-africans-on-the-shortlist-for-the-2026-africa-prize-for-engineering-innovation-2026-08-04</t>
+          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3 weeks ago - Two South African innovators have been shortlisted for the UK Royal Academy of Engineering’s Africa Prize for Engineering Innovation 2026. This is the continent’s richest award aimed at promoting engineering innovation and entrepreneurship ...</t>
+          <t>2 weeks ago - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -533,26 +537,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>subscriptions@creamermedia.co.za, chanel@engineeringnews.co.za, newsletters@creamermedia.co.za, advertising@creamermedia.co.za, newsdesk@engineeringnews.co.za</t>
-        </is>
-      </c>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
+          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1 week ago - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
+          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -565,17 +565,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Engineering Conferences in South Africa 2025-2026</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -583,7 +583,11 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -611,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
+          <t>Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -629,11 +633,7 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -684,17 +684,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>South Africa International Industrial Expo | Innovation Bridge</t>
+          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
+          <t>https://10times.com/southafrica/tradeshows</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
+          <t>6 days ago · South Africa trade shows, find and compare 966 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 172 upcoming expos in 2026-2027 1. SIDSSA, 2. BI + AI Innovation &amp; Tech Fest, 3. Investment Showcase, 4. South African Cheese Festival And Exhibition</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -707,17 +707,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show ...</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://madeinafricaevent.co.za/</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
+          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -725,22 +725,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>enquiries@aiexpoafrica.com</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
+          <t>Africa Tech Festival</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://manufacturingindaba.co.za/exhibition/</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -748,22 +752,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>support@informaconnect.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, dataprivacy@informaconnect.com, support@knect365.com, dataprivacy@knect365.com, customerservices@knect365.com</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>KZN Industrial Technology Exhibition</t>
+          <t>IT &amp; Technology Events in South Africa, List of all South ...</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://www.kznindustrial.co.za/</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
+          <t>Aug 17, 2026 · Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -771,26 +779,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>john@email.com</t>
-        </is>
-      </c>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Two landmark exhibitions set to transform industrial technology and renewable energy in South Africa</t>
+          <t>ELENEX Africa Johannesburg 2026 - TradeFairDates</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/two-landmark-exhibitions-set-to-transform-industrial-technology-and-renewable-energy-in-south-africa-2025-10-24</t>
+          <t>https://www.tradefairdates.com/ELENEX-Africa-M6915/Johannesburg.html</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>October 24, 2025 - South Africa’s industrial and clean energy sectors celebrated a landmark moment today with the official launch of RE+ South Africa 2026 and the Cape Industrial Technology Exhibition (CITE) 2027.</t>
+          <t>Jul 9, 2026 · The fair is deeply rooted in the dynamics and industrial growth of Johannesburg and demonstrates South Africa's role as a leading center for technological innovation in Africa.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -798,26 +802,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>subscriptions@creamermedia.co.za, chanel@engineeringnews.co.za, newsletters@creamermedia.co.za, advertising@creamermedia.co.za, newsdesk@engineeringnews.co.za</t>
-        </is>
-      </c>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Exhibition | Innovation Festival Durban | South Africa</t>
+          <t>South Africa International Industrial Expo | Innovation Bridge</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://www.innovationfestival.durban/exhibition</t>
+          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities.</t>
+          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -825,26 +825,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, Erika@innovate.durban, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, sithabile@innovate.durban, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Discover Innovation Hub's Pavilion at Organic &amp; Natural Products Expo - Organic &amp; Natural Products Portal</t>
+          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://www.organicandnaturalportal.com/innovation-hub-organic-expo/</t>
+          <t>https://madeinafricaevent.co.za/</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>3 weeks ago - Gathering producers, retailers, buyers, and conscious consumers under one roof, the expo serves as Africa’s premier showcase for sustainability, health, and wellness innovation. A standout highlight of this year’s exhibition is The Innovation Hub Pavilion, hosting a curated line-up of forward-thinking South African small, medium, and micro-enterprises (SMMEs).</t>
+          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -857,17 +853,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>International Science, Innovation &amp; Technology Expo (INSITE)</t>
+          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://www.dsti.gov.za/index.php/resource-center/27-temp/dst-links/3-international-science-innovation-a-technology-expo</t>
+          <t>https://manufacturingindaba.co.za/exhibition/</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>The essence of INSITE INSITE is an international, biennial must-see Science and Technology event in South Africa, the only one of its kind in Africa that creates new frontiers for global challenges · INSITE aims to assemble the worlds leading innovators and scientists in one place, stimulating ...</t>
+          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -880,17 +876,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Trade Shows Worldwide - South Africa - 2026/2027</t>
+          <t>KZN Industrial Technology Exhibition</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://www.eventseye.com/fairs/c1_trade-shows_south-africa.html</t>
+          <t>https://www.kznindustrial.co.za/</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>South Africa Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in South Africa</t>
+          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -898,22 +894,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>john@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AAXO - The Association of African Exhibition Organisers</t>
+          <t>Two landmark exhibitions set to transform industrial technology and renewable energy in South Africa</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.aaxo.co.za/</t>
+          <t>https://www.engineeringnews.co.za/article/two-landmark-exhibitions-set-to-transform-industrial-technology-and-renewable-energy-in-south-africa-2025-10-24</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>February 20, 2026 - CAPE TOWN, South Africa – The inaugural Festival of Eventing (FOE) brought together 350 event professionals, 85 speakers, and 10 countries under one roof for a two-day showcase of innovation, inspiration, and industry connection.</t>
+          <t>October 24, 2025 - South Africa’s industrial and clean energy sectors celebrated a landmark moment today with the official launch of RE+ South Africa 2026 and the Cape Industrial Technology Exhibition (CITE) 2027.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -921,22 +921,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>chanel@engineeringnews.co.za, newsdesk@engineeringnews.co.za, advertising@creamermedia.co.za, newsletters@creamermedia.co.za, subscriptions@creamermedia.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
+          <t>In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community’s challenges and how community members view the impact of these challenges on their daily lives.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -944,22 +948,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>Engineering for People Design Challenge | Department of ...</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
+          <t>Aug 4, 2025 · This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but under-resourced neighbourhood on the eastern edge of Johannesburg. Home to around 46,000 people, Makers Valley is a community rich in creativity, activism ...</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -969,24 +977,24 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
+          <t>web-editor@eng.cam.ac.uk, marketing@eng.cam.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EWB Design Challenge | Aston University</t>
+          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
+          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
+          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -999,17 +1007,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
+          <t>Oct 16, 2024 · STEM-focused NGO Engineers Without Borders UK has launched its 2025 Engineering for People Design Challenge. Organised in conjunction with sister organisation Engineers Without Borders South Africa, as well as the Makers Valley Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1017,26 +1025,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>ied@ied.org.uk</t>
-        </is>
-      </c>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Latest Community Engineering Design Competition Announced</t>
+          <t>Engineering For People Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
+          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
+          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1044,22 +1048,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Real-world research: Engineering team designs South African trolley system; science students investigate heavy metals | University of Wisconsin - Stout</t>
+          <t>Engineering for People Design Challenge - Engineers Without ...</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
+          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>May 15, 2025 - Research ranged from heavy metals ... Borders’ international design challenge. Nearly 90 students in 23 teams addressed the EWB challenge. One group focused on engineering a safer, more accessible transportation system in South ...</t>
+          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1067,26 +1075,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>dolanm@uwstout.edu, frischj@uwstout.edu</t>
-        </is>
-      </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Engineering for people, that’s the challenge | Engineers Without Borders</t>
+          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.rs-online.com/designspark/an-introduction-to-engineering-for-people-design-challenge</t>
+          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>That’s exactly what the annual Engineering for People Design Challenge asks participants to do. The competition, delivered in partnership by Engineers without Borders South Africa and Engineers Without Borders UK, encourages engineering students and those collaborating with engineers to broaden their awareness of how their decisions change the world.</t>
+          <t>Oct 24, 2024 · The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1094,22 +1098,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>team@crowdsolve.net</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of Engineering</t>
+          <t>EWB Design Challenge | Aston University</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
+          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1117,26 +1125,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
-        </is>
-      </c>
+      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
+          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
+          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
+          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1144,22 +1148,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>ied@ied.org.uk</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Launching Engineering for People Design challenge 2024 ...</t>
+          <t>Engineers Without Borders South ...</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.electronicspecifier.com/studentzone/studentzone-news/launching-engineering-for-people-design-challenge-2024-25-2/</t>
+          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>November 16, 2025 - Engineers Without Borders has launched the 2024/25 cycle of the award-winning Engineering for People Design Challenge in partnership with Engineers Without Borders South Africa and Makers Valley Partnership.</t>
+          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1264,17 +1272,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Engineering in South Africa: 24 Best universities Ranked</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://edurank.org/engineering/za/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1287,17 +1295,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
+          <t>Engineering in South Africa: 24 Best universities Ranked</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2210</t>
+          <t>https://edurank.org/engineering/za/</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
+          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1333,17 +1341,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>University of South Africa</t>
+          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-promotes-globally-recognised-engineering-qualifications</t>
+          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Unisa promotes globally recognised engineering qualifications</t>
+          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1356,17 +1364,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1379,17 +1387,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>5 Best Universities to Study Engineering in South Africa</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
+          <t>https://globalscholarships.com/best-universities-engineering-south-africa/</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>May 9, 2026 - Its diplomas and BEngTech degrees can support routes to registration with the Engineering Council of South Africa as engineering technicians or engineering technologists after the required practical experience. ... Degree/s Offered: Bachelor’s, Master’s, Ph.D. South Africa’s oldest university, the University of Cape Town, is one of the best engineering schools in South Africa.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1398,6 +1406,1613 @@
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 ...</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>https://techspojoburg.co.za/</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>tech expo South Africa</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>info@techspojoburg.co.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Africa Tech Festival</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>https://africatechfestival.com/</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>tech expo South Africa</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>support@informaconnect.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, dataprivacy@informaconnect.com, support@knect365.com, dataprivacy@knect365.com, customerservices@knect365.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7 ...</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>https://techspocapetown.co.za/</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Where Business, Tech and Innovation Collide in Cape Town! TECHSPO Cape Town is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>tech expo South Africa</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>info@techspocapetown.co.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>IT &amp; Technology Events in South Africa | 10times</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>https://10times.com/southafrica/technology</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Aug 26, 2026 · Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>tech expo South Africa</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>https://10times.com/johannesburg-za/technology</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>tech expo South Africa</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Tech Expo Africa - Enabling Development</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>https://techexpo.africa/</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Tech Expo Africa is a social enterprise connecting African businesses with top tech and business leaders to drive innovation.</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>tech expo South Africa</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>info@techexpo.africa</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>TECHSPO Johannesburg Technology ExpoJohannesburg Technology ...</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>https://techspojoburg.co.za/johannesburg-technology-expo/</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>TECHSPO Johannesburg is a 2-day technology expo taking place September 28 – 29, 2026 at the luxurious NH Johannesburg Sandton Hotel, Toronto, Ontario. TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>tech expo South Africa</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>tech expo South Africa</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>atinfo@techspo.coor, u003einfo@techspo.co</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Home - Mediatech Africa | South Africa</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>https://www.mediatech.co.za/</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>tech expo South Africa</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>claire@mediatech.co.za, simon@mediatech.co.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>https://africatechnologyexpo.com/</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>tech expo South Africa</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>info@sparkafrica.co, partner@africatechnologyexpo.com, johndoe@email.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Maker Faire Africa - Wikipedia</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Maker_Faire_Africa</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Maker Faire Africa, Cairo, October 2011 Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds (Nubian Cheetah). Maker Faire Africa aims to engage with on ...</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>maker faire South Africa</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Maker Faire - Wikipedia</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Maker_Faire</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Maker Faire is a convention of do it yourself (DIY) enthusiasts established by Make magazine in 2006. Participants come from a wide variety of interests, such as robotics, 3D printing, computers, arts and crafts, and hacker culture.</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>maker faire South Africa</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>HOME | MAKERS FEST</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>https://www.makersfestival.co.za/</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>On 8 &amp; 9 November 2025 at The Ostrich in Cape Town, join 2,000+ visitors each day for maker demos, a curated market, and family activities. It’s Africa’s first hands-on festival for creativity and craftsmanship — and everything you make, you take home.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>maker faire South Africa</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, example@mysite.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, warren@makersfestival.co.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Upcoming Faires - Maker Faire</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>https://makerfaire.com/upcoming-faires/</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>maker faire South Africa</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>pr@make.co, fancybox_sprite@2x.png, fancybox_loading@2x.gif, chosen-sprite@2x.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Maker Faire Africa — Grokipedia</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>https://grokipedia.com/page/maker_faire_africa</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Maker Faire Africa Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>maker faire South Africa</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Maker Faire |</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>https://makerfaire.com/</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>maker faire South Africa</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>pr@make.co, fancybox_sprite@2x.png, fancybox_loading@2x.gif, chosen-sprite@2x.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Aug 21, 2015 · DIRECTIONS THE CAPE TOWN MAKER FAIRE The Lookout, V&amp;A Waterfront Granger Bay Boulevard, V &amp; A Waterfront, Cape Town, 8002, South Africa Get Directions Fri Aug 21, 13:00 - Sun Aug 23, 17:00 The Lookout, V&amp;A Waterfront View Map Payments are secure and encrypted</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>maker faire South Africa</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>https://makerfairecapetown.wordpress.com/about/</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>maker faire South Africa</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>http://capetown.makerfaire.com/</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>maker faire South Africa</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>pr@make.co, fancybox_sprite@2x.png, fancybox_loading@2x.gif, chosen-sprite@2x.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>maker faire South Africa</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ASTEMI Competitions – SAASTA</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>All these Olympiads and Competitions have a positive impact on education and on educational institutions in South Africa, but there is still a need to build stronger collaboration among teachers, schools, universities and educational authorities in order to meet the challenges of STEM education in South Africa today.</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>High School STEM Competition | Southafrica 2024 - IEOM Society</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas.</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Samsung opens Solve for Tomorrow 2026 STEM competition to all South African public schools</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>February 27, 2026 - Samsung Electronics South Africa has opened applications for the 2026 edition of Solve for Tomorrow (SFT), its annual science, technology, engineering, and mathematics (STEM) competition aimed at Grade 10 and 11 learners.</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>https://www.samsung.com/za/solvefortomorrow/</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>South African Space Design Competition | Inspire Space ...</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>https://www.zasdc.org/</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Join the South African Space Design Competition to inspire space innovation, develop STEM skills, and compete for a trip to NASA. Perfect for high school students passionate about space.</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>user@domain.com, info@zasdc.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>High School STEM Competition | Capetown 2026</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the ‘first author’. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>ASTEMI SA</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>https://www.astemi.co.za/</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>StemCo - StemCo 2026 International Competitions</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>https://stemco.org/</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>June 10, 2026 - BEST YOURSELF WITH STEMCO! Platform for the world’s brightest. ... Thanks to the participating 25 countries in 2019. Singapore, Albania, Australia, Azerbaijan, Canada, Germany, India, Indonesia, Japan, Jordan, Kazakhstan, Kyrgyzstan, Malawi, Mongolia, Nigeria, Myanmar, South Africa, Tajikistan, Turkey, Turkmenistan, Ukraine, The United States, Uzbekistan, Vietnam</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>stemcomongolia@gmail.com, awaisnaeem786@gmail.com, education@missmaneducation.com, example@mail.com, info@missmaneducation.com, name@example.com, t.azizakhon@gmail.com, havtt@fermat.edu.vn, info.iksc@kangaroo.org.pk, bestyourself@stemco.org, hkoffice@missmaneducation.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>ASTEMI Competitions 2022 – SAASTA</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>https://saasta.ac.za/astemi-competitions-2</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026 Season - Africa's Global STEM Celebration</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>https://www.stemfestival.org/competitions/</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>April 30, 2026 - ... The Elementary, Junior, and Senior Robotics categories at STEM Festival are dedicated to advancing the World Robot Olympiad (WRO) across the Niger Delta and South-South Nigeria, working with ArcLights Foundation.</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Robotics Competition | WRO South Africa | Gauteng</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>https://www.wrosa.co.za/</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>WRO South Africa ( World Robot Olympiad ) is a robotics competition which brings together young people from all over the world to develop their creativity and problem-solving skills.</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in the leading UN-based global robotics competition, focusing on the critical area of agriculture and food security.</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, info@thecortexhub.africa, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Robotics for Good Youth Challenge South Africa</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa/</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Apr 25, 2025 · The Robotics for Good Youth Challenge South Africa is a national event in a global robotics competition on disaster response, leading to the AI for Good Summit 2025.</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>name@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Robotics for Good Youth Challenge South Africa</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Oct 31, 2025 · The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge, organized by ITU and The Cortex Hub, in partnership with Google.</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>name@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Roboticon 2026: South Africa Showcases Robotics for Culture ...</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>https://www.ubuntutimes.co.za/roboticon-2026-south-africa-showcases-robotics-for-culture-education-and-innovation/</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Jul 2, 2026 · The event, partnered with the World Robotics Olympiad, positions South Africa as a leader in educational robotics and entrepreneurial innovation.” South Africa’s robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation.</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>newspaper-rec300@2x.jpg, adverts@ubuntutimes.co.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Live Competitions — Nirvana Global Foundation</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>https://nirvanaglobalfoundation.org/competition.html</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Enjoy AI South Africa An international AI and robotics competition for young innovators. Teams build, program and compete with official ENJOY AI robotics kits across categories like Battle of Stars, Mining Expedition, Drone Cup and Inventions Trail — preparing learners for the global ENJOY AI stage.</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>coach@school.co.za, info@nirvanaglobalfoundation.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Home | Roboticon 2026</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>https://roboticon.resolute.education/</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Join us for the ultimate robotics showcase as Resolute proudly sponsors the World Robotics Olympiad (WRO) South Africa! This year, we're bringing together two worlds for the biggest robotics event of the year – Roboticon and the WRO Nationals, happening on the same day at the same venue.</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>The South African Institution of Civil Engineering</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>https://civils.org.za/</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Zutari Bursary Programme 2027 Opens Applications for Civil ...</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>https://www.globalsouthopportunities.com/2026/08/10/zutari/</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Aug 10, 2026 · Zutari has opened applications for its 2027 Engineering Bursary Programme, offering financial and professional development support to South African students pursuing studies in Civil Engineering and Electrical Engineering.</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>List of ALL Engineering Bursaries South Africa 2027</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>How much can I earn within the Engineering field in South Africa? The engineering sector in South Africa offers a wide range of career opportunities across fields such as civil, mechanical, electrical, chemical, mining, and industrial engineering. Salaries vary depending on qualifications, experience, and industry, with entry-level roles typically starting at moderate levels and increasing ...</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>SAICE’s 34th International Bridge Competition Inspires ...</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>https://southafricatoday.net/lifestyle/education/saices-34th-international-bridge-competition-inspires-tomorrows-engineers/</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Sep 1, 2025 · The South African Institution of Civil Engineering (SAICE) hosted its 34th International Bridge Building Competition at the Midrand Conference Centre, bringing together 21 teams of high school learners from across South Africa, alongside international participants from Eswatini, Uganda, and Zimbabwe.</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>https://safcec.org.za/</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>communication@safcec.org.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Home - SAICE</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>https://saice.org.za/</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>The South African Institution of Civil Engineering (SAICE) is the industry body for civil engineering professionals in South Africa. Our aim is to, promote growth, excellence and sustainability in the industry.</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>executiveadmin@saice.org.za, civilinfo@saice.org.za, barbara@avenue.co.za, marketing@saice.org.za, accounts@saice.org.za, communications@saice.org.za, membership@saice.org.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Jul 7, 2026 · 19 June 2026 marked an exciting celebration of Youth Month as aspiring young engineers from across Gauteng gathered for the 2026 SAICE Johannesburg Branch Schools Bridge Building Competition. Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in ...</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>How to compete at the WSZA National Competitions 2025</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>ASTEMI Competitions – SAASTA</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>List of ALL Engineering Bursaries South Africa 2027Competitions | Capetown 2026SAIMechEPRDW Engineering Bursaries 2027: Fund Your Future in Civil ...ASTEMI SA - Competition Directory</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Aerospace Engineers develop and test aircraft and spacecrafts. They are also responsible for the design, maintenance and management of R&amp;D for various types of spacecrafts, aircrafts, missiles and satellites. This sector of engineering is divided into 2 branches which overlap: astronautical engineering and aeronautical engineering. These profession... See full list on zabursaries.co.za Bioresource Engineering is a discipline that incorporates design, engineering, as well as biological sciences to enhance and increase the sustainability of the planet’s natural resources. Bioresource Engineers look for solutions to problems involving animals, plants, and the environment. Bioresource Engineers are responsible for designing, operatin... See full list on zabursaries.co.za Chemical Engineers use chemical processes to find new ways to produce goods – from pharmaceuticals, cleaning solvents and fuels, to textiles and even food. These professionals are also involved in creating new ways to improve industrial processes by use of better chemical systems, as well as to limit inefficiency and waste within the industrial set... See full list on zabursaries.co.za Civil Engineers oversee the design, planning and construction of major infrastructures such as railways, highways, bridges, skyscraper buildings and water reservoirs. They assess material and labour costs, project deadlines and environmental impacts which will affect their projects. These professionals can find employment in various sectors, includ... See full list on zabursaries.co.za Construction engineers deal with the design, planning, management and construction of major infrastructures, including buildings, bridges, airports, tunnels, roads, railroads, dams, facilities and the like. Construction engineering is a sub-division of the Civil Engineering sector. Some of the job responsibilities of a Construction Engineer, involv... See full list on zabursaries.co.za Electronics engineering deals with the design of electronic circuits, microcontrollers, microprocessors and other devices by way of active and non-linear electrical components. These professionals are responsible for designing, testing and maintaining of electronic parts and systems used in the automation, navigation, communication and related fiel... See full list on zabursaries.co.za Environmental Engineers create solutions for environmental problems, by making us of engineering principles, as well as chemistry, biology and soil science. Their work involves addressing global issues such as climate change, water and air pollution, waste disposal, public health, recycling and environmental sustainability. Professionals in this se... See full list on zabursaries.co.za Engineering defines the branch of technology and science that deals with maintenance, design, building, as well as the use of machines, engines, and structures. A qualification in Engineering (General) is great for a student who is still unsure about what aspect of Engineering they would like to branch into, and most Universities offer a General En... See full list on zabursaries.co.za Industrial Engineers are responsible for determining ways to improve employee management; as well as the management of machinery; manufacturing processes and other assets, in order to improve the operations of their company. These professionals study reports based on process efficiency and create strategies which will improve said processes – this ... See full list on zabursaries.co.za Instrumentation engineers focus on automated systems, pneumatic domains and the operation and principles of measuring instruments used herein. People in this sector generally work for manufacturing or chemical plants, with the aim of improving the productivity, stability, optimisation and reliability of the system in question. If you are looking fo... See full list on zabursaries.co.za Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the IEOM Cape Town, South ... The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession. 2 days ago · Unlock your future with the PRDW Bursary Programme 2027! Applications are now open for South African citizens and permanent residents pursuing a career in Civil, Mechanical, or Mechatronics Engineering. Don’t miss this chance to receive financial support for your studies—apply before the deadline on 28 August 2026 at 16:00. About the ... We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Competitions | Capetown 2026</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>PRDW Engineering Bursaries 2027: Fund Your Future in Civil ...</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>https://www.jobssouthafrica.co.za/skills-development/prdw-engineering-bursaries-2027-fund-your-future-in-civil-mechanical-or-mechatronics/</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>2 days ago · Unlock your future with the PRDW Bursary Programme 2027! Applications are now open for South African citizens and permanent residents pursuing a career in Civil, Mechanical, or Mechatronics Engineering. Don’t miss this chance to receive financial support for your studies—apply before the deadline on 28 August 2026 at 16:00. About the ...</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>ASTEMI SA - Competition Directory</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>https://www.astemi.co.za/competition-directory</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>SAIMechE</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>https://www.saimeche.org.za/</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Electrical Engineering Conferences in South Africa 2026/2027 ...</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>https://conferenceindex.org/conferences/electrical-engineering/south-africa</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Electrical Engineering Conferences in South Africa 2026 2027 2028 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and symposiums.</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>South African Institute of Electrical Engineers</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>https://www.saiee.org.za/</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Centres South African Institute of Electrical Engineers (SAIEE) About Us See Member Benefits</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>glueup-logo-white@2x.png, reception@saiee.org.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Zutari Bursary Programme 2027: Fully Funded Engineering ...</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>https://careersandopportunities.com/2026/08/07/bursary/</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Aug 7, 2026 · Applications are now open for the Zutari Bursary Programme 2027. Ten fully funded engineering bursaries are available for South African students studying Civil or Electrical Engineering. Apply by 31 August 2026.</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Sep 4, 2025 · 3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>How to compete at the WSZA National Competitions 2025</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Zutari Bursary Programme 2027 Opens Applications for Civil ...</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>https://www.globalsouthopportunities.com/2026/08/10/zutari/</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Aug 10, 2026 · Zutari has opened applications for its 2027 Engineering Bursary Programme, offering financial and professional development support to South African students pursuing studies in Civil Engineering and Electrical Engineering.</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>https://hackon.co.za/</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Build the Future with Entelect Hackathons</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>https://challenge.entelect.co.za/</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Build the Future with Entelect Hackathons Join South Africa’s premier optimisation-first developer competition platform. Compete, iterate, and outperform the best.</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Hackathons en South Africa</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>https://za.allhackathons.com/</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Aug 22, 2025 · Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>MoMo Hackathon 2026 - South Africa, Wed, 2 Sep. 2026 at 00:00 ...</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>https://momodevelopercommunity.mtn.com/events/momo-hackathon-2026-south-africa-16</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>MoMo Dev Community - MoMo Hackathon 2026 - South Africa - Wed, 2 Sep. 2026, at In Person South Africa - Johannesburg</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>support@insided.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Hackathons - challenge.entelect.co.za</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>https://challenge.entelect.co.za/hackathons</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>4 days ago · University Cup Compete against the best university teams across South Africa Prize Pool: Various cool prizes &amp; bragging rights!</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Hackathons | Sebaka</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>https://sebakasouthafrica.co.za/hackathons.html</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Sebaka Mentorship &amp; Hackathons — Build an AI Agent for Software Quality Engineering.</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Young Engineers Movement (YEM) - ORT SA</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update competition data 2026-08-26
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E106"/>
+  <dimension ref="A1:E112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,17 +469,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
+          <t>VUT inspires future engineers through Bridge Building Competition – Vaal University of Technology</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.poidata.io/report/engineer/south-africa</t>
+          <t>https://vut.ac.za/vut-inspires-future-engineers-through-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
+          <t>1 month ago - “VUT Ekhaya Alumni and SAICE STAR Vaal hosted the 2026 Bridge Building Competition, inspiring 16 Vaal schools through practical engineering, creativity and STEM education.”</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -492,17 +492,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Two South Africans on the shortlist for the 2026 Africa Prize for Engineering Innovation</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/two-south-africans-on-the-shortlist-for-the-2026-africa-prize-for-engineering-innovation-2026-08-04</t>
+          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3 weeks ago - Two South African innovators have been shortlisted for the UK Royal Academy of Engineering’s Africa Prize for Engineering Innovation 2026. This is the continent’s richest award aimed at promoting engineering innovation and entrepreneurship ...</t>
+          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -510,11 +510,7 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>chanel@engineeringnews.co.za, newsdesk@engineeringnews.co.za, advertising@creamermedia.co.za, newsletters@creamermedia.co.za, subscriptions@creamermedia.co.za</t>
-        </is>
-      </c>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -542,17 +538,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
+          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
+          <t>https://www.poidata.io/report/engineer/south-africa</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
+          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -565,17 +561,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
+          <t>Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -583,26 +579,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
+          <t>Two South Africans on the shortlist for the 2026 Africa Prize for Engineering Innovation</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.thecasecentre.org/products/view?id=189255</t>
+          <t>https://www.engineeringnews.co.za/article/two-south-africans-on-the-shortlist-for-the-2026-africa-prize-for-engineering-innovation-2026-08-04</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
+          <t>3 weeks ago - Two South African innovators have been shortlisted for the UK Royal Academy of Engineering’s Africa Prize for Engineering Innovation 2026. This is the continent’s richest award aimed at promoting engineering innovation and entrepreneurship ...</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -610,22 +602,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>newsletters@creamermedia.co.za, chanel@engineeringnews.co.za, subscriptions@creamermedia.co.za, newsdesk@engineeringnews.co.za, advertising@creamermedia.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Engineering Conferences in South Africa 2025-2026</t>
+          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
+          <t>https://www.thecasecentre.org/products/view?id=189255</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
+          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -638,17 +634,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>South Africa · South Korea · Spain · Sri Lanka · Sudan · Sweden · Switzerland · Syrian Arab Republic · Taiwan · Tajikistan · Tanzania · Thailand · Togo · Trinidad and Tobago · Tunisia · Turkey · Uganda · Ukraine · United Arab Emirates · United Kingdom ·</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -656,22 +652,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>South Africa · South Korea · Spain · Sri Lanka · Sudan · Sweden · Switzerland · Syrian Arab Republic · Taiwan · Tajikistan · Tanzania · Thailand · Togo · Trinidad and Tobago · Tunisia · Turkey · Uganda · Ukraine · United Arab Emirates · United Kingdom ·</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>6 days ago · South Africa trade shows, find and compare 966 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 172 upcoming expos in 2026-2027 1. SIDSSA, 2. BI + AI Innovation &amp; Tech Fest, 3. Investment Showcase, 4. South African Cheese Festival And Exhibition</t>
+          <t>South Africa trade shows, find and compare 966 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 172 upcoming expos in 2026-2027 1. SIDSSA, 2. BI + AI Innovation &amp; Tech Fest, 3. Investment Showcase, 4.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -707,17 +707,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show ...</t>
+          <t>Africa Tech Festival</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -727,24 +727,24 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>enquiries@aiexpoafrica.com</t>
+          <t>dataprivacy@informaconnect.com, support@informaconnect.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, dataprivacy@knect365.com, customerservices@knect365.com, support@knect365.com</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Africa Tech Festival</t>
+          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
+          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -752,26 +752,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>support@informaconnect.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, dataprivacy@informaconnect.com, support@knect365.com, dataprivacy@knect365.com, customerservices@knect365.com</t>
-        </is>
-      </c>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa, List of all South ...</t>
+          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://innovationweek.co.za/</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Aug 17, 2026 · Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>SA Innovation Week 2026 is South Africa's official national innovation platform accelerating implementation, commercialisation and impact.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -779,22 +775,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>info@pixal8media.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ELENEX Africa Johannesburg 2026 - TradeFairDates</t>
+          <t>IT &amp; Technology Events in South Africa | 10times</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://www.tradefairdates.com/ELENEX-Africa-M6915/Johannesburg.html</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Jul 9, 2026 · The fair is deeply rooted in the dynamics and industrial growth of Johannesburg and demonstrates South Africa's role as a leading center for technological innovation in Africa.</t>
+          <t>Big Data and Business Analytics Innovation Conference Johannesburg, South Africa IT &amp; Technology 100 Members Wed, 28 - Thu, 29 Oct 2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -807,17 +807,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>South Africa International Industrial Expo | Innovation Bridge</t>
+          <t>Electra Mining Africa | South Africa's Leading Mining and Industrial ...</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
+          <t>https://www.electramining.co.za/</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
+          <t>South Africa's Leading Mining Exhibition 7 - 11 September 2026 | JHB Expo Centre Nasrec Discover the biggest mining, industrial, electrical and power event in Africa. Connect with solution-providers, explore the latest technology and meet decision-makers who shape the future of the industry.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -825,22 +825,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>john@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://madeinafricaevent.co.za/</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
+          <t>AI Expo Africa 2026 - Join the Largest AI Event &amp; Trade Community in Africa TODAY! Our business audience is a buyer / supplier focused community and comprised of Enterprise decision makers / CxOs, allied to AI Cloud platform providers, Tier 1 / 2 deployment &amp; service providers, AI start ups / innovators, investors, educators, government and AI ecosystem community builders.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -848,22 +852,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>enquiries@aiexpoafrica.com</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
+          <t>ELENEX Africa Johannesburg 2026 - TradeFairDates</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://manufacturingindaba.co.za/exhibition/</t>
+          <t>https://www.tradefairdates.com/ELENEX-Africa-M6915/Johannesburg.html</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
+          <t>The fair is deeply rooted in the dynamics and industrial growth of Johannesburg and demonstrates South Africa's role as a leading center for technological innovation in Africa.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -876,17 +884,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>KZN Industrial Technology Exhibition</t>
+          <t>TECHSPO Cape Town 2027 - Technology Expo · October 6</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://www.kznindustrial.co.za/</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
+          <t>Where Business, Tech and Innovation Collide in Cape Town! TECHSPO Cape Town is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -896,24 +904,24 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>john@email.com</t>
+          <t>info@techspocapetown.co.za</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Two landmark exhibitions set to transform industrial technology and renewable energy in South Africa</t>
+          <t>TECHSPO Joburg 2026 - Technology Expo · October 10</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/two-landmark-exhibitions-set-to-transform-industrial-technology-and-renewable-energy-in-south-africa-2025-10-24</t>
+          <t>https://techspojoburg.co.za/</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>October 24, 2025 - South Africa’s industrial and clean energy sectors celebrated a landmark moment today with the official launch of RE+ South Africa 2026 and the Cape Industrial Technology Exhibition (CITE) 2027.</t>
+          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -923,24 +931,24 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>chanel@engineeringnews.co.za, newsdesk@engineeringnews.co.za, advertising@creamermedia.co.za, newsletters@creamermedia.co.za, subscriptions@creamermedia.co.za</t>
+          <t>info@techspojoburg.co.za</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community’s challenges and how community members view the impact of these challenges on their daily lives.</t>
+          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -948,26 +956,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
-        </is>
-      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of ...</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Aug 4, 2025 · This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but under-resourced neighbourhood on the eastern edge of Johannesburg. Home to around 46,000 people, Makers Valley is a community rich in creativity, activism ...</t>
+          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -977,24 +981,24 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>web-editor@eng.cam.ac.uk, marketing@eng.cam.ac.uk</t>
+          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
+          <t>EWB Design Challenge | Aston University</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
+          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
+          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1007,17 +1011,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Latest Community Engineering Design Competition Announced</t>
+          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
+          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Oct 16, 2024 · STEM-focused NGO Engineers Without Borders UK has launched its 2025 Engineering for People Design Challenge. Organised in conjunction with sister organisation Engineers Without Borders South Africa, as well as the Makers Valley Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg.</t>
+          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1025,22 +1029,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ied@ied.org.uk</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Engineering For People Design Challenge - EWBSA</t>
+          <t>Engineers Without Borders South ...</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
+          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
+          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1048,26 +1056,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
-        </is>
-      </c>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge - Engineers Without ...</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
+          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1080,17 +1084,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
+          <t>Engineering for People Design Challenge | Department of Engineering</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Oct 24, 2024 · The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
+          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1100,24 +1104,24 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>team@crowdsolve.net</t>
+          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>EWB Design Challenge | Aston University</t>
+          <t>Engineering for people, that’s the challenge | Engineers Without Borders</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
+          <t>https://www.rs-online.com/designspark/an-introduction-to-engineering-for-people-design-challenge</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
+          <t>That’s exactly what the annual Engineering for People Design Challenge asks participants to do. The competition, delivered in partnership by Engineers without Borders South Africa and Engineers Without Borders UK, encourages engineering students and those collaborating with engineers to broaden their awareness of how their decisions change the world.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1130,17 +1134,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
+          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
+          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
+          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1148,26 +1152,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>ied@ied.org.uk</t>
-        </is>
-      </c>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South ...</t>
+          <t>The status and challenges of industrial engineering in South Africa</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
+          <t>https://www.scielo.org.za/scielo.php?script=sci_arttext&amp;pid=S2224-78902016000100002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
+          <t>This resulted in an identity crisis for industrial engineers, who were caught between the Industrial Revolution and the new challenges of the information system era [5]. In addition, within the South African context, where major socioeconomic changes have occurred since 1994, IEs have been exposed to a number of unique challenges that are non-existent or less dominant in other fields.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1175,7 +1175,11 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>corne@sun.ac.za, admin@saiie.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1226,17 +1230,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;area=2200&amp;ranking=Overall&amp;country=ZAF</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1249,17 +1253,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1272,17 +1276,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Engineering in South Africa: 24 Best universities Ranked</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://edurank.org/engineering/za/</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1295,17 +1299,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Engineering in South Africa: 24 Best universities Ranked</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://edurank.org/engineering/za/</t>
+          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1318,17 +1322,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2025</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2025</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1341,17 +1345,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
+          <t>University Overall Rankings - Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
+          <t>University Overall Rankings - Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1364,17 +1368,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
+          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1387,17 +1391,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>5 Best Universities to Study Engineering in South Africa</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://globalscholarships.com/best-universities-engineering-south-africa/</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>May 9, 2026 - Its diplomas and BEngTech degrees can support routes to registration with the Engineering Council of South Africa as engineering technicians or engineering technologists after the required practical experience. ... Degree/s Offered: Bachelor’s, Master’s, Ph.D. South Africa’s oldest university, the University of Cape Town, is one of the best engineering schools in South Africa.</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1410,7 +1414,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 ...</t>
+          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1420,7 +1424,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
+          <t>1 month ago - TECHSPO Johannesburg 2026 is a two day technology expo taking place September 28th to 29th, 2026 at the luxurious Hyatt Regency Johannesburg, Johannesburg, South Africa. TECHSPO Johannesburg brings together developers, brands, marketers, technology ...</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1437,17 +1441,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Africa Tech Festival</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
+          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1457,24 +1461,24 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>support@informaconnect.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, dataprivacy@informaconnect.com, support@knect365.com, dataprivacy@knect365.com, customerservices@knect365.com</t>
+          <t>info@techspocapetown.co.za</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7 ...</t>
+          <t>IT &amp; Technology Events in South Africa, List of all South Africa Technology Business Expo &amp; Events</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Where Business, Tech and Innovation Collide in Cape Town! TECHSPO Cape Town is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
+          <t>New York Small Business Expo (Spring)07 MayNew York , USA · AFROZUM Fair · 07-09 May · Johannesburg , South Africa · AFROZUM Fair07-09 MayJohannesburg , South Africa · Nigeria Industries &amp; Manufacturing Summit · 18-20 May · Abuja , Nigeria ...</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1482,26 +1486,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>info@techspocapetown.co.za</t>
-        </is>
-      </c>
+      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Aug 26, 2026 · Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1509,22 +1509,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>atinfo@techspo.coor, u003einfo@techspo.co</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
+          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://10times.com/johannesburg-za/technology</t>
+          <t>https://africatechnologyexpo.com/</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1532,22 +1536,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>info@sparkafrica.co, partner@africatechnologyexpo.com, johndoe@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Tech Expo Africa - Enabling Development</t>
+          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://techexpo.africa/</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Tech Expo Africa is a social enterprise connecting African businesses with top tech and business leaders to drive innovation.</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1557,24 +1565,24 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>info@techexpo.africa</t>
+          <t>dataprivacy@informaconnect.com, support@informaconnect.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, dataprivacy@knect365.com, customerservices@knect365.com, support@knect365.com</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology ExpoJohannesburg Technology ...</t>
+          <t>IT Indaba 2026 – Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://techspojoburg.co.za/johannesburg-technology-expo/</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg is a 2-day technology expo taking place September 28 – 29, 2026 at the luxurious NH Johannesburg Sandton Hotel, Toronto, Ontario. TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
+          <t>The inaugural 2025 IT Indaba promises to bring together 3,000+ IT professionals and tech influencers who are involved in the procurement of systems, tools, platforms and services, along with user experience developers who deal with the core processes and client interfaces of the business.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1587,17 +1595,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
+          <t>Home - Mediatech Africa | South Africa</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
+          <t>https://www.mediatech.co.za/</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
+          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1607,24 +1615,24 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>atinfo@techspo.coor, u003einfo@techspo.co</t>
+          <t>claire@mediatech.co.za, simon@mediatech.co.za</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Home - Mediatech Africa | South Africa</t>
+          <t>FinancialContent - TECHSPO Cape Town 2026 Unites Business, Tech and Marketing Leaders for High-Impact Expo</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://www.mediatech.co.za/</t>
+          <t>https://markets.financialcontent.com/stocks/article/abnewswire-2026-4-8-techspo-cape-town-2026-unites-business-tech-and-marketing-leaders-for-high-impact-expo</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
+          <t>April 8, 2026 - Cape Town, South Africa - TECHSPO Cape Town Technology Expo returns October 1-2, 2026, to the V&amp;A Waterfront Cape Town Avenue Conference Venue, uniting business leaders, technologists, marketers, and innovators for a high-impact, two-day showcase ...</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1632,26 +1640,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>claire@mediatech.co.za, simon@mediatech.co.za</t>
-        </is>
-      </c>
+      <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
+          <t>Discover Tech Conferences Events &amp; Activities in South Africa | Eventbrite</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://africatechnologyexpo.com/</t>
+          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
+          <t>Save this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South AfricaShare this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1659,11 +1663,7 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>info@sparkafrica.co, partner@africatechnologyexpo.com, johndoe@email.com</t>
-        </is>
-      </c>
+      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Maker Faire Africa, Cairo, October 2011 Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds (Nubian Cheetah). Maker Faire Africa aims to engage with on ...</t>
+          <t>March 7, 2025 - Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds ...</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1724,7 +1724,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>On 8 &amp; 9 November 2025 at The Ostrich in Cape Town, join 2,000+ visitors each day for maker demos, a curated market, and family activities. It’s Africa’s first hands-on festival for creativity and craftsmanship — and everything you make, you take home.</t>
+          <t>On 8 &amp; 9 November 2025 at The Ostrich in Cape Town, join 2,000+ visitors each day for maker demos, a curated market, and family activities. It’s Africa’s first hands-on festival for creativity and craftsmanship — and everything you make, you take home. Tickets are on sale now.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, example@mysite.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, warren@makersfestival.co.za</t>
+          <t>8c4075d5481d476e945486754f783364@sentry.io, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, warren@makersfestival.co.za, example@mysite.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1751,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
+          <t>Aug 28, 2026 · The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>pr@make.co, fancybox_sprite@2x.png, fancybox_loading@2x.gif, chosen-sprite@2x.png</t>
+          <t>chosen-sprite@2x.png, pr@make.co, fancybox_loading@2x.gif, fancybox_sprite@2x.png</t>
         </is>
       </c>
     </row>
@@ -1778,7 +1778,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Maker Faire Africa Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
+          <t>Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
+          <t>A city’s Maker community, turned up to full volume. Hundreds of exhibitors, interactive zones, live talks, and a stage that lifts up expert makers and thought leaders alongside a few legendary guests.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>pr@make.co, fancybox_sprite@2x.png, fancybox_loading@2x.gif, chosen-sprite@2x.png</t>
+          <t>chosen-sprite@2x.png, pr@make.co, fancybox_loading@2x.gif, fancybox_sprite@2x.png</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Aug 21, 2015 · DIRECTIONS THE CAPE TOWN MAKER FAIRE The Lookout, V&amp;A Waterfront Granger Bay Boulevard, V &amp; A Waterfront, Cape Town, 8002, South Africa Get Directions Fri Aug 21, 13:00 - Sun Aug 23, 17:00 The Lookout, V&amp;A Waterfront View Map Payments are secure and encrypted</t>
+          <t>Aug 21, 2015 · We’re delighted to present the first ever Cape Town Maker Faire, hosted by Open Design in partnership with Trimble.Maker Faire is primarily designed as a forward-looking event, showcasing makers who are exploring new forms and new technologies.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1864,17 +1864,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
+          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>http://capetown.makerfaire.com/</t>
+          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
+          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1882,26 +1882,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>pr@make.co, fancybox_sprite@2x.png, fancybox_loading@2x.gif, chosen-sprite@2x.png</t>
-        </is>
-      </c>
+      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
+          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
+          <t>http://capetown.makerfaire.com/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
+          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1909,12 +1905,16 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>chosen-sprite@2x.png, pr@make.co, fancybox_loading@2x.gif, fancybox_sprite@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1937,17 +1937,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Southafrica 2024 - IEOM Society</t>
+          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
+          <t>https://www.samsung.com/za/solvefortomorrow/</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas.</t>
+          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1955,26 +1955,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Samsung opens Solve for Tomorrow 2026 STEM competition to all South African public schools</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>February 27, 2026 - Samsung Electronics South Africa has opened applications for the 2026 edition of Solve for Tomorrow (SFT), its annual science, technology, engineering, and mathematics (STEM) competition aimed at Grade 10 and 11 learners.</t>
+          <t>The IEOM High School/Middle School STEM Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1982,22 +1978,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
+          <t>South African Space Design Competition | Inspire Space Innovation ...</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/za/solvefortomorrow/</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
+          <t>Join the South African Space Design Competition to inspire space innovation, develop STEM skills, and compete for a trip to NASA. Perfect for high school students passionate about space.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2005,22 +2005,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>info@zasdc.org, user@domain.com</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space ...</t>
+          <t>High School STEM Competition | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Join the South African Space Design Competition to inspire space innovation, develop STEM skills, and compete for a trip to NASA. Perfect for high school students passionate about space.</t>
+          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2030,24 +2034,24 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>user@domain.com, info@zasdc.org</t>
+          <t>info@ieomsociety.org</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Capetown 2026</t>
+          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
+          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the ‘first author’. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
+          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2055,16 +2059,12 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ASTEMI SA</t>
+          <t>Astemi Sa</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2087,17 +2087,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>StemCo - StemCo 2026 International Competitions</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://stemco.org/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>June 10, 2026 - BEST YOURSELF WITH STEMCO! Platform for the world’s brightest. ... Thanks to the participating 25 countries in 2019. Singapore, Albania, Australia, Azerbaijan, Canada, Germany, India, Indonesia, Japan, Jordan, Kazakhstan, Kyrgyzstan, Malawi, Mongolia, Nigeria, Myanmar, South Africa, Tajikistan, Turkey, Turkmenistan, Ukraine, The United States, Uzbekistan, Vietnam</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2105,26 +2105,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>stemcomongolia@gmail.com, awaisnaeem786@gmail.com, education@missmaneducation.com, example@mail.com, info@missmaneducation.com, name@example.com, t.azizakhon@gmail.com, havtt@fermat.edu.vn, info.iksc@kangaroo.org.pk, bestyourself@stemco.org, hkoffice@missmaneducation.com</t>
-        </is>
-      </c>
+      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions 2022 – SAASTA</t>
+          <t>Applications for 2026 Samsung Solve For Tomorrow Now Open!</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://saasta.ac.za/astemi-competitions-2</t>
+          <t>https://news.samsung.com/za/applications-for-2026-samsung-solve-for-tomorrow-now-open</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries open until 06 March 2026. This is a transformative ...</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2137,17 +2133,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026 Season - Africa's Global STEM Celebration</t>
+          <t>Register your school for Samsung Solve for Tomorrow 2026</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://www.stemfestival.org/competitions/</t>
+          <t>https://www.sowetan.co.za/careers/2026-03-03-register-your-school-for-samsung-solve-for-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>April 30, 2026 - ... The Elementary, Junior, and Senior Robotics categories at STEM Festival are dedicated to advancing the World Robot Olympiad (WRO) across the Niger Delta and South-South Nigeria, working with ArcLights Foundation.</t>
+          <t>Register your school for Samsung Solve for Tomorrow 2026 STEM competition aims to transform and empower South African learners with critical skills to solve real-world challenges March 03, 2026 at 7:44 am</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2155,7 +2151,11 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ssasft@samsung.com</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2180,24 +2180,24 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com</t>
+          <t>605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
+          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in the leading UN-based global robotics competition, focusing on the critical area of agriculture and food security.</t>
+          <t>April 14, 2026 - This National Event, to be held at the Sandton Convention Centre in Johannesburg, South Africa, as part of AI for Good Impact Africa, at AI Expo Africa 2025, is a qualifying tournament leading to the Grand Finale in Geneva during the AI for ...</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2207,24 +2207,24 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, info@thecortexhub.africa, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com</t>
+          <t>name@example.com</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa</t>
+          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa/</t>
+          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Apr 25, 2025 · The Robotics for Good Youth Challenge South Africa is a national event in a global robotics competition on disaster response, leading to the AI for Good Summit 2025.</t>
+          <t>This is a call for learners and teams from across South Africa who are passionate about robotics, innovation, and making a difference. Whether you’re experienced or just starting, this competition welcomes anyone eager to learn and innovate.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2234,7 +2234,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>name@example.com</t>
+          <t>8c4075d5481d476e945486754f783364@sentry.io, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, info@thecortexhub.africa, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -2246,12 +2246,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa/</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Oct 31, 2025 · The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge, organized by ITU and The Cortex Hub, in partnership with Google.</t>
+          <t>Apr 25, 2025 · Experience the excitement as South African teams showcase their skills in a UN-based global robotics competition, focusing on the critical area of disaster response. This National Event is a qualifying tournament leading to the Grand Finale in Geneva during the AI for Good Global Summit 2025.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2278,7 +2278,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Jul 2, 2026 · The event, partnered with the World Robotics Olympiad, positions South Africa as a leader in educational robotics and entrepreneurial innovation.” South Africa’s robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation.</t>
+          <t>Jul 2, 2026 · South Africa’s robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation. Hosted at the Heartfelt Arena in Pretoria, the event is not only a showcase of technical skills but also a celebration of how robotics can address societal challenges.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2288,24 +2288,24 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>newspaper-rec300@2x.jpg, adverts@ubuntutimes.co.za</t>
+          <t>adverts@ubuntutimes.co.za, newspaper-rec300@2x.jpg</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Live Competitions — Nirvana Global Foundation</t>
+          <t>FIRST South Africa – Robotics Programs for School Children</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://nirvanaglobalfoundation.org/competition.html</t>
+          <t>https://firstsa.org/</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Enjoy AI South Africa An international AI and robotics competition for young innovators. Teams build, program and compete with official ENJOY AI robotics kits across categories like Battle of Stars, Mining Expedition, Drone Cup and Inventions Trail — preparing learners for the global ENJOY AI stage.</t>
+          <t>From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way. FIRST Tech Challenge students learn to think like engineers. Teams ...</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2313,26 +2313,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>coach@school.co.za, info@nirvanaglobalfoundation.org</t>
-        </is>
-      </c>
+      <c r="E77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Home | Roboticon 2026</t>
+          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://roboticon.resolute.education/</t>
+          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Join us for the ultimate robotics showcase as Resolute proudly sponsors the World Robotics Olympiad (WRO) South Africa! This year, we're bringing together two worlds for the biggest robotics event of the year – Roboticon and the WRO Nationals, happening on the same day at the same venue.</t>
+          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2345,68 +2341,76 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering</t>
+          <t>South African Robotics Competitions and Schools</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://civils.org.za/</t>
+          <t>https://www.sciencexpo.org.za/robotics.html</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
+          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr"/>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>madelien@imbewu.foundation, webmaster@sciencexpo.org.za, marna.vanzyl@imbewu.foundation</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Zutari Bursary Programme 2027 Opens Applications for Civil ...</t>
+          <t>Limpopo Learners Represent South Africa at Global Robotics Finals in Switzerland - African Times</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://www.globalsouthopportunities.com/2026/08/10/zutari/</t>
+          <t>https://www.atnews.co.za/limpopo-learners-represent-south-africa-at-global-robotics-finals-in-switzerland/</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Aug 10, 2026 · Zutari has opened applications for its 2027 Engineering Bursary Programme, offering financial and professional development support to South African students pursuing studies in Civil Engineering and Electrical Engineering.</t>
+          <t>July 7, 2026 - The international competition, taking place from 7 to 10 July 2026 at the Palexpo International Exhibition and Convention Centre in Geneva, brings together some of the world’s brightest young innovators to develop technological solutions to ...</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr"/>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>NkosiN@atnews.co.za, rampedim@atnews.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>List of ALL Engineering Bursaries South Africa 2027</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - AfrikaBot</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
+          <t>https://www.saiee.org.za/displaycustomlink.aspx?name=AfrikaBot</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>How much can I earn within the Engineering field in South Africa? The engineering sector in South Africa offers a wide range of career opportunities across fields such as civil, mechanical, electrical, chemical, mining, and industrial engineering. Salaries vary depending on qualifications, experience, and industry, with entry-level roles typically starting at moderate levels and increasing ...</t>
+          <t>AfrikaBot is affordable because you can build a competitive robot for a lot less with the correct advice. AfrikaBOT is South Africa's first robotics competition for high school teenagers and university undergraduates who are smart enough to build their own robots from electronic parts rather ...</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
+          <t>robotics competition South Africa</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
@@ -2414,17 +2418,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>SAICE’s 34th International Bridge Competition Inspires ...</t>
+          <t>Upcoming Civil Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://southafricatoday.net/lifestyle/education/saices-34th-international-bridge-competition-inspires-tomorrows-engineers/</t>
+          <t>https://conferencealerts.co.in/south-africa/civil-engineering</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Sep 1, 2025 · The South African Institution of Civil Engineering (SAICE) hosted its 34th International Bridge Building Competition at the Midrand Conference Centre, bringing together 21 teams of high school learners from across South Africa, alongside international participants from Eswatini, Uganda, and Zimbabwe.</t>
+          <t>International Civil engineering conferences in South africa 2025-2026 with invitation letter. A great opportunity to meet and learn from experts in your field.</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2437,17 +2441,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
+          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://safcec.org.za/</t>
+          <t>https://www.engineeringnews.co.za/article/saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini-2022-09-13</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng. Twelve schools participated in the grand finale, which saw great, ...</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2457,24 +2461,24 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>communication@safcec.org.za</t>
+          <t>newsletters@creamermedia.co.za, chanel@engineeringnews.co.za, subscriptions@creamermedia.co.za, newsdesk@engineeringnews.co.za, advertising@creamermedia.co.za</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Home - SAICE</t>
+          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://saice.org.za/</t>
+          <t>https://www.crown.co.za/construction-world/marketplace/22289-saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) is the industry body for civil engineering professionals in South Africa. Our aim is to, promote growth, excellence and sustainability in the industry.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2484,24 +2488,24 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>executiveadmin@saice.org.za, civilinfo@saice.org.za, barbara@avenue.co.za, marketing@saice.org.za, accounts@saice.org.za, communications@saice.org.za, membership@saice.org.za</t>
+          <t>ernao@crown.co.za, constr@crown.co.za</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
+          <t>Engineering the Future: 16 schools compete in SAICE’s 33rd International Bridge Building Competition - SAICE</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
+          <t>https://saice.org.za/press-releases/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Jul 7, 2026 · 19 June 2026 marked an exciting celebration of Youth Month as aspiring young engineers from across Gauteng gathered for the 2026 SAICE Johannesburg Branch Schools Bridge Building Competition. Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in ...</t>
+          <t>April 17, 2025 - The South African Institution of Civil Engineering (SAICE) hosted its 33rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2509,27 +2513,31 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>accounts@saice.org.za, marketing@saice.org.za, communications@saice.org.za, membership@saice.org.za, civilinfo@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>Upcoming Civil Engineering Conferences in South Africa 2025</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://www.allconferencealert.com/south-africa/civil-engineering-conference.html</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+          <t>September 7, 2025 - Find the list of upcoming Civil Engineering conferences in South Africa 2025 with invitation an letter.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
@@ -2537,45 +2545,49 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>SWM Communications | SAICE recognises civil engineering research excellence through national student competition</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://swmcommunications.co.za/press-office/saice-recognises-civil-engineering-research-excellence-through-national-student-competition/</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>April 1, 2026 - The event – which was sponsored by Sika, WorldsView, BVI, RIBCCS, and AF Consulting – was hosted at SAICE House in Midrand, Gauteng, and accredited for 0.2 CPD points. Students were invited to present their civil engineering university research and investigation project, which is part of the national curriculum for final year civil engineering undergraduate students.</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr"/>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>nthabeleng@saice.org.za, info@swmcommunications.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>List of ALL Engineering Bursaries South Africa 2027Competitions | Capetown 2026SAIMechEPRDW Engineering Bursaries 2027: Fund Your Future in Civil ...ASTEMI SA - Competition Directory</t>
+          <t>ICE Africa – Supporting Civil Engineers in Africa | Institution of Civil Engineers (ICE)</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
+          <t>https://www.ice.org.uk/about-us/what-we-do/ice-near-you/international/ice-africa/</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Aerospace Engineers develop and test aircraft and spacecrafts. They are also responsible for the design, maintenance and management of R&amp;D for various types of spacecrafts, aircrafts, missiles and satellites. This sector of engineering is divided into 2 branches which overlap: astronautical engineering and aeronautical engineering. These profession... See full list on zabursaries.co.za Bioresource Engineering is a discipline that incorporates design, engineering, as well as biological sciences to enhance and increase the sustainability of the planet’s natural resources. Bioresource Engineers look for solutions to problems involving animals, plants, and the environment. Bioresource Engineers are responsible for designing, operatin... See full list on zabursaries.co.za Chemical Engineers use chemical processes to find new ways to produce goods – from pharmaceuticals, cleaning solvents and fuels, to textiles and even food. These professionals are also involved in creating new ways to improve industrial processes by use of better chemical systems, as well as to limit inefficiency and waste within the industrial set... See full list on zabursaries.co.za Civil Engineers oversee the design, planning and construction of major infrastructures such as railways, highways, bridges, skyscraper buildings and water reservoirs. They assess material and labour costs, project deadlines and environmental impacts which will affect their projects. These professionals can find employment in various sectors, includ... See full list on zabursaries.co.za Construction engineers deal with the design, planning, management and construction of major infrastructures, including buildings, bridges, airports, tunnels, roads, railroads, dams, facilities and the like. Construction engineering is a sub-division of the Civil Engineering sector. Some of the job responsibilities of a Construction Engineer, involv... See full list on zabursaries.co.za Electronics engineering deals with the design of electronic circuits, microcontrollers, microprocessors and other devices by way of active and non-linear electrical components. These professionals are responsible for designing, testing and maintaining of electronic parts and systems used in the automation, navigation, communication and related fiel... See full list on zabursaries.co.za Environmental Engineers create solutions for environmental problems, by making us of engineering principles, as well as chemistry, biology and soil science. Their work involves addressing global issues such as climate change, water and air pollution, waste disposal, public health, recycling and environmental sustainability. Professionals in this se... See full list on zabursaries.co.za Engineering defines the branch of technology and science that deals with maintenance, design, building, as well as the use of machines, engines, and structures. A qualification in Engineering (General) is great for a student who is still unsure about what aspect of Engineering they would like to branch into, and most Universities offer a General En... See full list on zabursaries.co.za Industrial Engineers are responsible for determining ways to improve employee management; as well as the management of machinery; manufacturing processes and other assets, in order to improve the operations of their company. These professionals study reports based on process efficiency and create strategies which will improve said processes – this ... See full list on zabursaries.co.za Instrumentation engineers focus on automated systems, pneumatic domains and the operation and principles of measuring instruments used herein. People in this sector generally work for manufacturing or chemical plants, with the aim of improving the productivity, stability, optimisation and reliability of the system in question. If you are looking fo... See full list on zabursaries.co.za Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the IEOM Cape Town, South ... The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession. 2 days ago · Unlock your future with the PRDW Bursary Programme 2027! Applications are now open for South African citizens and permanent residents pursuing a career in Civil, Mechanical, or Mechatronics Engineering. Don’t miss this chance to receive financial support for your studies—apply before the deadline on 28 August 2026 at 16:00. About the ... We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>March 19, 2026 - organise seminars, workshops, visits and inter-universities competitions regarding civil engineering projects · For more information or to get involved please contact [email protected]. We have a volunteer member in South Africa who helps arrange ICE activities and promote our work.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -2583,49 +2595,45 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>Civil Engineering Conferences in South Africa 2025/2026/2027 - Conference Index</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://conferenceindex.org/conferences/civil-engineering/south-africa</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+          <t>Apr 13 International Conference on Architectural, Civil and Environmental Engineering (ICACEE) - Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>PRDW Engineering Bursaries 2027: Fund Your Future in Civil ...</t>
+          <t>Upcoming Civil engineering Conferences in Cape town 2025</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://www.jobssouthafrica.co.za/skills-development/prdw-engineering-bursaries-2027-fund-your-future-in-civil-mechanical-or-mechatronics/</t>
+          <t>https://conferencealerts.co.in/cape-town/civil-engineering</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2 days ago · Unlock your future with the PRDW Bursary Programme 2027! Applications are now open for South African citizens and permanent residents pursuing a career in Civil, Mechanical, or Mechatronics Engineering. Don’t miss this chance to receive financial support for your studies—apply before the deadline on 28 August 2026 at 16:00. About the ...</t>
+          <t>Civil engineering conferences in Cape town 2025 provide an exclusive global platform to meet and engage with experts and aspirants in various fields.</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -2633,22 +2641,22 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2205</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
@@ -2656,17 +2664,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>SAIMechE</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://www.saimeche.org.za/</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
+          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2679,22 +2687,22 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Electrical Engineering Conferences in South Africa 2026/2027 ...</t>
+          <t>List of ALL Engineering Bursaries South Africa 2027PRDW Bursaries 2027: Support for Civil, Mechanical ...ASTEMI Competitions – SAASTACompetitions | Capetown 2026Mechanical Engineering Bursaries 2023- 2024</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://conferenceindex.org/conferences/electrical-engineering/south-africa</t>
+          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Electrical Engineering Conferences in South Africa 2026 2027 2028 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and symposiums.</t>
+          <t>Aerospace Engineers develop and test aircraft and spacecrafts. They are also responsible for the design, maintenance and management of R&amp;D for various types of spacecrafts, aircrafts, missiles and satellites. This sector of engineering is divided into 2 branches which overlap: astronautical engineering and aeronautical engineering. These profession... See full list on zabursaries.co.za Bioresource Engineering is a discipline that incorporates design, engineering, as well as biological sciences to enhance and increase the sustainability of the planet’s natural resources. Bioresource Engineers look for solutions to problems involving animals, plants, and the environment. Bioresource Engineers are responsible for designing, operatin... See full list on zabursaries.co.za Chemical Engineers use chemical processes to find new ways to produce goods – from pharmaceuticals, cleaning solvents and fuels, to textiles and even food. These professionals are also involved in creating new ways to improve industrial processes by use of better chemical systems, as well as to limit inefficiency and waste within the industrial set... See full list on zabursaries.co.za Civil Engineers oversee the design, planning and construction of major infrastructures such as railways, highways, bridges, skyscraper buildings and water reservoirs. They assess material and labour costs, project deadlines and environmental impacts which will affect their projects. These professionals can find employment in various sectors, includ... See full list on zabursaries.co.za Construction engineers deal with the design, planning, management and construction of major infrastructures, including buildings, bridges, airports, tunnels, roads, railroads, dams, facilities and the like. Construction engineering is a sub-division of the Civil Engineering sector. Some of the job responsibilities of a Construction Engineer, involv... See full list on zabursaries.co.za Electronics engineering deals with the design of electronic circuits, microcontrollers, microprocessors and other devices by way of active and non-linear electrical components. These professionals are responsible for designing, testing and maintaining of electronic parts and systems used in the automation, navigation, communication and related fiel... See full list on zabursaries.co.za Environmental Engineers create solutions for environmental problems, by making us of engineering principles, as well as chemistry, biology and soil science. Their work involves addressing global issues such as climate change, water and air pollution, waste disposal, public health, recycling and environmental sustainability. Professionals in this se... See full list on zabursaries.co.za Engineering defines the branch of technology and science that deals with maintenance, design, building, as well as the use of machines, engines, and structures. A qualification in Engineering (General) is great for a student who is still unsure about what aspect of Engineering they would like to branch into, and most Universities offer a General En... See full list on zabursaries.co.za Industrial Engineers are responsible for determining ways to improve employee management; as well as the management of machinery; manufacturing processes and other assets, in order to improve the operations of their company. These professionals study reports based on process efficiency and create strategies which will improve said processes – this ... See full list on zabursaries.co.za Instrumentation engineers focus on automated systems, pneumatic domains and the operation and principles of measuring instruments used herein. People in this sector generally work for manufacturing or chemical plants, with the aim of improving the productivity, stability, optimisation and reliability of the system in question. If you are looking fo... See full list on zabursaries.co.za 3 days ago · PRDW Bursaries 2027: Civil, Mechanical, and Mechatronics Engineering PRDW is inviting South African citizens and permanent residents to apply for its 2027 Bursary Programme. This opportunity […] ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa. Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation. Mechanical Engineering bursaries are offered by many companies in South Africa each year to deserving candidates. Have a look at some of the companies..</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
@@ -2702,49 +2710,45 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers</t>
+          <t>PRDW Bursaries 2027: Support for Civil, Mechanical ...</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/</t>
+          <t>https://southafricaportal.com/prdw-engineering-bursaries-2027/</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Centres South African Institute of Electrical Engineers (SAIEE) About Us See Member Benefits</t>
+          <t>3 days ago · PRDW Bursaries 2027: Civil, Mechanical, and Mechatronics Engineering PRDW is inviting South African citizens and permanent residents to apply for its 2027 Bursary Programme. This opportunity […]</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, reception@saiee.org.za</t>
-        </is>
-      </c>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Zutari Bursary Programme 2027: Fully Funded Engineering ...</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://careersandopportunities.com/2026/08/07/bursary/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Aug 7, 2026 · Applications are now open for the Zutari Bursary Programme 2027. Ten fully funded engineering bursaries are available for South African students studying Civil or Electrical Engineering. Apply by 31 August 2026.</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
@@ -2752,72 +2756,72 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
+          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr"/>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
+          <t>Mechanical Engineering Bursaries 2023- 2024</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://bursaries-southafrica.co.za/bursaries-mechanical-engineering/</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Sep 4, 2025 · 3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>Mechanical Engineering bursaries are offered by many companies in South Africa each year to deserving candidates. Have a look at some of the companies..</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>SAIMechE</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://www.saimeche.org.za/</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
@@ -2825,17 +2829,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Zutari Bursary Programme 2027 Opens Applications for Civil ...</t>
+          <t>IEEE South Africa</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://www.globalsouthopportunities.com/2026/08/10/zutari/</t>
+          <t>http://www.ieee.org.za/</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Aug 10, 2026 · Zutari has opened applications for its 2027 Engineering Bursary Programme, offering financial and professional development support to South African students pursuing studies in Civil Engineering and Electrical Engineering.</t>
+          <t>The South African Section has around 1200 members and many subsections. It was formed in 1963 by the merger of the Institute of Radio Engineers (IRE, founded 1912) and the American Institute of Electrical Engineers (AIEE, founded 1884).</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2848,22 +2852,22 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
+          <t>Electrical Engineering Conferences in South Africa 2026/2027 ...</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://hackon.co.za/</t>
+          <t>https://conferenceindex.org/conferences/electrical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
+          <t>Electrical Engineering Conferences in South Africa 2026 2027 2028 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and symposiums.</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -2871,22 +2875,22 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Build the Future with Entelect Hackathons</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>https://challenge.entelect.co.za/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Build the Future with Entelect Hackathons Join South Africa’s premier optimisation-first developer competition platform. Compete, iterate, and outperform the best.</t>
+          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions.</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E101" t="inlineStr"/>
@@ -2894,22 +2898,22 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Hackathons en South Africa</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://za.allhackathons.com/</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Aug 22, 2025 · Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
+          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
@@ -2917,72 +2921,72 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>MoMo Hackathon 2026 - South Africa, Wed, 2 Sep. 2026 at 00:00 ...</t>
+          <t>Zutari Bursary Programme 2027: Fully Funded Engineering ...</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://momodevelopercommunity.mtn.com/events/momo-hackathon-2026-south-africa-16</t>
+          <t>https://careersandopportunities.com/2026/08/07/bursary/</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>MoMo Dev Community - MoMo Hackathon 2026 - South Africa - Wed, 2 Sep. 2026, at In Person South Africa - Johannesburg</t>
+          <t>Aug 7, 2026 · Applications are now open for the Zutari Bursary Programme 2027. Ten fully funded engineering bursaries are available for South African students studying Civil or Electrical Engineering. Apply by 31 August 2026.</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>support@insided.com</t>
-        </is>
-      </c>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Hackathons - challenge.entelect.co.za</t>
+          <t>South African Institute of Electrical Engineers</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://challenge.entelect.co.za/hackathons</t>
+          <t>https://www.saiee.org.za/</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>4 days ago · University Cup Compete against the best university teams across South Africa Prize Pool: Various cool prizes &amp; bragging rights!</t>
+          <t>All equipment from massive ships to tiny devices h ... Earn your CPD credits today! Read it here.</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E104" t="inlineStr"/>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>glueup-logo-white@2x.png, reception@saiee.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Hackathons | Sebaka</t>
+          <t>Zutari Bursary Programme 2027 Opens Applications for Civil ...</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://sebakasouthafrica.co.za/hackathons.html</t>
+          <t>https://www.globalsouthopportunities.com/2026/08/10/zutari/</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Sebaka Mentorship &amp; Hackathons — Build an AI Agent for Software Quality Engineering.</t>
+          <t>Aug 10, 2026 · Zutari has opened applications for its 2027 Engineering Bursary Programme, offering financial and professional development support to South African students pursuing studies in Civil Engineering and Electrical Engineering.</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
@@ -2990,29 +2994,167 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
+          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>https://hackon.co.za/</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Hackathons en South Africa</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>https://za.allhackathons.com/</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Aug 22, 2025 · Join us for an electrifying hackathon where innovation meets security and finance! This event brings together developers, data scientists, cybersecurity experts, and FinTech enthusiasts to …</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Hackathons - challenge.entelect.co.za</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>https://challenge.entelect.co.za/hackathons</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>5 days ago · A hands-on practice problem statement for Hack-ademy workshop attendees, joining in person or online. Compete against the best university teams across South Africa. Prize Pool: Various cool prizes &amp; bragging rights!</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Build the Future with Entelect Hackathons</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>https://challenge.entelect.co.za/</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Instead of focusing on building a once-off project, our hackathons centre around optimisation problems. Participants develop solutions that are tested, scored, and ranked based on performance, efficiency, and strategy.</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Unisa hosts first-ever Hackathon to ignite student learning ...</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-hosts-first-ever-Hackathon-to-ignite-student-learning-experience</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Jul 14, 2025 · The event supported key priorities of South Africa’s National Development Plan, Unisa’s Catalytic Niche Areas and the United Nations’ Sustainable Development Goals that relate to access to quality education, decent work and innovation.</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
           <t>Young Engineers Movement (YEM) - ORT SA</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr">
+      <c r="B111" t="inlineStr">
         <is>
           <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>The Young Engineers Movement (YEM) is an immersive engineering and technology hackathon designed to equip young South Africans with the skills, mindset and confidence needed to solve real-world challenges.</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
         <is>
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr">
+      <c r="E111" t="inlineStr">
         <is>
           <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
         </is>
       </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>CompeteHub - Where Champions Are Made</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>https://www.devpluxe.co.za/</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Join thousands of developers, designers, and innovators competing in South Africa ' s most impactful tech hackathons. We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update competition data 2026-08-27
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E112"/>
+  <dimension ref="A1:E121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>3 weeks ago - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -464,22 +464,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>VUT inspires future engineers through Bridge Building Competition – Vaal University of Technology</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://vut.ac.za/vut-inspires-future-engineers-through-bridge-building-competition/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1 month ago - “VUT Ekhaya Alumni and SAICE STAR Vaal hosted the 2026 Bridge Building Competition, inspiring 16 Vaal schools through practical engineering, creativity and STEM education.”</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -487,22 +491,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -510,22 +518,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2 weeks ago - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -538,17 +550,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.poidata.io/report/engineer/south-africa</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -561,17 +573,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Engineering Conferences in South Africa 2025-2026</t>
+          <t>2027 Africa Prize for Engineering Innovation Opens Applications</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
+          <t>https://www.globalsouthopportunities.com/2026/08/09/africa-134/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
+          <t>The Royal Academy of Engineering has opened applications for the 2027 Africa Prize for Engineering Innovation, providing African innovators with an opportunity to develop, strengthen and commercialise engineering solutions addressing important challenges across the continent.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -584,17 +596,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Two South Africans on the shortlist for the 2026 Africa Prize for Engineering Innovation</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/two-south-africans-on-the-shortlist-for-the-2026-africa-prize-for-engineering-innovation-2026-08-04</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>3 weeks ago - Two South African innovators have been shortlisted for the UK Royal Academy of Engineering’s Africa Prize for Engineering Innovation 2026. This is the continent’s richest award aimed at promoting engineering innovation and entrepreneurship ...</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa. Find out more</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -602,26 +614,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>newsletters@creamermedia.co.za, chanel@engineeringnews.co.za, subscriptions@creamermedia.co.za, newsdesk@engineeringnews.co.za, advertising@creamermedia.co.za</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
+          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.thecasecentre.org/products/view?id=189255</t>
+          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
+          <t>Eligibility Benchmark Requirements The Africa Prize is open to individuals or teams based in sub-Saharan Africa with a scalable engineering innovation that demonstrates social or environmental impact potential. Applicants must: Be citizens ordinarily residing in a sub-Saharan African country. Be over 18 years old and fluent in English.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -634,17 +642,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
+          <t>List of ALL Engineering Bursaries South Africa 2027</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>How much can I earn within the Engineering field in South Africa? The engineering sector in South Africa offers a wide range of career opportunities across fields such as civil, mechanical, electrical, chemical, mining, and industrial engineering. Salaries vary depending on qualifications, experience, and industry, with entry-level roles typically starting at moderate levels and increasing ...</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -652,26 +660,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>NASA space win: SA learners triumph at Kennedy Space Center</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://furtherafrica.com/2026/08/11/nasa-space-win-sa-learners-triumph-at-kennedy-space-center/</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>South Africa · South Korea · Spain · Sri Lanka · Sudan · Sweden · Switzerland · Syrian Arab Republic · Taiwan · Tajikistan · Tanzania · Thailand · Togo · Trinidad and Tobago · Tunisia · Turkey · Uganda · Ukraine · United Arab Emirates · United Kingdom ·</t>
+          <t>NASA space win for South Africa as seven Western Cape learners win the International Space Settlement Design Competition at Kennedy Space Center.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -694,7 +698,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>South Africa trade shows, find and compare 966 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 172 upcoming expos in 2026-2027 1. SIDSSA, 2. BI + AI Innovation &amp; Tech Fest, 3. Investment Showcase, 4.</t>
+          <t>South Africa trade shows, find and compare 964 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 174 upcoming expos in 2026-2027 1. South Africa Infrastructure &amp; Water Expo, 2.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -707,17 +711,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Africa Tech Festival</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
+          <t>AI Expo Africa 2026 - Join the Largest AI Event &amp; Trade Community in Africa TODAY! Our business audience is a buyer / supplier focused community and comprised of Enterprise decision makers / CxOs, allied to AI Cloud platform providers, Tier 1 / 2 deployment &amp; service providers, AI start ups / innovators, investors, educators, government and AI ecosystem community builders.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -727,24 +731,24 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>dataprivacy@informaconnect.com, support@informaconnect.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, dataprivacy@knect365.com, customerservices@knect365.com, support@knect365.com</t>
+          <t>enquiries@aiexpoafrica.com</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
+          <t>DigiMarCon Africa 2027 - Cape Town, South Africa · October 6</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://digimarconafrica.com/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
+          <t>The Premier Digital Marketing, Media and Advertising Conference &amp; Exhibition held annually in Cape Town, South Africa! Join your peers for 2 days jam packed with digital marketing best practices, latest trends and strategy, also check out the next generation of technology &amp; innovation; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year ...</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -752,22 +756,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>info@digimarconafrica.com</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
+          <t>Exhibitions in South Africa 2026-2027 - ExpoTobi</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://innovationweek.co.za/</t>
+          <t>https://expotobi.com/country/south-africa/exhibitions</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SA Innovation Week 2026 is South Africa's official national innovation platform accelerating implementation, commercialisation and impact.</t>
+          <t>All Exhibitions in South Africa 2026-2027 | Full and accurate description of events for various business sectors | Schedule, tickets, travel arrangements and participation</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -775,26 +783,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>info@pixal8media.co.za</t>
-        </is>
-      </c>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>Africa Tech Festival</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Big Data and Business Analytics Innovation Conference Johannesburg, South Africa IT &amp; Technology 100 Members Wed, 28 - Thu, 29 Oct 2026</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -802,22 +806,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>support@knect365.com, customerservices@informaconnect.com, dataprivacy@informaconnect.com, customerservices@knect365.com, support@informaconnect.com, salesenquiries@africatechfestival.com, dataprivacy@knect365.com</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Electra Mining Africa | South Africa's Leading Mining and Industrial ...</t>
+          <t>IT &amp; Technology Events in South Africa | 10times</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://www.electramining.co.za/</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>South Africa's Leading Mining Exhibition 7 - 11 September 2026 | JHB Expo Centre Nasrec Discover the biggest mining, industrial, electrical and power event in Africa. Connect with solution-providers, explore the latest technology and meet decision-makers who shape the future of the industry.</t>
+          <t>Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -825,26 +833,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>john@email.com</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
+          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://innovationweek.co.za/</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AI Expo Africa 2026 - Join the Largest AI Event &amp; Trade Community in Africa TODAY! Our business audience is a buyer / supplier focused community and comprised of Enterprise decision makers / CxOs, allied to AI Cloud platform providers, Tier 1 / 2 deployment &amp; service providers, AI start ups / innovators, investors, educators, government and AI ecosystem community builders.</t>
+          <t>SA Innovation Week 2026 is South Africa's official national innovation platform accelerating implementation, commercialisation and impact.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -854,24 +858,24 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>enquiries@aiexpoafrica.com</t>
+          <t>info@pixal8media.co.za</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ELENEX Africa Johannesburg 2026 - TradeFairDates</t>
+          <t>Proudly South African Buy Local Summit &amp; Expo 2026 | Innovation Bridge</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://www.tradefairdates.com/ELENEX-Africa-M6915/Johannesburg.html</t>
+          <t>https://innovationbridge.info/ibportal/content/proudly-south-african-buy-local-summit-expo-2026</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>The fair is deeply rooted in the dynamics and industrial growth of Johannesburg and demonstrates South Africa's role as a leading center for technological innovation in Africa.</t>
+          <t>The 14th edition of the Proudly South African Buy Local Summit &amp; Expo will take place on 16-17 March 2026 at the Sandton Convention Centre, Johannesburg. As Proudly South African's flagship annual event, the Summit &amp; Expo has evolved into the country's premier local procurement and localisation platform, convening key public and private sector stakeholders to strengthen domestic value ...</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -981,7 +985,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
+          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
         </is>
       </c>
     </row>
@@ -1084,17 +1088,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of Engineering</t>
+          <t>Engineering for people, that’s the challenge | Engineers Without Borders</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://www.rs-online.com/designspark/an-introduction-to-engineering-for-people-design-challenge</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
+          <t>That’s exactly what the annual Engineering for People Design Challenge asks participants to do. The competition, delivered in partnership by Engineers without Borders South Africa and Engineers Without Borders UK, encourages engineering students and those collaborating with engineers to broaden their awareness of how their decisions change the world.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1102,26 +1106,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
-        </is>
-      </c>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Engineering for people, that’s the challenge | Engineers Without Borders</t>
+          <t>Engineering for People Design Challenge | Department of Engineering</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.rs-online.com/designspark/an-introduction-to-engineering-for-people-design-challenge</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>That’s exactly what the annual Engineering for People Design Challenge asks participants to do. The competition, delivered in partnership by Engineers without Borders South Africa and Engineers Without Borders UK, encourages engineering students and those collaborating with engineers to broaden their awareness of how their decisions change the world.</t>
+          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1129,7 +1129,11 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1157,17 +1161,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>The status and challenges of industrial engineering in South Africa</t>
+          <t>Launching Engineering for People Design challenge 2024 ...</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.scielo.org.za/scielo.php?script=sci_arttext&amp;pid=S2224-78902016000100002</t>
+          <t>https://www.electronicspecifier.com/studentzone/studentzone-news/launching-engineering-for-people-design-challenge-2024-25-2/</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>This resulted in an identity crisis for industrial engineers, who were caught between the Industrial Revolution and the new challenges of the information system era [5]. In addition, within the South African context, where major socioeconomic changes have occurred since 1994, IEs have been exposed to a number of unique challenges that are non-existent or less dominant in other fields.</t>
+          <t>November 16, 2025 - Engineers Without Borders has launched the 2024/25 cycle of the award-winning Engineering for People Design Challenge in partnership with Engineers Without Borders South Africa and Makers Valley Partnership.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1175,11 +1179,7 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>corne@sun.ac.za, admin@saiie.co.za</t>
-        </is>
-      </c>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1276,17 +1276,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Engineering in South Africa: 24 Best universities Ranked</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://edurank.org/engineering/za/</t>
+          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1299,17 +1299,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Engineering in South Africa: 24 Best universities Ranked</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://edurank.org/engineering/za/</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1322,17 +1322,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2210</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1368,17 +1368,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
+          <t>University of South Africa</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
+          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-promotes-globally-recognised-engineering-qualifications</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
+          <t>Unisa promotes globally recognised engineering qualifications</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1391,17 +1391,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
+          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1414,17 +1414,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>Africa Tech Festival</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>https://techspojoburg.co.za/</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>1 month ago - TECHSPO Johannesburg 2026 is a two day technology expo taking place September 28th to 29th, 2026 at the luxurious Hyatt Regency Johannesburg, Johannesburg, South Africa. TECHSPO Johannesburg brings together developers, brands, marketers, technology ...</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation … 17-19 November 2026 Cape Town ...</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1434,24 +1434,24 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>info@techspojoburg.co.za</t>
+          <t>support@knect365.com, customerservices@informaconnect.com, dataprivacy@informaconnect.com, customerservices@knect365.com, support@informaconnect.com, salesenquiries@africatechfestival.com, dataprivacy@knect365.com</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>TECHSPO Technology Expo</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://techspo.co/</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
+          <t>TECHSPO is a Technology Expo Series with annual events in 50 international cities, across 20 countries. South Africa October 1 – 2, 2026 Cape Town, South ...</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1459,26 +1459,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>info@techspocapetown.co.za</t>
-        </is>
-      </c>
+      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa, List of all South Africa Technology Business Expo &amp; Events</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~…</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://www.industryevents.com/events/techspo-johannesburg-2026-technology-expo-internet-mobile-adtech-martech-saas</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>New York Small Business Expo (Spring)07 MayNew York , USA · AFROZUM Fair · 07-09 May · Johannesburg , South Africa · AFROZUM Fair07-09 MayJohannesburg , South Africa · Nigeria Industries &amp; Manufacturing Summit · 18-20 May · Abuja , Nigeria ...</t>
+          <t>TECHSPO Johannesburg Technology Expo returns September 28-29, 2026 to the NH Johannesburg Sandton Hotel in Johannesburg, South Africa.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1486,22 +1482,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>events@techspojoburg.co.za, support@industryevents.com, your@email.com, you@company.com, colleague@company.com</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
+          <t>Tech conferences in South Africa 2026 / 2027 - dev.events</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
+          <t>https://dev.events/AF/ZA/tech</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
+          <t>Best Tech conferences in South Africa 2026 / 2027 · The Principal Dev – Masterclass for Tech Leads · Clean Architecture Masterclass · OT SECURITY FIRST ...</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1509,26 +1509,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>atinfo@techspo.coor, u003einfo@techspo.co</t>
-        </is>
-      </c>
+      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
+          <t>IT &amp; Technology Events in South Africa - 10Times</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://africatechnologyexpo.com/</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
+          <t>The TECHSPO Technology Expo is set to take place in the bustling business hub of Sandton, Johannesburg, from September 28 to September 29, 2026.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1536,26 +1532,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>info@sparkafrica.co, partner@africatechnologyexpo.com, johndoe@email.com</t>
-        </is>
-      </c>
+      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
+          <t>Mediatech Africa (@mediatechafrica) · Johannesburg - Instagram</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://www.instagram.com/mediatechafrica/</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
+          <t>Africa's largest Pro AV, Film, Broadcast &amp; Live Event Tech Expo. 27 - 29 June 2028, Johannesburg .</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1563,26 +1555,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>dataprivacy@informaconnect.com, support@informaconnect.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, dataprivacy@knect365.com, customerservices@knect365.com, support@knect365.com</t>
-        </is>
-      </c>
+      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 – Africa's biggest IT Conference and Expo</t>
+          <t>Africa Technology Expo</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://africatechnologyexpo.com/</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>The inaugural 2025 IT Indaba promises to bring together 3,000+ IT professionals and tech influencers who are involved in the procurement of systems, tools, platforms and services, along with user experience developers who deal with the core processes and client interfaces of the business.</t>
+          <t>The Africa Technology Expo (ATE) is a first-of-its-kind, multi-year enterprise gathering at the intersection of Africa's potential and global opportunity.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1590,22 +1578,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>partner@africatechnologyexpo.com, johndoe@email.com, info@sparkafrica.co</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Home - Mediatech Africa | South Africa</t>
+          <t>Graintech Africa 2026 | Grain &amp; Allied Tech Expo Johannesburg</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://www.mediatech.co.za/</t>
+          <t>https://sa.graintechafrica.com/</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
+          <t>Join Graintech Africa 2026, 11–13 March in Johannesburg. Explore innovations in grain processing, milling, storage, packaging &amp; allied technologies.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1615,24 +1607,24 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>claire@mediatech.co.za, simon@mediatech.co.za</t>
+          <t>gtaexpo@graintechafrica.com</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>FinancialContent - TECHSPO Cape Town 2026 Unites Business, Tech and Marketing Leaders for High-Impact Expo</t>
+          <t>TECHSPO Events</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://markets.financialcontent.com/stocks/article/abnewswire-2026-4-8-techspo-cape-town-2026-unites-business-tech-and-marketing-leaders-for-high-impact-expo</t>
+          <t>https://techspo.co/events/</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>April 8, 2026 - Cape Town, South Africa - TECHSPO Cape Town Technology Expo returns October 1-2, 2026, to the V&amp;A Waterfront Cape Town Avenue Conference Venue, uniting business leaders, technologists, marketers, and innovators for a high-impact, two-day showcase ...</t>
+          <t>Johannesburg, South Africa. October 1 – 2, 2026. Cape Town, South Africa. October 8 – 9, 2026. Philadelphia, PA. October 14 – 15, 2026. Miami, FL. October 22 – ...</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1645,17 +1637,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Discover Tech Conferences Events &amp; Activities in South Africa | Eventbrite</t>
+          <t>zambia &amp; southern africa - Africa FarmTech Expos</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
+          <t>https://www.africafarmtechexpo.com/south/</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Save this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South AfricaShare this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South Africa</t>
+          <t>The Africa FarmTech Expos welcome international, regional and local companies that are involved in manufacture and supply of technologies, products and services ...</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1663,7 +1655,11 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>info@fwafrica.net</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1691,17 +1687,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Maker Faire - Wikipedia</t>
+          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Maker_Faire</t>
+          <t>https://makerfairecapetown.wordpress.com/about/</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Maker Faire is a convention of do it yourself (DIY) enthusiasts established by Make magazine in 2006. Participants come from a wide variety of interests, such as robotics, 3D printing, computers, arts and crafts, and hacker culture.</t>
+          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1714,17 +1710,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>HOME | MAKERS FEST</t>
+          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://www.makersfestival.co.za/</t>
+          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>On 8 &amp; 9 November 2025 at The Ostrich in Cape Town, join 2,000+ visitors each day for maker demos, a curated market, and family activities. It’s Africa’s first hands-on festival for creativity and craftsmanship — and everything you make, you take home. Tickets are on sale now.</t>
+          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1732,26 +1728,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>8c4075d5481d476e945486754f783364@sentry.io, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, warren@makersfestival.co.za, example@mysite.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Upcoming Faires - Maker Faire</t>
+          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://makerfaire.com/upcoming-faires/</t>
+          <t>http://capetown.makerfaire.com/</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Aug 28, 2026 · The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
+          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1761,24 +1753,24 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>chosen-sprite@2x.png, pr@make.co, fancybox_loading@2x.gif, fancybox_sprite@2x.png</t>
+          <t>chosen-sprite@2x.png, fancybox_sprite@2x.png, fancybox_loading@2x.gif, pr@make.co</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Maker Faire Africa — Grokipedia</t>
+          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://grokipedia.com/page/maker_faire_africa</t>
+          <t>https://contemporaryand.com/fr/events/maker-faire-africa-comes-to-johannesburg</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
+          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1791,17 +1783,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Maker Faire |</t>
+          <t>The Makers Hub</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://makerfaire.com/</t>
+          <t>https://www.decorex.co.za/cape-town/en-gb/visit/TheMakersHub.html</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>A city’s Maker community, turned up to full volume. Hundreds of exhibitors, interactive zones, live talks, and a stage that lifts up expert makers and thought leaders alongside a few legendary guests.</t>
+          <t>Explore unique handmade items, take part in interactive workshops, and engage directly with Cape Town’s vibrant maker community.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1811,24 +1803,24 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>chosen-sprite@2x.png, pr@make.co, fancybox_loading@2x.gif, fancybox_sprite@2x.png</t>
+          <t>decorexafrica@rxglobal.com</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
+          <t>Maker Faire Africa comes to Jo’Burg – AfriGadget</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
+          <t>https://www.afrigadget.com/2014/07/08/maker-faire-africa-comes-to-joburg/</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Aug 21, 2015 · We’re delighted to present the first ever Cape Town Maker Faire, hosted by Open Design in partnership with Trimble.Maker Faire is primarily designed as a forward-looking event, showcasing makers who are exploring new forms and new technologies.</t>
+          <t>Maker Faire Africa 2014 will bring together over 5,000 attendees, along with featured inventors, world-class makers, self-made entrepreneurs &amp; workshop experts from South Africa, across the continent, and around the world, to manufacture real solutions for some of Africa’s most pressing ...</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1841,17 +1833,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
+          <t>HOME | MAKERS FEST</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://makerfairecapetown.wordpress.com/about/</t>
+          <t>https://www.makersfestival.co.za/</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
+          <t>At Makers Festival SA, you get full access to every hands-on workshop, from woodworking and ceramics to leatherwork, painting, and more.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1859,22 +1851,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, example@mysite.com, 8c4075d5481d476e945486754f783364@sentry.io, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, warren@makersfestival.co.za, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
+          <t>Makers Festival SA 🛠️ (@makersfestival_sa) • Instagram photos ...</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
+          <t>https://www.instagram.com/makersfestival_sa/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
+          <t>8,503 Followers, 58 Following, 57 Posts - Makers Festival SA 🛠️ (@makersfestival_sa) on Instagram: "🛠️ Building Skills. Building Memories. 🏕️ 8th &amp; 9th November 2025 / Cape Town, SA 🪵 Founder @hutch_custom 📩 DM us - apply to be a MAKER 🫶🏼"</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1887,17 +1883,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
+          <t>Why Africa needs Maker Faire | ZDNET</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>http://capetown.makerfaire.com/</t>
+          <t>https://www.zdnet.com/article/why-africa-needs-maker-faire/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
+          <t>July 24, 2014 - Unlike other Maker Faires, Okafor said that it's not enough to simply hold the event in an African city and see who turns up. Two volunteers are currently working in South Africa to discover inventors in rural areas and neighbouring countries such as Zambia and Botswana who they can encourage to attend and show off their work.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1907,14 +1903,14 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>chosen-sprite@2x.png, pr@make.co, fancybox_loading@2x.gif, fancybox_sprite@2x.png</t>
+          <t>brand_licensing@ziffdavis.com</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1924,7 +1920,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>All these Olympiads and Competitions have a positive impact on education and on educational institutions in South Africa, but there is still a need to build stronger collaboration among teachers, schools, universities and educational authorities in order to meet the challenges of STEM education in South Africa today.</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1937,17 +1933,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
+          <t>Samsung opens Solve for Tomorrow 2026 STEM competition to all South African public schools</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/za/solvefortomorrow/</t>
+          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
+          <t>February 27, 2026 - Samsung Electronics South Africa has opened applications for the 2026 edition of Solve for Tomorrow (SFT), its annual science, technology, engineering, and mathematics (STEM) competition aimed at Grade 10 and 11 learners.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1960,17 +1956,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.samsung.com/za/solvefortomorrow/</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>The IEOM High School/Middle School STEM Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects.</t>
+          <t>Rooted in the belief that today’s youth hold the key to tomorrow’s progress, Solve for Tomorrow South Africa provides participants with the tools, mentorship, and platforms they need to turn ideas into action.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1978,26 +1974,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation ...</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Join the South African Space Design Competition to inspire space innovation, develop STEM skills, and compete for a trip to NASA. Perfect for high school students passionate about space.</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2005,26 +1997,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>info@zasdc.org, user@domain.com</t>
-        </is>
-      </c>
+      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Southafrica 2024 - IEOM Society</t>
+          <t>High School STEM Competition | Capetown 2026</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
+          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas.</t>
+          <t>High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas. Each submission can provide a summary of the STEM project. All projects must be presented at the IEOM Cape Town, South Africa 2026.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2041,17 +2029,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
+          <t>South African Space Design Competition | Inspire Space ...</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
+          <t>Join the South African Space Design Competition to inspire space innovation, develop STEM skills, and compete for a trip to NASA. Perfect for high school students passionate about space.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2059,12 +2047,16 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>info@zasdc.org, user@domain.com</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Astemi Sa</t>
+          <t>ASTEMI SA</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2087,17 +2079,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>StemCo - StemCo 2026 International Competitions</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://stemco.org/</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>June 10, 2026 - BEST YOURSELF WITH STEMCO! Platform for the world’s brightest. ... Thanks to the participating 25 countries in 2019. Singapore, Albania, Australia, Azerbaijan, Canada, Germany, India, Indonesia, Japan, Jordan, Kazakhstan, Kyrgyzstan, Malawi, Mongolia, Nigeria, Myanmar, South Africa, Tajikistan, Turkey, Turkmenistan, Ukraine, The United States, Uzbekistan, Vietnam</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2105,22 +2097,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>name@example.com, bestyourself@stemco.org, havtt@fermat.edu.vn, hkoffice@missmaneducation.com, info@missmaneducation.com, stemcomongolia@gmail.com, awaisnaeem786@gmail.com, example@mail.com, education@missmaneducation.com, info.iksc@kangaroo.org.pk, t.azizakhon@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Applications for 2026 Samsung Solve For Tomorrow Now Open!</t>
+          <t>High School STEM Competition | Southafrica 2024</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://news.samsung.com/za/applications-for-2026-samsung-solve-for-tomorrow-now-open</t>
+          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries open until 06 March 2026. This is a transformative ...</t>
+          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, ...</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2128,22 +2124,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Register your school for Samsung Solve for Tomorrow 2026</t>
+          <t>Competition – Eskom Expo for Young Scientists</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://www.sowetan.co.za/careers/2026-03-03-register-your-school-for-samsung-solve-for-tomorrow-2026/</t>
+          <t>https://exposcience.co.za/category/competition/</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Register your school for Samsung Solve for Tomorrow 2026 STEM competition aims to transform and empower South African learners with critical skills to solve real-world challenges March 03, 2026 at 7:44 am</t>
+          <t>Aqil Variava business cities Damien ... Gray STEMI Vuyo Nzimande · Eskom Expo for Young Scientists is an exposition, or science fair, where students have a chance to show others their projects about their own scientific investigations. At the annual prestigious Eskom Expo for Young Scientists International Science Fair (ISF), selected students from 35 Expo Regions in South Africa then compete ...</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2153,7 +2153,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>ssasft@samsung.com</t>
+          <t>support@exposcience.co.za</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2180,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com</t>
+          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>8c4075d5481d476e945486754f783364@sentry.io, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, info@thecortexhub.africa, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com</t>
+          <t>c183baa23371454f99f417f6616b724d@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, info@thecortexhub.africa, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -2288,7 +2288,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>adverts@ubuntutimes.co.za, newspaper-rec300@2x.jpg</t>
+          <t>newspaper-rec300@2x.jpg, adverts@ubuntutimes.co.za</t>
         </is>
       </c>
     </row>
@@ -2361,7 +2361,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>madelien@imbewu.foundation, webmaster@sciencexpo.org.za, marna.vanzyl@imbewu.foundation</t>
+          <t>madelien@imbewu.foundation, marna.vanzyl@imbewu.foundation, webmaster@sciencexpo.org.za</t>
         </is>
       </c>
     </row>
@@ -2388,7 +2388,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>NkosiN@atnews.co.za, rampedim@atnews.co.za</t>
+          <t>rampedim@atnews.co.za, NkosiN@atnews.co.za</t>
         </is>
       </c>
     </row>
@@ -2418,17 +2418,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Upcoming Civil Engineering Conferences in South Africa 2025-2026</t>
+          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://conferencealerts.co.in/south-africa/civil-engineering</t>
+          <t>https://www.engineeringnews.co.za/article/saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini-2022-09-13</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>International Civil engineering conferences in South africa 2025-2026 with invitation letter. A great opportunity to meet and learn from experts in your field.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng. Twelve schools participated in the grand finale, which saw great, ...</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2436,22 +2436,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>chanel@engineeringnews.co.za, newsletters@creamermedia.co.za, newsdesk@engineeringnews.co.za, subscriptions@creamermedia.co.za, advertising@creamermedia.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
+          <t>Engineering the Future: 16 schools compete in SAICE’s 33rd International Bridge Building Competition - SAICE</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini-2022-09-13</t>
+          <t>https://saice.org.za/press-releases/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng. Twelve schools participated in the grand finale, which saw great, ...</t>
+          <t>April 17, 2025 - The South African Institution of Civil Engineering (SAICE) hosted its 33rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2461,24 +2465,24 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>newsletters@creamermedia.co.za, chanel@engineeringnews.co.za, subscriptions@creamermedia.co.za, newsdesk@engineeringnews.co.za, advertising@creamermedia.co.za</t>
+          <t>membership@saice.org.za, civilinfo@saice.org.za, communications@saice.org.za, accounts@saice.org.za, marketing@saice.org.za</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
+          <t>Upcoming Civil Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://www.crown.co.za/construction-world/marketplace/22289-saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini</t>
+          <t>https://conferencealerts.co.in/south-africa/civil-engineering</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng.</t>
+          <t>International Civil engineering conferences in South africa 2025-2026 with invitation letter. A great opportunity to meet and learn from experts in your field.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2486,26 +2490,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>ernao@crown.co.za, constr@crown.co.za</t>
-        </is>
-      </c>
+      <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Engineering the Future: 16 schools compete in SAICE’s 33rd International Bridge Building Competition - SAICE</t>
+          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://saice.org.za/press-releases/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
+          <t>https://www.crown.co.za/construction-world/marketplace/22289-saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>April 17, 2025 - The South African Institution of Civil Engineering (SAICE) hosted its 33rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2515,7 +2515,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>accounts@saice.org.za, marketing@saice.org.za, communications@saice.org.za, membership@saice.org.za, civilinfo@saice.org.za</t>
+          <t>ernao@crown.co.za, constr@crown.co.za</t>
         </is>
       </c>
     </row>
@@ -2618,17 +2618,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Upcoming Civil engineering Conferences in Cape town 2025</t>
+          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://conferencealerts.co.in/cape-town/civil-engineering</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2205</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Civil engineering conferences in Cape town 2025 provide an exclusive global platform to meet and engage with experts and aspirants in various fields.</t>
+          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2641,17 +2641,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
+          <t>Upcoming Civil engineering Conferences in Cape town 2025</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2205</t>
+          <t>https://conferencealerts.co.in/cape-town/civil-engineering</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
+          <t>Civil engineering conferences in Cape town 2025 provide an exclusive global platform to meet and engage with experts and aspirants in various fields.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2664,17 +2664,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>South Africa students defeated the world to win nasa school ...</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://www.facebook.com/sanctview/posts/south-africa-students-defeated-the-world-to-win-nasa-school-engineering-competit/1361370549525718/</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
+          <t>Aug 11, 2026 · . Welabasha High School learner wins first place in Sasol mechanical technology competition. Thembeka Mathenjwa Sthole ▻ Welabasha High ...</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2687,17 +2687,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>List of ALL Engineering Bursaries South Africa 2027PRDW Bursaries 2027: Support for Civil, Mechanical ...ASTEMI Competitions – SAASTACompetitions | Capetown 2026Mechanical Engineering Bursaries 2023- 2024</t>
+          <t>Engineering for People Design Challenge</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
+          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Aerospace Engineers develop and test aircraft and spacecrafts. They are also responsible for the design, maintenance and management of R&amp;D for various types of spacecrafts, aircrafts, missiles and satellites. This sector of engineering is divided into 2 branches which overlap: astronautical engineering and aeronautical engineering. These profession... See full list on zabursaries.co.za Bioresource Engineering is a discipline that incorporates design, engineering, as well as biological sciences to enhance and increase the sustainability of the planet’s natural resources. Bioresource Engineers look for solutions to problems involving animals, plants, and the environment. Bioresource Engineers are responsible for designing, operatin... See full list on zabursaries.co.za Chemical Engineers use chemical processes to find new ways to produce goods – from pharmaceuticals, cleaning solvents and fuels, to textiles and even food. These professionals are also involved in creating new ways to improve industrial processes by use of better chemical systems, as well as to limit inefficiency and waste within the industrial set... See full list on zabursaries.co.za Civil Engineers oversee the design, planning and construction of major infrastructures such as railways, highways, bridges, skyscraper buildings and water reservoirs. They assess material and labour costs, project deadlines and environmental impacts which will affect their projects. These professionals can find employment in various sectors, includ... See full list on zabursaries.co.za Construction engineers deal with the design, planning, management and construction of major infrastructures, including buildings, bridges, airports, tunnels, roads, railroads, dams, facilities and the like. Construction engineering is a sub-division of the Civil Engineering sector. Some of the job responsibilities of a Construction Engineer, involv... See full list on zabursaries.co.za Electronics engineering deals with the design of electronic circuits, microcontrollers, microprocessors and other devices by way of active and non-linear electrical components. These professionals are responsible for designing, testing and maintaining of electronic parts and systems used in the automation, navigation, communication and related fiel... See full list on zabursaries.co.za Environmental Engineers create solutions for environmental problems, by making us of engineering principles, as well as chemistry, biology and soil science. Their work involves addressing global issues such as climate change, water and air pollution, waste disposal, public health, recycling and environmental sustainability. Professionals in this se... See full list on zabursaries.co.za Engineering defines the branch of technology and science that deals with maintenance, design, building, as well as the use of machines, engines, and structures. A qualification in Engineering (General) is great for a student who is still unsure about what aspect of Engineering they would like to branch into, and most Universities offer a General En... See full list on zabursaries.co.za Industrial Engineers are responsible for determining ways to improve employee management; as well as the management of machinery; manufacturing processes and other assets, in order to improve the operations of their company. These professionals study reports based on process efficiency and create strategies which will improve said processes – this ... See full list on zabursaries.co.za Instrumentation engineers focus on automated systems, pneumatic domains and the operation and principles of measuring instruments used herein. People in this sector generally work for manufacturing or chemical plants, with the aim of improving the productivity, stability, optimisation and reliability of the system in question. If you are looking fo... See full list on zabursaries.co.za 3 days ago · PRDW Bursaries 2027: Civil, Mechanical, and Mechatronics Engineering PRDW is inviting South African citizens and permanent residents to apply for its 2027 Bursary Programme. This opportunity […] ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa. Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation. Mechanical Engineering bursaries are offered by many companies in South Africa each year to deserving candidates. Have a look at some of the companies..</t>
+          <t>Engineering for People, our flagship university design challenge, has won Silver in the QS Reimagine Education Awards 2025, recognising its impact in empowering ... Missing: mechanical | Show results with: mechanical</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2710,17 +2710,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>PRDW Bursaries 2027: Support for Civil, Mechanical ...</t>
+          <t>Team South Africa wins NASA space engineering competition</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://southafricaportal.com/prdw-engineering-bursaries-2027/</t>
+          <t>https://www.facebook.com/100090360075633/posts/team-south-africa-has-won-a-nasa-space-engineering-competition-the-team-beat-oth/1035040346184625/</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>3 days ago · PRDW Bursaries 2027: Civil, Mechanical, and Mechatronics Engineering PRDW is inviting South African citizens and permanent residents to apply for its 2027 Bursary Programme. This opportunity […]</t>
+          <t>Team South Africa has won a NASA space engineering competition. The team beat other countries with their engineering and problem-solving skills. The victory is ...</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2733,17 +2733,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>What are the names of international level mechanical ... - Quora</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.quora.com/What-are-the-names-of-international-level-mechanical-engineering-competitions-for-a-college-student</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>Jun 10, 2015 · BAJA conducted by SAE(Society for automotive engineering),a competition for building ATV (terrain vehicle) is considered the biggest event for ... What are the various mechanical engineering competitions in ... What are the competitions for mechanical engineering students? More results from www.quora.com</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2756,17 +2756,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>CELEBRATING MANUFACTURING AND ENGINEERING ...</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.facebook.com/mersetasocial/videos/𝐖𝐀𝐓𝐂𝐇-𝐂𝐄𝐋𝐄𝐁𝐑𝐀𝐓𝐈𝐍𝐆-𝐌𝐀𝐍𝐔𝐅𝐀𝐂𝐓𝐔𝐑𝐈𝐍𝐆-𝐀𝐍𝐃-𝐄𝐍𝐆𝐈𝐍𝐄𝐄𝐑𝐈𝐍𝐆-𝐂𝐇𝐀𝐌𝐏𝐈𝐎𝐍𝐒-𝐀𝐓-𝐖𝐎𝐑𝐋𝐃𝐒𝐊𝐈𝐋𝐋𝐒-𝐒𝐎𝐔𝐓𝐇-𝐀/779762595201549/</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
+          <t>Mar 12, 2026 · The event highlighted the power of artisan development in creating opportunities for training, employment, and entrepreneurship in South Africa.</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2774,26 +2774,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Mechanical Engineering Bursaries 2023- 2024</t>
+          <t>ICME 2028: 22. International Conference on Mechanical ...</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://bursaries-southafrica.co.za/bursaries-mechanical-engineering/</t>
+          <t>https://waset.org/mechanical-engineering-conference-in-november-2028-in-cape-town</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Mechanical Engineering bursaries are offered by many companies in South Africa each year to deserving candidates. Have a look at some of the companies..</t>
+          <t>International Conference on Mechanical Engineering November 04-05, 2028 in Cape Town, South Africa. Early Bird Registration Deadline October 04, 2028 ...</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2806,17 +2802,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>SAIMechE</t>
+          <t>Real-world research: Engineering team designs South African ...</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://www.saimeche.org.za/</t>
+          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
+          <t>May 15, 2025 · Cross-disciplinary teams present prototypes at Research Day, Engineers Without Borders' design challenge addressed by nearly 90 students.</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2824,27 +2820,31 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>dolanm@uwstout.edu, frischj@uwstout.edu</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>IEEE South Africa</t>
+          <t>About Baja - SAE International</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>http://www.ieee.org.za/</t>
+          <t>https://www.sae.org/events/student/about/baja</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>The South African Section has around 1200 members and many subsections. It was formed in 1963 by the merger of the Institute of Radio Engineers (IRE, founded 1912) and the American Institute of Electrical Engineers (AIEE, founded 1884).</t>
+          <t>Baja SAE® consists of competitions that simulate real-world engineering design projects and their related challenges. May 20-23, 2027. Baja SAE South Africa</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
@@ -2852,22 +2852,22 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Electrical Engineering Conferences in South Africa 2026/2027 ...</t>
+          <t>WorldSkills Results</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://conferenceindex.org/conferences/electrical-engineering/south-africa</t>
+          <t>https://results.worldskills.org/results</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Electrical Engineering Conferences in South Africa 2026 2027 2028 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and symposiums.</t>
+          <t>WorldSkills Competition 2022 Special Edition South Africa Mechanical Engineering CAD 17. South Africa Plumbing and Heating 23.</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -2875,40 +2875,44 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+          <t>Johannesburg, S.A. - Next Engineers</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://www.nextengineers.org/en/locations/johannesburg</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions.</t>
+          <t>Johannesburg's Engineering Discovery has reached 3 170 Grade 8 learners across the city since launch in 2022. This year, the team is aiming to reach 1 000 more!</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr"/>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>nextengineers@protec.org.za, NextEngineers@fhi360.org</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>South African Institute of Electrical Engineers</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://www.saiee.org.za/</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
+          <t>South African Institute of Electrical Engineers (SAIEE) About Us See Member Benefits · Become a SAIEE Member today! SAIEE Membership · Earn CPD credits · About Training Academy · Join a SAIEE Centre near you! Centres · South African Institute of Electrical Engineers (SAIEE) 01 ·</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2916,7 +2920,11 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>reception@saiee.org.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2944,17 +2952,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers</t>
+          <t>List of ALL Engineering Bursaries South Africa 2027</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/</t>
+          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>All equipment from massive ships to tiny devices h ... Earn your CPD credits today! Read it here.</t>
+          <t>How much can I earn within the Engineering field in South Africa? The engineering sector in South Africa offers a wide range of career opportunities across fields such as civil, mechanical, electrical, chemical, mining, and industrial engineering. Salaries vary depending on qualifications, experience, and industry, with entry-level roles typically starting at moderate levels and increasing ...</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2962,26 +2970,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, reception@saiee.org.za</t>
-        </is>
-      </c>
+      <c r="E104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Zutari Bursary Programme 2027 Opens Applications for Civil ...</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://www.globalsouthopportunities.com/2026/08/10/zutari/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Aug 10, 2026 · Zutari has opened applications for its 2027 Engineering Bursary Programme, offering financial and professional development support to South African students pursuing studies in Civil Engineering and Electrical Engineering.</t>
+          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2989,27 +2993,31 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://hackon.co.za/</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
+          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
@@ -3017,22 +3025,22 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Hackathons en South Africa</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://za.allhackathons.com/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Aug 22, 2025 · Join us for an electrifying hackathon where innovation meets security and finance! This event brings together developers, data scientists, cybersecurity experts, and FinTech enthusiasts to …</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E107" t="inlineStr"/>
@@ -3040,22 +3048,22 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Hackathons - challenge.entelect.co.za</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://challenge.entelect.co.za/hackathons</t>
+          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>5 days ago · A hands-on practice problem statement for Hack-ademy workshop attendees, joining in person or online. Compete against the best university teams across South Africa. Prize Pool: Various cool prizes &amp; bragging rights!</t>
+          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
@@ -3063,22 +3071,22 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Build the Future with Entelect Hackathons</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - SAIEE National Student Project Competition</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>https://challenge.entelect.co.za/</t>
+          <t>https://www.saiee.org.za/calendar/EventDetails.aspx?eeid=29281</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Instead of focusing on building a once-off project, our hackathons centre around optimisation problems. Participants develop solutions that are tested, scored, and ranked based on performance, efficiency, and strategy.</t>
+          <t>The SAIEE National Students Project Competition will be held at the North-West University (Potchefstroom Campus) on 21 November 2019</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E109" t="inlineStr"/>
@@ -3086,22 +3094,22 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Unisa hosts first-ever Hackathon to ignite student learning ...</t>
+          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-hosts-first-ever-Hackathon-to-ignite-student-learning-experience</t>
+          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Jul 14, 2025 · The event supported key priorities of South Africa’s National Development Plan, Unisa’s Catalytic Niche Areas and the United Nations’ Sustainable Development Goals that relate to access to quality education, decent work and innovation.</t>
+          <t>March 12, 2026 - At the Centre for High Performance Computing (CHPC) Conference hosted in Cape Town at the end of last year, four current fourth-year electrical engineering students were crowned national champions in the Student Cluster Competition for 2025.</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E110" t="inlineStr"/>
@@ -3109,52 +3117,259 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Young Engineers Movement (YEM) - ORT SA</t>
+          <t>Student Design Competition | IEEE CASS</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
+          <t>https://ieee-cas.org/society-involvement/student-design-competition</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>The Young Engineers Movement (YEM) is an immersive engineering and technology hackathon designed to equip young South Africans with the skills, mindset and confidence needed to solve real-world challenges.</t>
+          <t>CASS will reimburse the travel costs for the trip to ISCAS 2026 for the four finalists, one for each region - Regions 1-7 (USA and Canada), Region 8 (Europe, Middle East, Africa), Region 9 (Latin America), and Region 10 (Asia, Australia, Pacific), as well as ISCAS registration.</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
-        </is>
-      </c>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
+          <t>The Home of South African Hackathons</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>https://hackon.co.za/</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Hackathons en South Africa</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>https://za.allhackathons.com/</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Geekulcha Annual Hackathon 2026 - Registration | Sonke Platform</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>https://sonke.gklink.co/event/gkhack26</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>GEEKULCHA ANNUAL HACKATHON 2026 Africa's premier hackathon that drives digital innovation and empowers the next generation of tech leaders.</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Build the Future with Entelect Hackathons</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>https://challenge.entelect.co.za/</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Build the Future with Entelect Hackathons Join South Africa's premier optimisation-first developer competition platform. Compete, iterate, and outperform the best.</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Unisa hosts first-ever Hackathon to ignite student learning experience</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-hosts-first-ever-Hackathon-to-ignite-student-learning-experience</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Unisa's Information and Communication Technology Portfolio, in collaboration with the College of Science, Engineering and Technology, held the first-ever Unisa Hackathon on 3 and 4 July 2025, marking a major step in the university's journey to embed digital innovation and entrepreneurship into the students learning experience.</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>AI Hackathon | Sebaka</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>https://sebakasouthafrica.co.za/index.html</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>AI Hackathon Build an AI Agent for Software Quality Engineering The future of software testing is intelligent, collaborative and AI-powered.</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Hackathon Timeline | Sebaka</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>https://sebakasouthafrica.co.za/events.html</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Sebaka Mentorship &amp; Hackathons — Build an AI Agent for Software Quality Engineering.</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Hackathons - challenge.entelect.co.za</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>https://challenge.entelect.co.za/hackathons</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>University Cup Compete against the best university teams across South Africa Prize Pool: Various cool prizes &amp; bragging rights!</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Young Engineers Movement (YEM) - ORT SA</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
           <t>CompeteHub - Where Champions Are Made</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr">
+      <c r="B121" t="inlineStr">
         <is>
           <t>https://www.devpluxe.co.za/</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>Join thousands of developers, designers, and innovators competing in South Africa ' s most impactful tech hackathons. We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>About DevPluxe Empowering South Africa ' s next generation of innovators We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
         <is>
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
+      <c r="E121" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update competition data 2026-08-28
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+          <t>3 weeks ago - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -464,26 +464,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>Sep 4, 2025 · 3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -493,24 +489,24 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>info@ieomsociety.org</t>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -520,24 +516,24 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+          <t>info@ieomsociety.org</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -545,12 +541,16 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -560,7 +560,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -573,17 +573,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2027 Africa Prize for Engineering Innovation Opens Applications</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.globalsouthopportunities.com/2026/08/09/africa-134/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>The Royal Academy of Engineering has opened applications for the 2027 Africa Prize for Engineering Innovation, providing African innovators with an opportunity to develop, strengthen and commercialise engineering solutions addressing important challenges across the continent.</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -596,7 +596,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -619,17 +619,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
+          <t>Two South Africans on the shortlist for the 2026 Africa Prize for Engineering Innovation</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
+          <t>https://www.engineeringnews.co.za/article/two-south-africans-on-the-shortlist-for-the-2026-africa-prize-for-engineering-innovation-2026-08-04</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Eligibility Benchmark Requirements The Africa Prize is open to individuals or teams based in sub-Saharan Africa with a scalable engineering innovation that demonstrates social or environmental impact potential. Applicants must: Be citizens ordinarily residing in a sub-Saharan African country. Be over 18 years old and fluent in English.</t>
+          <t>3 weeks ago - Two South African innovators have been shortlisted for the UK Royal Academy of Engineering’s Africa Prize for Engineering Innovation 2026. This is the continent’s richest award aimed at promoting engineering innovation and entrepreneurship ...</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -637,22 +637,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>chanel@engineeringnews.co.za, newsletters@creamermedia.co.za, advertising@creamermedia.co.za, subscriptions@creamermedia.co.za, newsdesk@engineeringnews.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>List of ALL Engineering Bursaries South Africa 2027</t>
+          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
+          <t>https://www.poidata.io/report/engineer/south-africa</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>How much can I earn within the Engineering field in South Africa? The engineering sector in South Africa offers a wide range of career opportunities across fields such as civil, mechanical, electrical, chemical, mining, and industrial engineering. Salaries vary depending on qualifications, experience, and industry, with entry-level roles typically starting at moderate levels and increasing ...</t>
+          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -665,17 +669,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>NASA space win: SA learners triumph at Kennedy Space Center</t>
+          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://furtherafrica.com/2026/08/11/nasa-space-win-sa-learners-triumph-at-kennedy-space-center/</t>
+          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>NASA space win for South Africa as seven Western Cape learners win the International Space Settlement Design Competition at Kennedy Space Center.</t>
+          <t>2 weeks ago - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -688,17 +692,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
+          <t>South Africa International Industrial Expo | Innovation Bridge</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/tradeshows</t>
+          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>South Africa trade shows, find and compare 964 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 174 upcoming expos in 2026-2027 1. South Africa Infrastructure &amp; Water Expo, 2.</t>
+          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -711,17 +715,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
+          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://madeinafricaevent.co.za/</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AI Expo Africa 2026 - Join the Largest AI Event &amp; Trade Community in Africa TODAY! Our business audience is a buyer / supplier focused community and comprised of Enterprise decision makers / CxOs, allied to AI Cloud platform providers, Tier 1 / 2 deployment &amp; service providers, AI start ups / innovators, investors, educators, government and AI ecosystem community builders.</t>
+          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -729,26 +733,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>enquiries@aiexpoafrica.com</t>
-        </is>
-      </c>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DigiMarCon Africa 2027 - Cape Town, South Africa · October 6</t>
+          <t>Two landmark exhibitions set to transform industrial technology and renewable energy in South Africa</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://digimarconafrica.com/</t>
+          <t>https://www.engineeringnews.co.za/article/two-landmark-exhibitions-set-to-transform-industrial-technology-and-renewable-energy-in-south-africa-2025-10-24</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>The Premier Digital Marketing, Media and Advertising Conference &amp; Exhibition held annually in Cape Town, South Africa! Join your peers for 2 days jam packed with digital marketing best practices, latest trends and strategy, also check out the next generation of technology &amp; innovation; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year ...</t>
+          <t>October 24, 2025 - South Africa’s industrial and clean energy sectors celebrated a landmark moment today with the official launch of RE+ South Africa 2026 and the Cape Industrial Technology Exhibition (CITE) 2027.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -758,24 +758,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>info@digimarconafrica.com</t>
+          <t>chanel@engineeringnews.co.za, newsletters@creamermedia.co.za, advertising@creamermedia.co.za, subscriptions@creamermedia.co.za, newsdesk@engineeringnews.co.za</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Exhibitions in South Africa 2026-2027 - ExpoTobi</t>
+          <t>KZN Industrial Technology Exhibition</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://expotobi.com/country/south-africa/exhibitions</t>
+          <t>https://www.kznindustrial.co.za/</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>All Exhibitions in South Africa 2026-2027 | Full and accurate description of events for various business sectors | Schedule, tickets, travel arrangements and participation</t>
+          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -783,22 +783,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>john@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Africa Tech Festival</t>
+          <t>Trade Shows Worldwide - South Africa - 2026/2027</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://www.eventseye.com/fairs/c1_trade-shows_south-africa.html</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
+          <t>South Africa Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in South Africa</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -806,26 +810,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>support@knect365.com, customerservices@informaconnect.com, dataprivacy@informaconnect.com, customerservices@knect365.com, support@informaconnect.com, salesenquiries@africatechfestival.com, dataprivacy@knect365.com</t>
-        </is>
-      </c>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>Exhibition | Innovation Festival Durban | South Africa</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://www.innovationfestival.durban/exhibition</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -833,22 +833,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, Erika@innovate.durban, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, sithabile@innovate.durban, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
+          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://innovationweek.co.za/</t>
+          <t>https://manufacturingindaba.co.za/exhibition/</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SA Innovation Week 2026 is South Africa's official national innovation platform accelerating implementation, commercialisation and impact.</t>
+          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -856,26 +860,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>info@pixal8media.co.za</t>
-        </is>
-      </c>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Proudly South African Buy Local Summit &amp; Expo 2026 | Innovation Bridge</t>
+          <t>International Science, Innovation &amp; Technology Expo (INSITE)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://innovationbridge.info/ibportal/content/proudly-south-african-buy-local-summit-expo-2026</t>
+          <t>https://www.dsti.gov.za/index.php/resource-center/27-temp/dst-links/3-international-science-innovation-a-technology-expo</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>The 14th edition of the Proudly South African Buy Local Summit &amp; Expo will take place on 16-17 March 2026 at the Sandton Convention Centre, Johannesburg. As Proudly South African's flagship annual event, the Summit &amp; Expo has evolved into the country's premier local procurement and localisation platform, convening key public and private sector stakeholders to strengthen domestic value ...</t>
+          <t>The essence of INSITE INSITE is an international, biennial must-see Science and Technology event in South Africa, the only one of its kind in Africa that creates new frontiers for global challenges · INSITE aims to assemble the worlds leading innovators and scientists in one place, stimulating ...</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -888,17 +888,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 - Technology Expo · October 6</t>
+          <t>Discover Innovation Hub's Pavilion at Organic &amp; Natural Products Expo - Organic &amp; Natural Products Portal</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://www.organicandnaturalportal.com/innovation-hub-organic-expo/</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Where Business, Tech and Innovation Collide in Cape Town! TECHSPO Cape Town is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology.</t>
+          <t>3 weeks ago - Gathering producers, retailers, buyers, and conscious consumers under one roof, the expo serves as Africa’s premier showcase for sustainability, health, and wellness innovation. A standout highlight of this year’s exhibition is The Innovation Hub Pavilion, hosting a curated line-up of forward-thinking South African small, medium, and micro-enterprises (SMMEs).</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -906,26 +906,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>info@techspocapetown.co.za</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TECHSPO Joburg 2026 - Technology Expo · October 10</t>
+          <t>Come and explore our exhibition of innovative discoveries at Science Forum South Africa 2024 | CSIR</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://techspojoburg.co.za/</t>
+          <t>https://www.csir.co.za/come-and-explore-our-exhibition-innovative-discoveries-science-forum-south-africa-2024</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
+          <t>December 3, 2024 - The exhibition launch will take place on Tuesday, 3 December 2024, with the opening address by Department of Science, Technology and Innovation Minister Dr Blade Nzimande.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -933,26 +929,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>info@techspojoburg.co.za</t>
-        </is>
-      </c>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
+          <t>In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community’s challenges and how community members view the impact of these challenges on their daily lives.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -960,22 +952,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
+          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -983,26 +979,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
-        </is>
-      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EWB Design Challenge | Aston University</t>
+          <t>Engineering for People Design Challenge | Department of ...</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
+          <t>Aug 4, 2025 · This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but under-resourced neighbourhood on the eastern edge of Johannesburg. Home to around 46,000 people, Makers Valley is a community rich in creativity, activism ...</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1010,22 +1002,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
+          <t>Engineering For People Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
+          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
+          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1035,24 +1031,24 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ied@ied.org.uk</t>
+          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South ...</t>
+          <t>Engineering for People Design Challenge - Engineers Without ...</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
+          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
+          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1065,17 +1061,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Latest Community Engineering Design Competition Announced</t>
+          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
+          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
+          <t>Oct 24, 2024 · The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1083,22 +1079,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>team@crowdsolve.net</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Engineering for people, that’s the challenge | Engineers Without Borders</t>
+          <t>EWB Design Challenge | Aston University</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.rs-online.com/designspark/an-introduction-to-engineering-for-people-design-challenge</t>
+          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>That’s exactly what the annual Engineering for People Design Challenge asks participants to do. The competition, delivered in partnership by Engineers without Borders South Africa and Engineers Without Borders UK, encourages engineering students and those collaborating with engineers to broaden their awareness of how their decisions change the world.</t>
+          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1111,17 +1111,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of Engineering</t>
+          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
+          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1131,24 +1131,24 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
+          <t>ied@ied.org.uk</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
+          <t>Engineers Without Borders South ...</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
+          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
+          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1161,17 +1161,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Launching Engineering for People Design challenge 2024 ...</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.electronicspecifier.com/studentzone/studentzone-news/launching-engineering-for-people-design-challenge-2024-25-2/</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>November 16, 2025 - Engineers Without Borders has launched the 2024/25 cycle of the award-winning Engineering for People Design Challenge in partnership with Engineers Without Borders South Africa and Makers Valley Partnership.</t>
+          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1184,17 +1184,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1202,22 +1202,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1225,22 +1229,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>National Student Competition | ORSSA</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;area=2200&amp;ranking=Overall&amp;country=ZAF</t>
+          <t>https://www.orssa.org.za/studentcomp</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>National Student Competitions The Operations Research Society of South Africa The home of decision intelligence The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1248,22 +1256,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, email@example.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1276,17 +1288,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Competitions – Enactus South Africa | National Expos ...</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://enactusza.org/what-we-do/competitions</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Explore our national and international competitions that empower students to tackle challenges with entrepreneurial solutions and social impact at the core.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1294,22 +1306,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>adminsa@enactus.org, xmadlanga@enactus.org, marketingsa@enactus.org, liso@enactus.org</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Engineering in South Africa: 24 Best universities Ranked</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://edurank.org/engineering/za/</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
+          <t>Sep 4, 2025 · 3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1317,22 +1333,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
+          <t>Engineering Competition For African Youth In Engineering ...</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2210</t>
+          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
+          <t>Aug 18, 2025 · The Africa Prize is open to individuals or teams based in sub-Saharan Africa with a scalable engineering innovation that demonstrates social or environmental impact potential.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1345,17 +1365,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2025</t>
+          <t>Engineering for People Design Challenge</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
+          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2025</t>
+          <t>Engineering for People, our flagship university design challenge, has won Silver in the QS Reimagine Education Awards 2025, recognising its impact in empowering ...</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1368,17 +1388,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>University of South Africa</t>
+          <t>Inspiring, building and shaping a future fit engineering community</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-promotes-globally-recognised-engineering-qualifications</t>
+          <t>https://www.ewb-international.org/home/inspiring-building-and-shaping-a-future-fit-engineering-community/</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Unisa promotes globally recognised engineering qualifications</t>
+          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, the Design Challenge has been delivered in ... Missing: competition | Show results with: competition</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1386,22 +1406,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>admin@ewb-international.org</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
+          <t>International science and technology competition 2026</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
+          <t>https://www.facebook.com/groups/443764394251719/posts/1259344422693708/</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
+          <t>Dec 20, 2025 · ... Engineering Technologies (ICISCET 2026) to be held from 14 - 16 October 2026 in Vanderbijlpark, South Africa. Submission Deadline:15 June ...</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1424,7 +1448,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation … 17-19 November 2026 Cape Town ...</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1434,24 +1458,24 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>support@knect365.com, customerservices@informaconnect.com, dataprivacy@informaconnect.com, customerservices@knect365.com, support@informaconnect.com, salesenquiries@africatechfestival.com, dataprivacy@knect365.com</t>
+          <t>salesenquiries@africatechfestival.com, dataprivacy@informaconnect.com, support@informaconnect.com, support@knect365.com, customerservices@informaconnect.com, customerservices@knect365.com, dataprivacy@knect365.com</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TECHSPO Technology Expo</t>
+          <t>IT &amp; Technology Events in South Africa | 10times</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://techspo.co/</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>TECHSPO is a Technology Expo Series with annual events in 50 international cities, across 20 countries. South Africa October 1 – 2, 2026 Cape Town, South ...</t>
+          <t>Aug 17, 2026 · Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1464,17 +1488,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~…</t>
+          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 ...</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://www.industryevents.com/events/techspo-johannesburg-2026-technology-expo-internet-mobile-adtech-martech-saas</t>
+          <t>https://techspojoburg.co.za/</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology Expo returns September 28-29, 2026 to the NH Johannesburg Sandton Hotel in Johannesburg, South Africa.</t>
+          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1482,26 +1506,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>events@techspojoburg.co.za, support@industryevents.com, your@email.com, you@company.com, colleague@company.com</t>
-        </is>
-      </c>
+      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Tech conferences in South Africa 2026 / 2027 - dev.events</t>
+          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://dev.events/AF/ZA/tech</t>
+          <t>https://10times.com/johannesburg-za/technology</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Best Tech conferences in South Africa 2026 / 2027 · The Principal Dev – Masterclass for Tech Leads · Clean Architecture Masterclass · OT SECURITY FIRST ...</t>
+          <t>19 hours ago · Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1514,17 +1534,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa - 10Times</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7 ...</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>The TECHSPO Technology Expo is set to take place in the bustling business hub of Sandton, Johannesburg, from September 28 to September 29, 2026.</t>
+          <t>Where Business, Tech and Innovation Collide in Cape Town! TECHSPO Cape Town is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1532,22 +1552,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>info@techspocapetown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Mediatech Africa (@mediatechafrica) · Johannesburg - Instagram</t>
+          <t>TECHSPO Johannesburg Technology ExpoJohannesburg Technology ...</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/mediatechafrica/</t>
+          <t>https://techspojoburg.co.za/johannesburg-technology-expo/</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Africa's largest Pro AV, Film, Broadcast &amp; Live Event Tech Expo. 27 - 29 June 2028, Johannesburg .</t>
+          <t>TECHSPO Johannesburg is a 2-day technology expo taking place September 28 – 29, 2026 at the luxurious NH Johannesburg Sandton Hotel, Toronto, Ontario. TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1560,17 +1584,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Africa Technology Expo</t>
+          <t>IT Indaba 2026 – Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://africatechnologyexpo.com/</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>The Africa Technology Expo (ATE) is a first-of-its-kind, multi-year enterprise gathering at the intersection of Africa's potential and global opportunity.</t>
+          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what’s next before everyone else does. Only 2,500 ...</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1578,26 +1602,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>partner@africatechnologyexpo.com, johndoe@email.com, info@sparkafrica.co</t>
-        </is>
-      </c>
+      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Graintech Africa 2026 | Grain &amp; Allied Tech Expo Johannesburg</t>
+          <t>TECHSPO Technology Expo</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://sa.graintechafrica.com/</t>
+          <t>https://techspo.co/</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Join Graintech Africa 2026, 11–13 March in Johannesburg. Explore innovations in grain processing, milling, storage, packaging &amp; allied technologies.</t>
+          <t>TECHSPO is a Technology Expo Series with annual events in 50 international cities, across 20 countries. South Africa October 1 – 2, 2026 Cape Town, South ...</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1605,26 +1625,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>gtaexpo@graintechafrica.com</t>
-        </is>
-      </c>
+      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>TECHSPO Events</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~…</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://techspo.co/events/</t>
+          <t>https://www.industryevents.com/events/techspo-johannesburg-2026-technology-expo-internet-mobile-adtech-martech-saas</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Johannesburg, South Africa. October 1 – 2, 2026. Cape Town, South Africa. October 8 – 9, 2026. Philadelphia, PA. October 14 – 15, 2026. Miami, FL. October 22 – ...</t>
+          <t>TECHSPO Johannesburg Technology Expo returns September 28-29, 2026 to the NH Johannesburg Sandton Hotel in Johannesburg, South Africa.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1632,22 +1648,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>your@email.com, events@techspojoburg.co.za, support@industryevents.com, you@company.com, colleague@company.com</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>zambia &amp; southern africa - Africa FarmTech Expos</t>
+          <t>Tech conferences in South Africa 2026 / 2027 - dev.events</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://www.africafarmtechexpo.com/south/</t>
+          <t>https://dev.events/AF/ZA/tech</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>The Africa FarmTech Expos welcome international, regional and local companies that are involved in manufacture and supply of technologies, products and services ...</t>
+          <t>Best Tech conferences in South Africa 2026 / 2027 · The Principal Dev – Masterclass for Tech Leads · Clean Architecture Masterclass · Escape 2026 · HR World Summit ...</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1655,11 +1675,7 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>info@fwafrica.net</t>
-        </is>
-      </c>
+      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1687,17 +1703,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
+          <t>Maker Faire - Wikipedia</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://makerfairecapetown.wordpress.com/about/</t>
+          <t>https://en.wikipedia.org/wiki/Maker_Faire</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
+          <t>May 3, 2026 - Maker Faires are also held in Europe, Asia, South America and Africa.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1710,17 +1726,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
+          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
+          <t>https://makerfairecapetown.wordpress.com/about/</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
+          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1753,24 +1769,24 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>chosen-sprite@2x.png, fancybox_sprite@2x.png, fancybox_loading@2x.gif, pr@make.co</t>
+          <t>fancybox_sprite@2x.png, fancybox_loading@2x.gif, chosen-sprite@2x.png, pr@make.co</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
+          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://contemporaryand.com/fr/events/maker-faire-africa-comes-to-johannesburg</t>
+          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
+          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1783,17 +1799,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>The Makers Hub</t>
+          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://www.decorex.co.za/cape-town/en-gb/visit/TheMakersHub.html</t>
+          <t>https://contemporaryand.com/en/events/maker-faire-africa-comes-to-johannesburg</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Explore unique handmade items, take part in interactive workshops, and engage directly with Cape Town’s vibrant maker community.</t>
+          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1801,11 +1817,7 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>decorexafrica@rxglobal.com</t>
-        </is>
-      </c>
+      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1853,7 +1865,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, example@mysite.com, 8c4075d5481d476e945486754f783364@sentry.io, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, warren@makersfestival.co.za, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com</t>
+          <t>warren@makersfestival.co.za, 8c4075d5481d476e945486754f783364@sentry.io, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, example@mysite.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -1883,17 +1895,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Why Africa needs Maker Faire | ZDNET</t>
+          <t>The Makers Hub</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://www.zdnet.com/article/why-africa-needs-maker-faire/</t>
+          <t>https://www.decorex.co.za/cape-town/en-gb/visit/TheMakersHub.html</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>July 24, 2014 - Unlike other Maker Faires, Okafor said that it's not enough to simply hold the event in an African city and see who turns up. Two volunteers are currently working in South Africa to discover inventors in rural areas and neighbouring countries such as Zambia and Botswana who they can encourage to attend and show off their work.</t>
+          <t>Explore unique handmade items, take part in interactive workshops, and engage directly with Cape Town’s vibrant maker community.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1903,14 +1915,14 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>brand_licensing@ziffdavis.com</t>
+          <t>decorexafrica@rxglobal.com</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1920,7 +1932,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>All these Olympiads and Competitions have a positive impact on education and on educational institutions in South Africa, but there is still a need to build stronger collaboration among teachers, schools, universities and educational authorities in order to meet the challenges of STEM education in South Africa today.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1933,17 +1945,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Samsung opens Solve for Tomorrow 2026 STEM competition to all South African public schools</t>
+          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
+          <t>https://www.samsung.com/za/solvefortomorrow/</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>February 27, 2026 - Samsung Electronics South Africa has opened applications for the 2026 edition of Solve for Tomorrow (SFT), its annual science, technology, engineering, and mathematics (STEM) competition aimed at Grade 10 and 11 learners.</t>
+          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1956,17 +1968,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
+          <t>High School STEM Competition | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/za/solvefortomorrow/</t>
+          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Rooted in the belief that today’s youth hold the key to tomorrow’s progress, Solve for Tomorrow South Africa provides participants with the tools, mentorship, and platforms they need to turn ideas into action.</t>
+          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1974,22 +1986,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>Astemi Sa</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.astemi.co.za/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>What is ASTEMI SA? The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible. We aim to increase participation in the activities of ASTEMI SA. We will encourage our members to lower the barriers of ...</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2012,7 +2028,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas. Each submission can provide a summary of the STEM project. All projects must be presented at the IEOM Cape Town, South Africa 2026.</t>
+          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the 'first author'. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2029,17 +2045,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space ...</t>
+          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Join the South African Space Design Competition to inspire space innovation, develop STEM skills, and compete for a trip to NASA. Perfect for high school students passionate about space.</t>
+          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2047,26 +2063,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>info@zasdc.org, user@domain.com</t>
-        </is>
-      </c>
+      <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ASTEMI SA</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2079,17 +2091,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>StemCo - StemCo 2026 International Competitions</t>
+          <t>Samsung, DBE Announce Top 20 Schools Selected to Advance to the Next ...</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://stemco.org/</t>
+          <t>https://news.samsung.com/za/samsung-dbe-announce-top-20-schools-selected-to-advance-to-the-next-level-of-2026-solve-for-tomorrow-competition</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>June 10, 2026 - BEST YOURSELF WITH STEMCO! Platform for the world’s brightest. ... Thanks to the participating 25 countries in 2019. Singapore, Albania, Australia, Azerbaijan, Canada, Germany, India, Indonesia, Japan, Jordan, Kazakhstan, Kyrgyzstan, Malawi, Mongolia, Nigeria, Myanmar, South Africa, Tajikistan, Turkey, Turkmenistan, Ukraine, The United States, Uzbekistan, Vietnam</t>
+          <t>At an event that took place on 14 April 2026, Samsung in partnership with the Department of Basic Education (DBE) officially announced the Top 20 schools that have been selected to advance to the next stages of the 2026 STEM-based (Science, Technology, Engineering and Mathematics) - Solve For Tomorrow (SFT) competition. In attendance was Mr. Simon Lee, the President and CEO of Samsung Africa ...</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2097,26 +2109,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>name@example.com, bestyourself@stemco.org, havtt@fermat.edu.vn, hkoffice@missmaneducation.com, info@missmaneducation.com, stemcomongolia@gmail.com, awaisnaeem786@gmail.com, example@mail.com, education@missmaneducation.com, info.iksc@kangaroo.org.pk, t.azizakhon@gmail.com</t>
-        </is>
-      </c>
+      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Southafrica 2024</t>
+          <t>NASA space win: SA learners triumph at Kennedy Space Center</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
+          <t>https://furtherafrica.com/2026/08/11/nasa-space-win-sa-learners-triumph-at-kennedy-space-center/</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, ...</t>
+          <t>Seven South African high school learners just won the International Space Settlement Design Competition at NASA's Kennedy Space Center — on their country's first-ever entry. The talent was never missing. The opportunity was. #SouthAfrica #STEM #SpaceTech</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2124,26 +2132,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Competition – Eskom Expo for Young Scientists</t>
+          <t>Applications for 2026 Samsung Solve For Tomorrow Now Open!</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://exposcience.co.za/category/competition/</t>
+          <t>https://news.samsung.com/za/applications-for-2026-samsung-solve-for-tomorrow-now-open</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Aqil Variava business cities Damien ... Gray STEMI Vuyo Nzimande · Eskom Expo for Young Scientists is an exposition, or science fair, where students have a chance to show others their projects about their own scientific investigations. At the annual prestigious Eskom Expo for Young Scientists International Science Fair (ISF), selected students from 35 Expo Regions in South Africa then compete ...</t>
+          <t>The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries open until 06 March 2026. This is a transformative ...</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2151,11 +2155,7 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>support@exposcience.co.za</t>
-        </is>
-      </c>
+      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com</t>
+          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2197,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>April 14, 2026 - This National Event, to be held at the Sandton Convention Centre in Johannesburg, South Africa, as part of AI for Good Impact Africa, at AI Expo Africa 2025, is a qualifying tournament leading to the Grand Finale in Geneva during the AI for ...</t>
+          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge, organized by ITU and The Cortex Hub, in partnership with Google.</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>This is a call for learners and teams from across South Africa who are passionate about robotics, innovation, and making a difference. Whether you’re experienced or just starting, this competition welcomes anyone eager to learn and innovate.</t>
+          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in the leading UN-based global robotics competition, focusing on the critical area of agriculture and food security.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2234,14 +2234,14 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>c183baa23371454f99f417f6616b724d@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, info@thecortexhub.africa, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com</t>
+          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, info@thecortexhub.africa, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa</t>
+          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2251,7 +2251,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Apr 25, 2025 · Experience the excitement as South African teams showcase their skills in a UN-based global robotics competition, focusing on the critical area of disaster response. This National Event is a qualifying tournament leading to the Grand Finale in Geneva during the AI for Good Global Summit 2025.</t>
+          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in a UN-based global robotics competition, focusing on the critical area of disaster response.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2268,7 +2268,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Roboticon 2026: South Africa Showcases Robotics for Culture ...</t>
+          <t>Roboticon 2026: South Africa Showcases Robotics for Culture, Education ...</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2278,7 +2278,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Jul 2, 2026 · South Africa’s robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation. Hosted at the Heartfelt Arena in Pretoria, the event is not only a showcase of technical skills but also a celebration of how robotics can address societal challenges.</t>
+          <t>The event, partnered with the World Robotics Olympiad, positions South Africa as a leader in educational robotics and entrepreneurial innovation." South Africa's robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2288,24 +2288,24 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>newspaper-rec300@2x.jpg, adverts@ubuntutimes.co.za</t>
+          <t>adverts@ubuntutimes.co.za, newspaper-rec300@2x.jpg</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>FIRST South Africa – Robotics Programs for School Children</t>
+          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://firstsa.org/</t>
+          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way. FIRST Tech Challenge students learn to think like engineers. Teams ...</t>
+          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop their creativity and problem-solving skills through challenging and educational robotics competitions.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2318,17 +2318,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
+          <t>FIRST LEGO League Challenge Events - FIRST South Africa</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
+          <t>https://firstsa.org/challenge-events/</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
+          <t>After all teams have finished their Judging sessions and Robot Games, there will be a Closing Ceremony, where all participants will receive medals and the Awards will be handed out. Teams have the opportunity to win awards in various categories, but the FIRST LEGO League Core Values remain the focus. List of Awards Challenge Event/Tournament ...</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2341,17 +2341,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>South African Robotics Competitions and Schools</t>
+          <t>Home | Roboticon 2026</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://www.sciencexpo.org.za/robotics.html</t>
+          <t>https://roboticon.resolute.education/</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
+          <t>Join us for the ultimate robotics showcase as Resolute proudly sponsors the World Robotics Olympiad (WRO) South Africa! This year, we're bringing together two worlds for the biggest robotics event of the year - Roboticon and the WRO Nationals, happening on the same day at the same venue.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2359,26 +2359,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>madelien@imbewu.foundation, marna.vanzyl@imbewu.foundation, webmaster@sciencexpo.org.za</t>
-        </is>
-      </c>
+      <c r="E79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Limpopo Learners Represent South Africa at Global Robotics Finals in Switzerland - African Times</t>
+          <t>Robo Rumble 2026 - University of Limpopo</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://www.atnews.co.za/limpopo-learners-represent-south-africa-at-global-robotics-finals-in-switzerland/</t>
+          <t>https://www.ul.ac.za/robo-rumble-2026/</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>July 7, 2026 - The international competition, taking place from 7 to 10 July 2026 at the Palexpo International Exhibition and Convention Centre in Geneva, brings together some of the world’s brightest young innovators to develop technological solutions to ...</t>
+          <t>The UL Digital Hub proudly presents Robo Rumble 2026, a groundbreaking national STEM and innovation competition delivered in partnership with AlgoAtWork and powered by Engen South Africa. This dynamic initiative invites bright minds from across the country to explore the future of technology, creativity, and problem-solving. Robo Rumble 2026 is built on a structured innovation pipeline ...</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2388,24 +2384,24 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>rampedim@atnews.co.za, NkosiN@atnews.co.za</t>
+          <t>enrolment@ul.ac.za</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - AfrikaBot</t>
+          <t>ROBO-RUMBLE 2026 — Innovation in Motion</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/displaycustomlink.aspx?name=AfrikaBot</t>
+          <t>https://roborumble.net/</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>AfrikaBot is affordable because you can build a competitive robot for a lot less with the correct advice. AfrikaBOT is South Africa's first robotics competition for high school teenagers and university undergraduates who are smart enough to build their own robots from electronic parts rather ...</t>
+          <t>South Africa's premier youth robotics &amp; technology competition. Robo Wars, Drone Racing, Grand Prix &amp; Innovation Challenge. August 2026.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2418,17 +2414,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
+          <t>The South African Institution of Civil Engineering</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini-2022-09-13</t>
+          <t>https://civils.org.za/</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng. Twelve schools participated in the grand finale, which saw great, ...</t>
+          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2436,26 +2432,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>chanel@engineeringnews.co.za, newsletters@creamermedia.co.za, newsdesk@engineeringnews.co.za, subscriptions@creamermedia.co.za, advertising@creamermedia.co.za</t>
-        </is>
-      </c>
+      <c r="E82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Engineering the Future: 16 schools compete in SAICE’s 33rd International Bridge Building Competition - SAICE</t>
+          <t>Civil Expo ITs 2026</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://saice.org.za/press-releases/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
+          <t>https://civilexpoits2026.com/</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>April 17, 2025 - The South African Institution of Civil Engineering (SAICE) hosted its 33rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
+          <t>Hi Cipo Pals! Civil Expo ITs 2026 Sovereign Structures, Resilient Societies This national civil engineering competition is your chance to put your engineering precision to the test and build real-world structural solutions. Step up and prove your skills on a national stage!</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2465,24 +2457,24 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>membership@saice.org.za, civilinfo@saice.org.za, communications@saice.org.za, accounts@saice.org.za, marketing@saice.org.za</t>
+          <t>civilexpo.sipilits@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Upcoming Civil Engineering Conferences in South Africa 2025-2026</t>
+          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://conferencealerts.co.in/south-africa/civil-engineering</t>
+          <t>https://safcec.org.za/</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>International Civil engineering conferences in South africa 2025-2026 with invitation letter. A great opportunity to meet and learn from experts in your field.</t>
+          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2490,22 +2482,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>communication@safcec.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
+          <t>Form-Scaff sponsors SAICE bridge building competition 2026</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://www.crown.co.za/construction-world/marketplace/22289-saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini</t>
+          <t>https://www.facebook.com/formscaffza/posts/building-bridges-testing-ideas-inspiring-future-engineerson-friday-21-august-202/1521870209968920/</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng.</t>
+          <t>2 days ago · SAICE International Bridge Building Competition, supporting an initiative that challenges young minds to put engineering principles, creativity ...</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2513,26 +2509,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>ernao@crown.co.za, constr@crown.co.za</t>
-        </is>
-      </c>
+      <c r="E85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Upcoming Civil Engineering Conferences in South Africa 2025</t>
+          <t>Engineering for People Design Challenge Launches in South ...</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://www.allconferencealert.com/south-africa/civil-engineering-conference.html</t>
+          <t>https://www.linkedin.com/posts/ewbsa_engineering-for-people-design-challenge-launch-activity-7485656340049231872-lSGJ</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>September 7, 2025 - Find the list of upcoming Civil Engineering conferences in South Africa 2025 with invitation an letter.</t>
+          <t>Jul 22, 2026 · We are bringing the Engineering for People Design Challenge to universities across South Africa. engineering students design with communities ... Missing: competition | Show results with: competition</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2545,17 +2537,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>SWM Communications | SAICE recognises civil engineering research excellence through national student competition</t>
+          <t>SAICE Bridge Building Competition 🏗 The South African ...</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://swmcommunications.co.za/press-office/saice-recognises-civil-engineering-research-excellence-through-national-student-competition/</t>
+          <t>https://www.facebook.com/EdenSchoolsDurban/posts/-saice-bridge-building-competition-️the-south-african-institution-of-civil-engin/1569775861605451/</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>April 1, 2026 - The event – which was sponsored by Sika, WorldsView, BVI, RIBCCS, and AF Consulting – was hosted at SAICE House in Midrand, Gauteng, and accredited for 0.2 CPD points. Students were invited to present their civil engineering university research and investigation project, which is part of the national curriculum for final year civil engineering undergraduate students.</t>
+          <t>Their annual Bridge Building Competition introduces high school learners to engineering principles through hands-on construction. This flagship STEM ...</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2563,26 +2555,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>nthabeleng@saice.org.za, info@swmcommunications.co.za</t>
-        </is>
-      </c>
+      <c r="E87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ICE Africa – Supporting Civil Engineers in Africa | Institution of Civil Engineers (ICE)</t>
+          <t>The Bridge-building competition once again saw grade 11 and ...</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://www.ice.org.uk/about-us/what-we-do/ice-near-you/international/ice-africa/</t>
+          <t>https://www.facebook.com/sanralza/posts/the-bridge-building-competition-once-again-saw-grade-11-and-12-learners-particip/881766283981029/</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>March 19, 2026 - organise seminars, workshops, visits and inter-universities competitions regarding civil engineering projects · For more information or to get involved please contact [email protected]. We have a volunteer member in South Africa who helps arrange ICE activities and promote our work.</t>
+          <t>Aug 14, 2024 · The South African Institution of Civil Engineering (SAICE) initiated the bridge building competition to further high school learners' use of ...</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2595,17 +2583,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Civil Engineering Conferences in South Africa 2025/2026/2027 - Conference Index</t>
+          <t>Power Construction Civil Engineering Bursary Programme 2026</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://conferenceindex.org/conferences/civil-engineering/south-africa</t>
+          <t>https://www.edupstairs.org/power-construction-civil-engineering-bursary-programme-2026-2/</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Apr 13 International Conference on Architectural, Civil and Environmental Engineering (ICACEE) - Cape Town, South Africa</t>
+          <t>3 days ago · Power Construction Bursary Programme 2026 for Civil Engineering students from Gouda, Saron, Tulbagh and Porterville. Apply by 01 June 2026.</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2613,22 +2601,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>you@example.com, sifisomhlongo@edupstairs.org</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
+          <t>SAICE AQUALIBRIUM COMPETITION We are incredibly proud ...</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2205</t>
+          <t>https://www.facebook.com/MountviewSecondarySchool/videos/saice-aqualibrium-competitionwe-are-incredibly-proud-of-our-three-learners-andil/970492698885421/</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
+          <t>Mar 26, 2026 · The competition, hosted by the South African Institution of Civil Engineering (SAICE), challenges learners to apply practical engineering skills ...</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2641,17 +2633,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Upcoming Civil engineering Conferences in Cape town 2025</t>
+          <t>Becoming a Chartered Engineer in Africa - LinkedIn</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://conferencealerts.co.in/cape-town/civil-engineering</t>
+          <t>https://www.linkedin.com/posts/lokibenjere_in-many-parts-of-africa-particularly-southern-activity-7379451557467115520-mx4u</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Civil engineering conferences in Cape town 2025 provide an exclusive global platform to meet and engage with experts and aspirants in various fields.</t>
+          <t>Oct 2, 2025 · This global competition means that top South African engineers often receive offers from abroad, creating a "brain drain" effect that further ...</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2664,17 +2656,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>South Africa students defeated the world to win nasa school ...</t>
+          <t>Engineering for People Design Challenge Launches in South ...</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/sanctview/posts/south-africa-students-defeated-the-world-to-win-nasa-school-engineering-competit/1361370549525718/</t>
+          <t>https://www.linkedin.com/posts/ewbsa_engineering-for-people-design-challenge-launch-activity-7485656340049231872-lSGJ</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Aug 11, 2026 · . Welabasha High School learner wins first place in Sasol mechanical technology competition. Thembeka Mathenjwa Sthole ▻ Welabasha High ...</t>
+          <t>Jul 22, 2026 · We are bringing the Engineering for People Design Challenge to universities across South Africa. engineering students design with communities ... Missing: competition | Show results with: competition</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2687,17 +2679,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge</t>
+          <t>South Africa's future artisans, technicians and innovators are ...</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
+          <t>https://www.facebook.com/SasolLTD/posts/south-africas-future-artisans-technicians-and-innovators-are-preparing-to-showca/1392391599661358/</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Engineering for People, our flagship university design challenge, has won Silver in the QS Reimagine Education Awards 2025, recognising its impact in empowering ... Missing: mechanical | Show results with: mechanical</t>
+          <t>6 hours ago · The national competition takes place from 30 September to 2 October 2026, celebrating the talent, determination and innovation of South Africa's ...</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2710,17 +2702,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Team South Africa wins NASA space engineering competition</t>
+          <t>Engineering for People Design Challenge</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/100090360075633/posts/team-south-africa-has-won-a-nasa-space-engineering-competition-the-team-beat-oth/1035040346184625/</t>
+          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Team South Africa has won a NASA space engineering competition. The team beat other countries with their engineering and problem-solving skills. The victory is ...</t>
+          <t>Engineering for People, our flagship university design challenge, has won Silver in the QS Reimagine Education Awards 2025, recognising its impact in empowering ... Missing: mechanical | Show results with: mechanical</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2733,17 +2725,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>What are the names of international level mechanical ... - Quora</t>
+          <t>South Africa students defeated the world to win nasa school ...</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://www.quora.com/What-are-the-names-of-international-level-mechanical-engineering-competitions-for-a-college-student</t>
+          <t>https://www.facebook.com/sanctview/posts/south-africa-students-defeated-the-world-to-win-nasa-school-engineering-competit/1361370549525718/</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Jun 10, 2015 · BAJA conducted by SAE(Society for automotive engineering),a competition for building ATV (terrain vehicle) is considered the biggest event for ... What are the various mechanical engineering competitions in ... What are the competitions for mechanical engineering students? More results from www.quora.com</t>
+          <t>Aug 11, 2026 · Recent posts · Welabasha High School learner wins first place in Sasol mechanical technology competition.</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2756,17 +2748,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CELEBRATING MANUFACTURING AND ENGINEERING ...</t>
+          <t>What are the names of international level mechanical ... - Quora</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/mersetasocial/videos/𝐖𝐀𝐓𝐂𝐇-𝐂𝐄𝐋𝐄𝐁𝐑𝐀𝐓𝐈𝐍𝐆-𝐌𝐀𝐍𝐔𝐅𝐀𝐂𝐓𝐔𝐑𝐈𝐍𝐆-𝐀𝐍𝐃-𝐄𝐍𝐆𝐈𝐍𝐄𝐄𝐑𝐈𝐍𝐆-𝐂𝐇𝐀𝐌𝐏𝐈𝐎𝐍𝐒-𝐀𝐓-𝐖𝐎𝐑𝐋𝐃𝐒𝐊𝐈𝐋𝐋𝐒-𝐒𝐎𝐔𝐓𝐇-𝐀/779762595201549/</t>
+          <t>https://www.quora.com/What-are-the-names-of-international-level-mechanical-engineering-competitions-for-a-college-student</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Mar 12, 2026 · The event highlighted the power of artisan development in creating opportunities for training, employment, and entrepreneurship in South Africa.</t>
+          <t>Jun 10, 2015 · BAJA conducted by SAE(Society for automotive engineering),a competition for building ATV (terrain vehicle) is considered the biggest event for ... What are the various mechanical engineering competitions in ... What are the international competitions for undergraduate ... More results from www.quora.com</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2789,7 +2781,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>International Conference on Mechanical Engineering November 04-05, 2028 in Cape Town, South Africa. Early Bird Registration Deadline October 04, 2028 ...</t>
+          <t>International Conference on Mechanical Engineering November 04-05, 2028 in Cape Town, South Africa. Registration Deadline October 04, 2028 Conference Dates ...</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2802,17 +2794,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Real-world research: Engineering team designs South African ...</t>
+          <t>The AAKRUTI Innovation Competition 2026 invites students to ...</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
+          <t>https://www.facebook.com/MecadSolidWorks/videos/the-aakruti-innovation-competition-2026-invites-students-to-tackle-real-engineer/976560255335388/</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>May 15, 2025 · Cross-disciplinary teams present prototypes at Research Day, Engineers Without Borders' design challenge addressed by nearly 90 students.</t>
+          <t>May 22, 2026 · MECAD Systems - Solidworks South Africa ... Our Mechanical Engineering students are transforming concepts into real-world solutions through ...</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2820,26 +2812,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>dolanm@uwstout.edu, frischj@uwstout.edu</t>
-        </is>
-      </c>
+      <c r="E98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>About Baja - SAE International</t>
+          <t>Build the Future Spotlight: Team Mechanical Bulls</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://www.sae.org/events/student/about/baja</t>
+          <t>https://community.firstinspires.org/build-the-future-spotlight-team-mechanical-bulls</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Baja SAE® consists of competitions that simulate real-world engineering design projects and their related challenges. May 20-23, 2027. Baja SAE South Africa</t>
+          <t>FIRST Robotics Competition team Mechanical Bulls is spreading the impact of STEM around the world.</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2852,17 +2840,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>WorldSkills Results</t>
+          <t>Real-world research: Engineering team designs South African ...</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://results.worldskills.org/results</t>
+          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>WorldSkills Competition 2022 Special Edition South Africa Mechanical Engineering CAD 17. South Africa Plumbing and Heating 23.</t>
+          <t>May 15, 2025 · Cross-disciplinary teams present prototypes at Research Day, Engineers Without Borders' design challenge addressed by nearly 90 students.</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2870,22 +2858,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>dolanm@uwstout.edu, frischj@uwstout.edu</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Johannesburg, S.A. - Next Engineers</t>
+          <t>WorldSkills Results</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>https://www.nextengineers.org/en/locations/johannesburg</t>
+          <t>https://results.worldskills.org/results</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Johannesburg's Engineering Discovery has reached 3 170 Grade 8 learners across the city since launch in 2022. This year, the team is aiming to reach 1 000 more!</t>
+          <t>2024 South Africa Mechatronics. South Africa Mechanical Engineering CAD 21. Aircraft Maintenance 22. South Africa Plumbing and Heating 30. South ...</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2893,26 +2885,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>nextengineers@protec.org.za, NextEngineers@fhi360.org</t>
-        </is>
-      </c>
+      <c r="E101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers</t>
+          <t>Cars4Mars - TryEngineering.org Powered by IEEE</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/</t>
+          <t>https://tryengineering.org/event/cars4mars/</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers (SAIEE) About Us See Member Benefits · Become a SAIEE Member today! SAIEE Membership · Earn CPD credits · About Training Academy · Join a SAIEE Centre near you! Centres · South African Institute of Electrical Engineers (SAIEE) 01 ·</t>
+          <t>Cars4Mars is a robotics competition to design and build a Mars Rover Prototype. Competition starts – 1 May 2026 … hydraulics and electrical systems.</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2920,26 +2908,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>reception@saiee.org.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+      <c r="E102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Zutari Bursary Programme 2027: Fully Funded Engineering ...</t>
+          <t>South Africa's future artisans, technicians and innovators are ...</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://careersandopportunities.com/2026/08/07/bursary/</t>
+          <t>https://www.facebook.com/SasolLTD/posts/south-africas-future-artisans-technicians-and-innovators-are-preparing-to-showca/1392391599661358/</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Aug 7, 2026 · Applications are now open for the Zutari Bursary Programme 2027. Ten fully funded engineering bursaries are available for South African students studying Civil or Electrical Engineering. Apply by 31 August 2026.</t>
+          <t>6 hours ago · The National Competition in electrical engineering starting from today on the 16 until Thursday 18 August 2022 at Ekurhuleni East TVET College ...</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2952,17 +2936,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>List of ALL Engineering Bursaries South Africa 2027</t>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
+          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>How much can I earn within the Engineering field in South Africa? The engineering sector in South Africa offers a wide range of career opportunities across fields such as civil, mechanical, electrical, chemical, mining, and industrial engineering. Salaries vary depending on qualifications, experience, and industry, with entry-level roles typically starting at moderate levels and increasing ...</t>
+          <t>Student Chapter Design Contest (Africa) Serving the electrical energy conversion professional worldwide. Chapter Design Contest (Africa) Deadline: April 30, ...</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2975,17 +2959,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>CMU-Africa students shine at global electronics conference</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.africa.engineering.cmu.edu/news/2026/01/16-ieee-conference.html</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
+          <t>Jan 16, 2026 · SPEC 2025, held in Johannesburg, South Africa, is part of the Power Electronics Society, in the field of electrical engineering.</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2995,24 +2979,24 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>info@ieomsociety.org</t>
+          <t>africa-info@andrew.cmu.edu</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>Electricity challenges a top issue at African engineering ...</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://standardmicrogrid.com/content/electricity-challenges-top-issue-african-engineering-innovation-competition</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
+          <t>Electricity challenges a top issue at African engineering innovation competition. Engineering innovations to boost off-grid power and stop electricity theft ...</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -3025,17 +3009,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>South Africa introduces IoEWR for engineers - LinkedIn</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.linkedin.com/posts/mangosuthu-university-of-technology_mut-ioewr-engineeringexcellence-activity-7316443789068320768-mOs4</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>Apr 11, 2025 · This global competition means that top South African engineers often receive offers from abroad, creating a "brain drain" effect that further ...</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3048,17 +3032,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
+          <t>Engineering for People Design Challenge Grand Finals</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
+          <t>https://www.linkedin.com/posts/ewbsa_engineeringimpact-engineeringeducation-activity-7473789877885722624-QS1Q</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
+          <t>Jun 19, 2026 · View organization page for Engineers Without Borders South Africa ... Software Developer•GDGoC FUTMinna Technical Lead•Electrical and Electronics ...</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3071,17 +3055,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - SAIEE National Student Project Competition</t>
+          <t>2026 IEEE PES/IAS PowerAfrica Conference: HOME PAGE</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/calendar/EventDetails.aspx?eeid=29281</t>
+          <t>https://ieee-powerafrica.org/</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>The SAIEE National Students Project Competition will be held at the North-West University (Potchefstroom Campus) on 21 November 2019</t>
+          <t>Scheduled to take place in Safari Park,Nairobi, Kenya, from 21st –25th September 2026, the conference will convene stakeholders from academia, industry, ...</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3094,17 +3078,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>Real-world research: Engineering team designs South African ...</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>March 12, 2026 - At the Centre for High Performance Computing (CHPC) Conference hosted in Cape Town at the end of last year, four current fourth-year electrical engineering students were crowned national champions in the Student Cluster Competition for 2025.</t>
+          <t>May 15, 2025 · Cross-disciplinary teams present prototypes at Research Day, Engineers Without Borders' design challenge addressed by nearly 90 students.</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3112,22 +3096,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>dolanm@uwstout.edu, frischj@uwstout.edu</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Student Design Competition | IEEE CASS</t>
+          <t>The Gauteng Department of Education - Facebook</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://ieee-cas.org/society-involvement/student-design-competition</t>
+          <t>https://www.facebook.com/gauteng.edu/posts/pretoriatuinesos-inside-the-electrical-technology-and-electronics-workshop-learn/1496498595832609/</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>CASS will reimburse the travel costs for the trip to ISCAS 2026 for the four finalists, one for each region - Regions 1-7 (USA and Canada), Region 8 (Europe, Middle East, Africa), Region 9 (Latin America), and Region 10 (Asia, Australia, Pacific), as well as ISCAS registration.</t>
+          <t>Aug 17, 2026 · The National Competition in electrical engineering starting from today on the 16 until Thursday 18 August 2022 at Ekurhuleni East TVET College ...</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3140,7 +3128,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>The Home of South African Hackathons</t>
+          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3173,7 +3161,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
+          <t>Aug 22, 2025 · Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -3186,17 +3174,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Geekulcha Annual Hackathon 2026 - Registration | Sonke Platform</t>
+          <t>Build the Future with Entelect Hackathons</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>https://sonke.gklink.co/event/gkhack26</t>
+          <t>https://challenge.entelect.co.za/</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>GEEKULCHA ANNUAL HACKATHON 2026 Africa's premier hackathon that drives digital innovation and empowers the next generation of tech leaders.</t>
+          <t>Build the Future with Entelect Hackathons Join South Africa’s premier optimisation-first developer competition platform. Compete, iterate, and outperform the best.</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3209,17 +3197,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Build the Future with Entelect Hackathons</t>
+          <t>Geekulcha Annual Hackathon 2026 - Registration | Sonke Platform</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>https://challenge.entelect.co.za/</t>
+          <t>https://sonke.gklink.co/event/gkhack26</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Build the Future with Entelect Hackathons Join South Africa's premier optimisation-first developer competition platform. Compete, iterate, and outperform the best.</t>
+          <t>GEEKULCHA ANNUAL HACKATHON 2026 Africa's premier hackathon that drives digital innovation and empowers the next generation of tech leaders.</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3232,17 +3220,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Unisa hosts first-ever Hackathon to ignite student learning experience</t>
+          <t>Hackathons - challenge.entelect.co.za</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-hosts-first-ever-Hackathon-to-ignite-student-learning-experience</t>
+          <t>https://challenge.entelect.co.za/hackathons</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Unisa's Information and Communication Technology Portfolio, in collaboration with the College of Science, Engineering and Technology, held the first-ever Unisa Hackathon on 3 and 4 July 2025, marking a major step in the university's journey to embed digital innovation and entrepreneurship into the students learning experience.</t>
+          <t>Aug 21, 2026 · Hackathons Explore competitions, manage your teams, review the leaderboards and submit solutions.</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -3255,17 +3243,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>AI Hackathon | Sebaka</t>
+          <t>ICEP - Tshwane Varsity Hackathon</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>https://sebakasouthafrica.co.za/index.html</t>
+          <t>https://tvh.icep.co.za/</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>AI Hackathon Build an AI Agent for Software Quality Engineering The future of software testing is intelligent, collaborative and AI-powered.</t>
+          <t>Tshwane Varsity Hackathon South Africa's premier inter-university hackathon competition. Join hundreds of students for 53 hours of coding, innovation, and`` fun!</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3273,22 +3261,26 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>MagasengQM@tut.ac.za, info@tvh.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Hackathon Timeline | Sebaka</t>
+          <t>Join us as 55 young innovators showcase the engineering ...</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>https://sebakasouthafrica.co.za/events.html</t>
+          <t>https://www.facebook.com/ortsajhb/posts/join-us-as-55-young-innovators-showcase-the-engineering-coding-and-technology-so/1473351191493113/</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Sebaka Mentorship &amp; Hackathons — Build an AI Agent for Software Quality Engineering.</t>
+          <t>Jun 26, 2026 · Join us as 55 young innovators showcase the engineering, coding, and technology solutions during the Young Engineers Movement (YEM) Hackathon. ...</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3301,17 +3293,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Hackathons - challenge.entelect.co.za</t>
+          <t>Tech hackathons in Africa 2026 / 2027 - dev.events</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>https://challenge.entelect.co.za/hackathons</t>
+          <t>https://dev.events/hackathons/AF/tech</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>University Cup Compete against the best university teams across South Africa Prize Pool: Various cool prizes &amp; bragging rights!</t>
+          <t>Best Tech hackathons in Africa 2026 / 2027 · The Principal Dev – Masterclass for Tech Leads · Clean Architecture Masterclass · Africa Deep Tech Challenge 2026.</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -3324,17 +3316,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Young Engineers Movement (YEM) - ORT SA</t>
+          <t>Faurecia South Africa's Post - LinkedIn</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
+          <t>https://www.linkedin.com/posts/forvia-faurecia-south-africa_calling-all-future-engineers-join-activity-7437386283603279872-NGpQ</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
+          <t>Mar 10, 2026 · cia South Africa's Engineering Hackathon FORVIA South motivated, curious, and driven young engineers. When: 27 March 2026 Where: FORVIA Cape ...</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -3342,26 +3334,22 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
-        </is>
-      </c>
+      <c r="E120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>CompeteHub - Where Champions Are Made</t>
+          <t>55 Learners From Underserved Schools to Shine at Hackathon!</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>https://www.devpluxe.co.za/</t>
+          <t>https://www.goodthingsguy.com/55-learners-underserved-schools-yem-hackathon/</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>About DevPluxe Empowering South Africa ' s next generation of innovators We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
+          <t>Jun 17, 2026 · The event is a multi-day programme hosted by ORT South Africa running from 22 to 26 June 2026 in Johannesburg.</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -3369,7 +3357,11 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr"/>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>198031-featured-75x75@2.5x.jpeg, 198013-featured-75x75@2.5x.jpg, 198031-featured-75x75@3x.jpeg, 197895-featured-75x75@2x.jpg, 198091-featured-75x75@3x.jpg, 198019-featured-75x75@2.5x.jpg, 197895-featured-75x75@1.5x.jpg, 197895-featured-75x75@2.5x.jpg, 198013-featured-75x75@1.5x.jpg, 198019-featured-75x75@1.5x.jpg, 197895-featured-75x75@3x.jpg, 198019-featured-75x75@2x.jpg, 198091-featured-75x75@1.5x.jpg, 198091-featured-75x75@2x.jpg, 198031-featured-75x75@1.5x.jpeg, 198013-featured-75x75@2x.jpg, 198013-featured-75x75@3x.jpg, 198091-featured-75x75@2.5x.jpg, 198019-featured-75x75@3x.jpg, 198031-featured-75x75@2x.jpeg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update competition data 2026-08-29
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -469,17 +469,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
+          <t>Two South Africans on the shortlist for the 2026 Africa Prize for Engineering Innovation</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.engineeringnews.co.za/article/two-south-africans-on-the-shortlist-for-the-2026-africa-prize-for-engineering-innovation-2026-08-04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sep 4, 2025 · 3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>3 weeks ago - Two South African innovators have been shortlisted for the UK Royal Academy of Engineering’s Africa Prize for Engineering Innovation 2026. This is the continent’s richest award aimed at promoting engineering innovation and entrepreneurship ...</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -489,24 +489,24 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+          <t>advertising@creamermedia.co.za, chanel@engineeringnews.co.za, newsdesk@engineeringnews.co.za, subscriptions@creamermedia.co.za, newsletters@creamermedia.co.za</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.poidata.io/report/engineer/south-africa</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -514,26 +514,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>2 weeks ago - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -541,26 +537,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -568,22 +560,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+          <t>Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
+          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -596,17 +592,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.thecasecentre.org/products/view?id=189255</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa. Find out more</t>
+          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -619,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Two South Africans on the shortlist for the 2026 Africa Prize for Engineering Innovation</t>
+          <t>Engineering conferences in South Africa 2026-2027</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/two-south-africans-on-the-shortlist-for-the-2026-africa-prize-for-engineering-innovation-2026-08-04</t>
+          <t>https://conferencenext.com/conferences/south-africa/engineering</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>3 weeks ago - Two South African innovators have been shortlisted for the UK Royal Academy of Engineering’s Africa Prize for Engineering Innovation 2026. This is the continent’s richest award aimed at promoting engineering innovation and entrepreneurship ...</t>
+          <t>Researchers, academicians, students, scholars, investors, and professionals can attend Engineering conferences in South Africa. You just need to select an event, complete the registration process, pay fees, and receive an invitation letter.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -639,24 +635,24 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>chanel@engineeringnews.co.za, newsletters@creamermedia.co.za, advertising@creamermedia.co.za, subscriptions@creamermedia.co.za, newsdesk@engineeringnews.co.za</t>
+          <t>michaeljjacobson1@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.poidata.io/report/engineer/south-africa</t>
+          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
+          <t>South Africa · South Korea · Spain · Sri Lanka · Sudan · Sweden · Switzerland · Syrian Arab Republic · Taiwan · Tajikistan · Tanzania · Thailand · Togo · Trinidad and Tobago · Tunisia · Turkey · Uganda · Ukraine · United Arab Emirates · United Kingdom ·</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -669,17 +665,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
+          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
+          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2 weeks ago - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
+          <t>Engineering design competition is open to teams of engineering students from any university program in West Africa.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -738,17 +734,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Two landmark exhibitions set to transform industrial technology and renewable energy in South Africa</t>
+          <t>KZN Industrial Technology Exhibition</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/two-landmark-exhibitions-set-to-transform-industrial-technology-and-renewable-energy-in-south-africa-2025-10-24</t>
+          <t>https://www.kznindustrial.co.za/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>October 24, 2025 - South Africa’s industrial and clean energy sectors celebrated a landmark moment today with the official launch of RE+ South Africa 2026 and the Cape Industrial Technology Exhibition (CITE) 2027.</t>
+          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -758,24 +754,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>chanel@engineeringnews.co.za, newsletters@creamermedia.co.za, advertising@creamermedia.co.za, subscriptions@creamermedia.co.za, newsdesk@engineeringnews.co.za</t>
+          <t>john@email.com</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>KZN Industrial Technology Exhibition</t>
+          <t>Two landmark exhibitions set to transform industrial technology and renewable energy in South Africa</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://www.kznindustrial.co.za/</t>
+          <t>https://www.engineeringnews.co.za/article/two-landmark-exhibitions-set-to-transform-industrial-technology-and-renewable-energy-in-south-africa-2025-10-24</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
+          <t>October 24, 2025 - South Africa’s industrial and clean energy sectors celebrated a landmark moment today with the official launch of RE+ South Africa 2026 and the Cape Industrial Technology Exhibition (CITE) 2027.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -785,7 +781,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>john@email.com</t>
+          <t>advertising@creamermedia.co.za, chanel@engineeringnews.co.za, newsdesk@engineeringnews.co.za, subscriptions@creamermedia.co.za, newsletters@creamermedia.co.za</t>
         </is>
       </c>
     </row>
@@ -835,7 +831,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, Erika@innovate.durban, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, sithabile@innovate.durban, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com</t>
+          <t>sithabile@innovate.durban, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, Erika@innovate.durban, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -865,17 +861,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>International Science, Innovation &amp; Technology Expo (INSITE)</t>
+          <t>Come and explore our exhibition of innovative discoveries at Science Forum South Africa 2024 | CSIR</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://www.dsti.gov.za/index.php/resource-center/27-temp/dst-links/3-international-science-innovation-a-technology-expo</t>
+          <t>https://www.csir.co.za/come-and-explore-our-exhibition-innovative-discoveries-science-forum-south-africa-2024</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>The essence of INSITE INSITE is an international, biennial must-see Science and Technology event in South Africa, the only one of its kind in Africa that creates new frontiers for global challenges · INSITE aims to assemble the worlds leading innovators and scientists in one place, stimulating ...</t>
+          <t>December 3, 2024 - The exhibition launch will take place on Tuesday, 3 December 2024, with the opening address by Department of Science, Technology and Innovation Minister Dr Blade Nzimande.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -911,17 +907,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Come and explore our exhibition of innovative discoveries at Science Forum South Africa 2024 | CSIR</t>
+          <t>International Science, Innovation &amp; Technology Expo (INSITE)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.csir.co.za/come-and-explore-our-exhibition-innovative-discoveries-science-forum-south-africa-2024</t>
+          <t>https://www.dsti.gov.za/index.php/resource-center/27-temp/dst-links/3-international-science-innovation-a-technology-expo</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>December 3, 2024 - The exhibition launch will take place on Tuesday, 3 December 2024, with the opening address by Department of Science, Technology and Innovation Minister Dr Blade Nzimande.</t>
+          <t>The essence of INSITE INSITE is an international, biennial must-see Science and Technology event in South Africa, the only one of its kind in Africa that creates new frontiers for global challenges · INSITE aims to assemble the worlds leading innovators and scientists in one place, stimulating ...</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -934,17 +930,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>Engineering For People Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community’s challenges and how community members view the impact of these challenges on their daily lives.</t>
+          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -961,17 +957,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
+          <t>In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community's challenges and how community members view the impact of these challenges on their daily lives.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -979,22 +975,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of ...</t>
+          <t>Engineering for People Design Challenge - Engineers Without Borders UK</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Aug 4, 2025 · This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but under-resourced neighbourhood on the eastern edge of Johannesburg. Home to around 46,000 people, Makers Valley is a community rich in creativity, activism ...</t>
+          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1002,26 +1002,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
-        </is>
-      </c>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Engineering For People Design Challenge - EWBSA</t>
+          <t>Engineering for People Design Challenge returns to Johannesburg!</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
+          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
+          <t>Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1029,26 +1025,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
-        </is>
-      </c>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge - Engineers Without ...</t>
+          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
+          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
+          <t>The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1056,22 +1048,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>team@crowdsolve.net</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Oct 24, 2024 · The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
+          <t>STEM-focused NGO Engineers Without Borders UK has launched its 2025 Engineering for People Design Challenge. Organised in conjunction with sister organisation Engineers Without Borders South Africa, as well as the Makers Valley Partnership, this year's challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1079,26 +1075,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>team@crowdsolve.net</t>
-        </is>
-      </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>EWB Design Challenge | Aston University</t>
+          <t>Engineering for People Design Challenge | Department of Engineering</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
+          <t>This year's design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but under-resourced neighbourhood on the eastern edge of Johannesburg. Home to around 46,000 people, Makers Valley is a community rich in creativity, activism ...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1106,22 +1098,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>web-editor@eng.cam.ac.uk, marketing@eng.cam.ac.uk</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
+          <t>Bambasonke Design Challenge Empowers Engineering Students in SA - LinkedIn</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
+          <t>https://www.linkedin.com/posts/activity-7470764395091001345-GwCR</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
+          <t>By joining forces, student engineers have the chance to bridge societal gaps, uplift those in vulnerable positions, and contribute to building a more inclusive and prosperous South Africa.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1129,26 +1125,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>ied@ied.org.uk</t>
-        </is>
-      </c>
+      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South ...</t>
+          <t>Engineers Without Borders | OU Design Show 2025</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
+          <t>https://www.oudesignshow.org/designathon</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
+          <t>Makers Valley is a vibrant community of makers, creatives, and social enterprises in Johannesburg, South Africa. Engineers Without Borders UK has partnered with Makers Valley to engage students in design challenges focused on addressing local challenges and promoting sustainable development.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1161,17 +1153,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Latest Community Engineering Design Competition Announced</t>
+          <t>EWB-SA: Mid-Year Update - LinkedIn</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
+          <t>https://www.linkedin.com/pulse/ewb-sa-mid-year-update-ewbsa-uxo9f</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
+          <t>We wrapped up an extraordinary cycle of the 2023/24 Engineering for People Design Challenge in December 2024, with students across South Africa applying their creativity and empathy to solve real ...</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1194,7 +1186,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1221,7 +1213,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1258,14 +1250,14 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, email@example.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com</t>
+          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, email@example.com, 8c4075d5481d476e945486754f783364@sentry.io, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1275,7 +1267,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
+          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1288,17 +1280,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Competitions – Enactus South Africa | National Expos ...</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://enactusza.org/what-we-do/competitions</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Explore our national and international competitions that empower students to tackle challenges with entrepreneurial solutions and social impact at the core.</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1308,24 +1300,24 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>adminsa@enactus.org, xmadlanga@enactus.org, marketingsa@enactus.org, liso@enactus.org</t>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
+          <t>Competitions - Enactus South Africa | National Expos, Challenges ...</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://enactusza.org/what-we-do/competitions</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Sep 4, 2025 · 3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>Explore our national and international competitions that empower students to tackle challenges with entrepreneurial solutions and social impact at the core.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1335,24 +1327,24 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+          <t>marketingsa@enactus.org, adminsa@enactus.org, liso@enactus.org, xmadlanga@enactus.org</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Engineering Competition For African Youth In Engineering ...</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Aug 18, 2025 · The Africa Prize is open to individuals or teams based in sub-Saharan Africa with a scalable engineering innovation that demonstrates social or environmental impact potential.</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1365,17 +1357,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge</t>
+          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
+          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Engineering for People, our flagship university design challenge, has won Silver in the QS Reimagine Education Awards 2025, recognising its impact in empowering ...</t>
+          <t>Eligibility Benchmark Requirements The Africa Prize is open to individuals or teams based in sub-Saharan Africa with a scalable engineering innovation that demonstrates social or environmental impact potential. Applicants must: Be citizens ordinarily residing in a sub-Saharan African country. Be over 18 years old and fluent in English.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1388,17 +1380,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Inspiring, building and shaping a future fit engineering community</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.ewb-international.org/home/inspiring-building-and-shaping-a-future-fit-engineering-community/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, the Design Challenge has been delivered in ... Missing: competition | Show results with: competition</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1406,26 +1398,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>admin@ewb-international.org</t>
-        </is>
-      </c>
+      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>International science and technology competition 2026</t>
+          <t>2027 Africa Prize for Engineering Innovation Opens Applications</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/443764394251719/posts/1259344422693708/</t>
+          <t>https://www.globalsouthopportunities.com/2026/08/09/africa-134/</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Dec 20, 2025 · ... Engineering Technologies (ICISCET 2026) to be held from 14 - 16 October 2026 in Vanderbijlpark, South Africa. Submission Deadline:15 June ...</t>
+          <t>The Royal Academy of Engineering has opened applications for the 2027 Africa Prize for Engineering Innovation, providing African innovators with an opportunity to develop, strengthen and commercialise engineering solutions addressing important challenges across the continent.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1438,17 +1426,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Africa Tech Festival</t>
+          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://techspojoburg.co.za/</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
+          <t>1 month ago - TECHSPO Johannesburg 2026 is a two day technology expo taking place September 28th to 29th, 2026 at the luxurious Hyatt Regency Johannesburg, Johannesburg, South Africa. TECHSPO Johannesburg brings together developers, brands, marketers, technology ...</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1458,14 +1446,14 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>salesenquiries@africatechfestival.com, dataprivacy@informaconnect.com, support@informaconnect.com, support@knect365.com, customerservices@informaconnect.com, customerservices@knect365.com, dataprivacy@knect365.com</t>
+          <t>info@techspojoburg.co.za</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>IT &amp; Technology Events in South Africa, List of all South Africa Technology Business Expo &amp; Events</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1475,7 +1463,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Aug 17, 2026 · Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>New York Small Business Expo (Spring)07 MayNew York , USA · AFROZUM Fair · 07-09 May · Johannesburg , South Africa · AFROZUM Fair07-09 MayJohannesburg , South Africa · Nigeria Industries &amp; Manufacturing Summit · 18-20 May · Abuja , Nigeria ...</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1488,17 +1476,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 ...</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://techspojoburg.co.za/</t>
+          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
+          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1506,22 +1494,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>atinfo@techspo.coor, u003einfo@techspo.co</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
+          <t>Home - Mediatech Africa | South Africa</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://10times.com/johannesburg-za/technology</t>
+          <t>https://www.mediatech.co.za/</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>19 hours ago · Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1529,22 +1521,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>simon@mediatech.co.za, claire@mediatech.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7 ...</t>
+          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://africatechnologyexpo.com/</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Where Business, Tech and Innovation Collide in Cape Town! TECHSPO Cape Town is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
+          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1554,24 +1550,24 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>info@techspocapetown.co.za</t>
+          <t>info@sparkafrica.co, johndoe@email.com, partner@africatechnologyexpo.com</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology ExpoJohannesburg Technology ...</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://techspojoburg.co.za/johannesburg-technology-expo/</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg is a 2-day technology expo taking place September 28 – 29, 2026 at the luxurious NH Johannesburg Sandton Hotel, Toronto, Ontario. TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
+          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1579,22 +1575,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>info@techspocapetown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 – Africa's biggest IT Conference and Expo</t>
+          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what’s next before everyone else does. Only 2,500 ...</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1602,22 +1602,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>salesenquiries@africatechfestival.com, support@informaconnect.com, support@knect365.com, dataprivacy@knect365.com, customerservices@informaconnect.com, customerservices@knect365.com, dataprivacy@informaconnect.com</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>TECHSPO Technology Expo</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference - AI Expo Africa | 28 - 29 October SCC Johannesburg South Africa</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://techspo.co/</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>TECHSPO is a Technology Expo Series with annual events in 50 international cities, across 20 countries. South Africa October 1 – 2, 2026 Cape Town, South ...</t>
+          <t>(2 Day Event) 28th-29th October 2026 Sandton Convention Centre, JHB, South Africa · AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade ...</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1625,22 +1629,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>enquiries@aiexpoafrica.com</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~…</t>
+          <t>Discover Tech Conferences Events &amp; Activities in South Africa | Eventbrite</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://www.industryevents.com/events/techspo-johannesburg-2026-technology-expo-internet-mobile-adtech-martech-saas</t>
+          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology Expo returns September 28-29, 2026 to the NH Johannesburg Sandton Hotel in Johannesburg, South Africa.</t>
+          <t>Save this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South AfricaShare this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1648,26 +1656,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>your@email.com, events@techspojoburg.co.za, support@industryevents.com, you@company.com, colleague@company.com</t>
-        </is>
-      </c>
+      <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Tech conferences in South Africa 2026 / 2027 - dev.events</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://dev.events/AF/ZA/tech</t>
+          <t>https://www.industryevents.com/events/techspo-johannesburg-2026-technology-expo-internet-mobile-adtech-martech-saas</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Best Tech conferences in South Africa 2026 / 2027 · The Principal Dev – Masterclass for Tech Leads · Clean Architecture Masterclass · Escape 2026 · HR World Summit ...</t>
+          <t>TECHSPO Johannesburg – Where Business, Tech and Innovation Collide in Johannesburg, South Africa. TECHSPO Johannesburg Technology Expo returns September 28-29, 2026 to the NH Johannesburg Sandton Hotel in Johannesburg, South Africa.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1675,7 +1679,11 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>you@company.com, your@email.com, colleague@company.com, events@techspojoburg.co.za, support@industryevents.com</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1749,17 +1757,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
+          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>http://capetown.makerfaire.com/</t>
+          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
+          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1767,26 +1775,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>fancybox_sprite@2x.png, fancybox_loading@2x.gif, chosen-sprite@2x.png, pr@make.co</t>
-        </is>
-      </c>
+      <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
+          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
+          <t>http://capetown.makerfaire.com/</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
+          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1794,22 +1798,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>fancybox_loading@2x.gif, fancybox_sprite@2x.png, pr@make.co, chosen-sprite@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
+          <t>Blog : Maker Faire Africa</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://contemporaryand.com/en/events/maker-faire-africa-comes-to-johannesburg</t>
+          <t>http://makerfaireafrica.com/blog/</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
+          <t>December 31, 2021 - You can help them out on the new South African crowdfunding site, ThundaFund. ... One of the most ambitions items at Maker Faire Africa this year in Johannesburg, South Africa is Samuel Ngobeni’s “art car”. He’s a designer from Germinston, who has spent the last three years building his ANIMAL car, from the ground up, that means the frame and all.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1822,17 +1830,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Jo’Burg – AfriGadget</t>
+          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://www.afrigadget.com/2014/07/08/maker-faire-africa-comes-to-joburg/</t>
+          <t>https://contemporaryand.com/en/events/maker-faire-africa-comes-to-johannesburg</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Maker Faire Africa 2014 will bring together over 5,000 attendees, along with featured inventors, world-class makers, self-made entrepreneurs &amp; workshop experts from South Africa, across the continent, and around the world, to manufacture real solutions for some of Africa’s most pressing ...</t>
+          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1845,17 +1853,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>HOME | MAKERS FEST</t>
+          <t>The Makers Hub</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://www.makersfestival.co.za/</t>
+          <t>https://www.decorex.co.za/cape-town/en-gb/visit/TheMakersHub.html</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>At Makers Festival SA, you get full access to every hands-on workshop, from woodworking and ceramics to leatherwork, painting, and more.</t>
+          <t>Explore unique handmade items, take part in interactive workshops, and engage directly with Cape Town’s vibrant maker community.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1865,24 +1873,24 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>warren@makersfestival.co.za, 8c4075d5481d476e945486754f783364@sentry.io, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, example@mysite.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com</t>
+          <t>decorexafrica@rxglobal.com</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Makers Festival SA 🛠️ (@makersfestival_sa) • Instagram photos ...</t>
+          <t>Maker Faire Africa comes to Jo’Burg – AfriGadget</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/makersfestival_sa/</t>
+          <t>https://www.afrigadget.com/2014/07/08/maker-faire-africa-comes-to-joburg/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>8,503 Followers, 58 Following, 57 Posts - Makers Festival SA 🛠️ (@makersfestival_sa) on Instagram: "🛠️ Building Skills. Building Memories. 🏕️ 8th &amp; 9th November 2025 / Cape Town, SA 🪵 Founder @hutch_custom 📩 DM us - apply to be a MAKER 🫶🏼"</t>
+          <t>Maker Faire Africa 2014 will bring together over 5,000 attendees, along with featured inventors, world-class makers, self-made entrepreneurs &amp; workshop experts from South Africa, across the continent, and around the world, to manufacture real solutions for some of Africa’s most pressing ...</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1895,17 +1903,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>The Makers Hub</t>
+          <t>Makers Festival SA 🛠️ (@makersfestival_sa) • Instagram photos ...</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://www.decorex.co.za/cape-town/en-gb/visit/TheMakersHub.html</t>
+          <t>https://www.instagram.com/makersfestival_sa/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Explore unique handmade items, take part in interactive workshops, and engage directly with Cape Town’s vibrant maker community.</t>
+          <t>8,503 Followers, 58 Following, 57 Posts - Makers Festival SA 🛠️ (@makersfestival_sa) on Instagram: "🛠️ Building Skills. Building Memories. 🏕️ 8th &amp; 9th November 2025 / Cape Town, SA 🪵 Founder @hutch_custom 📩 DM us - apply to be a MAKER 🫶🏼"</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1913,11 +1921,7 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>decorexafrica@rxglobal.com</t>
-        </is>
-      </c>
+      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1945,17 +1949,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/za/solvefortomorrow/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1968,17 +1972,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Southafrica 2024 - IEOM Society</t>
+          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
+          <t>https://www.samsung.com/za/solvefortomorrow/</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas.</t>
+          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1986,26 +1990,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Astemi Sa</t>
+          <t>High School STEM Competition | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/</t>
+          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>What is ASTEMI SA? The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible. We aim to increase participation in the activities of ASTEMI SA. We will encourage our members to lower the barriers of ...</t>
+          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2013,22 +2013,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Capetown 2026</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the 'first author'. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
+          <t>The IEOM High School/Middle School STEM Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2045,17 +2049,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
+          <t>Astemi Sa</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
+          <t>https://www.astemi.co.za/</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
+          <t>What is ASTEMI SA? The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible. We aim to increase participation in the activities of ASTEMI SA. We will encourage our members to lower the barriers of ...</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2068,17 +2072,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2114,17 +2118,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>NASA space win: SA learners triumph at Kennedy Space Center</t>
+          <t>Register your school for Samsung Solve for Tomorrow 2026</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://furtherafrica.com/2026/08/11/nasa-space-win-sa-learners-triumph-at-kennedy-space-center/</t>
+          <t>https://www.sowetan.co.za/careers/2026-03-03-register-your-school-for-samsung-solve-for-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Seven South African high school learners just won the International Space Settlement Design Competition at NASA's Kennedy Space Center — on their country's first-ever entry. The talent was never missing. The opportunity was. #SouthAfrica #STEM #SpaceTech</t>
+          <t>Register your school for Samsung Solve for Tomorrow 2026 STEM competition aims to transform and empower South African learners with critical skills to solve real-world challenges March 03, 2026 at 7:44 am</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2132,7 +2136,11 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ssasft@samsung.com</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2180,7 +2188,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com</t>
+          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -2214,17 +2222,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
+          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa/</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in the leading UN-based global robotics competition, focusing on the critical area of agriculture and food security.</t>
+          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in a UN-based global robotics competition, focusing on the critical area of disaster response.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2234,24 +2242,24 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, info@thecortexhub.africa, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com</t>
+          <t>name@example.com</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
+          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa/</t>
+          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in a UN-based global robotics competition, focusing on the critical area of disaster response.</t>
+          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in the leading UN-based global robotics competition, focusing on the critical area of agriculture and food security.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2261,7 +2269,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>name@example.com</t>
+          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, info@thecortexhub.africa, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -2295,17 +2303,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
+          <t>Live Competitions — Nirvana Global Foundation</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
+          <t>https://nirvanaglobalfoundation.org/competition.html</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop their creativity and problem-solving skills through challenging and educational robotics competitions.</t>
+          <t>Enjoy AI South Africa An international AI and robotics competition for young innovators. Teams build, program and compete with official ENJOY AI robotics kits across categories like Battle of Stars, Mining Expedition, Drone Cup and Inventions Trail — preparing learners for the global ENJOY AI stage.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2313,22 +2321,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>you@email.com, coach@school.co.za, info@nirvanaglobalfoundation.org</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>FIRST LEGO League Challenge Events - FIRST South Africa</t>
+          <t>FIRST South Africa - Robotics Programs for School Children</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://firstsa.org/challenge-events/</t>
+          <t>https://firstsa.org/</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>After all teams have finished their Judging sessions and Robot Games, there will be a Closing Ceremony, where all participants will receive medals and the Awards will be handed out. Teams have the opportunity to win awards in various categories, but the FIRST LEGO League Core Values remain the focus. List of Awards Challenge Event/Tournament ...</t>
+          <t>FIRST® LEGO ® League FIRST® LEGO ® League guides youth through STEM learning and exploration at an early age. From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2341,17 +2353,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Home | Roboticon 2026</t>
+          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://roboticon.resolute.education/</t>
+          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Join us for the ultimate robotics showcase as Resolute proudly sponsors the World Robotics Olympiad (WRO) South Africa! This year, we're bringing together two worlds for the biggest robotics event of the year - Roboticon and the WRO Nationals, happening on the same day at the same venue.</t>
+          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop their creativity and problem-solving skills through challenging and educational robotics competitions.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2364,17 +2376,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Robo Rumble 2026 - University of Limpopo</t>
+          <t>Home | Roboticon 2026</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://www.ul.ac.za/robo-rumble-2026/</t>
+          <t>https://roboticon.resolute.education/</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>The UL Digital Hub proudly presents Robo Rumble 2026, a groundbreaking national STEM and innovation competition delivered in partnership with AlgoAtWork and powered by Engen South Africa. This dynamic initiative invites bright minds from across the country to explore the future of technology, creativity, and problem-solving. Robo Rumble 2026 is built on a structured innovation pipeline ...</t>
+          <t>Join us for the ultimate robotics showcase as Resolute proudly sponsors the World Robotics Olympiad (WRO) South Africa! This year, we're bringing together two worlds for the biggest robotics event of the year - Roboticon and the WRO Nationals, happening on the same day at the same venue.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2382,11 +2394,7 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>enrolment@ul.ac.za</t>
-        </is>
-      </c>
+      <c r="E80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2414,17 +2422,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering</t>
+          <t>RoadEng Civil Engineer - Alternative to Complicated CAD</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://civils.org.za/</t>
+          <t>https://www.bing.com/aclick?ld=e8xUZ4ioxsW5QmsutJAwQ9GTVUCUxFpLo4nwUHEtN1raTBZn6dckIigpjwYbmX9hQf4xNfnHsLDyDxzld8sBYgRNK9Pilt8IYkO6HHBk28jli7yFEuvrwP3rY43Za_uAgqkKFfrdc9WJVhMy7Nh0MfAv8Gil3bPyWDEUyMGT5KwOnSRCeH5neCFgOK-cMHXFYzH75Dj0k0ktut69vlpYvbInMv-ys&amp;u=aHR0cHMlM2ElMmYlMmZ3d3cuc29mdHJlZS5jb20lMmZwcm9kdWN0cyUyZmNvcnJpZG9yLWRlc2lnbiUyZnJvYWRlbmclM2Ztc2Nsa2lkJTNkMzYyMTQ2YmQ4YjFkMThiMmE5MzQyYzJmNTEwZDYxNmQ&amp;rlid=362146bd8b1d18b2a9342c2f510d616d</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
+          <t>Built for road engineering, fast &amp; interactive even with large LiDAR, DEM, &amp; drone data. RoadEng is a user-friendly civil design software, specialized in rural infrastructure.</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2432,22 +2440,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>support@softree.com</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Civil Expo ITs 2026</t>
+          <t>The South African Institution of Civil Engineering</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://civilexpoits2026.com/</t>
+          <t>https://civils.org.za/</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Hi Cipo Pals! Civil Expo ITs 2026 Sovereign Structures, Resilient Societies This national civil engineering competition is your chance to put your engineering precision to the test and build real-world structural solutions. Step up and prove your skills on a national stage!</t>
+          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2455,26 +2467,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>civilexpo.sipilits@gmail.com</t>
-        </is>
-      </c>
+      <c r="E83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://safcec.org.za/</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
+          <t>Sep 4, 2025 · The Africa Prize for Engineering Innovation is the continent’s largest award dedicated to fostering engineering innovation. Its mission is to stimulate, celebrate, and reward ingenuity and entrepreneurship across sub-Saharan Africa.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2484,24 +2492,24 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>communication@safcec.org.za</t>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Form-Scaff sponsors SAICE bridge building competition 2026</t>
+          <t>Civil Expo ITs 2026</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/formscaffza/posts/building-bridges-testing-ideas-inspiring-future-engineerson-friday-21-august-202/1521870209968920/</t>
+          <t>https://civilexpoits2026.com/</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2 days ago · SAICE International Bridge Building Competition, supporting an initiative that challenges young minds to put engineering principles, creativity ...</t>
+          <t>Hi Cipo Pals! Civil Expo ITs 2026 Sovereign Structures, Resilient Societies This national civil engineering competition is your chance to put your engineering precision to the test and build real-world structural solutions. Step up and prove your skills on a national stage!</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2509,22 +2517,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>civilexpo.sipilits@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge Launches in South ...</t>
+          <t>ICE Africa – Supporting Civil Engineers in Africa</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/posts/ewbsa_engineering-for-people-design-challenge-launch-activity-7485656340049231872-lSGJ</t>
+          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Jul 22, 2026 · We are bringing the Engineering for People Design Challenge to universities across South Africa. engineering students design with communities ... Missing: competition | Show results with: competition</t>
+          <t>Click your country to find local events, competitions, and information on how you can get more involved. At the heart of everything we do in South Africa is ICE-SA, the volunteer ICE local association (formerly known as the Joint Civils Division).</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2537,17 +2549,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>SAICE Bridge Building Competition 🏗 The South African ...</t>
+          <t>Engineering for People Design Challenge Launches in South ...</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/EdenSchoolsDurban/posts/-saice-bridge-building-competition-️the-south-african-institution-of-civil-engin/1569775861605451/</t>
+          <t>https://www.linkedin.com/posts/ewbsa_engineering-for-people-design-challenge-launch-activity-7485656340049231872-lSGJ</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Their annual Bridge Building Competition introduces high school learners to engineering principles through hands-on construction. This flagship STEM ...</t>
+          <t>Jul 22, 2026 · We are bringing the Engineering for People Design Challenge to universities across South Africa. engineering students design with communities ... Missing: competition | Show results with: competition</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2560,17 +2572,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>The Bridge-building competition once again saw grade 11 and ...</t>
+          <t>Civil Engineering Needs To Fill Thousands of Jobs. This ...</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/sanralza/posts/the-bridge-building-competition-once-again-saw-grade-11-and-12-learners-particip/881766283981029/</t>
+          <t>https://www.bentley.com/en/blog/civil-engineering-needs-to-fill-thousands-of-jobs-this-contest-starts-with-introducing-middle-and-high-schoolers-to-the-field/</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Aug 14, 2024 · The South African Institution of Civil Engineering (SAICE) initiated the bridge building competition to further high school learners' use of ...</t>
+          <t>Jul 8, 2026 · The AASHTO Bridge Challenge contest compresses a full engineering job into one project. Bentley supplies sponsorship, free software, and judges.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2583,17 +2595,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Power Construction Civil Engineering Bursary Programme 2026</t>
+          <t>The South African Institution of Civil Engineering (SAICE ...</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://www.edupstairs.org/power-construction-civil-engineering-bursary-programme-2026-2/</t>
+          <t>https://www.facebook.com/100069805516530/posts/the-south-african-institution-of-civil-engineering-saice-hosted-the-2026-aqualib/1241182688218570/</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>3 days ago · Power Construction Bursary Programme 2026 for Civil Engineering students from Gouda, Saron, Tulbagh and Porterville. Apply by 01 June 2026.</t>
+          <t>Mar 20, 2026 · This global competition brings together students and young professionals from across the globe to develop innovative solutions to real-life ...</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2601,26 +2613,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>you@example.com, sifisomhlongo@edupstairs.org</t>
-        </is>
-      </c>
+      <c r="E89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>SAICE AQUALIBRIUM COMPETITION We are incredibly proud ...</t>
+          <t>The Bridge-building competition once again saw grade 11 and ...</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/MountviewSecondarySchool/videos/saice-aqualibrium-competitionwe-are-incredibly-proud-of-our-three-learners-andil/970492698885421/</t>
+          <t>https://www.facebook.com/sanralza/posts/the-bridge-building-competition-once-again-saw-grade-11-and-12-learners-particip/881766283981029/</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Mar 26, 2026 · The competition, hosted by the South African Institution of Civil Engineering (SAICE), challenges learners to apply practical engineering skills ...</t>
+          <t>Aug 14, 2024 · The South African Institution of Civil Engineering (SAICE) initiated the bridge building competition to further high school learners' use of ...</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2633,17 +2641,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Becoming a Chartered Engineer in Africa - LinkedIn</t>
+          <t>Bridges for bridging the skills gap in civil engineering. | EBSCOhost</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/posts/lokibenjere_in-many-parts-of-africa-particularly-southern-activity-7379451557467115520-mx4u</t>
+          <t>https://openurl.ebsco.com/contentitem/gcd:99622195</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Oct 2, 2025 · This global competition means that top South African engineers often receive offers from abroad, creating a "brain drain" effect that further ...</t>
+          <t>Abstract. The article offers information on the annual AECOM-SAICE International Bridge Building Competition, organised by SAICE, held in August 2014 at the ...</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2666,7 +2674,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Jul 22, 2026 · We are bringing the Engineering for People Design Challenge to universities across South Africa. engineering students design with communities ... Missing: competition | Show results with: competition</t>
+          <t>Jul 22, 2026 · We are bringing the Engineering for People Design Challenge to universities across South Africa. engineering students design with communities ...</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2689,7 +2697,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>6 hours ago · The national competition takes place from 30 September to 2 October 2026, celebrating the talent, determination and innovation of South Africa's ...</t>
+          <t>24 hours ago · The national competition takes place from 30 September to 2 October 2026, celebrating the talent, determination and innovation of South Africa's ...</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2725,17 +2733,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>South Africa students defeated the world to win nasa school ...</t>
+          <t>What are the names of international level mechanical ... - Quora</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/sanctview/posts/south-africa-students-defeated-the-world-to-win-nasa-school-engineering-competit/1361370549525718/</t>
+          <t>https://www.quora.com/What-are-the-names-of-international-level-mechanical-engineering-competitions-for-a-college-student</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Aug 11, 2026 · Recent posts · Welabasha High School learner wins first place in Sasol mechanical technology competition.</t>
+          <t>Jun 10, 2015 · BAJA conducted by SAE(Society for automotive engineering),a competition for building ATV (terrain vehicle) is considered the biggest event for ...</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2748,17 +2756,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>What are the names of international level mechanical ... - Quora</t>
+          <t>South Africa students defeated the world to win nasa school ...</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://www.quora.com/What-are-the-names-of-international-level-mechanical-engineering-competitions-for-a-college-student</t>
+          <t>https://www.facebook.com/sanctview/posts/south-africa-students-defeated-the-world-to-win-nasa-school-engineering-competit/1361370549525718/</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Jun 10, 2015 · BAJA conducted by SAE(Society for automotive engineering),a competition for building ATV (terrain vehicle) is considered the biggest event for ... What are the various mechanical engineering competitions in ... What are the international competitions for undergraduate ... More results from www.quora.com</t>
+          <t>Aug 11, 2026 · Recent posts · Welabasha High School learner wins first place in Sasol mechanical technology competition.</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2781,7 +2789,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>International Conference on Mechanical Engineering November 04-05, 2028 in Cape Town, South Africa. Registration Deadline October 04, 2028 Conference Dates ...</t>
+          <t>ICME 2028: 22. International Conference on Mechanical Engineering. November 04-05, 2028 in Cape Town, South Africa. HYBRID. Cape Town.</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2794,17 +2802,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>The AAKRUTI Innovation Competition 2026 invites students to ...</t>
+          <t>Real-world research: Engineering team designs South African ...</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/MecadSolidWorks/videos/the-aakruti-innovation-competition-2026-invites-students-to-tackle-real-engineer/976560255335388/</t>
+          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>May 22, 2026 · MECAD Systems - Solidworks South Africa ... Our Mechanical Engineering students are transforming concepts into real-world solutions through ...</t>
+          <t>May 15, 2025 · Cross-disciplinary teams present prototypes at Research Day, Engineers Without Borders' design challenge addressed by nearly 90 students.</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2812,22 +2820,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>frischj@uwstout.edu, dolanm@uwstout.edu</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Build the Future Spotlight: Team Mechanical Bulls</t>
+          <t>About Baja - SAE International</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://community.firstinspires.org/build-the-future-spotlight-team-mechanical-bulls</t>
+          <t>https://www.sae.org/events/student/about/baja</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>FIRST Robotics Competition team Mechanical Bulls is spreading the impact of STEM around the world.</t>
+          <t>Baja SAE® consists of competitions that simulate real-world engineering design projects and their related challenges. May 20-23, 2027. Baja SAE South Africa</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2840,17 +2852,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Real-world research: Engineering team designs South African ...</t>
+          <t>WorldSkills Results</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
+          <t>https://results.worldskills.org/results</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>May 15, 2025 · Cross-disciplinary teams present prototypes at Research Day, Engineers Without Borders' design challenge addressed by nearly 90 students.</t>
+          <t>2024 South Africa Mechatronics. South Africa Mechanical Engineering CAD 21. Aircraft Maintenance 22. South Africa Plumbing and Heating 30. South ...</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2858,26 +2870,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>dolanm@uwstout.edu, frischj@uwstout.edu</t>
-        </is>
-      </c>
+      <c r="E100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>WorldSkills Results</t>
+          <t>Johannesburg, S.A. - Next Engineers</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>https://results.worldskills.org/results</t>
+          <t>https://www.nextengineers.org/en/locations/johannesburg</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2024 South Africa Mechatronics. South Africa Mechanical Engineering CAD 21. Aircraft Maintenance 22. South Africa Plumbing and Heating 30. South ...</t>
+          <t>Johannesburg's Engineering Discovery has reached 3 170 Grade 8 learners across the city since launch in 2022. This year, the team is aiming to reach 1 000 more!</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2885,22 +2893,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>NextEngineers@fhi360.org, nextengineers@protec.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Cars4Mars - TryEngineering.org Powered by IEEE</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://tryengineering.org/event/cars4mars/</t>
+          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Cars4Mars is a robotics competition to design and build a Mars Rover Prototype. Competition starts – 1 May 2026 … hydraulics and electrical systems.</t>
+          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2913,17 +2925,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>South Africa's future artisans, technicians and innovators are ...</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - SAIEE National Student Project Competition</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/SasolLTD/posts/south-africas-future-artisans-technicians-and-innovators-are-preparing-to-showca/1392391599661358/</t>
+          <t>https://www.saiee.org.za/calendar/EventDetails.aspx?eeid=29281</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>6 hours ago · The National Competition in electrical engineering starting from today on the 16 until Thursday 18 August 2022 at Ekurhuleni East TVET College ...</t>
+          <t>The SAIEE National Students Project Competition will be held at the North-West University (Potchefstroom Campus) on 21 November 2019</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2936,17 +2948,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
+          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
+          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Student Chapter Design Contest (Africa) Serving the electrical energy conversion professional worldwide. Chapter Design Contest (Africa) Deadline: April 30, ...</t>
+          <t>March 12, 2026 - At the Centre for High Performance Computing (CHPC) Conference hosted in Cape Town at the end of last year, four current fourth-year electrical engineering students were crowned national champions in the Student Cluster Competition for 2025.</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2959,17 +2971,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>CMU-Africa students shine at global electronics conference</t>
+          <t>Student Design Competition | IEEE CASS</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://www.africa.engineering.cmu.edu/news/2026/01/16-ieee-conference.html</t>
+          <t>https://ieee-cas.org/society-involvement/student-design-competition</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Jan 16, 2026 · SPEC 2025, held in Johannesburg, South Africa, is part of the Power Electronics Society, in the field of electrical engineering.</t>
+          <t>CASS will reimburse the travel costs for the trip to ISCAS 2026 for the four finalists, one for each region - Regions 1-7 (USA and Canada), Region 8 (Europe, Middle East, Africa), Region 9 (Latin America), and Region 10 (Asia, Australia, Pacific), as well as ISCAS registration.</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2977,26 +2989,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>africa-info@andrew.cmu.edu</t>
-        </is>
-      </c>
+      <c r="E105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Electricity challenges a top issue at African engineering ...</t>
+          <t>Top 100 Electrical Engineering Companies in South Africa (2026) | ensun</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://standardmicrogrid.com/content/electricity-challenges-top-issue-african-engineering-innovation-competition</t>
+          <t>https://ensun.io/search/electrical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Electricity challenges a top issue at African engineering innovation competition. Engineering innovations to boost off-grid power and stop electricity theft ...</t>
+          <t>The competitive landscape is marked by both established firms and emerging startups, driving innovation and efficiency. Additionally, South Africa’s position in the broader global market allows for potential collaborations and export opportunities, particularly in green technologies. Understanding these factors is essential for anyone looking to engage with the Electrical Engineering sector in South Africa, as they influence the overall business environment and potential for growth.</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -3009,17 +3017,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>South Africa introduces IoEWR for engineers - LinkedIn</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - IEEE ZA 5G Competition</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/posts/mangosuthu-university-of-technology_mut-ioewr-engineeringexcellence-activity-7316443789068320768-mOs4</t>
+          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51397</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Apr 11, 2025 · This global competition means that top South African engineers often receive offers from abroad, creating a "brain drain" effect that further ...</t>
+          <t>Form templates: Template for a Cover Sheet for the Competition on Ideas, Designs and Applications for 5G and Beyond South Africa (.docx) [Click to Download] Template for a Resume for the Student (.docx) [Click to Download] ... Help (FAQ) • Privacy Statement • Terms &amp; Conditions The SAIEE is ...</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3032,17 +3040,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge Grand Finals</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - SA Computing Olympiad stars hold their own in international competition</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/posts/ewbsa_engineeringimpact-engineeringeducation-activity-7473789877885722624-QS1Q</t>
+          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51457</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Jun 19, 2026 · View organization page for Engineers Without Borders South Africa ... Software Developer•GDGoC FUTMinna Technical Lead•Electrical and Electronics ...</t>
+          <t>July 20, 2021 - For the other three South African team members, this was their first IOI. Brent Butkow finished ranked 342, Jean Weight finished in 287th position and Faran Steenkamp was ranked 280. In addition to the serious IOI contest days, host country Singapore arranged several fun events where Faran Steenkamp was placed third in the sponsored Code Cup, and won a cash prize of 200 USD.</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3055,17 +3063,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026 IEEE PES/IAS PowerAfrica Conference: HOME PAGE</t>
+          <t>Electrical Engineering Conferences in South Africa 2025/2026/2027 - Conference Index</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>https://ieee-powerafrica.org/</t>
+          <t>https://conferenceindex.org/conferences/electrical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Scheduled to take place in Safari Park,Nairobi, Kenya, from 21st –25th September 2026, the conference will convene stakeholders from academia, industry, ...</t>
+          <t>Electrical Engineering Conferences in South Africa 2025 2026 2027 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and ...</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3078,17 +3086,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Real-world research: Engineering team designs South African ...</t>
+          <t>7 Electrical Engineering Degree Programs in South Africa - Study Abroad | educations.com</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
+          <t>https://www.educations.com/electrical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>May 15, 2025 · Cross-disciplinary teams present prototypes at Research Day, Engineers Without Borders' design challenge addressed by nearly 90 students.</t>
+          <t>Find the best fit for you - Compare 7 in Engineering Programs Electrical Engineering in South Africa for 2025/2026</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3096,26 +3104,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>dolanm@uwstout.edu, frischj@uwstout.edu</t>
-        </is>
-      </c>
+      <c r="E110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>The Gauteng Department of Education - Facebook</t>
+          <t>Electrical Engineering in South Africa: Best universities Ranked</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/gauteng.edu/posts/pretoriatuinesos-inside-the-electrical-technology-and-electronics-workshop-learn/1496498595832609/</t>
+          <t>https://edurank.org/engineering/electrical/za/</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Aug 17, 2026 · The National Competition in electrical engineering starting from today on the 16 until Thursday 18 August 2022 at Ekurhuleni East TVET College ...</t>
+          <t>March 2, 2025 - Below is the list of 24 best universities for Electrical Engineering in South Africa ranked based on their research performance: a graph of 827K citations received by 40.9K academic papers made by these universities was used to calculate ratings and create the top.</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3128,17 +3132,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
+          <t>Join us as 55 young innovators showcase the engineering ...</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>https://hackon.co.za/</t>
+          <t>https://www.facebook.com/ortsajhb/posts/join-us-as-55-young-innovators-showcase-the-engineering-coding-and-technology-so/1473351191493113/</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
+          <t>Jun 26, 2026 · Join us as 55 young innovators showcase the engineering, coding, and technology solutions during the Young Engineers Movement (YEM) Hackathon. ...</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -3151,17 +3155,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Hackathons en South Africa</t>
+          <t>Tech hackathons in Africa 2026 / 2027 - dev.events</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>https://za.allhackathons.com/</t>
+          <t>https://dev.events/hackathons/AF/tech</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Aug 22, 2025 · Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
+          <t>Best Tech hackathons in Africa 2026 / 2027 · The Principal Dev – Masterclass for Tech Leads · Clean Architecture Masterclass · Africa Deep Tech Challenge 2026.</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -3174,17 +3178,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Build the Future with Entelect Hackathons</t>
+          <t>ORT South Africa's Young Engineers Movement Hackathon</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>https://challenge.entelect.co.za/</t>
+          <t>https://www.linkedin.com/posts/good-things-guy_55-learners-from-underserved-schools-to-shine-activity-7473009611185217539-Ye7_</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Build the Future with Entelect Hackathons Join South Africa’s premier optimisation-first developer competition platform. Compete, iterate, and outperform the best.</t>
+          <t>Jun 17, 2026 · The event is a multi-day programme hosted by ORT South Africa running from 22 to 26 June 2026 in Johannesburg.</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3197,17 +3201,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Geekulcha Annual Hackathon 2026 - Registration | Sonke Platform</t>
+          <t>55 Learners From Underserved Schools to Shine at Hackathon!</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>https://sonke.gklink.co/event/gkhack26</t>
+          <t>https://www.goodthingsguy.com/55-learners-underserved-schools-yem-hackathon/</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>GEEKULCHA ANNUAL HACKATHON 2026 Africa's premier hackathon that drives digital innovation and empowers the next generation of tech leaders.</t>
+          <t>Jun 17, 2026 · The event is a multi-day programme hosted by ORT South Africa running from 22 to 26 June 2026 in Johannesburg.</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3215,22 +3219,26 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>198091-featured-75x75@2x.jpg, 197913-featured-75x75@3x.jpg, 198091-featured-75x75@1.5x.jpg, 197913-featured-75x75@2.5x.jpg, 198091-featured-75x75@3x.jpg, 196675-featured-75x75@1.5x.jpg, 197913-featured-75x75@2x.jpg, 196675-featured-75x75@2.5x.jpg, 196675-featured-75x75@2x.jpg, 196675-featured-75x75@3x.jpg, 197913-featured-75x75@1.5x.jpg, 198091-featured-75x75@2.5x.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Hackathons - challenge.entelect.co.za</t>
+          <t>Ocean Hackathon® Cape Town - Global Fund for Coral Reefs</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>https://challenge.entelect.co.za/hackathons</t>
+          <t>https://globalfundcoralreefs.org/reef-plus/events/ocean-hackathon-cape-town/</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Aug 21, 2026 · Hackathons Explore competitions, manage your teams, review the leaderboards and submit solutions.</t>
+          <t>The Ocean Hackathon® is a 48-hour innovation sprint, teams of hackers, engineers, When? 17–19 October 2025 🌍 Where? Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -3238,22 +3246,26 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>mohammad.al-tawaha@undp.org, thando@oceanhub.africa, _@astro-renderers.BsLwzaai.css</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>ICEP - Tshwane Varsity Hackathon</t>
+          <t>Global South AI Safety Hackathon | Apart Research</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>https://tvh.icep.co.za/</t>
+          <t>https://apartresearch.com/sprints/global-south-ais-hackathon-2026-06-19-to-2026-06-21</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Tshwane Varsity Hackathon South Africa's premier inter-university hackathon competition. Join hundreds of students for 53 hours of coding, innovation, and`` fun!</t>
+          <t>Jun 19, 2026 · The Global South AI Safety Hackathon brings together researchers, engineers, and policy professionals across Latin America, Africa, and Asia ...</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3263,24 +3275,24 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>MagasengQM@tut.ac.za, info@tvh.co.za</t>
+          <t>sprints@apartresearch.com, example@email.com</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Join us as 55 young innovators showcase the engineering ...</t>
+          <t>Just 4 days left to apply for the Mintek-SCI Grad Hackathon ...</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/ortsajhb/posts/join-us-as-55-young-innovators-showcase-the-engineering-coding-and-technology-so/1473351191493113/</t>
+          <t>https://x.com/Mintek_RSA/status/2081711307800093135</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Jun 26, 2026 · Join us as 55 young innovators showcase the engineering, coding, and technology solutions during the Young Engineers Movement (YEM) Hackathon. ...</t>
+          <t>Jul 27, 2026 · Just 4 days left to apply for the Mintek-SCI Grad Hackathon 2026! South Africa's minerals, mining, and metallurgy sector.</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3293,17 +3305,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Tech hackathons in Africa 2026 / 2027 - dev.events</t>
+          <t>Africa Ignite Hackathon - HackerEarth</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>https://dev.events/hackathons/AF/tech</t>
+          <t>https://www.hackerearth.com/challenges/hackathon/africa-ignite-hackathon/</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Best Tech hackathons in Africa 2026 / 2027 · The Principal Dev – Masterclass for Tech Leads · Clean Architecture Masterclass · Africa Deep Tech Challenge 2026.</t>
+          <t>The Africa Ignite Hackathon is a regional innovation challenge designed to empower developers, startups, and tech enthusiasts across Sub-Saharan Africa</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -3316,17 +3328,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Faurecia South Africa's Post - LinkedIn</t>
+          <t>W3Node Conference &amp; Hackathon</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/posts/forvia-faurecia-south-africa_calling-all-future-engineers-join-activity-7437386283603279872-NGpQ</t>
+          <t>https://w3node.io/</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Mar 10, 2026 · cia South Africa's Engineering Hackathon FORVIA South motivated, curious, and driven young engineers. When: 27 March 2026 Where: FORVIA Cape ...</t>
+          <t>South Africa. November. 12-14 2026. Africa's premier Developer conference. //About. w3node. Welcome to Africa's Premier Web3 Developer Conference and Hackathon.</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -3334,22 +3346,26 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr"/>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>hello@w3africa.io</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>55 Learners From Underserved Schools to Shine at Hackathon!</t>
+          <t>Siemens Energy South Africa Hackathon - Facebook</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>https://www.goodthingsguy.com/55-learners-underserved-schools-yem-hackathon/</t>
+          <t>https://www.facebook.com/SiemensEnergy/videos/siemens-energy-south-africa-hackathon/966581709250326/</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Jun 17, 2026 · The event is a multi-day programme hosted by ORT South Africa running from 22 to 26 June 2026 in Johannesburg.</t>
+          <t>May 7, 2026 · Students from across Gauteng, South Africa joined the Siemens Energy South Africa Just Energy Transition (JET) Hackathon to take on ...</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -3357,11 +3373,7 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>198031-featured-75x75@2.5x.jpeg, 198013-featured-75x75@2.5x.jpg, 198031-featured-75x75@3x.jpeg, 197895-featured-75x75@2x.jpg, 198091-featured-75x75@3x.jpg, 198019-featured-75x75@2.5x.jpg, 197895-featured-75x75@1.5x.jpg, 197895-featured-75x75@2.5x.jpg, 198013-featured-75x75@1.5x.jpg, 198019-featured-75x75@1.5x.jpg, 197895-featured-75x75@3x.jpg, 198019-featured-75x75@2x.jpg, 198091-featured-75x75@1.5x.jpg, 198091-featured-75x75@2x.jpg, 198031-featured-75x75@1.5x.jpeg, 198013-featured-75x75@2x.jpg, 198013-featured-75x75@3x.jpg, 198091-featured-75x75@2.5x.jpg, 198019-featured-75x75@3x.jpg, 198031-featured-75x75@2x.jpeg</t>
-        </is>
-      </c>
+      <c r="E121" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update competition data 2026-08-30
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>3 weeks ago - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -464,22 +464,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Two South Africans on the shortlist for the 2026 Africa Prize for Engineering Innovation</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/two-south-africans-on-the-shortlist-for-the-2026-africa-prize-for-engineering-innovation-2026-08-04</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>3 weeks ago - Two South African innovators have been shortlisted for the UK Royal Academy of Engineering’s Africa Prize for Engineering Innovation 2026. This is the continent’s richest award aimed at promoting engineering innovation and entrepreneurship ...</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -489,24 +493,24 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>advertising@creamermedia.co.za, chanel@engineeringnews.co.za, newsdesk@engineeringnews.co.za, subscriptions@creamermedia.co.za, newsletters@creamermedia.co.za</t>
+          <t>info@ieomsociety.org</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
+          <t>Team South Africa wins at NASA space engineering competition</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.poidata.io/report/engineer/south-africa</t>
+          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
+          <t>South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -519,17 +523,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2 weeks ago - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
+          <t>To promote excellence in Science, Technology, Engineering, Mathematics and Innovation in South African schools.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -542,17 +546,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -560,26 +564,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Engineering Conferences in South Africa 2025-2026</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -587,22 +587,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
+          <t>PDF 2026 South Africa Engineering Competition</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.thecasecentre.org/products/view?id=189255</t>
+          <t>https://library.ukzn.ac.za/wp-content/uploads/2026/08/About-Competition.pdf</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
+          <t>Best Regards, The 2026 SA Engineering Competition Team University of KwaZulu-Natal • Elsevier</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -615,17 +619,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Engineering conferences in South Africa 2026-2027</t>
+          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://conferencenext.com/conferences/south-africa/engineering</t>
+          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Researchers, academicians, students, scholars, investors, and professionals can attend Engineering conferences in South Africa. You just need to select an event, complete the registration process, pay fees, and receive an invitation letter.</t>
+          <t>Eligibility Benchmark Requirements The Africa Prize is open to individuals or teams based in sub-Saharan Africa with a scalable engineering innovation that demonstrates social or environmental impact potential. Applicants must: Be citizens ordinarily residing in a sub-Saharan African country. Be over 18 years old and fluent in English.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -633,26 +637,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>michaeljjacobson1@gmail.com</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>South Africa · South Korea · Spain · Sri Lanka · Sudan · Sweden · Switzerland · Syrian Arab Republic · Taiwan · Tajikistan · Tanzania · Thailand · Togo · Trinidad and Tobago · Tunisia · Turkey · Uganda · Ukraine · United Arab Emirates · United Kingdom ·</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -665,17 +665,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
+          <t>2027 Africa Prize for Engineering Innovation Opens Applications</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
+          <t>https://www.globalsouthopportunities.com/2026/08/09/africa-134/</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Engineering design competition is open to teams of engineering students from any university program in West Africa.</t>
+          <t>The Royal Academy of Engineering has opened applications for the 2027 Africa Prize for Engineering Innovation, providing African innovators with an opportunity to develop, strengthen and commercialise engineering solutions addressing important challenges across the continent.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -711,17 +711,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
+          <t>KZN Industrial Technology Exhibition</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://madeinafricaevent.co.za/</t>
+          <t>https://www.kznindustrial.co.za/</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
+          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -729,22 +729,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>john@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>KZN Industrial Technology Exhibition</t>
+          <t>Two landmark exhibitions set to transform industrial technology and renewable energy in South Africa</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://www.kznindustrial.co.za/</t>
+          <t>https://www.engineeringnews.co.za/article/two-landmark-exhibitions-set-to-transform-industrial-technology-and-renewable-energy-in-south-africa-2025-10-24</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
+          <t>October 24, 2025 - South Africa’s industrial and clean energy sectors celebrated a landmark moment today with the official launch of RE+ South Africa 2026 and the Cape Industrial Technology Exhibition (CITE) 2027.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -754,24 +758,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>john@email.com</t>
+          <t>chanel@engineeringnews.co.za, advertising@creamermedia.co.za, newsdesk@engineeringnews.co.za, newsletters@creamermedia.co.za, subscriptions@creamermedia.co.za</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Two landmark exhibitions set to transform industrial technology and renewable energy in South Africa</t>
+          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/two-landmark-exhibitions-set-to-transform-industrial-technology-and-renewable-energy-in-south-africa-2025-10-24</t>
+          <t>https://madeinafricaevent.co.za/</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>October 24, 2025 - South Africa’s industrial and clean energy sectors celebrated a landmark moment today with the official launch of RE+ South Africa 2026 and the Cape Industrial Technology Exhibition (CITE) 2027.</t>
+          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -779,26 +783,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>advertising@creamermedia.co.za, chanel@engineeringnews.co.za, newsdesk@engineeringnews.co.za, subscriptions@creamermedia.co.za, newsletters@creamermedia.co.za</t>
-        </is>
-      </c>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Trade Shows Worldwide - South Africa - 2026/2027</t>
+          <t>Exhibition | Innovation Festival Durban | South Africa</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://www.eventseye.com/fairs/c1_trade-shows_south-africa.html</t>
+          <t>https://www.innovationfestival.durban/exhibition</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>South Africa Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in South Africa</t>
+          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -806,22 +806,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Erika@innovate.durban, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, sithabile@innovate.durban, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Exhibition | Innovation Festival Durban | South Africa</t>
+          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://www.innovationfestival.durban/exhibition</t>
+          <t>https://manufacturingindaba.co.za/exhibition/</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities.</t>
+          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -829,26 +833,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>sithabile@innovate.durban, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, Erika@innovate.durban, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
+          <t>Trade Shows Worldwide - South Africa - 2026/2027</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://manufacturingindaba.co.za/exhibition/</t>
+          <t>https://www.eventseye.com/fairs/c1_trade-shows_south-africa.html</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
+          <t>South Africa Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in South Africa</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -861,17 +861,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Come and explore our exhibition of innovative discoveries at Science Forum South Africa 2024 | CSIR</t>
+          <t>Discover Innovation Hub's Pavilion at Organic &amp; Natural Products Expo - Organic &amp; Natural Products Portal</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://www.csir.co.za/come-and-explore-our-exhibition-innovative-discoveries-science-forum-south-africa-2024</t>
+          <t>https://www.organicandnaturalportal.com/innovation-hub-organic-expo/</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>December 3, 2024 - The exhibition launch will take place on Tuesday, 3 December 2024, with the opening address by Department of Science, Technology and Innovation Minister Dr Blade Nzimande.</t>
+          <t>3 weeks ago - Gathering producers, retailers, buyers, and conscious consumers under one roof, the expo serves as Africa’s premier showcase for sustainability, health, and wellness innovation. A standout highlight of this year’s exhibition is The Innovation Hub Pavilion, hosting a curated line-up of forward-thinking South African small, medium, and micro-enterprises (SMMEs).</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -884,17 +884,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Discover Innovation Hub's Pavilion at Organic &amp; Natural Products Expo - Organic &amp; Natural Products Portal</t>
+          <t>Come and explore our exhibition of innovative discoveries at Science Forum South Africa 2024 | CSIR</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://www.organicandnaturalportal.com/innovation-hub-organic-expo/</t>
+          <t>https://www.csir.co.za/come-and-explore-our-exhibition-innovative-discoveries-science-forum-south-africa-2024</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>3 weeks ago - Gathering producers, retailers, buyers, and conscious consumers under one roof, the expo serves as Africa’s premier showcase for sustainability, health, and wellness innovation. A standout highlight of this year’s exhibition is The Innovation Hub Pavilion, hosting a curated line-up of forward-thinking South African small, medium, and micro-enterprises (SMMEs).</t>
+          <t>December 3, 2024 - The exhibition launch will take place on Tuesday, 3 December 2024, with the opening address by Department of Science, Technology and Innovation Minister Dr Blade Nzimande.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -930,17 +930,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Engineering For People Design Challenge - EWBSA</t>
+          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
+          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
+          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -948,11 +948,7 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
-        </is>
-      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -967,7 +963,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community's challenges and how community members view the impact of these challenges on their daily lives.</t>
+          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -977,24 +973,24 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
+          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge - Engineers Without Borders UK</t>
+          <t>EWB Design Challenge | Aston University</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
+          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
+          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1007,17 +1003,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge returns to Johannesburg!</t>
+          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
+          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
+          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1025,22 +1021,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ied@ied.org.uk</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
+          <t>Engineers Without Borders South ...</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
+          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
+          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1048,11 +1048,7 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>team@crowdsolve.net</t>
-        </is>
-      </c>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1067,7 +1063,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>STEM-focused NGO Engineers Without Borders UK has launched its 2025 Engineering for People Design Challenge. Organised in conjunction with sister organisation Engineers Without Borders South Africa, as well as the Makers Valley Partnership, this year's challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg.</t>
+          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1090,7 +1086,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>This year's design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but under-resourced neighbourhood on the eastern edge of Johannesburg. Home to around 46,000 people, Makers Valley is a community rich in creativity, activism ...</t>
+          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1100,24 +1096,24 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>web-editor@eng.cam.ac.uk, marketing@eng.cam.ac.uk</t>
+          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge Empowers Engineering Students in SA - LinkedIn</t>
+          <t>Engineering for people, that’s the challenge | Engineers Without Borders</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/posts/activity-7470764395091001345-GwCR</t>
+          <t>https://www.rs-online.com/designspark/an-introduction-to-engineering-for-people-design-challenge</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>By joining forces, student engineers have the chance to bridge societal gaps, uplift those in vulnerable positions, and contribute to building a more inclusive and prosperous South Africa.</t>
+          <t>That’s exactly what the annual Engineering for People Design Challenge asks participants to do. The competition, delivered in partnership by Engineers without Borders South Africa and Engineers Without Borders UK, encourages engineering students and those collaborating with engineers to broaden their awareness of how their decisions change the world.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1130,17 +1126,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Engineers Without Borders | OU Design Show 2025</t>
+          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.oudesignshow.org/designathon</t>
+          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Makers Valley is a vibrant community of makers, creatives, and social enterprises in Johannesburg, South Africa. Engineers Without Borders UK has partnered with Makers Valley to engage students in design challenges focused on addressing local challenges and promoting sustainable development.</t>
+          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1153,17 +1149,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>EWB-SA: Mid-Year Update - LinkedIn</t>
+          <t>The status and challenges of industrial engineering in South Africa</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/pulse/ewb-sa-mid-year-update-ewbsa-uxo9f</t>
+          <t>https://www.scielo.org.za/scielo.php?script=sci_arttext&amp;pid=S2224-78902016000100002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>We wrapped up an extraordinary cycle of the 2023/24 Engineering for People Design Challenge in December 2024, with students across South Africa applying their creativity and empathy to solve real ...</t>
+          <t>This resulted in an identity crisis for industrial engineers, who were caught between the Industrial Revolution and the new challenges of the information system era [5]. In addition, within the South African context, where major socioeconomic changes have occurred since 1994, IEs have been exposed to a number of unique challenges that are non-existent or less dominant in other fields.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1171,22 +1167,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>corne@sun.ac.za, admin@saiie.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1194,26 +1194,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1221,26 +1217,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>National Student Competition | ORSSA</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://www.orssa.org.za/studentcomp</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;area=2200&amp;ranking=Overall&amp;country=ZAF</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>National Student Competitions The Operations Research Society of South Africa The home of decision intelligence The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1248,26 +1240,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, email@example.com, 8c4075d5481d476e945486754f783364@sentry.io, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
+          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1280,17 +1268,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1298,26 +1286,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Competitions - Enactus South Africa | National Expos, Challenges ...</t>
+          <t>Engineering in South Africa: 24 Best universities Ranked</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://enactusza.org/what-we-do/competitions</t>
+          <t>https://edurank.org/engineering/za/</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Explore our national and international competitions that empower students to tackle challenges with entrepreneurial solutions and social impact at the core.</t>
+          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1325,26 +1309,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>marketingsa@enactus.org, adminsa@enactus.org, liso@enactus.org, xmadlanga@enactus.org</t>
-        </is>
-      </c>
+      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>University Overall Rankings - Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>University Overall Rankings - Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1357,17 +1337,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
+          <t>University of South Africa</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
+          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-promotes-globally-recognised-engineering-qualifications</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Eligibility Benchmark Requirements The Africa Prize is open to individuals or teams based in sub-Saharan Africa with a scalable engineering innovation that demonstrates social or environmental impact potential. Applicants must: Be citizens ordinarily residing in a sub-Saharan African country. Be over 18 years old and fluent in English.</t>
+          <t>Unisa promotes globally recognised engineering qualifications</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1380,17 +1360,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1403,17 +1383,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2027 Africa Prize for Engineering Innovation Opens Applications</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.globalsouthopportunities.com/2026/08/09/africa-134/</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>The Royal Academy of Engineering has opened applications for the 2027 Africa Prize for Engineering Innovation, providing African innovators with an opportunity to develop, strengthen and commercialise engineering solutions addressing important challenges across the continent.</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1426,7 +1406,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 (Internet ...</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1436,7 +1416,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>1 month ago - TECHSPO Johannesburg 2026 is a two day technology expo taking place September 28th to 29th, 2026 at the luxurious Hyatt Regency Johannesburg, Johannesburg, South Africa. TECHSPO Johannesburg brings together developers, brands, marketers, technology ...</t>
+          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1444,26 +1424,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>info@techspojoburg.co.za</t>
-        </is>
-      </c>
+      <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa, List of all South Africa Technology Business Expo &amp; Events</t>
+          <t>Africa Tech Festival</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>New York Small Business Expo (Spring)07 MayNew York , USA · AFROZUM Fair · 07-09 May · Johannesburg , South Africa · AFROZUM Fair07-09 MayJohannesburg , South Africa · Nigeria Industries &amp; Manufacturing Summit · 18-20 May · Abuja , Nigeria ...</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1471,22 +1447,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>support@informaconnect.com, customerservices@knect365.com, customerservices@informaconnect.com, salesenquiries@africatechfestival.com, dataprivacy@knect365.com, support@knect365.com, dataprivacy@informaconnect.com</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 - 7, 2027 ...</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
+          <t>The annual TECHSPO Cape Town 2027 Technology Expo returns October 6th to 7th, 2027 to the V&amp;A Waterfront Cape Town Avenue Conference Venue in Cape Town. TECHSPO Cape Town Technology Expo is the must-attend event to: Experience the Future of Technology &amp; Innovation Discover cutting-edge tech, game-changing tools, and innovators shaping tomorrow's digital world. See the latest advancements in ...</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1496,24 +1476,24 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>atinfo@techspo.coor, u003einfo@techspo.co</t>
+          <t>info@techspocapetown.co.za</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Home - Mediatech Africa | South Africa</t>
+          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://www.mediatech.co.za/</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
+          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1521,26 +1501,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>simon@mediatech.co.za, claire@mediatech.co.za</t>
-        </is>
-      </c>
+      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
+          <t>TECHSPO Johannesburg Technology ExpoJohannesburg Technology Expo ...</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://africatechnologyexpo.com/</t>
+          <t>https://techspojoburg.co.za/johannesburg-technology-expo/</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
+          <t>TECHSPO Johannesburg is a 2-day technology expo taking place September 28 - 29, 2026 at the luxurious NH Johannesburg Sandton Hotel, Toronto, Ontario. TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1548,26 +1524,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>info@sparkafrica.co, johndoe@email.com, partner@africatechnologyexpo.com</t>
-        </is>
-      </c>
+      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://10times.com/johannesburg-za/technology</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
+          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1575,26 +1547,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>info@techspocapetown.co.za</t>
-        </is>
-      </c>
+      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
+          <t>Tech Expo Africa - Enabling Development</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://techexpo.africa/</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
+          <t>Tech Expo Africa is a social enterprise connecting African businesses with top tech and business leaders to drive innovation.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1604,14 +1572,14 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>salesenquiries@africatechfestival.com, support@informaconnect.com, support@knect365.com, dataprivacy@knect365.com, customerservices@informaconnect.com, customerservices@knect365.com, dataprivacy@informaconnect.com</t>
+          <t>info@techexpo.africa</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference - AI Expo Africa | 28 - 29 October SCC Johannesburg South Africa</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1621,7 +1589,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>(2 Day Event) 28th-29th October 2026 Sandton Convention Centre, JHB, South Africa · AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade ...</t>
+          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1638,17 +1606,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Discover Tech Conferences Events &amp; Activities in South Africa | Eventbrite</t>
+          <t>IT &amp; Technology Events in South Africa | 10times</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Save this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South AfricaShare this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South Africa</t>
+          <t>Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1661,7 +1629,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~…</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1671,7 +1639,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg – Where Business, Tech and Innovation Collide in Johannesburg, South Africa. TECHSPO Johannesburg Technology Expo returns September 28-29, 2026 to the NH Johannesburg Sandton Hotel in Johannesburg, South Africa.</t>
+          <t>Exhibitions &amp; Tradeshows on 22 Sept 2026 - 23 Sept 2026 in South Africa. TECHSPO Johannesburg - Where Business, Tech and Innovation Collide in…</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1681,7 +1649,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>you@company.com, your@email.com, colleague@company.com, events@techspojoburg.co.za, support@industryevents.com</t>
+          <t>colleague@company.com, you@company.com, support@industryevents.com, your@email.com, events@techspojoburg.co.za</t>
         </is>
       </c>
     </row>
@@ -1698,7 +1666,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>March 7, 2025 - Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds ...</t>
+          <t>Maker Faire Africa, Cairo, October 2011 Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds (Nubian Cheetah). Maker Faire Africa aims to engage with on ...</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1721,7 +1689,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>May 3, 2026 - Maker Faires are also held in Europe, Asia, South America and Africa.</t>
+          <t>Maker Faire is a convention of do it yourself (DIY) enthusiasts established by Make magazine in 2006. Participants come from a wide variety of interests, such as robotics, 3D printing, computers, arts and crafts, and hacker culture.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1734,17 +1702,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
+          <t>Upcoming Faires - Maker Faire</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://makerfairecapetown.wordpress.com/about/</t>
+          <t>https://makerfaire.com/upcoming-faires/</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
+          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1752,22 +1720,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>fancybox_loading@2x.gif, pr@make.co, fancybox_sprite@2x.png, chosen-sprite@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
+          <t>Maker Faire |</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
+          <t>https://makerfaire.com/</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
+          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1775,22 +1747,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>pr@make.co</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
+          <t>Maker Faire Africa — Grokipedia</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>http://capetown.makerfaire.com/</t>
+          <t>https://grokipedia.com/page/maker_faire_africa</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
+          <t>Maker Faire Africa Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1798,26 +1774,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>fancybox_loading@2x.gif, fancybox_sprite@2x.png, pr@make.co, chosen-sprite@2x.png</t>
-        </is>
-      </c>
+      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Blog : Maker Faire Africa</t>
+          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>http://makerfaireafrica.com/blog/</t>
+          <t>https://capetown.makerfaire.com/</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>December 31, 2021 - You can help them out on the new South African crowdfunding site, ThundaFund. ... One of the most ambitions items at Maker Faire Africa this year in Johannesburg, South Africa is Samuel Ngobeni’s “art car”. He’s a designer from Germinston, who has spent the last three years building his ANIMAL car, from the ground up, that means the frame and all.</t>
+          <t>Jump into the Make: community and bring a Maker Faire to your town, city, or region! Spark curiosity, rally makers of all ages, and plug your local scene into a global movement fueled by creativity, resilience, innovation, and hands-on learning.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1825,22 +1797,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>fancybox_loading@2x.gif, pr@make.co, fancybox_sprite@2x.png, chosen-sprite@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
+          <t>Home | Makers Fest</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://contemporaryand.com/en/events/maker-faire-africa-comes-to-johannesburg</t>
+          <t>https://www.makersfestival.co.za/</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
+          <t>On 8 &amp; 9 November 2025 at The Ostrich in Cape Town, join 2,000+ visitors each day for maker demos, a curated market, and family activities. It's Africa's first hands-on festival for creativity and craftsmanship — and everything you make, you take home.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1848,22 +1824,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, warren@makersfestival.co.za, example@mysite.com</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>The Makers Hub</t>
+          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://www.decorex.co.za/cape-town/en-gb/visit/TheMakersHub.html</t>
+          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Explore unique handmade items, take part in interactive workshops, and engage directly with Cape Town’s vibrant maker community.</t>
+          <t>DIRECTIONS THE CAPE TOWN MAKER FAIRE The Lookout, V&amp;A Waterfront Granger Bay Boulevard, V &amp; A Waterfront, Cape Town, 8002, South Africa Get Directions Fri Aug 21, 13:00 - Sun Aug 23, 17:00 The Lookout, V&amp;A Waterfront View Map Payments are secure and encrypted</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1871,26 +1851,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>decorexafrica@rxglobal.com</t>
-        </is>
-      </c>
+      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Jo’Burg – AfriGadget</t>
+          <t>About | Explore Unique Maker Culture — Join Now — Makers Fair</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://www.afrigadget.com/2014/07/08/maker-faire-africa-comes-to-joburg/</t>
+          <t>https://www.makersfair.co.za/about</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Maker Faire Africa 2014 will bring together over 5,000 attendees, along with featured inventors, world-class makers, self-made entrepreneurs &amp; workshop experts from South Africa, across the continent, and around the world, to manufacture real solutions for some of Africa’s most pressing ...</t>
+          <t>Discover South African and Pan-African craftsmanship at Makers Fair, a women-led event celebrating sustainable design, art, and culture. Join us today!</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1898,22 +1874,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>user@domain.com</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Makers Festival SA 🛠️ (@makersfestival_sa) • Instagram photos ...</t>
+          <t>Maker Faire groups | Meetup</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/makersfestival_sa/</t>
+          <t>https://www.meetup.com/topics/maker-faire/za/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>8,503 Followers, 58 Following, 57 Posts - Makers Festival SA 🛠️ (@makersfestival_sa) on Instagram: "🛠️ Building Skills. Building Memories. 🏕️ 8th &amp; 9th November 2025 / Cape Town, SA 🪵 Founder @hutch_custom 📩 DM us - apply to be a MAKER 🫶🏼"</t>
+          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1995,17 +1975,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Southafrica 2024 - IEOM Society</t>
+          <t>High School STEM Competition | Capetown 2026</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
+          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas.</t>
+          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the 'first author'. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2022,17 +2002,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Astemi Sa</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.astemi.co.za/</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The IEOM High School/Middle School STEM Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects.</t>
+          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2040,26 +2020,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Astemi Sa</t>
+          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/</t>
+          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>What is ASTEMI SA? The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible. We aim to increase participation in the activities of ASTEMI SA. We will encourage our members to lower the barriers of ...</t>
+          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2072,17 +2048,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
+          <t>The IEOM High School/Middle School STEM Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2090,22 +2066,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Samsung, DBE Announce Top 20 Schools Selected to Advance to the Next ...</t>
+          <t>Applications for 2026 Samsung Solve For Tomorrow Now Open!</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://news.samsung.com/za/samsung-dbe-announce-top-20-schools-selected-to-advance-to-the-next-level-of-2026-solve-for-tomorrow-competition</t>
+          <t>https://news.samsung.com/za/applications-for-2026-samsung-solve-for-tomorrow-now-open</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>At an event that took place on 14 April 2026, Samsung in partnership with the Department of Basic Education (DBE) officially announced the Top 20 schools that have been selected to advance to the next stages of the 2026 STEM-based (Science, Technology, Engineering and Mathematics) - Solve For Tomorrow (SFT) competition. In attendance was Mr. Simon Lee, the President and CEO of Samsung Africa ...</t>
+          <t>The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries open until 06 March 2026. This is a transformative ...</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2118,17 +2098,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Register your school for Samsung Solve for Tomorrow 2026</t>
+          <t>Samsung, DBE Announce Top 20 Schools Selected to Advance to the Next ...</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://www.sowetan.co.za/careers/2026-03-03-register-your-school-for-samsung-solve-for-tomorrow-2026/</t>
+          <t>https://news.samsung.com/za/samsung-dbe-announce-top-20-schools-selected-to-advance-to-the-next-level-of-2026-solve-for-tomorrow-competition</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Register your school for Samsung Solve for Tomorrow 2026 STEM competition aims to transform and empower South African learners with critical skills to solve real-world challenges March 03, 2026 at 7:44 am</t>
+          <t>At an event that took place on 14 April 2026, Samsung in partnership with the Department of Basic Education (DBE) officially announced the Top 20 schools that have been selected to advance to the next stages of the 2026 STEM-based (Science, Technology, Engineering and Mathematics) - Solve For Tomorrow (SFT) competition. In attendance was Mr. Simon Lee, the President and CEO of Samsung Africa ...</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2136,26 +2116,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>ssasft@samsung.com</t>
-        </is>
-      </c>
+      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Applications for 2026 Samsung Solve For Tomorrow Now Open!</t>
+          <t>Register your school for Samsung Solve for Tomorrow 2026</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://news.samsung.com/za/applications-for-2026-samsung-solve-for-tomorrow-now-open</t>
+          <t>https://www.sowetan.co.za/careers/2026-03-03-register-your-school-for-samsung-solve-for-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries open until 06 March 2026. This is a transformative ...</t>
+          <t>Register your school for Samsung Solve for Tomorrow 2026 STEM competition aims to transform and empower South African learners with critical skills to solve real-world challenges March 03, 2026 at 7:44 am</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2163,7 +2139,11 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ssasft@samsung.com</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2188,7 +2168,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com</t>
+          <t>605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -2269,7 +2249,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, info@thecortexhub.africa, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com</t>
+          <t>605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, info@thecortexhub.africa, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2276,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>adverts@ubuntutimes.co.za, newspaper-rec300@2x.jpg</t>
+          <t>newspaper-rec300@2x.jpg, adverts@ubuntutimes.co.za</t>
         </is>
       </c>
     </row>
@@ -2422,17 +2402,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>RoadEng Civil Engineer - Alternative to Complicated CAD</t>
+          <t>Home [civilexpoits2026.com]</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://www.bing.com/aclick?ld=e8xUZ4ioxsW5QmsutJAwQ9GTVUCUxFpLo4nwUHEtN1raTBZn6dckIigpjwYbmX9hQf4xNfnHsLDyDxzld8sBYgRNK9Pilt8IYkO6HHBk28jli7yFEuvrwP3rY43Za_uAgqkKFfrdc9WJVhMy7Nh0MfAv8Gil3bPyWDEUyMGT5KwOnSRCeH5neCFgOK-cMHXFYzH75Dj0k0ktut69vlpYvbInMv-ys&amp;u=aHR0cHMlM2ElMmYlMmZ3d3cuc29mdHJlZS5jb20lMmZwcm9kdWN0cyUyZmNvcnJpZG9yLWRlc2lnbiUyZnJvYWRlbmclM2Ztc2Nsa2lkJTNkMzYyMTQ2YmQ4YjFkMThiMmE5MzQyYzJmNTEwZDYxNmQ&amp;rlid=362146bd8b1d18b2a9342c2f510d616d</t>
+          <t>https://civilexpoits2026.com/</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Built for road engineering, fast &amp; interactive even with large LiDAR, DEM, &amp; drone data. RoadEng is a user-friendly civil design software, specialized in rural infrastructure.</t>
+          <t>This national civil engineering competition is your chance to put your engineering precision to the test and build real-world structural solutions. Step up and prove your skills on a national stage!</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2442,24 +2422,24 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>support@softree.com</t>
+          <t>civilexpo.sipilits@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering</t>
+          <t>SAICE's 34th International Bridge Competition Inspires Tomorrow's ...</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://civils.org.za/</t>
+          <t>https://southafricatoday.net/lifestyle/education/saices-34th-international-bridge-competition-inspires-tomorrows-engineers/</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
+          <t>The South African Institution of Civil Engineering (SAICE) hosted its 34th International Bridge Building Competition at the Midrand Conference Centre, bringing together 21 teams of high school learners from across South Africa, alongside international participants from Eswatini, Uganda, and Zimbabwe.</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2472,7 +2452,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2482,7 +2462,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Sep 4, 2025 · The Africa Prize for Engineering Innovation is the continent’s largest award dedicated to fostering engineering innovation. Its mission is to stimulate, celebrate, and reward ingenuity and entrepreneurship across sub-Saharan Africa.</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2492,24 +2472,24 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Civil Expo ITs 2026</t>
+          <t>ICE Africa - Supporting Civil Engineers in Africa</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://civilexpoits2026.com/</t>
+          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Hi Cipo Pals! Civil Expo ITs 2026 Sovereign Structures, Resilient Societies This national civil engineering competition is your chance to put your engineering precision to the test and build real-world structural solutions. Step up and prove your skills on a national stage!</t>
+          <t>ICE Africa supports civil engineers across the continent, providing access to qualifications, training, and networking opportunities for professional growth.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2517,26 +2497,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>civilexpo.sipilits@gmail.com</t>
-        </is>
-      </c>
+      <c r="E85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ICE Africa – Supporting Civil Engineers in Africa</t>
+          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
+          <t>https://safcec.org.za/</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Click your country to find local events, competitions, and information on how you can get more involved. At the heart of everything we do in South Africa is ICE-SA, the volunteer ICE local association (formerly known as the Joint Civils Division).</t>
+          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2544,22 +2520,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>communication@safcec.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge Launches in South ...</t>
+          <t>Engineering the Future: 16 schools compete in SAICE's 33rd ...</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/posts/ewbsa_engineering-for-people-design-challenge-launch-activity-7485656340049231872-lSGJ</t>
+          <t>https://southafricatoday.net/lifestyle/education/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Jul 22, 2026 · We are bringing the Engineering for People Design Challenge to universities across South Africa. engineering students design with communities ... Missing: competition | Show results with: competition</t>
+          <t>The South African Institution of Civil Engineering (SAICE) hosted its 33 rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland. The very first SAICE Bridge Building Competition was held in 1991, and it aimed to encourage high school learners to apply their knowledge of mathematics and science in a ...</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2572,17 +2552,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Civil Engineering Needs To Fill Thousands of Jobs. This ...</t>
+          <t>The South African Institution of Civil Engineering (SAICE)</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://www.bentley.com/en/blog/civil-engineering-needs-to-fill-thousands-of-jobs-this-contest-starts-with-introducing-middle-and-high-schoolers-to-the-field/</t>
+          <t>https://www.facebook.com/SAICECIVIL/posts/enter-for-the-2026-saice-national-awardsnominations-are-open-and-were-looking-fo/1419225983581060/</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Jul 8, 2026 · The AASHTO Bridge Challenge contest compresses a full engineering job into one project. Bentley supplies sponsorship, free software, and judges.</t>
+          <t>Enter for the 2026 SAICE National Awards! Nominations are open, and we're looking for the projects that truly made a difference where it matters most. The Community-Based Project of the Year is...</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2595,17 +2575,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE ...</t>
+          <t>Home - SAICE</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/100069805516530/posts/the-south-african-institution-of-civil-engineering-saice-hosted-the-2026-aqualib/1241182688218570/</t>
+          <t>https://saice.org.za/</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Mar 20, 2026 · This global competition brings together students and young professionals from across the globe to develop innovative solutions to real-life ...</t>
+          <t>The South African Institution of Civil Engineering (SAICE) is the industry body for civil engineering professionals in South Africa. Our aim is to, promote growth, excellence and sustainability in the industry.</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2613,22 +2593,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>civilinfo@saice.org.za, marketing@saice.org.za, accounts@saice.org.za, membership@saice.org.za, executiveadmin@saice.org.za, communications@saice.org.za, barbara@avenue.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>The Bridge-building competition once again saw grade 11 and ...</t>
+          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/sanralza/posts/the-bridge-building-competition-once-again-saw-grade-11-and-12-learners-particip/881766283981029/</t>
+          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Aug 14, 2024 · The South African Institution of Civil Engineering (SAICE) initiated the bridge building competition to further high school learners' use of ...</t>
+          <t>19 June 2026 marked an exciting celebration of Youth Month as aspiring young engineers from across Gauteng gathered for the 2026 SAICE Johannesburg Branch Schools Bridge Building Competition. Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in ...</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2641,17 +2625,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Bridges for bridging the skills gap in civil engineering. | EBSCOhost</t>
+          <t>Awards 2025 - SAICE</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://openurl.ebsco.com/contentitem/gcd:99622195</t>
+          <t>https://saice.org.za/awards-2025/</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Abstract. The article offers information on the annual AECOM-SAICE International Bridge Building Competition, organised by SAICE, held in August 2014 at the ...</t>
+          <t>Learn about SAICE's award categories, submission guidelines, key dates and how to nominate project and professionals.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2659,22 +2643,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>civilinfo@saice.org.za, marketing@saice.org.za, accounts@saice.org.za, membership@saice.org.za, communications@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge Launches in South ...</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/posts/ewbsa_engineering-for-people-design-challenge-launch-activity-7485656340049231872-lSGJ</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Jul 22, 2026 · We are bringing the Engineering for People Design Challenge to universities across South Africa. engineering students design with communities ...</t>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2687,17 +2675,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>South Africa's future artisans, technicians and innovators are ...</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/SasolLTD/posts/south-africas-future-artisans-technicians-and-innovators-are-preparing-to-showca/1392391599661358/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>24 hours ago · The national competition takes place from 30 September to 2 October 2026, celebrating the talent, determination and innovation of South Africa's ...</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2710,17 +2698,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Engineering for People, our flagship university design challenge, has won Silver in the QS Reimagine Education Awards 2025, recognising its impact in empowering ... Missing: mechanical | Show results with: mechanical</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2728,22 +2716,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>What are the names of international level mechanical ... - Quora</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://www.quora.com/What-are-the-names-of-international-level-mechanical-engineering-competitions-for-a-college-student</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Jun 10, 2015 · BAJA conducted by SAE(Society for automotive engineering),a competition for building ATV (terrain vehicle) is considered the biggest event for ...</t>
+          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2756,17 +2748,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>South Africa students defeated the world to win nasa school ...</t>
+          <t>PDF 2026 South Africa Engineering Competition</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/sanctview/posts/south-africa-students-defeated-the-world-to-win-nasa-school-engineering-competit/1361370549525718/</t>
+          <t>https://library.ukzn.ac.za/wp-content/uploads/2026/08/About-Competition.pdf</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Aug 11, 2026 · Recent posts · Welabasha High School learner wins first place in Sasol mechanical technology competition.</t>
+          <t>Best Regards, The 2026 SA Engineering Competition Team University of KwaZulu-Natal • Elsevier</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2779,17 +2771,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ICME 2028: 22. International Conference on Mechanical ...</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://waset.org/mechanical-engineering-conference-in-november-2028-in-cape-town</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>ICME 2028: 22. International Conference on Mechanical Engineering. November 04-05, 2028 in Cape Town, South Africa. HYBRID. Cape Town.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2797,22 +2789,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Real-world research: Engineering team designs South African ...</t>
+          <t>Competitions South Africa - Live Giveaways &amp; Prize Draws | Freehub</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
+          <t>https://freehub.co.za/competitions/</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>May 15, 2025 · Cross-disciplinary teams present prototypes at Research Day, Engineers Without Borders' design challenge addressed by nearly 90 students.</t>
+          <t>Browse live South African competitions, giveaways and prize draws. Find car, cash, voucher, tech and holiday competitions with clear entry rules and official source links.</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2820,26 +2816,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>frischj@uwstout.edu, dolanm@uwstout.edu</t>
-        </is>
-      </c>
+      <c r="E98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>About Baja - SAE International</t>
+          <t>South African Competitions Worth Entering Today | Freehub</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://www.sae.org/events/student/about/baja</t>
+          <t>https://freehub.co.za/</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Baja SAE® consists of competitions that simulate real-world engineering design projects and their related challenges. May 20-23, 2027. Baja SAE South Africa</t>
+          <t>Find South African competitions worth checking today, with curated picks, clear closing dates, entry-cost labels and official promoter links.</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2852,17 +2844,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>WorldSkills Results</t>
+          <t>PDF Apply Now! Worldskills South Africa National Competition 2025</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://results.worldskills.org/results</t>
+          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2024 South Africa Mechatronics. South Africa Mechanical Engineering CAD 21. Aircraft Maintenance 22. South Africa Plumbing and Heating 30. South ...</t>
+          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2875,17 +2867,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Johannesburg, S.A. - Next Engineers</t>
+          <t>SAIMechE</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>https://www.nextengineers.org/en/locations/johannesburg</t>
+          <t>https://www.saimeche.org.za/</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Johannesburg's Engineering Discovery has reached 3 170 Grade 8 learners across the city since launch in 2022. This year, the team is aiming to reach 1 000 more!</t>
+          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2893,26 +2885,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>NextEngineers@fhi360.org, nextengineers@protec.org.za</t>
-        </is>
-      </c>
+      <c r="E101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
+          <t>Cars4Mars - TryEngineering.org Powered by IEEE</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
+          <t>https://tryengineering.org/event/cars4mars/</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
+          <t>Cars4Mars is a robotics competition to design and build a Mars Rover Prototype. Competition starts – 1 May 2026 … hydraulics and electrical systems.</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2925,17 +2913,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - SAIEE National Student Project Competition</t>
+          <t>Join us as 55 young innovators showcase the engineering ...</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/calendar/EventDetails.aspx?eeid=29281</t>
+          <t>https://www.facebook.com/ortsajhb/posts/join-us-as-55-young-innovators-showcase-the-engineering-coding-and-technology-so/1473351191493113/</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>The SAIEE National Students Project Competition will be held at the North-West University (Potchefstroom Campus) on 21 November 2019</t>
+          <t>Jun 26, 2026 · Join us as 55 young innovators showcase the engineering, coding, and technology solutions they've developed during the Young Engineers Movement ...</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2948,17 +2936,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>CMU-Africa students shine at global electronics conference</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://www.africa.engineering.cmu.edu/news/2026/01/16-ieee-conference.html</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>March 12, 2026 - At the Centre for High Performance Computing (CHPC) Conference hosted in Cape Town at the end of last year, four current fourth-year electrical engineering students were crowned national champions in the Student Cluster Competition for 2025.</t>
+          <t>Jan 16, 2026 · SPEC 2025, held in Johannesburg, South Africa, is part of the Power Electronics Society, in the field of electrical engineering.</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2966,22 +2954,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>africa-info@andrew.cmu.edu</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Student Design Competition | IEEE CASS</t>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://ieee-cas.org/society-involvement/student-design-competition</t>
+          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>CASS will reimburse the travel costs for the trip to ISCAS 2026 for the four finalists, one for each region - Regions 1-7 (USA and Canada), Region 8 (Europe, Middle East, Africa), Region 9 (Latin America), and Region 10 (Asia, Australia, Pacific), as well as ISCAS registration.</t>
+          <t>Student Chapter Design Contest (Africa) Serving the electrical energy conversion professional worldwide. Chapter Design Contest (Africa) Deadline: April 30, ...</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2994,17 +2986,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Top 100 Electrical Engineering Companies in South Africa (2026) | ensun</t>
+          <t>Electricity challenges a top issue at African engineering ...</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://ensun.io/search/electrical-engineering/south-africa</t>
+          <t>https://standardmicrogrid.com/content/electricity-challenges-top-issue-african-engineering-innovation-competition</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>The competitive landscape is marked by both established firms and emerging startups, driving innovation and efficiency. Additionally, South Africa’s position in the broader global market allows for potential collaborations and export opportunities, particularly in green technologies. Understanding these factors is essential for anyone looking to engage with the Electrical Engineering sector in South Africa, as they influence the overall business environment and potential for growth.</t>
+          <t>Electricity challenges a top issue at African engineering innovation competition. Engineering innovations to boost off-grid power and stop electricity theft ... Missing: electrical | Show results with: electrical</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -3017,17 +3009,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - IEEE ZA 5G Competition</t>
+          <t>Engineering for People Design Challenge Grand Finals</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51397</t>
+          <t>https://www.linkedin.com/posts/ewbsa_engineeringimpact-engineeringeducation-activity-7473789877885722624-QS1Q</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Form templates: Template for a Cover Sheet for the Competition on Ideas, Designs and Applications for 5G and Beyond South Africa (.docx) [Click to Download] Template for a Resume for the Student (.docx) [Click to Download] ... Help (FAQ) • Privacy Statement • Terms &amp; Conditions The SAIEE is ...</t>
+          <t>Jun 19, 2026 · View organization page for Engineers Without Borders South Africa ... Software Developer•GDGoC FUTMinna Technical Lead•Electrical and Electronics ...</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3040,17 +3032,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - SA Computing Olympiad stars hold their own in international competition</t>
+          <t>Engineering for People Design Challenge</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51457</t>
+          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>July 20, 2021 - For the other three South African team members, this was their first IOI. Brent Butkow finished ranked 342, Jean Weight finished in 287th position and Faran Steenkamp was ranked 280. In addition to the serious IOI contest days, host country Singapore arranged several fun events where Faran Steenkamp was placed third in the sponsored Code Cup, and won a cash prize of 200 USD.</t>
+          <t>Engineering for People, our flagship university design challenge, has won Silver in the QS Reimagine Education Awards 2025, recognising its impact in empowering ... Missing: electrical | Show results with: electrical</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3063,17 +3055,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Electrical Engineering Conferences in South Africa 2025/2026/2027 - Conference Index</t>
+          <t>Real-world research: Engineering team designs South African ...</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>https://conferenceindex.org/conferences/electrical-engineering/south-africa</t>
+          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Electrical Engineering Conferences in South Africa 2025 2026 2027 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and ...</t>
+          <t>May 15, 2025 · Cross-disciplinary teams present prototypes at Research Day, Engineers Without Borders' design challenge addressed by nearly 90 students.</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3081,22 +3073,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>frischj@uwstout.edu, dolanm@uwstout.edu</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>7 Electrical Engineering Degree Programs in South Africa - Study Abroad | educations.com</t>
+          <t>Stephen Theron's Post - LinkedIn</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>https://www.educations.com/electrical-engineering/south-africa</t>
+          <t>https://www.linkedin.com/posts/stephen-theron_sasolsolarchallenge-tvetafrica-solarev-activity-7498683354414858240-K6vq</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Find the best fit for you - Compare 7 in Engineering Programs Electrical Engineering in South Africa for 2025/2026</t>
+          <t>3 days ago · He's leading 12 fellow TVET students building a solar-powered EV for South Africa's national solar car challenge — a competition no SA team has ...</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3104,22 +3100,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>retshegofaditswemashigo55@gmail.com, nretshegofaditswemashigo55@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Electrical Engineering in South Africa: Best universities Ranked</t>
+          <t>WE HAVE A WINNER! What happens when you combine ...</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://edurank.org/engineering/electrical/za/</t>
+          <t>https://www.facebook.com/100095556341859/posts/-𝑾𝑬-𝑯𝑨𝑽𝑬-𝑨-𝑾𝑰𝑵𝑵𝑬𝑹-what-happens-when-you-combine-industrial-engineering-ai-a-big-/1251805024681364/</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>March 2, 2025 - Below is the list of 24 best universities for Electrical Engineering in South Africa ranked based on their research performance: a graph of 827K citations received by 40.9K academic papers made by these universities was used to calculate ratings and create the top.</t>
+          <t>Aug 12, 2026 · Competing against Industrial Engineering undergraduates from universities across South Africa, the challenge was to develop a solution using ...</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3155,17 +3155,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Tech hackathons in Africa 2026 / 2027 - dev.events</t>
+          <t>55 Learners From Underserved Schools to Shine at Hackathon!</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>https://dev.events/hackathons/AF/tech</t>
+          <t>https://www.goodthingsguy.com/55-learners-underserved-schools-yem-hackathon/</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Best Tech hackathons in Africa 2026 / 2027 · The Principal Dev – Masterclass for Tech Leads · Clean Architecture Masterclass · Africa Deep Tech Challenge 2026.</t>
+          <t>Jun 17, 2026 · The event is a multi-day programme hosted by ORT South Africa running from 22 to 26 June 2026 in Johannesburg.</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -3173,7 +3173,11 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>197912-featured-75x75@2x.jpeg, 197912-featured-75x75@2.5x.jpeg, 198065-featured-75x75@1.5x.jpg, 198065-featured-75x75@2.5x.jpg, 198167-featured-75x75@1.5x.jpg, 198032-featured-75x75@2.5x.jpg, 198065-featured-75x75@3x.jpg, 197912-featured-75x75@3x.jpeg, 198032-featured-75x75@1.5x.jpg, 198065-featured-75x75@2x.jpg, 198167-featured-75x75@2x.jpg, 198032-featured-75x75@3x.jpg, 197912-featured-75x75@1.5x.jpeg, 198167-featured-75x75@2.5x.jpg, 198167-featured-75x75@3x.jpg, 198032-featured-75x75@2x.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3201,17 +3205,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>55 Learners From Underserved Schools to Shine at Hackathon!</t>
+          <t>Tech hackathons in Africa 2026 / 2027 - dev.events</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>https://www.goodthingsguy.com/55-learners-underserved-schools-yem-hackathon/</t>
+          <t>https://dev.events/hackathons/AF/tech</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Jun 17, 2026 · The event is a multi-day programme hosted by ORT South Africa running from 22 to 26 June 2026 in Johannesburg.</t>
+          <t>Tech hackathons in Africa 2026 ・ for experienced software engineers. Feb 27 - Dec 25 ・ the #1 tech conference listing. curated by tech community.</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3219,11 +3223,7 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>198091-featured-75x75@2x.jpg, 197913-featured-75x75@3x.jpg, 198091-featured-75x75@1.5x.jpg, 197913-featured-75x75@2.5x.jpg, 198091-featured-75x75@3x.jpg, 196675-featured-75x75@1.5x.jpg, 197913-featured-75x75@2x.jpg, 196675-featured-75x75@2.5x.jpg, 196675-featured-75x75@2x.jpg, 196675-featured-75x75@3x.jpg, 197913-featured-75x75@1.5x.jpg, 198091-featured-75x75@2.5x.jpg</t>
-        </is>
-      </c>
+      <c r="E115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>mohammad.al-tawaha@undp.org, thando@oceanhub.africa, _@astro-renderers.BsLwzaai.css</t>
+          <t>thando@oceanhub.africa, _@astro-renderers.BsLwzaai.css, mohammad.al-tawaha@undp.org</t>
         </is>
       </c>
     </row>
@@ -3275,24 +3275,24 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>sprints@apartresearch.com, example@email.com</t>
+          <t>example@email.com, sprints@apartresearch.com</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Just 4 days left to apply for the Mintek-SCI Grad Hackathon ...</t>
+          <t>Africa Ignite Hackathon - HackerEarth</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>https://x.com/Mintek_RSA/status/2081711307800093135</t>
+          <t>https://www.hackerearth.com/challenges/hackathon/africa-ignite-hackathon/</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Jul 27, 2026 · Just 4 days left to apply for the Mintek-SCI Grad Hackathon 2026! South Africa's minerals, mining, and metallurgy sector.</t>
+          <t>The Africa Ignite Hackathon is a regional innovation challenge designed to empower developers, startups, and tech enthusiasts across Sub-Saharan Africa</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3305,17 +3305,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Africa Ignite Hackathon - HackerEarth</t>
+          <t>Siemens Energy South Africa Hackathon - Facebook</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>https://www.hackerearth.com/challenges/hackathon/africa-ignite-hackathon/</t>
+          <t>https://www.facebook.com/SiemensEnergy/videos/siemens-energy-south-africa-hackathon/966581709250326/</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>The Africa Ignite Hackathon is a regional innovation challenge designed to empower developers, startups, and tech enthusiasts across Sub-Saharan Africa</t>
+          <t>May 7, 2026 · Students from across Gauteng, South Africa joined the Siemens Energy South Africa Just Energy Transition (JET) Hackathon to take on ...</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -3328,17 +3328,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>W3Node Conference &amp; Hackathon</t>
+          <t>Tech job opportunity AND money to be won : r/southafrica</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>https://w3node.io/</t>
+          <t>https://www.reddit.com/r/southafrica/comments/x8umad/tech_job_opportunity_and_money_to_be_won/</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>South Africa. November. 12-14 2026. Africa's premier Developer conference. //About. w3node. Welcome to Africa's Premier Web3 Developer Conference and Hackathon.</t>
+          <t>Sep 8, 2022 · Boston Consulting Group (BCG) is holding a hackathon on 28-29 October across its offices in Europe, Middle East, South America and Africa to ...</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -3346,26 +3346,22 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>hello@w3africa.io</t>
-        </is>
-      </c>
+      <c r="E120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Siemens Energy South Africa Hackathon - Facebook</t>
+          <t>Mintek</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/SiemensEnergy/videos/siemens-energy-south-africa-hackathon/966581709250326/</t>
+          <t>https://x.com/Mintek_RSA/status/2072666153650938330</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>May 7, 2026 · Students from across Gauteng, South Africa joined the Siemens Energy South Africa Just Energy Transition (JET) Hackathon to take on ...</t>
+          <t>Jul 2, 2026 · The #MintekSCI Grad Hackathon 2026 invites innovative solutions for South Africa's minerals, mining, and metallurgy sector.</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">

</xml_diff>

<commit_message>
Update competition data 2026-08-31
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>South African Space Design Competition | Inspire Space ...</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>Join the South African Space Design Competition to inspire space innovation, develop STEM skills, and compete for a trip to NASA.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -466,24 +466,24 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>info@ieomsociety.org</t>
+          <t>info@zasdc.org, user@domain.com</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>Team South Africa has won a NASA space engineering ...</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.facebook.com/61558499280968/posts/team-south-africa-has-won-a-nasa-space-engineering-competition-the-team-beat-oth/122242230842283309/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+          <t>Aug 8, 2026 · Team South Africa has won a NASA space engineering competition. The team beat other countries with their engineering and problem-solving skills.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -491,26 +491,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Team South Africa wins at NASA space engineering competition</t>
+          <t>Engineering for People Design Challenge</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
+          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
+          <t>Engineering for People, our flagship university design challenge, has won Silver in the QS Reimagine Education Awards 2025, recognising its impact in empowering ...</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -523,17 +519,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>SA's Team Wins Global Space Engineering Competition at NASA!</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.goodthingsguy.com/sa-team-wins-at-nasa/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>To promote excellence in Science, Technology, Engineering, Mathematics and Innovation in South African schools.</t>
+          <t>Aug 14, 2026 · SA's first-ever team to compete in the International Space Settlement Design Competition has returned home from NASA as world champions!</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -541,22 +537,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>198115-featured-75x75@3x.jpg, 198201-featured-75x75@3x.jpg, 198201-featured-75x75@1.5x.jpg, 198115-featured-75x75@2x.jpg, 198119-featured-75x75@2.5x.jpg, 198119-featured-75x75@2x.jpg, 198201-featured-75x75@2x.jpg, 198208-featured-75x75@3x.jpg, 198208-featured-75x75@2.5x.jpg, 198119-featured-75x75@1.5x.jpg, 198191-featured-75x75@2.5x.jpg, 198208-featured-75x75@1.5x.jpg, 198115-featured-75x75@1.5x.jpg, 198191-featured-75x75@3x.jpg, 198201-featured-75x75@2.5x.jpg, 198119-featured-75x75@3x.jpg, 198208-featured-75x75@2x.jpg, 198115-featured-75x75@2.5x.jpg, 198191-featured-75x75@1.5x.jpg, 198191-featured-75x75@2x.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>South African Learners Win NASA Space Engineering ...</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://www.linkedin.com/posts/business-tech-africa_seven-south-african-learners-made-history-activity-7492930299115528192-HOEY</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
+          <t>Aug 11, 2026 · Seven South African learners made history by winning an international space engineering competition at NASA - National Aeronautics and Space ...</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -569,17 +569,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
+          <t>The 2026 South Africa Engineering Competition Online - LibCal</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://ukzn.libcal.com/event/17342211</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>From: 2:30 PM, Tuesday, September 1, 2026 ; To: 4:00 PM, Tuesday, September 15, 2026 ; Time Zone: Central Africa Time (change) ; Online: This is an online event.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -589,24 +589,24 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
+          <t>HlongwaneS2@ukzn.ac.za</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PDF 2026 South Africa Engineering Competition</t>
+          <t>Robotics for Good Youth Challenge South Africa</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://library.ukzn.ac.za/wp-content/uploads/2026/08/About-Competition.pdf</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Best Regards, The 2026 SA Engineering Competition Team University of KwaZulu-Natal • Elsevier</t>
+          <t>Experience the excitement as South African teams showcase their skills in the leading UN-based global robotics competition, focusing on the critical area of ...</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -614,22 +614,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>name@example.com</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
+          <t>South Africa students defeated the world to win nasa school ...</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
+          <t>https://www.facebook.com/sanctview/posts/south-africa-students-defeated-the-world-to-win-nasa-school-engineering-competit/1361370549525718/</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Eligibility Benchmark Requirements The Africa Prize is open to individuals or teams based in sub-Saharan Africa with a scalable engineering innovation that demonstrates social or environmental impact potential. Applicants must: Be citizens ordinarily residing in a sub-Saharan African country. Be over 18 years old and fluent in English.</t>
+          <t>Aug 11, 2026 · South Africa students defeated the world to win nasa school engineering competition.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -642,17 +646,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>GRW Engineering in South Africa - The Case Centre</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.thecasecentre.org/products/view</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief ...</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -665,17 +669,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2027 Africa Prize for Engineering Innovation Opens Applications</t>
+          <t>[As Received] Seven South African high school students have ...</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://www.globalsouthopportunities.com/2026/08/09/africa-134/</t>
+          <t>https://www.reddit.com/r/DownSouth/comments/1vjq89i/as_received_seven_south_african_high_school/</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>The Royal Academy of Engineering has opened applications for the 2027 Africa Prize for Engineering Innovation, providing African innovators with an opportunity to develop, strengthen and commercialise engineering solutions addressing important challenges across the continent.</t>
+          <t>Aug 9, 2026 · [As Received] Seven South African high school students have made history by winning the International Space Settlement Design Competition at ...</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -688,17 +692,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>South Africa International Industrial Expo | Innovation Bridge</t>
+          <t>Africa Tech Festival</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -706,22 +710,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>customerservices@knect365.com, dataprivacy@knect365.com, support@informaconnect.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, support@knect365.com, dataprivacy@informaconnect.com</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>KZN Industrial Technology Exhibition</t>
+          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://www.kznindustrial.co.za/</t>
+          <t>https://10times.com/southafrica/tradeshows</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
+          <t>South Africa trade shows, find and compare 965 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 169 upcoming expos in 2026-2027 1. Investment Showcase, 2. South African Cheese Festival And ...</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -729,26 +737,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>john@email.com</t>
-        </is>
-      </c>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Two landmark exhibitions set to transform industrial technology and renewable energy in South Africa</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/two-landmark-exhibitions-set-to-transform-industrial-technology-and-renewable-energy-in-south-africa-2025-10-24</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>October 24, 2025 - South Africa’s industrial and clean energy sectors celebrated a landmark moment today with the official launch of RE+ South Africa 2026 and the Cape Industrial Technology Exhibition (CITE) 2027.</t>
+          <t>AI Expo Africa 2026 - Join the Largest AI Event &amp; Trade Community in Africa TODAY! Our business audience is a buyer / supplier focused community and comprised of Enterprise decision makers / CxOs, allied to AI Cloud platform providers, Tier 1 / 2 deployment &amp; service providers, AI start ups / innovators, investors, educators, government and AI ecosystem community builders.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -758,24 +762,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>chanel@engineeringnews.co.za, advertising@creamermedia.co.za, newsdesk@engineeringnews.co.za, newsletters@creamermedia.co.za, subscriptions@creamermedia.co.za</t>
+          <t>enquiries@aiexpoafrica.com</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
+          <t>Exhibition | Innovation Festival Durban | South Africa</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://madeinafricaevent.co.za/</t>
+          <t>https://www.innovationfestival.durban/exhibition</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
+          <t>Exhibition Opportunities BENEFITS FOR YOUR PARTICIPATING IN THE EXHIBITION: An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities. Opportunity to market your Brand. Exposure on print, electronic and social media platforms.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -783,22 +787,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>8c4075d5481d476e945486754f783364@sentry.io, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, sithabile@innovate.durban, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, Erika@innovate.durban, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Exhibition | Innovation Festival Durban | South Africa</t>
+          <t>Electra Mining Africa | South Africa's Leading Mining and Industrial ...</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://www.innovationfestival.durban/exhibition</t>
+          <t>https://www.electramining.co.za/</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities.</t>
+          <t>South Africa's Leading Mining Exhibition 7 - 11 September 2026 | JHB Expo Centre Nasrec Discover the biggest mining, industrial, electrical and power event in Africa. Connect with solution-providers, explore the latest technology and meet decision-makers who shape the future of the industry.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -808,24 +816,24 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Erika@innovate.durban, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, sithabile@innovate.durban, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com</t>
+          <t>john@email.com</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
+          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://manufacturingindaba.co.za/exhibition/</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
+          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -838,17 +846,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Trade Shows Worldwide - South Africa - 2026/2027</t>
+          <t>ELENEX Africa Johannesburg 2026 - TradeFairDates</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://www.eventseye.com/fairs/c1_trade-shows_south-africa.html</t>
+          <t>https://www.tradefairdates.com/ELENEX-Africa-M6915/Johannesburg.html</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>South Africa Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in South Africa</t>
+          <t>The fair is deeply rooted in the dynamics and industrial growth of Johannesburg and demonstrates South Africa's role as a leading center for technological innovation in Africa.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -861,17 +869,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Discover Innovation Hub's Pavilion at Organic &amp; Natural Products Expo - Organic &amp; Natural Products Portal</t>
+          <t>IT &amp; Technology Events in South Africa | 10times</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://www.organicandnaturalportal.com/innovation-hub-organic-expo/</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>3 weeks ago - Gathering producers, retailers, buyers, and conscious consumers under one roof, the expo serves as Africa’s premier showcase for sustainability, health, and wellness innovation. A standout highlight of this year’s exhibition is The Innovation Hub Pavilion, hosting a curated line-up of forward-thinking South African small, medium, and micro-enterprises (SMMEs).</t>
+          <t>Big Data and Business Analytics Innovation Conference Johannesburg, South Africa IT &amp; Technology 100 Members Wed, 28 - Thu, 29 Oct 2026</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -884,17 +892,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Come and explore our exhibition of innovative discoveries at Science Forum South Africa 2024 | CSIR</t>
+          <t>Exhibitions in South Africa 2026-2027 - ExpoTobi</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://www.csir.co.za/come-and-explore-our-exhibition-innovative-discoveries-science-forum-south-africa-2024</t>
+          <t>https://expotobi.com/country/south-africa/exhibitions</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>December 3, 2024 - The exhibition launch will take place on Tuesday, 3 December 2024, with the opening address by Department of Science, Technology and Innovation Minister Dr Blade Nzimande.</t>
+          <t>All Exhibitions in South Africa 2026-2027 | Full and accurate description of events for various business sectors | Schedule, tickets, travel arrangements and participation</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -907,17 +915,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>International Science, Innovation &amp; Technology Expo (INSITE)</t>
+          <t>AI Expo Africa 2026 - Africa-Europe Innovation Platform</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.dsti.gov.za/index.php/resource-center/27-temp/dst-links/3-international-science-innovation-a-technology-expo</t>
+          <t>https://www.africaeuropeinnovation.net/event/ai-expo-africa-2026/</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>The essence of INSITE INSITE is an international, biennial must-see Science and Technology event in South Africa, the only one of its kind in Africa that creates new frontiers for global challenges · INSITE aims to assemble the worlds leading innovators and scientists in one place, stimulating ...</t>
+          <t>AI Expo Africa is the continent's largest Artificial Intelligence and Intelligent Automation trade show and conference, connecting enterprise buyers with ...</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -930,17 +938,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
+          <t>Engineering - Wikipedia</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
+          <t>https://en.wikipedia.org/wiki/Engineering</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
+          <t>The steam engine, the major driver in the Industrial Revolution, underscores the importance of engineering in modern history. This beam engine is on display in the Technical University of Madrid. Engineering is the practice of systematically applying natural science and mathematics to design and improve systems, devices, or processes that solve problems under constraints. It is typically ...</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -953,17 +961,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>Engineer - Wikipedia</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://en.wikipedia.org/wiki/Engineer</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
+          <t>Engineers develop new technological solutions. During the engineering design process, the responsibilities of the engineer may include defining problems, conducting and narrowing research, analyzing criteria, finding and analyzing solutions, and making decisions.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -971,26 +979,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
-        </is>
-      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EWB Design Challenge | Aston University</t>
+          <t>Engineering - Simple English Wikipedia, the free encyclopedia</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
+          <t>https://simple.wikipedia.org/wiki/Engineering</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
+          <t>People who do engineering are called engineers. They learn engineering at a college or university. Engineers usually design or build things. Some engineers also use science, mathematics, and other skills to solve problems in technology.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1003,17 +1007,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
+          <t>Engineering.com</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
+          <t>https://www.engineering.com/</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
+          <t>6 days ago · Engineering information and connections for the global community of engineers. Find engineering webinars, research, articles, games, videos, jobs and calculators.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1021,26 +1025,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>ied@ied.org.uk</t>
-        </is>
-      </c>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South ...</t>
+          <t>Engineering | Definition, History, Functions, &amp; Facts |...</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
+          <t>https://www.britannica.com/technology/engineering</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
+          <t>Jul 27, 2026 · engineering, the application of science to the optimum conversion of the resources of nature to the uses of humankind.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1053,17 +1053,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Latest Community Engineering Design Competition Announced</t>
+          <t>1: What is Engineering? - Engineering LibreTexts</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
+          <t>https://eng.libretexts.org/Bookshelves/Introductory_Engineering/Introduction_to_Engineering_-_Thinking_Like_an_Engineer/01:_What_is_Engineering</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
+          <t>This page defines engineering as a distinct discipline from science and technology, highlighting its invisible yet impactful role in daily life and public trust. It discusses the historical …</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1071,22 +1071,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>info@libretexts.org</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of Engineering</t>
+          <t>Types of engineering explained with examples and career options</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://engineering.oregonstate.edu/academics/discover-engineering/types-engineering-explained-examples-and-career-options</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
+          <t>Explore every type of engineering — from architectural engineering to nuclear engineering — with real-world examples and career opportunities. Discover which engineering field might be a good fit for you.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1096,24 +1100,24 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
+          <t>askengineering@oregonstate.edu</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Engineering for people, that’s the challenge | Engineers Without Borders</t>
+          <t>What is engineering? | Live Science</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.rs-online.com/designspark/an-introduction-to-engineering-for-people-design-challenge</t>
+          <t>https://www.livescience.com/47499-what-is-engineering.html</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>That’s exactly what the annual Engineering for People Design Challenge asks participants to do. The competition, delivered in partnership by Engineers without Borders South Africa and Engineers Without Borders UK, encourages engineering students and those collaborating with engineers to broaden their awareness of how their decisions change the world.</t>
+          <t>Feb 28, 2022 · Engineering is the application of science and mathematics to solve problems. Engineers figure out how things work and find practical uses for scientific discoveries.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1121,22 +1125,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>help@magazinesdirect.com</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
+          <t>What is Engineering? Definition, introduction and a brief history</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
+          <t>https://pressbooks.bccampus.ca/engineeringinsociety/chapter/chapter-1/</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
+          <t>Engineering is the creative application of science, mathematical methods, and empirical evidence to the innovation, design, construction, and maintenance of structures, machines, materials, devices, systems, processes, and organizations.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1149,17 +1157,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>The status and challenges of industrial engineering in South Africa</t>
+          <t>What does an engineer do? - CareerExplorer</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.scielo.org.za/scielo.php?script=sci_arttext&amp;pid=S2224-78902016000100002</t>
+          <t>https://www.careerexplorer.com/careers/engineer/</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>This resulted in an identity crisis for industrial engineers, who were caught between the Industrial Revolution and the new challenges of the information system era [5]. In addition, within the South African context, where major socioeconomic changes have occurred since 1994, IEs have been exposed to a number of unique challenges that are non-existent or less dominant in other fields.</t>
+          <t>Choosing an engineering field is a significant decision that requires careful consideration of personal interests, skills, and career goals. Remember that your choice of engineering specialization does not have to be permanent.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1169,24 +1177,24 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>corne@sun.ac.za, admin@saiie.co.za</t>
+          <t>7877ad02a37049bcb77ea0be94bf5a9e@o168256.ingest.sentry.io</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
+          <t>2026 South Africa Engineering Competition - notices.ukzn.ac.za</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
+          <t>https://notices.ukzn.ac.za/content/GetFile.aspx?id=96047</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
+          <t>UKZN and Elsevier. If you are an engineering student (undergraduate or postgraduate), don't miss joining the challenge to solve real-world cases using Engineering Village and Knovel.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1199,17 +1207,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1217,22 +1225,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;area=2200&amp;ranking=Overall&amp;country=ZAF</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1240,22 +1252,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
+          <t>Engineering Students Rise to Industry Challenge - cput.ac.za</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
+          <t>https://www.cput.ac.za/component/rsblog/engineering-students-rise-to-industry-challenge?Itemid=101</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
+          <t>BeautyInTech, an African beauty technology and innovation company, challenged CPUT engineering students to reimagine the handheld liquid dispenser, and asked them for ideas. CPUT used the competition as a launchpad for something bigger - giving students the basis to tackle this challenge, and whatever innovation challenges come next.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1268,17 +1284,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>National Student Competition | ORSSA</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://www.orssa.org.za/studentcomp</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>National Student Competitions The Operations Research Society of South Africa The home of decision intelligence The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1286,22 +1302,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, email@example.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Engineering in South Africa: 24 Best universities Ranked</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://edurank.org/engineering/za/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
+          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1314,17 +1334,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2025</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2025</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1332,22 +1352,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>University of South Africa</t>
+          <t>Competitions - Enactus South Africa | National Expos, Challenges ...</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-promotes-globally-recognised-engineering-qualifications</t>
+          <t>https://enactusza.org/what-we-do/competitions</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Unisa promotes globally recognised engineering qualifications</t>
+          <t>Explore our national and international competitions that empower students to tackle challenges with entrepreneurial solutions and social impact at the core.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1355,22 +1379,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>xmadlanga@enactus.org, adminsa@enactus.org, liso@enactus.org, marketingsa@enactus.org</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
+          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
+          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
+          <t>Eligibility Benchmark Requirements The Africa Prize is open to individuals or teams based in sub-Saharan Africa with a scalable engineering innovation that demonstrates social or environmental impact potential. Applicants must: Be citizens ordinarily residing in a sub-Saharan African country. Be over 18 years old and fluent in English.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1383,17 +1411,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1406,7 +1434,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 (Internet ...</t>
+          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1416,7 +1444,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
+          <t>July 30, 2026 - TECHSPO Johannesburg 2026 is a two day technology expo taking place September 28th to 29th, 2026 at the luxurious Hyatt Regency Johannesburg, Johannesburg, South Africa. TECHSPO Johannesburg brings together developers, brands, marketers, technology ...</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1424,22 +1452,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>info@techspojoburg.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Africa Tech Festival</t>
+          <t>IT &amp; Technology Events in South Africa, List of all South Africa Technology Business Expo &amp; Events</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
+          <t>New York Small Business Expo (Spring)07 MayNew York , USA · AFROZUM Fair · 07-09 May · Johannesburg , South Africa · AFROZUM Fair07-09 MayJohannesburg , South Africa · Nigeria Industries &amp; Manufacturing Summit · 18-20 May · Abuja , Nigeria ...</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1447,26 +1479,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>support@informaconnect.com, customerservices@knect365.com, customerservices@informaconnect.com, salesenquiries@africatechfestival.com, dataprivacy@knect365.com, support@knect365.com, dataprivacy@informaconnect.com</t>
-        </is>
-      </c>
+      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 - 7, 2027 ...</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>The annual TECHSPO Cape Town 2027 Technology Expo returns October 6th to 7th, 2027 to the V&amp;A Waterfront Cape Town Avenue Conference Venue in Cape Town. TECHSPO Cape Town Technology Expo is the must-attend event to: Experience the Future of Technology &amp; Innovation Discover cutting-edge tech, game-changing tools, and innovators shaping tomorrow's digital world. See the latest advancements in ...</t>
+          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1476,24 +1504,24 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>info@techspocapetown.co.za</t>
+          <t>u003einfo@techspo.co, atinfo@techspo.coor</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
+          <t>Home - Mediatech Africa | South Africa</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://www.mediatech.co.za/</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
+          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1501,22 +1529,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>claire@mediatech.co.za, simon@mediatech.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology ExpoJohannesburg Technology Expo ...</t>
+          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://techspojoburg.co.za/johannesburg-technology-expo/</t>
+          <t>https://africatechnologyexpo.com/</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg is a 2-day technology expo taking place September 28 - 29, 2026 at the luxurious NH Johannesburg Sandton Hotel, Toronto, Ontario. TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
+          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1524,22 +1556,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>partner@africatechnologyexpo.com, johndoe@email.com, info@sparkafrica.co</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://10times.com/johannesburg-za/technology</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1547,22 +1583,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>info@techspocapetown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Tech Expo Africa - Enabling Development</t>
+          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://techexpo.africa/</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Tech Expo Africa is a social enterprise connecting African businesses with top tech and business leaders to drive innovation.</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1572,24 +1612,24 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>info@techexpo.africa</t>
+          <t>customerservices@knect365.com, dataprivacy@knect365.com, support@informaconnect.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, support@knect365.com, dataprivacy@informaconnect.com</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
+          <t>Discover Tech Conferences Events &amp; Activities in South Africa | Eventbrite</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
+          <t>Save this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South AfricaShare this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1597,26 +1637,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>enquiries@aiexpoafrica.com</t>
-        </is>
-      </c>
+      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>IT Indaba 2026 – Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>The inaugural 2025 IT Indaba promises to bring together 3,000+ IT professionals and tech influencers who are involved in the procurement of systems, tools, platforms and services, along with user experience developers who deal with the core processes and client interfaces of the business.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1629,17 +1665,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~…</t>
+          <t>IT &amp; Technology Events in Johannesburg, List of all Johannesburg Technology Business Expo &amp; Events in South Africa</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://www.industryevents.com/events/techspo-johannesburg-2026-technology-expo-internet-mobile-adtech-martech-saas</t>
+          <t>https://10times.com/johannesburg-za/technology</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Exhibitions &amp; Tradeshows on 22 Sept 2026 - 23 Sept 2026 in South Africa. TECHSPO Johannesburg - Where Business, Tech and Innovation Collide in…</t>
+          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1647,26 +1683,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>colleague@company.com, you@company.com, support@industryevents.com, your@email.com, events@techspojoburg.co.za</t>
-        </is>
-      </c>
+      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Maker Faire Africa - Wikipedia</t>
+          <t>Maker culture - Wikipedia</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Maker_Faire_Africa</t>
+          <t>https://en.wikipedia.org/wiki/Maker_culture</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Maker Faire Africa, Cairo, October 2011 Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds (Nubian Cheetah). Maker Faire Africa aims to engage with on ...</t>
+          <t>Maker culture encourages novel applications of technologies, and the exploration of intersections between traditionally separate domains and ways of working including metalworking, calligraphy, filmmaking, and computer programming.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1679,17 +1711,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Maker Faire - Wikipedia</t>
+          <t>MakerWorld: Download Free 3D Models</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Maker_Faire</t>
+          <t>https://makerworld.com/</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Maker Faire is a convention of do it yourself (DIY) enthusiasts established by Make magazine in 2006. Participants come from a wide variety of interests, such as robotics, 3D printing, computers, arts and crafts, and hacker culture.</t>
+          <t>Leading 3D printing model community for designers and makers. Download thousands of 3D models and stl models for free, and your No.1 option for multicolor 3D models.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1702,17 +1734,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Upcoming Faires - Maker Faire</t>
+          <t>MAKER Definition &amp; Meaning - Merriam-Webster</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://makerfaire.com/upcoming-faires/</t>
+          <t>https://www.merriam-webster.com/dictionary/maker</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
+          <t>4 days ago · The meaning of MAKER is one that makes. How to use maker in a sentence.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1722,24 +1754,24 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>fancybox_loading@2x.gif, pr@make.co, fancybox_sprite@2x.png, chosen-sprite@2x.png</t>
+          <t>325506e3332d487999567a7bc91d151d@bug-reporting-xalgha6.m-w.com, icon_FB_active@2x.png, 485x364@2x.jpg, poetry-3533-c1127e17993b9df02a3cd810ffa02f2a@2x.jpg, alt-68472e2f61868-12424-2bd56b87b38dfc9715277f54861cc33b@2x.jpg, icon_heart_default@2x.png, old%20words%20for%20stupid%20muttonhead-6190-50dfd94054d4595c843d6b1a81fc9196@2x.jpg, alt-68362132d8a91-12386-1aa35da5ca39141e6146bf929773f6a9@1x.jpg, sticky-social-icons-sprite@2x.png, icon.pron@2x.png, 485x364@1x.jpg, dog-running-with-ball-6949-8f7cb15ae040661a7f354b16b0ffd663@2x.jpg, poetry-3533-c1127e17993b9df02a3cd810ffa02f2a@1x.jpg, icon_heart_active@2x.png, skateboard-dog-hat-13601-75a1345ca35ed9e5634be2453f9f21a9@2x.jpg, alt-68362132d8a91-12386-1aa35da5ca39141e6146bf929773f6a9@2x.jpg, uncommon%20phobia%20doraphobia-1072-c1849a46b563601d175e5564be040cb9@1x.jpg, alt-657775b8b94e6-11003-656ebc9b8ac9f59662e8742aabd756b9@1x.jpg, icon_cite_default@2x.png, old%20words%20for%20stupid%20muttonhead-6190-50dfd94054d4595c843d6b1a81fc9196@1x.jpg, skateboard-dog-hat-13601-75a1345ca35ed9e5634be2453f9f21a9@1x.jpg, carrot@2x.png, man%20sitting%20in%20a%20chair%20looking%20confused-9966-606d9b0c372ee2138e77733a68b16b24@1x.jpg, icon.pron.hover@2x.png, alt-69987e038fe3e-13165-a718b91a08bcb238b5957488228d2428@2x.jpg, icon_cite_active@2x.png, alt-663a3d0c0f0fc-11473-5f855bd7e243e60d2c1bcf6ef08a4145@1x.jpg, alt-657775b8b94e6-11003-656ebc9b8ac9f59662e8742aabd756b9@2x.jpg, to%20whom%20it%20may%20concern%20typed%20on%20a%20typewriter-9898-33d8deaf608b55f91b0fde92abddf080@1x.jpg, uncommon%20phobia%20doraphobia-1072-c1849a46b563601d175e5564be040cb9@2x.jpg, mw-logo-245x245@1x.png, alt-69987e038fe3e-13165-a718b91a08bcb238b5957488228d2428@1x.jpg, to%20whom%20it%20may%20concern%20typed%20on%20a%20typewriter-9898-33d8deaf608b55f91b0fde92abddf080@2x.jpg, icon_FB_default@2x.png, alt-68472e2f61868-12424-2bd56b87b38dfc9715277f54861cc33b@1x.jpg, man%20sitting%20in%20a%20chair%20looking%20confused-9966-606d9b0c372ee2138e77733a68b16b24@2x.jpg, dog-running-with-ball-6949-8f7cb15ae040661a7f354b16b0ffd663@1x.jpg, alt-663a3d0c0f0fc-11473-5f855bd7e243e60d2c1bcf6ef08a4145@2x.jpg, WOTDpodcastlogo343W@2x.jpg</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Maker Faire |</t>
+          <t>MakerLab</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://makerfaire.com/</t>
+          <t>https://makerworld.com/en/makerlab</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
+          <t>No modeling skills required, no complex steps — with MakerLab, craft one-of-a-kind models with fun and ease. Create stunningly detailed 3D models from a single image with Tripo 3.1 Ultra. Create more detailed, lifelike busts with Make My Statue 2.0. From image to figurine, crafted in unique styles.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1747,26 +1779,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>pr@make.co</t>
-        </is>
-      </c>
+      <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Maker Faire Africa — Grokipedia</t>
+          <t>Chrome Music Lab - Song Maker</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://grokipedia.com/page/maker_faire_africa</t>
+          <t>https://musiclab.chromeexperiments.com/Song-Maker</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Maker Faire Africa Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
+          <t>Song Maker, an experiment in Chrome Music Lab, is a simple way for anyone to make and share a song.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1779,17 +1807,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
+          <t>Make: Community – A Community for Makers</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://capetown.makerfaire.com/</t>
+          <t>https://make.co/</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Jump into the Make: community and bring a Maker Faire to your town, city, or region! Spark curiosity, rally makers of all ages, and plug your local scene into a global movement fueled by creativity, resilience, innovation, and hands-on learning.</t>
+          <t>Since 2005, we’ve been the heartbeat of the global maker movement, inspiring millions through Make: Magazine, Maker Faire, and a thriving community of DIY innovators, tinkerers, and inventors.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1797,26 +1825,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>fancybox_loading@2x.gif, pr@make.co, fancybox_sprite@2x.png, chosen-sprite@2x.png</t>
-        </is>
-      </c>
+      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Home | Makers Fest</t>
+          <t>Maker Pro | Electronics Projects and Tutorials</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://www.makersfestival.co.za/</t>
+          <t>https://maker.pro/</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>On 8 &amp; 9 November 2025 at The Ostrich in Cape Town, join 2,000+ visitors each day for maker demos, a curated market, and family activities. It's Africa's first hands-on festival for creativity and craftsmanship — and everything you make, you take home.</t>
+          <t>Aug 18, 2026 · We provide a place for makers like you to share your designs, collaborate with one another, and learn how to take your product to market.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1824,26 +1848,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, warren@makersfestival.co.za, example@mysite.com</t>
-        </is>
-      </c>
+      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
+          <t>Make: DIY Projects and Ideas for Makers |</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
+          <t>https://makezine.com/</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>DIRECTIONS THE CAPE TOWN MAKER FAIRE The Lookout, V&amp;A Waterfront Granger Bay Boulevard, V &amp; A Waterfront, Cape Town, 8002, South Africa Get Directions Fri Aug 21, 13:00 - Sun Aug 23, 17:00 The Lookout, V&amp;A Waterfront View Map Payments are secure and encrypted</t>
+          <t>Make: celebrates your right to tweak, hack, and bend any technology to your will.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1851,22 +1871,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>pr@make.co</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>About | Explore Unique Maker Culture — Join Now — Makers Fair</t>
+          <t>Makeronline: Download Free 3D Printing Models and Print Now</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://www.makersfair.co.za/about</t>
+          <t>https://makeronline.com/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Discover South African and Pan-African craftsmanship at Makers Fair, a women-led event celebrating sustainable design, art, and culture. Join us today!</t>
+          <t>Discover and download free 3D printing models and files, start printing amazing designs today. Click to get started!</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1874,26 +1898,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>user@domain.com</t>
-        </is>
-      </c>
+      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Maker Faire groups | Meetup</t>
+          <t>Cricut® | Smart Cutting Machines, Materials, Tools &amp; More</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/topics/maker-faire/za/</t>
+          <t>https://cricut.com/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
+          <t>Design your idea, your way. Make it real with Cricut. Take our short quiz to discover which cutting machine is right for you. Our fits-in-any-space cutting machine for popular projects like full-color stickers, custom cards, T-shirts &amp; so much more.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1929,17 +1949,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.samsung.com/za/solvefortomorrow/</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1952,17 +1972,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/za/solvefortomorrow/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2075,17 +2095,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Applications for 2026 Samsung Solve For Tomorrow Now Open!</t>
+          <t>Competition - School Summit Africa</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://news.samsung.com/za/applications-for-2026-samsung-solve-for-tomorrow-now-open</t>
+          <t>https://schoolsummit.africa/competition/</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries open until 06 March 2026. This is a transformative ...</t>
+          <t>African Students Innovation Challenge The Inter-School STEM Innovations Challenge is a groundbreaking initiative aimed at nurturing creativity, critical thinking, and problem-solving skills among secondary school students through Science, Technology, Engineering, and Mathematics (STEM). This challenge is designed to foster real-world innovation by providing young learners with a platform to ...</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2098,17 +2118,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Samsung, DBE Announce Top 20 Schools Selected to Advance to the Next ...</t>
+          <t>Applications for 2026 Samsung Solve For Tomorrow Now Open!</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://news.samsung.com/za/samsung-dbe-announce-top-20-schools-selected-to-advance-to-the-next-level-of-2026-solve-for-tomorrow-competition</t>
+          <t>https://news.samsung.com/za/applications-for-2026-samsung-solve-for-tomorrow-now-open</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>At an event that took place on 14 April 2026, Samsung in partnership with the Department of Basic Education (DBE) officially announced the Top 20 schools that have been selected to advance to the next stages of the 2026 STEM-based (Science, Technology, Engineering and Mathematics) - Solve For Tomorrow (SFT) competition. In attendance was Mr. Simon Lee, the President and CEO of Samsung Africa ...</t>
+          <t>The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries open until 06 March 2026. This is a transformative ...</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2148,17 +2168,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Robotics Competition | WRO South Africa | Gauteng</t>
+          <t>Robotics for Good Youth Challenge South Africa</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>https://www.wrosa.co.za/</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa/</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>WRO South Africa ( World Robot Olympiad ) is a robotics competition which brings together young people from all over the world to develop their creativity and problem-solving skills.</t>
+          <t>This global competition is open to any individual or team willing to design, build, and code a robot to address the proposed challenge of disaster response in ...</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2168,24 +2188,24 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com</t>
+          <t>name@example.com</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
+          <t>Robotics for Good Youth Challenge - The Cortex Hub</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
+          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge, organized by ITU and The Cortex Hub, in partnership with Google.</t>
+          <t>The Robotics for Good Youth Challenge national competition will be held in Johannesburg, South Africa, at the Sandton Convention Centre on the 31st October 2025 ...</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2195,24 +2215,24 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>name@example.com</t>
+          <t>78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, info@thecortexhub.africa, 8c4075d5481d476e945486754f783364@sentry.io, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
+          <t>Robotics for Good Youth Challenge South Africa</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa/</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in a UN-based global robotics competition, focusing on the critical area of disaster response.</t>
+          <t>The Robotics for Good Youth Challenge is the leading UN-based global robotics championship, inviting students aged 10 to 18 to develop AI and robotics-based ...</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2229,17 +2249,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
+          <t>Oakhill teams celebrate robotics success - Knysna-Plett Herald</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
+          <t>https://www.knysnaplettherald.com/News/Article/Local-News/oakhill-teams-celebrate-robotics-success-202608271131</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in the leading UN-based global robotics competition, focusing on the critical area of agriculture and food security.</t>
+          <t>7 hours ago · The WRO is an international robotics competition in which learners design, build and programme autonomous robots to tackle technical challenges.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2247,26 +2267,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, info@thecortexhub.africa, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Roboticon 2026: South Africa Showcases Robotics for Culture, Education ...</t>
+          <t>Robotics for Good Youth Challenge South Africa - Limpopo</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://www.ubuntutimes.co.za/roboticon-2026-south-africa-showcases-robotics-for-culture-education-and-innovation/</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-limpopo/</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>The event, partnered with the World Robotics Olympiad, positions South Africa as a leader in educational robotics and entrepreneurial innovation." South Africa's robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation.</t>
+          <t>This global competition is open to any individual or team willing to design, build, and program a robot to address the proposed food security challenge on the ...</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2276,24 +2292,24 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>newspaper-rec300@2x.jpg, adverts@ubuntutimes.co.za</t>
+          <t>name@example.com</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Live Competitions — Nirvana Global Foundation</t>
+          <t>There is still hope : r/southafrica - Reddit</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://nirvanaglobalfoundation.org/competition.html</t>
+          <t>https://www.reddit.com/r/southafrica/comments/1889qd2/there_is_still_hope/</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Enjoy AI South Africa An international AI and robotics competition for young innovators. Teams build, program and compete with official ENJOY AI robotics kits across categories like Battle of Stars, Mining Expedition, Drone Cup and Inventions Trail — preparing learners for the global ENJOY AI stage.</t>
+          <t>Dec 1, 2023 · That's besides the robotics tournament we watched where the kids used Lego robotics sets to complete a programmed obstacle course. Just ...</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2301,26 +2317,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>you@email.com, coach@school.co.za, info@nirvanaglobalfoundation.org</t>
-        </is>
-      </c>
+      <c r="E77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>FIRST South Africa - Robotics Programs for School Children</t>
+          <t>FIRST Global Challenge</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://firstsa.org/</t>
+          <t>https://first.global/fgc/</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>FIRST® LEGO ® League FIRST® LEGO ® League guides youth through STEM learning and exploration at an early age. From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way.</t>
+          <t>The FIRST Global Challenge is an olympics-style, international robotics competition that takes place in a different country each year. ... South Africa ...</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2333,17 +2345,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
+          <t>Home | Roboticon 2026</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
+          <t>https://roboticon.resolute.education/</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop their creativity and problem-solving skills through challenging and educational robotics competitions.</t>
+          <t>Resolute Roboticon is a platform for schools to showcase their robotics and coding skills by competing in a fun, exciting competition.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2356,17 +2368,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Home | Roboticon 2026</t>
+          <t>Future robot rockstars of the Karoo! Winners of the 2026 World ...</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://roboticon.resolute.education/</t>
+          <t>https://www.facebook.com/SKASOUTHAFRICA/posts/future-robot-rockstars-of-the-karoo-winners-of-the-2026-world-robot-olympiad-pro/1677140377749131/</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Join us for the ultimate robotics showcase as Resolute proudly sponsors the World Robotics Olympiad (WRO) South Africa! This year, we're bringing together two worlds for the biggest robotics event of the year - Roboticon and the WRO Nationals, happening on the same day at the same venue.</t>
+          <t>Aug 17, 2026 · Winners of the 2026 World Robot Olympiad Provincial Competition at Carnarvon High School, Northern Cape — hosted with pride by NRF-SARAO. These ...</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2379,17 +2391,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ROBO-RUMBLE 2026 — Innovation in Motion</t>
+          <t>Wrapping up an incredible afternoon here at Carnarvon High ...</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://roborumble.net/</t>
+          <t>https://www.facebook.com/SKASOUTHAFRICA/videos/wrapping-up-an-incredible-afternoon-here-at-carnarvon-high-school-for-the-2026-w/1529989865024526/</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>South Africa's premier youth robotics &amp; technology competition. Robo Wars, Drone Racing, Grand Prix &amp; Innovation Challenge. August 2026.</t>
+          <t>Aug 15, 2026 · Mentors from Team South Africa discuss the impact of the FIRST Global robotics competition on youth development. They explain their ...</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2402,17 +2414,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Home [civilexpoits2026.com]</t>
+          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://civilexpoits2026.com/</t>
+          <t>https://www.engineeringnews.co.za/article/saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini-2022-09-13</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>This national civil engineering competition is your chance to put your engineering precision to the test and build real-world structural solutions. Step up and prove your skills on a national stage!</t>
+          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng. Twelve schools participated in the grand finale, which saw great, ...</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2422,24 +2434,24 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>civilexpo.sipilits@gmail.com</t>
+          <t>advertising@creamermedia.co.za, chanel@engineeringnews.co.za, subscriptions@creamermedia.co.za, newsletters@creamermedia.co.za, newsdesk@engineeringnews.co.za</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SAICE's 34th International Bridge Competition Inspires Tomorrow's ...</t>
+          <t>Engineering the Future: 16 schools compete in SAICE’s 33rd International Bridge Building Competition - SAICE</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://southafricatoday.net/lifestyle/education/saices-34th-international-bridge-competition-inspires-tomorrows-engineers/</t>
+          <t>https://saice.org.za/press-releases/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) hosted its 34th International Bridge Building Competition at the Midrand Conference Centre, bringing together 21 teams of high school learners from across South Africa, alongside international participants from Eswatini, Uganda, and Zimbabwe.</t>
+          <t>April 17, 2025 - The South African Institution of Civil Engineering (SAICE) hosted its 33rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2447,22 +2459,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>membership@saice.org.za, communications@saice.org.za, marketing@saice.org.za, accounts@saice.org.za, civilinfo@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
+          <t>Upcoming Civil Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://conferencealerts.co.in/south-africa/civil-engineering</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>International Civil engineering conferences in South africa 2025-2026 with invitation letter. A great opportunity to meet and learn from experts in your field.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2470,26 +2486,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
-        </is>
-      </c>
+      <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ICE Africa - Supporting Civil Engineers in Africa</t>
+          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
+          <t>https://www.crown.co.za/construction-world/marketplace/22289-saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>ICE Africa supports civil engineers across the continent, providing access to qualifications, training, and networking opportunities for professional growth.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2497,22 +2509,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>ernao@crown.co.za, constr@crown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
+          <t>Upcoming Civil Engineering Conferences in South Africa 2025</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://safcec.org.za/</t>
+          <t>https://www.allconferencealert.com/south-africa/civil-engineering-conference.html</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
+          <t>September 7, 2025 - Find the list of upcoming Civil Engineering conferences in South Africa 2025 with invitation an letter.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2520,26 +2536,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>communication@safcec.org.za</t>
-        </is>
-      </c>
+      <c r="E86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Engineering the Future: 16 schools compete in SAICE's 33rd ...</t>
+          <t>SWM Communications | SAICE recognises civil engineering research excellence through national student competition</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://southafricatoday.net/lifestyle/education/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
+          <t>https://swmcommunications.co.za/press-office/saice-recognises-civil-engineering-research-excellence-through-national-student-competition/</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) hosted its 33 rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland. The very first SAICE Bridge Building Competition was held in 1991, and it aimed to encourage high school learners to apply their knowledge of mathematics and science in a ...</t>
+          <t>April 1, 2026 - The event – which was sponsored by Sika, WorldsView, BVI, RIBCCS, and AF Consulting – was hosted at SAICE House in Midrand, Gauteng, and accredited for 0.2 CPD points. Students were invited to present their civil engineering university research and investigation project, which is part of the national curriculum for final year civil engineering undergraduate students.</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2547,22 +2559,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>info@swmcommunications.co.za, nthabeleng@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE)</t>
+          <t>ICE Africa – Supporting Civil Engineers in Africa | Institution of Civil Engineers (ICE)</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/SAICECIVIL/posts/enter-for-the-2026-saice-national-awardsnominations-are-open-and-were-looking-fo/1419225983581060/</t>
+          <t>https://www.ice.org.uk/about-us/what-we-do/ice-near-you/international/ice-africa/</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Enter for the 2026 SAICE National Awards! Nominations are open, and we're looking for the projects that truly made a difference where it matters most. The Community-Based Project of the Year is...</t>
+          <t>March 19, 2026 - organise seminars, workshops, visits and inter-universities competitions regarding civil engineering projects · For more information or to get involved please contact [email protected]. We have a volunteer member in South Africa who helps arrange ICE activities and promote our work.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2575,17 +2591,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Home - SAICE</t>
+          <t>Upcoming Civil engineering Conferences in Cape town 2025</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://saice.org.za/</t>
+          <t>https://conferencealerts.co.in/cape-town/civil-engineering</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) is the industry body for civil engineering professionals in South Africa. Our aim is to, promote growth, excellence and sustainability in the industry.</t>
+          <t>Civil engineering conferences in Cape town 2025 provide an exclusive global platform to meet and engage with experts and aspirants in various fields.</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2593,26 +2609,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>civilinfo@saice.org.za, marketing@saice.org.za, accounts@saice.org.za, membership@saice.org.za, executiveadmin@saice.org.za, communications@saice.org.za, barbara@avenue.co.za</t>
-        </is>
-      </c>
+      <c r="E89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
+          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2205</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>19 June 2026 marked an exciting celebration of Youth Month as aspiring young engineers from across Gauteng gathered for the 2026 SAICE Johannesburg Branch Schools Bridge Building Competition. Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in ...</t>
+          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2625,17 +2637,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Awards 2025 - SAICE</t>
+          <t>Civil Engineering Conferences in South Africa 2025/2026/2027 - Conference Index</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://saice.org.za/awards-2025/</t>
+          <t>https://conferenceindex.org/conferences/civil-engineering/south-africa</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Learn about SAICE's award categories, submission guidelines, key dates and how to nominate project and professionals.</t>
+          <t>Apr 13 International Conference on Architectural, Civil and Environmental Engineering (ICACEE) - Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2643,26 +2655,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>civilinfo@saice.org.za, marketing@saice.org.za, accounts@saice.org.za, membership@saice.org.za, communications@saice.org.za</t>
-        </is>
-      </c>
+      <c r="E91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>2026 South Africa Engineering Competition</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://notices.ukzn.ac.za/content/GetFile.aspx?id=96047</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+          <t>UKZN and Elsevier. If you are an engineering student (undergraduate or postgraduate), don't miss joining the challenge to solve real-world cases using Engineering Village and Knovel.</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2675,17 +2683,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2698,17 +2706,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2716,11 +2724,7 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2748,17 +2752,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>PDF 2026 South Africa Engineering Competition</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://library.ukzn.ac.za/wp-content/uploads/2026/08/About-Competition.pdf</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Best Regards, The 2026 SA Engineering Competition Team University of KwaZulu-Natal • Elsevier</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2766,22 +2770,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2798,17 +2806,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Competitions South Africa - Live Giveaways &amp; Prize Draws | Freehub</t>
+          <t>Mechanical Engineering Apprenticeship Jobs in South Africa ... - LinkedIn</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://freehub.co.za/competitions/</t>
+          <t>https://za.linkedin.com/jobs/mechanical-engineering-apprenticeship-jobs</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Browse live South African competitions, giveaways and prize draws. Find car, cash, voucher, tech and holiday competitions with clear entry rules and official source links.</t>
+          <t>Today's top 190 Mechanical Engineering Apprenticeship jobs in South Africa. Leverage your professional network, and get hired. New Mechanical Engineering Apprenticeship jobs added daily.</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2821,17 +2829,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>South African Competitions Worth Entering Today | Freehub</t>
+          <t>Competitions South Africa - Live Giveaways &amp; Prize Draws | Freehub</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://freehub.co.za/</t>
+          <t>https://freehub.co.za/competitions/</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Find South African competitions worth checking today, with curated picks, clear closing dates, entry-cost labels and official promoter links.</t>
+          <t>Browse live South African competitions, giveaways and prize draws. Find car, cash, voucher, tech and holiday competitions with clear entry rules and official source links.</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2890,17 +2898,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Cars4Mars - TryEngineering.org Powered by IEEE</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://tryengineering.org/event/cars4mars/</t>
+          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Cars4Mars is a robotics competition to design and build a Mars Rover Prototype. Competition starts – 1 May 2026 … hydraulics and electrical systems.</t>
+          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2913,17 +2921,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Join us as 55 young innovators showcase the engineering ...</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - SAIEE National Student Project Competition</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/ortsajhb/posts/join-us-as-55-young-innovators-showcase-the-engineering-coding-and-technology-so/1473351191493113/</t>
+          <t>https://www.saiee.org.za/calendar/EventDetails.aspx?eeid=29281</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Jun 26, 2026 · Join us as 55 young innovators showcase the engineering, coding, and technology solutions they've developed during the Young Engineers Movement ...</t>
+          <t>The SAIEE National Students Project Competition will be held at the North-West University (Potchefstroom Campus) on 21 November 2019</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2936,17 +2944,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>CMU-Africa students shine at global electronics conference</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - IEEE ZA 5G Competition</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://www.africa.engineering.cmu.edu/news/2026/01/16-ieee-conference.html</t>
+          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51397</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Jan 16, 2026 · SPEC 2025, held in Johannesburg, South Africa, is part of the Power Electronics Society, in the field of electrical engineering.</t>
+          <t>Form templates: Template for a Cover Sheet for the Competition on Ideas, Designs and Applications for 5G and Beyond South Africa (.docx) [Click to Download] Template for a Resume for the Student (.docx) [Click to Download] ... Help (FAQ) • Privacy Statement • Terms &amp; Conditions The SAIEE is ...</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2954,26 +2962,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>africa-info@andrew.cmu.edu</t>
-        </is>
-      </c>
+      <c r="E104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
+          <t>Student Design Competition | IEEE CASS</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
+          <t>https://ieee-cas.org/society-involvement/student-design-competition</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Student Chapter Design Contest (Africa) Serving the electrical energy conversion professional worldwide. Chapter Design Contest (Africa) Deadline: April 30, ...</t>
+          <t>CASS will reimburse the travel costs for the trip to ISCAS 2026 for the four finalists, one for each region - Regions 1-7 (USA and Canada), Region 8 (Europe, Middle East, Africa), Region 9 (Latin America), and Region 10 (Asia, Australia, Pacific), as well as ISCAS registration.</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2986,17 +2990,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Electricity challenges a top issue at African engineering ...</t>
+          <t>Top 100 Electrical Engineering Companies in South Africa (2026) | ensun</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://standardmicrogrid.com/content/electricity-challenges-top-issue-african-engineering-innovation-competition</t>
+          <t>https://ensun.io/search/electrical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Electricity challenges a top issue at African engineering innovation competition. Engineering innovations to boost off-grid power and stop electricity theft ... Missing: electrical | Show results with: electrical</t>
+          <t>The competitive landscape is marked by both established firms and emerging startups, driving innovation and efficiency. Additionally, South Africa’s position in the broader global market allows for potential collaborations and export opportunities, particularly in green technologies. Understanding these factors is essential for anyone looking to engage with the Electrical Engineering sector in South Africa, as they influence the overall business environment and potential for growth.</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -3009,17 +3013,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge Grand Finals</t>
+          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/posts/ewbsa_engineeringimpact-engineeringeducation-activity-7473789877885722624-QS1Q</t>
+          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Jun 19, 2026 · View organization page for Engineers Without Borders South Africa ... Software Developer•GDGoC FUTMinna Technical Lead•Electrical and Electronics ...</t>
+          <t>March 12, 2026 - At the Centre for High Performance Computing (CHPC) Conference hosted in Cape Town at the end of last year, four current fourth-year electrical engineering students were crowned national champions in the Student Cluster Competition for 2025.</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3032,17 +3036,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - SA Computing Olympiad stars hold their own in international competition</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
+          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51457</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Engineering for People, our flagship university design challenge, has won Silver in the QS Reimagine Education Awards 2025, recognising its impact in empowering ... Missing: electrical | Show results with: electrical</t>
+          <t>July 20, 2021 - For the other three South African team members, this was their first IOI. Brent Butkow finished ranked 342, Jean Weight finished in 287th position and Faran Steenkamp was ranked 280. In addition to the serious IOI contest days, host country Singapore arranged several fun events where Faran Steenkamp was placed third in the sponsored Code Cup, and won a cash prize of 200 USD.</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3055,17 +3059,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Real-world research: Engineering team designs South African ...</t>
+          <t>Electrical Engineering Conferences in South Africa 2025/2026/2027 - Conference Index</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>https://www.uwstout.edu/about-us/news-center/real-world-research-engineering-team-designs-south-african-trolley-system-science-students</t>
+          <t>https://conferenceindex.org/conferences/electrical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>May 15, 2025 · Cross-disciplinary teams present prototypes at Research Day, Engineers Without Borders' design challenge addressed by nearly 90 students.</t>
+          <t>Electrical Engineering Conferences in South Africa 2025 2026 2027 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and ...</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3073,26 +3077,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>frischj@uwstout.edu, dolanm@uwstout.edu</t>
-        </is>
-      </c>
+      <c r="E109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Stephen Theron's Post - LinkedIn</t>
+          <t>7 Electrical Engineering Degree Programs in South Africa - Study Abroad | educations.com</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/posts/stephen-theron_sasolsolarchallenge-tvetafrica-solarev-activity-7498683354414858240-K6vq</t>
+          <t>https://www.educations.com/electrical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>3 days ago · He's leading 12 fellow TVET students building a solar-powered EV for South Africa's national solar car challenge — a competition no SA team has ...</t>
+          <t>Find the best fit for you - Compare 7 in Engineering Programs Electrical Engineering in South Africa for 2025/2026</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3100,26 +3100,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>retshegofaditswemashigo55@gmail.com, nretshegofaditswemashigo55@gmail.com</t>
-        </is>
-      </c>
+      <c r="E110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>WE HAVE A WINNER! What happens when you combine ...</t>
+          <t>Electrical Engineering in South Africa: Best universities Ranked</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/100095556341859/posts/-𝑾𝑬-𝑯𝑨𝑽𝑬-𝑨-𝑾𝑰𝑵𝑵𝑬𝑹-what-happens-when-you-combine-industrial-engineering-ai-a-big-/1251805024681364/</t>
+          <t>https://edurank.org/engineering/electrical/za/</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Aug 12, 2026 · Competing against Industrial Engineering undergraduates from universities across South Africa, the challenge was to develop a solution using ...</t>
+          <t>March 2, 2025 - Below is the list of 24 best universities for Electrical Engineering in South Africa ranked based on their research performance: a graph of 827K citations received by 40.9K academic papers made by these universities was used to calculate ratings and create the top.</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3142,7 +3138,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Jun 26, 2026 · Join us as 55 young innovators showcase the engineering, coding, and technology solutions during the Young Engineers Movement (YEM) Hackathon. ...</t>
+          <t>Jun 26, 2026 · Join us as 55 young innovators showcase the engineering, coding, and technology solutions they've developed during the Young Engineers Movement ...</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -3165,7 +3161,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Jun 17, 2026 · The event is a multi-day programme hosted by ORT South Africa running from 22 to 26 June 2026 in Johannesburg.</t>
+          <t>Jun 17, 2026 · Learners from underserved South African schools will showcase their engineering and technology skills at the YEM Hackathon!</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -3175,24 +3171,24 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>197912-featured-75x75@2x.jpeg, 197912-featured-75x75@2.5x.jpeg, 198065-featured-75x75@1.5x.jpg, 198065-featured-75x75@2.5x.jpg, 198167-featured-75x75@1.5x.jpg, 198032-featured-75x75@2.5x.jpg, 198065-featured-75x75@3x.jpg, 197912-featured-75x75@3x.jpeg, 198032-featured-75x75@1.5x.jpg, 198065-featured-75x75@2x.jpg, 198167-featured-75x75@2x.jpg, 198032-featured-75x75@3x.jpg, 197912-featured-75x75@1.5x.jpeg, 198167-featured-75x75@2.5x.jpg, 198167-featured-75x75@3x.jpg, 198032-featured-75x75@2x.jpg</t>
+          <t>198115-featured-75x75@3x.jpg, 198201-featured-75x75@3x.jpg, 198201-featured-75x75@1.5x.jpg, 198115-featured-75x75@2x.jpg, 198119-featured-75x75@2.5x.jpg, 198119-featured-75x75@2x.jpg, 198201-featured-75x75@2x.jpg, 198208-featured-75x75@3x.jpg, 198208-featured-75x75@2.5x.jpg, 198119-featured-75x75@1.5x.jpg, 198191-featured-75x75@2.5x.jpg, 198208-featured-75x75@1.5x.jpg, 198115-featured-75x75@1.5x.jpg, 198191-featured-75x75@3x.jpg, 198201-featured-75x75@2.5x.jpg, 198119-featured-75x75@3x.jpg, 198208-featured-75x75@2x.jpg, 198115-featured-75x75@2.5x.jpg, 198191-featured-75x75@1.5x.jpg, 198191-featured-75x75@2x.jpg</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>ORT South Africa's Young Engineers Movement Hackathon</t>
+          <t>Tech hackathons in Africa 2026 / 2027 - dev.events</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/posts/good-things-guy_55-learners-from-underserved-schools-to-shine-activity-7473009611185217539-Ye7_</t>
+          <t>https://dev.events/hackathons/AF/tech</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Jun 17, 2026 · The event is a multi-day programme hosted by ORT South Africa running from 22 to 26 June 2026 in Johannesburg.</t>
+          <t>Best Tech hackathons in Africa 2026 / 2027 · The Principal Dev – Masterclass for Tech Leads · Clean Architecture Masterclass · DSH Pitch · GNSS 4 Disaster Risk ...</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3205,17 +3201,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Tech hackathons in Africa 2026 / 2027 - dev.events</t>
+          <t>Faurecia South Africa's Post - LinkedIn</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>https://dev.events/hackathons/AF/tech</t>
+          <t>https://www.linkedin.com/posts/forvia-faurecia-south-africa_calling-all-future-engineers-join-activity-7437386283603279872-NGpQ</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Tech hackathons in Africa 2026 ・ for experienced software engineers. Feb 27 - Dec 25 ・ the #1 tech conference listing. curated by tech community.</t>
+          <t>Mar 10, 2026 · Join FORVIA Faurecia South Africa's Engineering Hackathon FORVIA South Africa is searching for motivated, curious, and driven young engineers ...</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3228,17 +3224,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Ocean Hackathon® Cape Town - Global Fund for Coral Reefs</t>
+          <t>Global South AI Safety Hackathon | Apart Research</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>https://globalfundcoralreefs.org/reef-plus/events/ocean-hackathon-cape-town/</t>
+          <t>https://apartresearch.com/sprints/global-south-ais-hackathon-2026-06-19-to-2026-06-21</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>The Ocean Hackathon® is a 48-hour innovation sprint, teams of hackers, engineers, When? 17–19 October 2025 🌍 Where? Cape Town, South Africa</t>
+          <t>Jun 19, 2026 · The Global South AI Safety Hackathon brings together researchers, engineers, and policy professionals across Latin America, Africa, and Asia ...</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -3248,24 +3244,24 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>thando@oceanhub.africa, _@astro-renderers.BsLwzaai.css, mohammad.al-tawaha@undp.org</t>
+          <t>sprints@apartresearch.com, example@email.com</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Global South AI Safety Hackathon | Apart Research</t>
+          <t>Africa Ignite Hackathon - HackerEarth</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>https://apartresearch.com/sprints/global-south-ais-hackathon-2026-06-19-to-2026-06-21</t>
+          <t>https://www.hackerearth.com/challenges/hackathon/africa-ignite-hackathon/</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Jun 19, 2026 · The Global South AI Safety Hackathon brings together researchers, engineers, and policy professionals across Latin America, Africa, and Asia ...</t>
+          <t>The Africa Ignite Hackathon is a regional innovation challenge designed to empower developers, startups, and tech enthusiasts across Sub-Saharan Africa to build ...</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3273,26 +3269,22 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t>example@email.com, sprints@apartresearch.com</t>
-        </is>
-      </c>
+      <c r="E117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Africa Ignite Hackathon - HackerEarth</t>
+          <t>Siemens Energy South Africa Hackathon - Facebook</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>https://www.hackerearth.com/challenges/hackathon/africa-ignite-hackathon/</t>
+          <t>https://www.facebook.com/SiemensEnergy/videos/siemens-energy-south-africa-hackathon/966581709250326/</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>The Africa Ignite Hackathon is a regional innovation challenge designed to empower developers, startups, and tech enthusiasts across Sub-Saharan Africa</t>
+          <t>May 7, 2026 · Students from across Gauteng, South Africa joined the Siemens Energy South Africa Just Energy Transition (JET) Hackathon to take on ...</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3305,17 +3297,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Siemens Energy South Africa Hackathon - Facebook</t>
+          <t>Tech job opportunity AND money to be won : r/southafrica</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/SiemensEnergy/videos/siemens-energy-south-africa-hackathon/966581709250326/</t>
+          <t>https://www.reddit.com/r/southafrica/comments/x8umad/tech_job_opportunity_and_money_to_be_won/</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>May 7, 2026 · Students from across Gauteng, South Africa joined the Siemens Energy South Africa Just Energy Transition (JET) Hackathon to take on ...</t>
+          <t>Sep 8, 2022 · Boston Consulting Group (BCG) is holding a hackathon on 28-29 October across its offices in Europe, Middle East, South America and Africa to ...</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -3328,17 +3320,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Tech job opportunity AND money to be won : r/southafrica</t>
+          <t>W3Node Conference &amp; Hackathon</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/southafrica/comments/x8umad/tech_job_opportunity_and_money_to_be_won/</t>
+          <t>https://w3node.io/</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Sep 8, 2022 · Boston Consulting Group (BCG) is holding a hackathon on 28-29 October across its offices in Europe, Middle East, South America and Africa to ...</t>
+          <t>South Africa. November. 12-14 2026. Africa's premier Developer conference. //About. w3node. Welcome to Africa's Premier Web3 Developer Conference and Hackathon.</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -3346,7 +3338,11 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr"/>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>hello@w3africa.io</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">

</xml_diff>

<commit_message>
Update competition data 2026-09-01
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -466,7 +466,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>info@zasdc.org, user@domain.com</t>
+          <t>user@domain.com, info@zasdc.org</t>
         </is>
       </c>
     </row>
@@ -539,24 +539,24 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>198115-featured-75x75@3x.jpg, 198201-featured-75x75@3x.jpg, 198201-featured-75x75@1.5x.jpg, 198115-featured-75x75@2x.jpg, 198119-featured-75x75@2.5x.jpg, 198119-featured-75x75@2x.jpg, 198201-featured-75x75@2x.jpg, 198208-featured-75x75@3x.jpg, 198208-featured-75x75@2.5x.jpg, 198119-featured-75x75@1.5x.jpg, 198191-featured-75x75@2.5x.jpg, 198208-featured-75x75@1.5x.jpg, 198115-featured-75x75@1.5x.jpg, 198191-featured-75x75@3x.jpg, 198201-featured-75x75@2.5x.jpg, 198119-featured-75x75@3x.jpg, 198208-featured-75x75@2x.jpg, 198115-featured-75x75@2.5x.jpg, 198191-featured-75x75@1.5x.jpg, 198191-featured-75x75@2x.jpg</t>
+          <t>198274-featured-75x75@2.5x.jpg, 198366-featured-75x75@3x.jpg, 198322-featured-75x75@2.5x.jpg, 198322-featured-75x75@2x.jpg, 198274-featured-75x75@2x.jpg, 198261-featured-75x75@1.5x.jpg, 198366-featured-75x75@1.5x.jpg, 198322-featured-75x75@3x.jpg, 198261-featured-75x75@2.5x.jpg, 198274-featured-75x75@1.5x.jpg, 197529-featured-75x75@2.5x.jpeg, 198322-featured-75x75@1.5x.jpg, 198261-featured-75x75@2x.jpg, 198366-featured-75x75@2.5x.jpg, 197529-featured-75x75@1.5x.jpeg, 198261-featured-75x75@3x.jpg, 198274-featured-75x75@3x.jpg, 197529-featured-75x75@3x.jpeg, 198366-featured-75x75@2x.jpg, 197529-featured-75x75@2x.jpeg</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>South African Learners Win NASA Space Engineering ...</t>
+          <t>The 2026 South Africa Engineering Competition Online - LibCal</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/posts/business-tech-africa_seven-south-african-learners-made-history-activity-7492930299115528192-HOEY</t>
+          <t>https://ukzn.libcal.com/event/17342211</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Aug 11, 2026 · Seven South African learners made history by winning an international space engineering competition at NASA - National Aeronautics and Space ...</t>
+          <t>From: 2:30 PM, Tuesday, September 1, 2026 ; To: 4:00 PM, Tuesday, September 15, 2026 ; Time Zone: Central Africa Time (change) ; Online: This is an online event.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -564,22 +564,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>HlongwaneS2@ukzn.ac.za</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>The 2026 South Africa Engineering Competition Online - LibCal</t>
+          <t>South African Learners Win NASA Space Engineering ...</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://ukzn.libcal.com/event/17342211</t>
+          <t>https://www.linkedin.com/posts/business-tech-africa_seven-south-african-learners-made-history-activity-7492930299115528192-HOEY</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>From: 2:30 PM, Tuesday, September 1, 2026 ; To: 4:00 PM, Tuesday, September 15, 2026 ; Time Zone: Central Africa Time (change) ; Online: This is an online event.</t>
+          <t>Aug 11, 2026 · Seven South African learners made history by winning an international space engineering competition at NASA - National Aeronautics and Space ...</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -587,11 +591,7 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>HlongwaneS2@ukzn.ac.za</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -692,17 +692,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Africa Tech Festival</t>
+          <t>AI Expo Africa 2026 - Africa-Europe Innovation Platform</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://www.africaeuropeinnovation.net/event/ai-expo-africa-2026/</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
+          <t>AI Expo Africa is the continent's largest Artificial Intelligence and Intelligent Automation trade show and conference, connecting enterprise buyers with ... Missing: exhibition | Show results with: exhibition</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -710,26 +710,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>customerservices@knect365.com, dataprivacy@knect365.com, support@informaconnect.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, support@knect365.com, dataprivacy@informaconnect.com</t>
-        </is>
-      </c>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
+          <t>Africa Tech Festival</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/tradeshows</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>South Africa trade shows, find and compare 965 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 169 upcoming expos in 2026-2027 1. Investment Showcase, 2. South African Cheese Festival And ...</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech ...</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -737,22 +733,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>dataprivacy@knect365.com, dataprivacy@informaconnect.com, support@knect365.com, salesenquiries@africatechfestival.com, customerservices@knect365.com, customerservices@informaconnect.com, support@informaconnect.com</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
+          <t>Africa Automation Technology Fair</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://www.africaautomationtechnologyfair.com/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AI Expo Africa 2026 - Join the Largest AI Event &amp; Trade Community in Africa TODAY! Our business audience is a buyer / supplier focused community and comprised of Enterprise decision makers / CxOs, allied to AI Cloud platform providers, Tier 1 / 2 deployment &amp; service providers, AI start ups / innovators, investors, educators, government and AI ecosystem community builders.</t>
+          <t>The inaugural Africa Automation Indaba, taking place from 13–14 May 2026, is a landmark conference dedicated to advancing automation, process control, and ...</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -762,24 +762,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>enquiries@aiexpoafrica.com</t>
+          <t>aatf@rxglobal.com</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Exhibition | Innovation Festival Durban | South Africa</t>
+          <t>AI Expo Africa 2026, 28-29th Oct JHB SA (@ai_expo_africa)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://www.innovationfestival.durban/exhibition</t>
+          <t>https://www.instagram.com/ai_expo_africa/</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Exhibition Opportunities BENEFITS FOR YOUR PARTICIPATING IN THE EXHIBITION: An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities. Opportunity to market your Brand. Exposure on print, electronic and social media platforms.</t>
+          <t>Africa's largest Enterprise AI &amp; Intelligent Automation Trade Show &amp; Conference uniting buyers, suppliers &amp; investors in Africa EARLY ON SALE NOW. Follow.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -787,26 +787,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>8c4075d5481d476e945486754f783364@sentry.io, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, sithabile@innovate.durban, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, Erika@innovate.durban, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Electra Mining Africa | South Africa's Leading Mining and Industrial ...</t>
+          <t>AI for Good Impact Africa - ITU</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://www.electramining.co.za/</t>
+          <t>https://aiforgood.itu.int/event/impact-africa/</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>South Africa's Leading Mining Exhibition 7 - 11 September 2026 | JHB Expo Centre Nasrec Discover the biggest mining, industrial, electrical and power event in Africa. Connect with solution-providers, explore the latest technology and meet decision-makers who shape the future of the industry.</t>
+          <t>AI for Good Impact Africa will take place on 31 October in Johannesburg and coincide with the AI Expo Africa on 29-31 October 2025. Schedule. 09:30-09:45.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -816,24 +812,24 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>john@email.com</t>
+          <t>name@example.com</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
+          <t>2026 ISMRM-ISMRT Annual Meeting and Exhibition - Forum I</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://echo.ismrm.org/program/ISMRM2026/at-a-glance/session/220</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
+          <t>2026 ISMRM-ISMRT Annual Meeting and Exhibition • 09-14 May 2026 • Cape Town, South Africa. ISMRT Education Session. Forum I: Innovators and Innovations in ...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -846,17 +842,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ELENEX Africa Johannesburg 2026 - TradeFairDates</t>
+          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://www.tradefairdates.com/ELENEX-Africa-M6915/Johannesburg.html</t>
+          <t>https://10times.com/southafrica/tradeshows</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>The fair is deeply rooted in the dynamics and industrial growth of Johannesburg and demonstrates South Africa's role as a leading center for technological innovation in Africa.</t>
+          <t>TECHSPO Cape Town is an influential technology expo that serves as a hub where business, tech, and innovation converge. Taking place at the Avenue Conference ...</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -869,17 +865,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>T&amp;D Africa Conference &amp; Expo | Transmission &amp; Distribution</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://africaenergyindaba.com/events/td-africa/</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Big Data and Business Analytics Innovation Conference Johannesburg, South Africa IT &amp; Technology 100 Members Wed, 28 - Thu, 29 Oct 2026</t>
+          <t>The T&amp;D Africa (Transmission &amp; Distribution) Conference &amp; Expo is set to take place from 2 - 4 March 2027 at CTICC, Cape Town South Africa.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -892,17 +888,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Exhibitions in South Africa 2026-2027 - ExpoTobi</t>
+          <t>National Skills Fund at Innovation Expo and Youth Colloquium ...</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://expotobi.com/country/south-africa/exhibitions</t>
+          <t>https://www.facebook.com/NSF.1998/posts/join-us-today-as-we-go-big-at-the-innovation-expo-youth-colloquiumthe-national-s/1087629487109320/</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>All Exhibitions in South Africa 2026-2027 | Full and accurate description of events for various business sectors | Schedule, tickets, travel arrangements and participation</t>
+          <t>1 day ago · The Expo, which is in its third year running, is taking place on 9-18 June 2017. Including the NPA, over 200 exhibitors are taking part. They ...</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -915,17 +911,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AI Expo Africa 2026 - Africa-Europe Innovation Platform</t>
+          <t>“AfriHack 2026 Kicks Off with Major Partnerships Driving Digital ...</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.africaeuropeinnovation.net/event/ai-expo-africa-2026/</t>
+          <t>https://www.ednews.africa/p/afrihack-2026-kicks-off-with-major</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AI Expo Africa is the continent's largest Artificial Intelligence and Intelligent Automation trade show and conference, connecting enterprise buyers with ...</t>
+          <t>15 minutes ago · AfriHack 2026 will be held in two cities: Johannesburg (4–6 September) at the CAPACITI Hub in Braamfontein, and Cape Town (18–20 September) at ...</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -933,22 +929,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ednews.africa@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Engineering - Wikipedia</t>
+          <t>Engineering For People Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Engineering</t>
+          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>The steam engine, the major driver in the Industrial Revolution, underscores the importance of engineering in modern history. This beam engine is on display in the Technical University of Madrid. Engineering is the practice of systematically applying natural science and mathematics to design and improve systems, devices, or processes that solve problems under constraints. It is typically ...</t>
+          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -956,22 +956,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Engineer - Wikipedia</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Engineer</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Engineers develop new technological solutions. During the engineering design process, the responsibilities of the engineer may include defining problems, conducting and narrowing research, analyzing criteria, finding and analyzing solutions, and making decisions.</t>
+          <t>In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community's challenges and how community members view the impact of these challenges on their daily lives.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -979,22 +983,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Engineering - Simple English Wikipedia, the free encyclopedia</t>
+          <t>PDF Engineering ENGINEERING FOR PEOPLE Design challenge DESIGN CHALLENGE ...</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://simple.wikipedia.org/wiki/Engineering</t>
+          <t>https://www.ewb-uk.org/wp-content/uploads/2024/08/2024_25_Engineering_for_People_Design_Challenge_Makers_Valley.pdf</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>People who do engineering are called engineers. They learn engineering at a college or university. Engineers usually design or build things. Some engineers also use science, mathematics, and other skills to solve problems in technology.</t>
+          <t>Makers Makers Valley Valley Johannesburg, Johannesburg, South South Africa Africa The Engineering for People Design Challenge has been delivered in the UK and Ireland since 2011, South Africa and the USA since 2019, and Cameroon in 2022. It is an educational programme based on a concept developed originally by Engineers Without Borders Australia. The production of this document has been led by ...</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1007,17 +1015,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Engineering.com</t>
+          <t>Engineering for People Design Challenge returns to Johannesburg!</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.engineering.com/</t>
+          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>6 days ago · Engineering information and connections for the global community of engineers. Find engineering webinars, research, articles, games, videos, jobs and calculators.</t>
+          <t>Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1030,17 +1038,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Engineering | Definition, History, Functions, &amp; Facts |...</t>
+          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.britannica.com/technology/engineering</t>
+          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Jul 27, 2026 · engineering, the application of science to the optimum conversion of the resources of nature to the uses of humankind.</t>
+          <t>The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1048,22 +1056,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>team@crowdsolve.net</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1: What is Engineering? - Engineering LibreTexts</t>
+          <t>Engineering for People Design Challenge | Department of Engineering</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://eng.libretexts.org/Bookshelves/Introductory_Engineering/Introduction_to_Engineering_-_Thinking_Like_an_Engineer/01:_What_is_Engineering</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>This page defines engineering as a distinct discipline from science and technology, highlighting its invisible yet impactful role in daily life and public trust. It discusses the historical …</t>
+          <t>This year's design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but under-resourced neighbourhood on the eastern edge of Johannesburg. Home to around 46,000 people, Makers Valley is a community rich in creativity, activism ...</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1073,24 +1085,24 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>info@libretexts.org</t>
+          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Types of engineering explained with examples and career options</t>
+          <t>Bambasonke Design Challenge Empowers Engineering Students in SA - LinkedIn</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://engineering.oregonstate.edu/academics/discover-engineering/types-engineering-explained-examples-and-career-options</t>
+          <t>https://www.linkedin.com/posts/activity-7470764395091001345-GwCR</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Explore every type of engineering — from architectural engineering to nuclear engineering — with real-world examples and career opportunities. Discover which engineering field might be a good fit for you.</t>
+          <t>By joining forces, student engineers have the chance to bridge societal gaps, uplift those in vulnerable positions, and contribute to building a more inclusive and prosperous South Africa.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1098,26 +1110,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>askengineering@oregonstate.edu</t>
-        </is>
-      </c>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>What is engineering? | Live Science</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.livescience.com/47499-what-is-engineering.html</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Feb 28, 2022 · Engineering is the application of science and mathematics to solve problems. Engineers figure out how things work and find practical uses for scientific discoveries.</t>
+          <t>STEM-focused NGO Engineers Without Borders UK has launched its 2025 Engineering for People Design Challenge. Organised in conjunction with sister organisation Engineers Without Borders South Africa, as well as the Makers Valley Partnership, this year's challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1125,26 +1133,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>help@magazinesdirect.com</t>
-        </is>
-      </c>
+      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>What is Engineering? Definition, introduction and a brief history</t>
+          <t>Engineers Without Borders | OU Design Show 2025</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://pressbooks.bccampus.ca/engineeringinsociety/chapter/chapter-1/</t>
+          <t>https://www.oudesignshow.org/designathon</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Engineering is the creative application of science, mathematical methods, and empirical evidence to the innovation, design, construction, and maintenance of structures, machines, materials, devices, systems, processes, and organizations.</t>
+          <t>Makers Valley is a vibrant community of makers, creatives, and social enterprises in Johannesburg, South Africa. Engineers Without Borders UK has partnered with Makers Valley to engage students in design challenges focused on addressing local challenges and promoting sustainable development.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1157,17 +1161,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>What does an engineer do? - CareerExplorer</t>
+          <t>Engineering for People Design Challenge</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.careerexplorer.com/careers/engineer/</t>
+          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Choosing an engineering field is a significant decision that requires careful consideration of personal interests, skills, and career goals. Remember that your choice of engineering specialization does not have to be permanent.</t>
+          <t>Aligned with UNESCO's call for greater complexity in engineering education, the Design Challenge uses project-based learning to immerse students in real-world ...</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1175,11 +1179,7 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>7877ad02a37049bcb77ea0be94bf5a9e@o168256.ingest.sentry.io</t>
-        </is>
-      </c>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>UKZN and Elsevier. If you are an engineering student (undergraduate or postgraduate), don't miss joining the challenge to solve real-world cases using Engineering Village and Knovel.</t>
+          <t>UKZN and Elsevier. If you are an engineering student (undergraduate or postgraduate), don’t miss joining the challenge to solve real-world cases using Engineering Village and Knovel.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1244,7 +1244,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1261,17 +1261,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Engineering Students Rise to Industry Challenge - cput.ac.za</t>
+          <t>National Student Competition | ORSSA</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://www.cput.ac.za/component/rsblog/engineering-students-rise-to-industry-challenge?Itemid=101</t>
+          <t>https://www.orssa.org.za/studentcomp</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>BeautyInTech, an African beauty technology and innovation company, challenged CPUT engineering students to reimagine the handheld liquid dispenser, and asked them for ideas. CPUT used the competition as a launchpad for something bigger - giving students the basis to tackle this challenge, and whatever innovation challenges come next.</t>
+          <t>The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1279,22 +1279,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, email@example.com, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>National Student Competition | ORSSA</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://www.orssa.org.za/studentcomp</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>National Student Competitions The Operations Research Society of South Africa The home of decision intelligence The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
+          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1302,26 +1306,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, email@example.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
+          <t>Sep 4, 2025 · The Africa Prize for Engineering Innovation is open to individuals or teams based in sub-Saharan Africa who have a scalable engineering innovation with social or environmental impact potential.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1329,22 +1329,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
+          <t>Competitions – Enactus South Africa | National Expos ...</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://enactusza.org/what-we-do/competitions</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>Explore our national and international competitions that empower students to tackle challenges with entrepreneurial solutions and social impact at the core.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1354,24 +1358,24 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+          <t>liso@enactus.org, marketingsa@enactus.org, adminsa@enactus.org, xmadlanga@enactus.org</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Competitions - Enactus South Africa | National Expos, Challenges ...</t>
+          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://enactusza.org/what-we-do/competitions</t>
+          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Explore our national and international competitions that empower students to tackle challenges with entrepreneurial solutions and social impact at the core.</t>
+          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1379,26 +1383,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>xmadlanga@enactus.org, adminsa@enactus.org, liso@enactus.org, marketingsa@enactus.org</t>
-        </is>
-      </c>
+      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
+          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
+          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Eligibility Benchmark Requirements The Africa Prize is open to individuals or teams based in sub-Saharan Africa with a scalable engineering innovation that demonstrates social or environmental impact potential. Applicants must: Be citizens ordinarily residing in a sub-Saharan African country. Be over 18 years old and fluent in English.</t>
+          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1411,17 +1411,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;area=2200&amp;ranking=Overall&amp;country=ZAF</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1434,17 +1434,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>Africa Tech Festival</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>https://techspojoburg.co.za/</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>July 30, 2026 - TECHSPO Johannesburg 2026 is a two day technology expo taking place September 28th to 29th, 2026 at the luxurious Hyatt Regency Johannesburg, Johannesburg, South Africa. TECHSPO Johannesburg brings together developers, brands, marketers, technology ...</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech ...</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1454,24 +1454,24 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>info@techspojoburg.co.za</t>
+          <t>dataprivacy@knect365.com, dataprivacy@informaconnect.com, support@knect365.com, salesenquiries@africatechfestival.com, customerservices@knect365.com, customerservices@informaconnect.com, support@informaconnect.com</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa, List of all South Africa Technology Business Expo &amp; Events</t>
+          <t>TECHSPO Technology Expo</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://techspo.co/</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>New York Small Business Expo (Spring)07 MayNew York , USA · AFROZUM Fair · 07-09 May · Johannesburg , South Africa · AFROZUM Fair07-09 MayJohannesburg , South Africa · Nigeria Industries &amp; Manufacturing Summit · 18-20 May · Abuja , Nigeria ...</t>
+          <t>Johannesburg, South Africa. October 1 – 2, 2026. Cape Town, South Africa. October 8 – 9, 2026. Philadelphia, PA. October 14 – 15, 2026. Miami, FL. October 22 – ...</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1484,17 +1484,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
+          <t>Tech conferences in South Africa 2026 / 2027 - dev.events</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
+          <t>https://dev.events/AF/ZA/tech</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
+          <t>Best Tech conferences in South Africa 2026 / 2027 · The Principal Dev – Masterclass for Tech Leads · Clean Architecture Masterclass · Escape 2026 · HR World Summit ...</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1502,26 +1502,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>u003einfo@techspo.co, atinfo@techspo.coor</t>
-        </is>
-      </c>
+      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Home - Mediatech Africa | South Africa</t>
+          <t>IT &amp; Technology Events in South Africa | 10times</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://www.mediatech.co.za/</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
+          <t>The KZN AI Summit is set to take place in the vibrant city of Durban, South Africa, from September 3 to September 4, 2026. This premier event will gather ...</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1529,26 +1525,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>claire@mediatech.co.za, simon@mediatech.co.za</t>
-        </is>
-      </c>
+      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
+          <t>TECHSPO Cape Town 2026 - Vendelux</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://africatechnologyexpo.com/</t>
+          <t>https://vendelux.com/app/event/techspo-cape-town-2026/09979c20-a8e9-4c48-bd76-bda4fa906dae</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
+          <t>TECHSPO Cape Town 2026 welcomes innovators, marketers, and tech enthusiasts to the V&amp;A Waterfront Cape Town Avenue Conference Venue on October 1-2. Over these ...</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1558,24 +1550,24 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>partner@africatechnologyexpo.com, johndoe@email.com, info@sparkafrica.co</t>
+          <t>support@vendelux.com</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>Mediatech Africa (@mediatechafrica) · Johannesburg - Instagram</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://www.instagram.com/mediatechafrica/</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
+          <t>Africa's largest Pro AV, Film, Broadcast &amp; Live Event Tech Expo. 27 - 29 June 2028, Johannesburg .</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1583,26 +1575,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>info@techspocapetown.co.za</t>
-        </is>
-      </c>
+      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~…</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://www.industryevents.com/events/techspo-johannesburg-2026-technology-expo-internet-mobile-adtech-martech-saas</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
+          <t>TECHSPO Johannesburg Technology Expo returns September 28-29, 2026 to the NH Johannesburg Sandton Hotel in Johannesburg, South Africa. This must-attend, two-day ...</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1612,24 +1600,24 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>customerservices@knect365.com, dataprivacy@knect365.com, support@informaconnect.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, support@knect365.com, dataprivacy@informaconnect.com</t>
+          <t>support@industryevents.com, colleague@company.com, events@techspojoburg.co.za, your@email.com, you@company.com</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Discover Tech Conferences Events &amp; Activities in South Africa | Eventbrite</t>
+          <t>Top Startup Events in Africa for 2026 - StartupBlink Blog</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
+          <t>https://www.startupblink.com/blog/top-startup-events-in-africa/</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Save this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South AfricaShare this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South Africa</t>
+          <t>Aug 19, 2026 · Discover top startup events in Africa for 2026, including major conferences, investor summits, fintech events, and AI and deep-tech ...</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1642,17 +1630,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 – Africa's biggest IT Conference and Expo</t>
+          <t>Discover Tech Conferences Events &amp; Activities in South Africa</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>The inaugural 2025 IT Indaba promises to bring together 3,000+ IT professionals and tech influencers who are involved in the procurement of systems, tools, platforms and services, along with user experience developers who deal with the core processes and client interfaces of the business.</t>
+          <t>Tech conferences Events and Things to do in South Africa ; WomenHack - Cape Town - Employer Ticket - September 9, 2026. Wed, Sep 9 • 6:00 PM. Bo-Kaap · Cape Town.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1665,17 +1653,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in Johannesburg, List of all Johannesburg Technology Business Expo &amp; Events in South Africa</t>
+          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th ...</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://10times.com/johannesburg-za/technology</t>
+          <t>https://africatechnologyexpo.com/</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience.</t>
+          <t>The Africa Technology Expo (ATE) is a first-of-its-kind, multi-year enterprise gathering at the intersection of Africa's potential and global opportunity. Built ...</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1683,22 +1671,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>info@sparkafrica.co, johndoe@email.com, partner@africatechnologyexpo.com</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Maker culture - Wikipedia</t>
+          <t>Maker Faire - Wikipedia</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Maker_culture</t>
+          <t>https://en.wikipedia.org/wiki/Maker_Faire</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Maker culture encourages novel applications of technologies, and the exploration of intersections between traditionally separate domains and ways of working including metalworking, calligraphy, filmmaking, and computer programming.</t>
+          <t>Maker Faire is a convention of do it yourself (DIY) enthusiasts established by Make magazine in 2006. Participants come from a wide variety of interests, ...</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1711,17 +1703,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>MakerWorld: Download Free 3D Models</t>
+          <t>Maker Faire Africa - Wikipedia</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://makerworld.com/</t>
+          <t>https://en.wikipedia.org/wiki/Maker_Faire_Africa</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Leading 3D printing model community for designers and makers. Download thousands of 3D models and stl models for free, and your No.1 option for multicolor 3D models.</t>
+          <t>The aim of a Maker Faire Africa is to create a space on the African continent where Afrigadget-type innovations, inventions and initiatives can be sought, identified, brought to life, supported, amplified and propagated.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1734,17 +1726,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MAKER Definition &amp; Meaning - Merriam-Webster</t>
+          <t>Maker Faire Africa - Facebook</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://www.merriam-webster.com/dictionary/maker</t>
+          <t>https://www.facebook.com/MFAJoburg/</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>4 days ago · The meaning of MAKER is one that makes. How to use maker in a sentence.</t>
+          <t>Jul 24, 2020 · Pizza, beer &amp; wine will be served during the film and a brief Q&amp;A about the Maker Movement will take place directly after the film, for anyone who wishes to participate.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1752,26 +1744,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>325506e3332d487999567a7bc91d151d@bug-reporting-xalgha6.m-w.com, icon_FB_active@2x.png, 485x364@2x.jpg, poetry-3533-c1127e17993b9df02a3cd810ffa02f2a@2x.jpg, alt-68472e2f61868-12424-2bd56b87b38dfc9715277f54861cc33b@2x.jpg, icon_heart_default@2x.png, old%20words%20for%20stupid%20muttonhead-6190-50dfd94054d4595c843d6b1a81fc9196@2x.jpg, alt-68362132d8a91-12386-1aa35da5ca39141e6146bf929773f6a9@1x.jpg, sticky-social-icons-sprite@2x.png, icon.pron@2x.png, 485x364@1x.jpg, dog-running-with-ball-6949-8f7cb15ae040661a7f354b16b0ffd663@2x.jpg, poetry-3533-c1127e17993b9df02a3cd810ffa02f2a@1x.jpg, icon_heart_active@2x.png, skateboard-dog-hat-13601-75a1345ca35ed9e5634be2453f9f21a9@2x.jpg, alt-68362132d8a91-12386-1aa35da5ca39141e6146bf929773f6a9@2x.jpg, uncommon%20phobia%20doraphobia-1072-c1849a46b563601d175e5564be040cb9@1x.jpg, alt-657775b8b94e6-11003-656ebc9b8ac9f59662e8742aabd756b9@1x.jpg, icon_cite_default@2x.png, old%20words%20for%20stupid%20muttonhead-6190-50dfd94054d4595c843d6b1a81fc9196@1x.jpg, skateboard-dog-hat-13601-75a1345ca35ed9e5634be2453f9f21a9@1x.jpg, carrot@2x.png, man%20sitting%20in%20a%20chair%20looking%20confused-9966-606d9b0c372ee2138e77733a68b16b24@1x.jpg, icon.pron.hover@2x.png, alt-69987e038fe3e-13165-a718b91a08bcb238b5957488228d2428@2x.jpg, icon_cite_active@2x.png, alt-663a3d0c0f0fc-11473-5f855bd7e243e60d2c1bcf6ef08a4145@1x.jpg, alt-657775b8b94e6-11003-656ebc9b8ac9f59662e8742aabd756b9@2x.jpg, to%20whom%20it%20may%20concern%20typed%20on%20a%20typewriter-9898-33d8deaf608b55f91b0fde92abddf080@1x.jpg, uncommon%20phobia%20doraphobia-1072-c1849a46b563601d175e5564be040cb9@2x.jpg, mw-logo-245x245@1x.png, alt-69987e038fe3e-13165-a718b91a08bcb238b5957488228d2428@1x.jpg, to%20whom%20it%20may%20concern%20typed%20on%20a%20typewriter-9898-33d8deaf608b55f91b0fde92abddf080@2x.jpg, icon_FB_default@2x.png, alt-68472e2f61868-12424-2bd56b87b38dfc9715277f54861cc33b@1x.jpg, man%20sitting%20in%20a%20chair%20looking%20confused-9966-606d9b0c372ee2138e77733a68b16b24@2x.jpg, dog-running-with-ball-6949-8f7cb15ae040661a7f354b16b0ffd663@1x.jpg, alt-663a3d0c0f0fc-11473-5f855bd7e243e60d2c1bcf6ef08a4145@2x.jpg, WOTDpodcastlogo343W@2x.jpg</t>
-        </is>
-      </c>
+      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>MakerLab</t>
+          <t>Maker Faire |</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://makerworld.com/en/makerlab</t>
+          <t>https://makerfaire.com/</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>No modeling skills required, no complex steps — with MakerLab, craft one-of-a-kind models with fun and ease. Create stunningly detailed 3D models from a single image with Tripo 3.1 Ultra. Create more detailed, lifelike busts with Make My Statue 2.0. From image to figurine, crafted in unique styles.</t>
+          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1779,22 +1767,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>fancybox_loading@2x.gif, fancybox_sprite@2x.png, chosen-sprite@2x.png, pr@make.co</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Chrome Music Lab - Song Maker</t>
+          <t>About | Maker Faire Cape Town: Make • Create • Craft</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://musiclab.chromeexperiments.com/Song-Maker</t>
+          <t>https://makerfairecapetown.wordpress.com/about/</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Song Maker, an experiment in Chrome Music Lab, is a simple way for anyone to make and share a song.</t>
+          <t>Maker Faire is a community-based learning event that inspires everyone to become a maker and connect to people and projects in their local community. Yet, Maker ...</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1807,17 +1799,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Make: Community – A Community for Makers</t>
+          <t>Maker Faire Cape Town 2015 - PlanetJune Blog</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://make.co/</t>
+          <t>https://www.planetjune.com/blog/maker-faire-cape-town-2015/</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Since 2005, we’ve been the heartbeat of the global maker movement, inspiring millions through Make: Magazine, Maker Faire, and a thriving community of DIY innovators, tinkerers, and inventors.</t>
+          <t>Aug 24, 2015 · Yesterday, I attended the first annual Maker Faire in Cape Town and it was inspiring – there was lots to see and explore.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1830,17 +1822,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Maker Pro | Electronics Projects and Tutorials</t>
+          <t>Why Africa needs Maker Faire | ZDNET</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://maker.pro/</t>
+          <t>https://www.zdnet.com/article/why-africa-needs-maker-faire/</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Aug 18, 2026 · We provide a place for makers like you to share your designs, collaborate with one another, and learn how to take your product to market.</t>
+          <t>Jul 23, 2014 · The organiser of Maker Faire Africa talks to ZDNet about why he wants to build a network of inventors.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1853,17 +1845,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Make: DIY Projects and Ideas for Makers |</t>
+          <t>Cape Town Mini Maker Faire (@ctminimakerfaire) - Instagram</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://makezine.com/</t>
+          <t>https://www.instagram.com/ctminimakerfaire/</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Make: celebrates your right to tweak, hack, and bend any technology to your will.</t>
+          <t>Cape Town Mini Maker Faire opens today at 14h00 at the Cape Town Science Centre in Observatory! Come and see the innovatie ideas South African #makers have been ...</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1871,26 +1863,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>pr@make.co</t>
-        </is>
-      </c>
+      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Makeronline: Download Free 3D Printing Models and Print Now</t>
+          <t>Maker Faire Africa Workshop at Afrofuture - Dezeen</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://makeronline.com/</t>
+          <t>https://www.dezeen.com/2013/05/22/maker-faire-africa-workshop-at-afrofuture/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Discover and download free 3D printing models and files, start printing amazing designs today. Click to get started!</t>
+          <t>May 22, 2013 · The workshop was a taster for the larger two to three day events that Maker Faire Africa put on in African cities for local makers to exhibit ...</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1903,17 +1891,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Cricut® | Smart Cutting Machines, Materials, Tools &amp; More</t>
+          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://cricut.com/</t>
+          <t>https://contemporaryand.com/en/events/maker-faire-africa-comes-to-johannesburg</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Design your idea, your way. Make it real with Cricut. Take our short quiz to discover which cutting machine is right for you. Our fits-in-any-space cutting machine for popular projects like full-color stickers, custom cards, T-shirts &amp; so much more.</t>
+          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will ...</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1926,17 +1914,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>How To Enter | Get Involved Today - Inspire Space Innovation — South ...</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.zasdc.org/compete</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>All these Olympiads and Competitions have a positive impact on education and on educational institutions in South Africa, but there is still a need to build stronger collaboration among teachers, schools, universities and educational authorities in order to meet the challenges of STEM education in South Africa today.</t>
+          <t>Join the South African Space Design Competition to inspire youth in STEM, showcase innovative space settlement concepts, and gain national and international exposure.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1944,22 +1932,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>user@domain.com, info@zasdc.org</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/za/solvefortomorrow/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
+          <t>All these Olympiads and Competitions have a positive impact on education and on educational institutions in South Africa, but there is still a need to build stronger collaboration among teachers, schools, universities and educational authorities in order to meet the challenges of STEM education in South Africa today.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1972,17 +1964,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>South African Space Design Competition | Inspire Space Innovation ...</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>Join the South African Space Design Competition to inspire space innovation, develop STEM skills, and compete for a trip to NASA. Perfect for high school students passionate about space.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1990,22 +1982,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>user@domain.com, info@zasdc.org</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Capetown 2026</t>
+          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
+          <t>https://www.samsung.com/za/solvefortomorrow/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the 'first author'. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
+          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2013,26 +2009,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Astemi Sa</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
+          <t>The IEOM High School/Middle School STEM Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2040,22 +2032,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2068,17 +2064,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Astemi Sa</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.astemi.co.za/</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>The IEOM High School/Middle School STEM Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects.</t>
+          <t>What is ASTEMI SA? The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible. We aim to increase participation in the activities of ASTEMI SA. We will encourage our members to lower the barriers of ...</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2086,26 +2082,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Competition - School Summit Africa</t>
+          <t>High School STEM Competition | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://schoolsummit.africa/competition/</t>
+          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>African Students Innovation Challenge The Inter-School STEM Innovations Challenge is a groundbreaking initiative aimed at nurturing creativity, critical thinking, and problem-solving skills among secondary school students through Science, Technology, Engineering, and Mathematics (STEM). This challenge is designed to foster real-world innovation by providing young learners with a platform to ...</t>
+          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2113,22 +2105,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Applications for 2026 Samsung Solve For Tomorrow Now Open!</t>
+          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://news.samsung.com/za/applications-for-2026-samsung-solve-for-tomorrow-now-open</t>
+          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries open until 06 March 2026. This is a transformative ...</t>
+          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2141,17 +2137,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Register your school for Samsung Solve for Tomorrow 2026</t>
+          <t>Top 20 Schools in Samsung Solve For Tomorrow Competition ...</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://www.sowetan.co.za/careers/2026-03-03-register-your-school-for-samsung-solve-for-tomorrow-2026/</t>
+          <t>https://www.facebook.com/100065237850533/posts/top-20-schools-in-samsung-solve-for-tomorrow-competition-2026is-your-region-repr/1336320708552512/</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Register your school for Samsung Solve for Tomorrow 2026 STEM competition aims to transform and empower South African learners with critical skills to solve real-world challenges March 03, 2026 at 7:44 am</t>
+          <t>Apr 22, 2026 · The competition is designed to promote Science, Technology, Engineering, and Math (STEM) education among high school learners, with a focus to ...</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2159,26 +2155,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>ssasft@samsung.com</t>
-        </is>
-      </c>
+      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa</t>
+          <t>Robotics Competition | WRO South Africa | Gauteng</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa/</t>
+          <t>https://www.wrosa.co.za/</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>This global competition is open to any individual or team willing to design, build, and code a robot to address the proposed challenge of disaster response in ...</t>
+          <t>WRO South Africa ( World Robot Olympiad ) is a robotics competition which brings together young people from all over the world to develop their creativity and problem-solving skills.</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2188,24 +2180,24 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>name@example.com</t>
+          <t>8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge - The Cortex Hub</t>
+          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge national competition will be held in Johannesburg, South Africa, at the Sandton Convention Centre on the 31st October 2025 ...</t>
+          <t>April 14, 2026 - This National Event, to be held at the Sandton Convention Centre in Johannesburg, South Africa, as part of AI for Good Impact Africa, at AI Expo Africa 2025, is a qualifying tournament leading to the Grand Finale in Geneva during the AI for ...</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2215,24 +2207,24 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, info@thecortexhub.africa, 8c4075d5481d476e945486754f783364@sentry.io, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
+          <t>name@example.com</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa</t>
+          <t>FIRST South Africa – Robotics Programs for School Children</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
+          <t>https://firstsa.org/</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge is the leading UN-based global robotics championship, inviting students aged 10 to 18 to develop AI and robotics-based ...</t>
+          <t>From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way. FIRST Tech Challenge students learn to think like engineers. Teams ...</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2240,26 +2232,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>name@example.com</t>
-        </is>
-      </c>
+      <c r="E74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Oakhill teams celebrate robotics success - Knysna-Plett Herald</t>
+          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://www.knysnaplettherald.com/News/Article/Local-News/oakhill-teams-celebrate-robotics-success-202608271131</t>
+          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>7 hours ago · The WRO is an international robotics competition in which learners design, build and programme autonomous robots to tackle technical challenges.</t>
+          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2272,17 +2260,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa - Limpopo</t>
+          <t>South African Robotics Competitions and Schools</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-limpopo/</t>
+          <t>https://www.sciencexpo.org.za/robotics.html</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>This global competition is open to any individual or team willing to design, build, and program a robot to address the proposed food security challenge on the ...</t>
+          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2292,24 +2280,24 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>name@example.com</t>
+          <t>madelien@imbewu.foundation, marna.vanzyl@imbewu.foundation, webmaster@sciencexpo.org.za</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>There is still hope : r/southafrica - Reddit</t>
+          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/southafrica/comments/1889qd2/there_is_still_hope/</t>
+          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Dec 1, 2023 · That's besides the robotics tournament we watched where the kids used Lego robotics sets to complete a programmed obstacle course. Just ...</t>
+          <t>The Robotics for Good Youth Challenge national competition will be held in Johannesburg, South Africa, at the Sandton Convention Centre on the 31st October 2025.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2317,22 +2305,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, info@thecortexhub.africa, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>FIRST Global Challenge</t>
+          <t>Limpopo Learners Represent South Africa at Global Robotics Finals in Switzerland - African Times</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://first.global/fgc/</t>
+          <t>https://www.atnews.co.za/limpopo-learners-represent-south-africa-at-global-robotics-finals-in-switzerland/</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>The FIRST Global Challenge is an olympics-style, international robotics competition that takes place in a different country each year. ... South Africa ...</t>
+          <t>July 7, 2026 - The international competition, taking place from 7 to 10 July 2026 at the Palexpo International Exhibition and Convention Centre in Geneva, brings together some of the world’s brightest young innovators to develop technological solutions to ...</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2340,22 +2332,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>NkosiN@atnews.co.za, rampedim@atnews.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Home | Roboticon 2026</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - AfrikaBot</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://roboticon.resolute.education/</t>
+          <t>https://www.saiee.org.za/displaycustomlink.aspx?name=AfrikaBot</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Resolute Roboticon is a platform for schools to showcase their robotics and coding skills by competing in a fun, exciting competition.</t>
+          <t>AfrikaBot is affordable because you can build a competitive robot for a lot less with the correct advice. AfrikaBOT is South Africa's first robotics competition for high school teenagers and university undergraduates who are smart enough to build their own robots from electronic parts rather ...</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2368,17 +2364,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Future robot rockstars of the Karoo! Winners of the 2026 World ...</t>
+          <t>WorldSkillsZA Mobile Robotics Provincial Competition 2024</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/SKASOUTHAFRICA/posts/future-robot-rockstars-of-the-karoo-winners-of-the-2026-world-robot-olympiad-pro/1677140377749131/</t>
+          <t>https://worldskillsza.dhet.gov.za/site/WSZA-Prov-Comp/Provincial-Competitions.aspx</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Aug 17, 2026 · Winners of the 2026 World Robot Olympiad Provincial Competition at Carnarvon High School, Northern Cape — hosted with pride by NRF-SARAO. These ...</t>
+          <t>The WorldSkills South Africa (WSZA) will be having its Mobile Robotics Combined Provincial Competitions in Lephalale TVET College from the 07th - 10th October 2023. the first 3 days will be focused on training and the last day will be the actual Mobile Robotics competition.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2391,17 +2387,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Wrapping up an incredible afternoon here at Carnarvon High ...</t>
+          <t>South African Schools attend SITA Robotics Challenge</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/SKASOUTHAFRICA/videos/wrapping-up-an-incredible-afternoon-here-at-carnarvon-high-school-for-the-2026-w/1529989865024526/</t>
+          <t>https://www.education.gov.za/ArchivedDocuments/ArchivedArticles/SITARoboticsChallenge.aspx</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Aug 15, 2026 · Mentors from Team South Africa discuss the impact of the FIRST Global robotics competition on youth development. They explain their ...</t>
+          <t>The 2024 SITA (State Information Technology Agency) Robotics Challenge took place in Summerstrand, Gqeberha at the Radisson Blu Hotel and Southern Sun Marine Hotel from 25 – 26 September 2024.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2409,22 +2405,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>callcentre@dbe.gov.za, certification@dbe.gov.za</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
+          <t>2026 South Africa Engineering Competition</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini-2022-09-13</t>
+          <t>https://notices.ukzn.ac.za/content/GetFile.aspx?id=96047</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng. Twelve schools participated in the grand finale, which saw great, ...</t>
+          <t>UKZN and Elsevier. If you are an engineering student (undergraduate or postgraduate), don't miss joining the challenge to solve real-world cases using Engineering Village and Knovel.</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2432,26 +2432,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>advertising@creamermedia.co.za, chanel@engineeringnews.co.za, subscriptions@creamermedia.co.za, newsletters@creamermedia.co.za, newsdesk@engineeringnews.co.za</t>
-        </is>
-      </c>
+      <c r="E82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Engineering the Future: 16 schools compete in SAICE’s 33rd International Bridge Building Competition - SAICE</t>
+          <t>Competition Ts and Cs - SAICE</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://saice.org.za/press-releases/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
+          <t>https://saice.org.za/competition-ts-and-cs/</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>April 17, 2025 - The South African Institution of Civil Engineering (SAICE) hosted its 33rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
+          <t>Preamble These Terms and Conditions govern participation in the Know Your Sector Competition ("the Competition") conducted by the South African Institute of Civil Engineering ("SAICE"). Definitions SAICE: Shall mean the South African Institute of Civil Engineering. The Competition: Shall mean SAICE's Know Your Sector Competition. Entrant: Shall mean any individual who enters the ...</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2461,24 +2457,24 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>membership@saice.org.za, communications@saice.org.za, marketing@saice.org.za, accounts@saice.org.za, civilinfo@saice.org.za</t>
+          <t>communications@saice.org.za, marketing@saice.org.za, civilinfo@saice.org.za, membership@saice.org.za, accounts@saice.org.za</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Upcoming Civil Engineering Conferences in South Africa 2025-2026</t>
+          <t>Civil Engineering Conferences in South Africa 2026/2027/2028</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://conferencealerts.co.in/south-africa/civil-engineering</t>
+          <t>https://conferenceindex.org/conferences/civil-engineering/south-africa</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>International Civil engineering conferences in South africa 2025-2026 with invitation letter. A great opportunity to meet and learn from experts in your field.</t>
+          <t>Civil Engineering Conferences in South Africa 2026 2027 2028 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and symposiums.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2491,17 +2487,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
+          <t>Engineering the future: 16 schools compete in SAICE's 33rd ...</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://www.crown.co.za/construction-world/marketplace/22289-saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini</t>
+          <t>https://www.southafricanbusiness.co.za/08/2024/construction-and-engineering/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) hosted its 33rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2509,26 +2505,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>ernao@crown.co.za, constr@crown.co.za</t>
-        </is>
-      </c>
+      <c r="E85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Upcoming Civil Engineering Conferences in South Africa 2025</t>
+          <t>Civil Expo ITs 2026</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://www.allconferencealert.com/south-africa/civil-engineering-conference.html</t>
+          <t>https://civilexpoits2026.com/</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>September 7, 2025 - Find the list of upcoming Civil Engineering conferences in South Africa 2025 with invitation an letter.</t>
+          <t>Hi Cipo Pals! Civil Expo ITs 2026 Sovereign Structures, Resilient Societies This national civil engineering competition is your chance to put your engineering precision to the test and build real-world structural solutions. Step up and prove your skills on a national stage!</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2536,22 +2528,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>civilexpo.sipilits@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>SWM Communications | SAICE recognises civil engineering research excellence through national student competition</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://swmcommunications.co.za/press-office/saice-recognises-civil-engineering-research-excellence-through-national-student-competition/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>April 1, 2026 - The event – which was sponsored by Sika, WorldsView, BVI, RIBCCS, and AF Consulting – was hosted at SAICE House in Midrand, Gauteng, and accredited for 0.2 CPD points. Students were invited to present their civil engineering university research and investigation project, which is part of the national curriculum for final year civil engineering undergraduate students.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2561,24 +2557,24 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>info@swmcommunications.co.za, nthabeleng@saice.org.za</t>
+          <t>info@ieomsociety.org</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ICE Africa – Supporting Civil Engineers in Africa | Institution of Civil Engineers (ICE)</t>
+          <t>SAICE's 34th International bridge competition inspires tomorrow's engineers</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://www.ice.org.uk/about-us/what-we-do/ice-near-you/international/ice-africa/</t>
+          <t>https://www.crown.co.za/africa-updates/33867-saice-s-34th-international-bridge-competition-inspires-tomorrow-s-engineers</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>March 19, 2026 - organise seminars, workshops, visits and inter-universities competitions regarding civil engineering projects · For more information or to get involved please contact [email protected]. We have a volunteer member in South Africa who helps arrange ICE activities and promote our work.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) hosted its 34th International Bridge Building Competition at the Midrand Conference Centre, bringing together 21 teams of high school learners from across South Africa, alongside international participants from Eswatini, Uganda, and Zimbabwe.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2591,17 +2587,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Upcoming Civil engineering Conferences in Cape town 2025</t>
+          <t>The South African Institution of Civil Engineering (SAICE)</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://conferencealerts.co.in/cape-town/civil-engineering</t>
+          <t>https://www.facebook.com/SAICECIVIL/posts/enter-for-the-2026-saice-national-awardsnominations-are-open-and-were-looking-fo/1419225983581060/</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Civil engineering conferences in Cape town 2025 provide an exclusive global platform to meet and engage with experts and aspirants in various fields.</t>
+          <t>Enter for the 2026 SAICE National Awards! Nominations are open, and we're looking for the projects that truly made a difference where it matters most. The Community-Based Project of the Year is...</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2614,17 +2610,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
+          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2205</t>
+          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
+          <t>19 June 2026 marked an exciting celebration of Youth Month as aspiring young engineers from across Gauteng gathered for the 2026 SAICE Johannesburg Branch Schools Bridge Building Competition. Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in ...</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2637,17 +2633,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Civil Engineering Conferences in South Africa 2025/2026/2027 - Conference Index</t>
+          <t>Home - SAICE</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://conferenceindex.org/conferences/civil-engineering/south-africa</t>
+          <t>https://saice.org.za/</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Apr 13 International Conference on Architectural, Civil and Environmental Engineering (ICACEE) - Cape Town, South Africa</t>
+          <t>The South African Institution of Civil Engineering (SAICE) is the industry body for civil engineering professionals in South Africa. Our aim is to, promote growth, excellence and sustainability in the industry.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2655,22 +2651,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>executiveadmin@saice.org.za, communications@saice.org.za, marketing@saice.org.za, barbara@avenue.co.za, civilinfo@saice.org.za, membership@saice.org.za, accounts@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026 South Africa Engineering Competition</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://notices.ukzn.ac.za/content/GetFile.aspx?id=96047</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>UKZN and Elsevier. If you are an engineering student (undergraduate or postgraduate), don't miss joining the challenge to solve real-world cases using Engineering Village and Knovel.</t>
+          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2683,17 +2683,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>Engineering Competition For African Youth In Engineering ...</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+          <t>Aug 18, 2025 · This call invites engineers and innovators from across sub-Saharan Africa to apply with scalable innovations that address pressing social and environmental challenges.</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2706,7 +2706,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2716,7 +2716,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2729,17 +2729,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
+          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2747,22 +2747,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions.</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2770,26 +2774,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2806,17 +2806,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Mechanical Engineering Apprenticeship Jobs in South Africa ... - LinkedIn</t>
+          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://za.linkedin.com/jobs/mechanical-engineering-apprenticeship-jobs</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2210</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Today's top 190 Mechanical Engineering Apprenticeship jobs in South Africa. Leverage your professional network, and get hired. New Mechanical Engineering Apprenticeship jobs added daily.</t>
+          <t>&gt;&gt; Industrial and Manufacturing Engineering · &gt;&gt; Mechanical Engineering · &gt;&gt; Ocean Engineering · Environmental Science · Mathematics · Medicine · &gt;&gt; Anatomy · &gt;&gt; Anesthesiology and Pain Medicine · &gt;&gt; Cardiology and Cardiovascular Medicine · &gt;&gt; Critical Care and Intensive Care Medicine ·</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2829,17 +2829,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Competitions South Africa - Live Giveaways &amp; Prize Draws | Freehub</t>
+          <t>Best Mechanical Engineering Companies in South Africa</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://freehub.co.za/competitions/</t>
+          <t>https://engineeringness.com/best-mechanical-engineering-companies-in-south-africa/</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Browse live South African competitions, giveaways and prize draws. Find car, cash, voucher, tech and holiday competitions with clear entry rules and official source links.</t>
+          <t>October 4, 2025 - This article showcases our top picks for the best South Africa based Mechanical Engineering companies. These startups and companies are taking a variety of approaches to innovating the Mechanical Engineering industry, but are all exceptional companies well worth a follow.</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2852,17 +2852,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>PDF Apply Now! Worldskills South Africa National Competition 2025</t>
+          <t>Mechanical Engineering Conferences in South Africa 2026/2027/2028 - Conference Index</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
+          <t>https://conferenceindex.org/conferences/mechanical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
+          <t>Nov 04 International Conference on Tribology and Interface Engineering (ICTIE) - Cape Town, South Africa · Nov 04 International Conference on Mechanical and Systems Engineering (ICMSE) - Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2875,17 +2875,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>SAIMechE</t>
+          <t>Mechanical Engineering events - South Africa Group - Institution of Mechanical Engineers</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>https://www.saimeche.org.za/</t>
+          <t>https://nearyou.imeche.org/near-you/middle-east-and-africa/south-africa/events</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
+          <t>For details of Mechanical Engineering events organised by South Africa Group, please click the above link.</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2898,17 +2898,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
+          <t>2026 South Africa Engineering Competition</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
+          <t>https://notices.ukzn.ac.za/content/GetFile.aspx?id=96047</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
+          <t>UKZN and Elsevier. If you are an engineering student (undergraduate or postgraduate), don't miss joining the challenge to solve real-world cases using Engineering Village and Knovel.</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2921,17 +2921,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - SAIEE National Student Project Competition</t>
+          <t>Competitions | ESG</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/calendar/EventDetails.aspx?eeid=29281</t>
+          <t>https://za.rs-online.com/web/content/m/competition</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>The SAIEE National Students Project Competition will be held at the North-West University (Potchefstroom Campus) on 21 November 2019</t>
+          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2939,22 +2939,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>example@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - IEEE ZA 5G Competition</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51397</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Form templates: Template for a Cover Sheet for the Competition on Ideas, Designs and Applications for 5G and Beyond South Africa (.docx) [Click to Download] Template for a Resume for the Student (.docx) [Click to Download] ... Help (FAQ) • Privacy Statement • Terms &amp; Conditions The SAIEE is ...</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2967,17 +2971,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Student Design Competition | IEEE CASS</t>
+          <t>Electrical Engineering Conferences in South Africa 2026/2027/2028</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://ieee-cas.org/society-involvement/student-design-competition</t>
+          <t>https://conferenceindex.org/conferences/electrical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>CASS will reimburse the travel costs for the trip to ISCAS 2026 for the four finalists, one for each region - Regions 1-7 (USA and Canada), Region 8 (Europe, Middle East, Africa), Region 9 (Latin America), and Region 10 (Asia, Australia, Pacific), as well as ISCAS registration.</t>
+          <t>Electrical Engineering Conferences in South Africa 2026 2027 2028 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and symposiums.</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2990,17 +2994,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Top 100 Electrical Engineering Companies in South Africa (2026) | ensun</t>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa)</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://ensun.io/search/electrical-engineering/south-africa</t>
+          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>The competitive landscape is marked by both established firms and emerging startups, driving innovation and efficiency. Additionally, South Africa’s position in the broader global market allows for potential collaborations and export opportunities, particularly in green technologies. Understanding these factors is essential for anyone looking to engage with the Electrical Engineering sector in South Africa, as they influence the overall business environment and potential for growth.</t>
+          <t>IEEE-IAS Industrial Power Conversion Systems Department Serving the electrical energy conversion professional worldwide</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -3013,17 +3017,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>March 12, 2026 - At the Centre for High Performance Computing (CHPC) Conference hosted in Cape Town at the end of last year, four current fourth-year electrical engineering students were crowned national champions in the Student Cluster Competition for 2025.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3031,22 +3035,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - SA Computing Olympiad stars hold their own in international competition</t>
+          <t>Engineering students compete in global high-performance computing ...</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51457</t>
+          <t>https://ebe.uct.ac.za/articles/2026-05-29-engineering-students-compete-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>July 20, 2021 - For the other three South African team members, this was their first IOI. Brent Butkow finished ranked 342, Jean Weight finished in 287th position and Faran Steenkamp was ranked 280. In addition to the serious IOI contest days, host country Singapore arranged several fun events where Faran Steenkamp was placed third in the sponsored Code Cup, and won a cash prize of 200 USD.</t>
+          <t>At the Centre for High Performance Computing (CHPC) Conference hosted in Cape Town at the end of last year, four current fourth-year electrical engineering students were crowned national champions in the Student Cluster Competition for 2025. Now, Team UCT is preparing to represent South Africa at the global finals in Germany later this year.</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3054,22 +3062,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>ebe-faculty@uct.ac.za</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Electrical Engineering Conferences in South Africa 2025/2026/2027 - Conference Index</t>
+          <t>Eskom Bursary Programme South Africa 2026 - EduFunds SA</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>https://conferenceindex.org/conferences/electrical-engineering/south-africa</t>
+          <t>https://www.edufunds.co.za/eskom-bursary-programme-south-africa-2026/</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Electrical Engineering Conferences in South Africa 2025 2026 2027 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and ...</t>
+          <t>Apply for the Eskom Bursary Programme South Africa 2026. Funding for BEng/BSc engineering students in Chemical, Civil, Electrical, Mechanical, Industrial, and Metallurgy disciplines. Apply by 14 November 2025.</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3077,22 +3089,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Admin@edufunds.co.za, candidate.support@ci.hr</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>7 Electrical Engineering Degree Programs in South Africa - Study Abroad | educations.com</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>https://www.educations.com/electrical-engineering/south-africa</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Find the best fit for you - Compare 7 in Engineering Programs Electrical Engineering in South Africa for 2025/2026</t>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3105,17 +3121,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Electrical Engineering in South Africa: Best universities Ranked</t>
+          <t>Zutari Bursary Programme 2027 Opens Applications for Civil and ...</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://edurank.org/engineering/electrical/za/</t>
+          <t>https://www.globalsouthopportunities.com/2026/08/10/zutari/</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>March 2, 2025 - Below is the list of 24 best universities for Electrical Engineering in South Africa ranked based on their research performance: a graph of 827K citations received by 40.9K academic papers made by these universities was used to calculate ratings and create the top.</t>
+          <t>Zutari has opened applications for its 2027 Engineering Bursary Programme, offe